<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Thu 09/17/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2658" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2659" uniqueCount="324">
   <si>
     <t>Sudeep</t>
   </si>
@@ -5779,9 +5779,10 @@
     <col min="18" max="18" width="13.42578125" style="133" customWidth="1" collapsed="1"/>
     <col min="19" max="19" width="13.42578125" style="133" customWidth="1"/>
     <col min="20" max="20" width="11.28515625" style="133" customWidth="1"/>
-    <col min="21" max="21" width="10.42578125" style="133" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="22" width="10.7109375" style="133" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="28" width="9.140625" style="133"/>
+    <col min="21" max="21" width="10.42578125" style="133" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="10.7109375" style="133" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="23" width="9.140625" style="133" collapsed="1"/>
+    <col min="24" max="28" width="9.140625" style="133"/>
     <col min="29" max="29" width="14.140625" style="133" customWidth="1"/>
     <col min="30" max="30" width="12" style="133" customWidth="1"/>
     <col min="31" max="31" width="15.85546875" style="133" customWidth="1"/>
@@ -5824,7 +5825,9 @@
       <c r="R2" s="256">
         <v>46281</v>
       </c>
-      <c r="S2" s="256"/>
+      <c r="S2" s="256">
+        <v>46282</v>
+      </c>
       <c r="T2" s="183"/>
       <c r="U2" s="184" t="s">
         <v>281</v>
@@ -5886,7 +5889,9 @@
       <c r="R3" s="179" t="s">
         <v>237</v>
       </c>
-      <c r="S3" s="179"/>
+      <c r="S3" s="179" t="s">
+        <v>236</v>
+      </c>
       <c r="T3" s="180"/>
       <c r="U3" s="189"/>
       <c r="V3" s="180"/>
@@ -5950,15 +5955,17 @@
       <c r="R4" s="158">
         <v>-149</v>
       </c>
-      <c r="S4" s="158"/>
+      <c r="S4" s="158">
+        <v>-21850</v>
+      </c>
       <c r="T4" s="211"/>
       <c r="U4" s="171">
         <f t="shared" ref="U4:U30" si="0">SUM(H4:T4)</f>
-        <v>-40798</v>
+        <v>-62648</v>
       </c>
       <c r="V4" s="149">
         <f t="shared" ref="V4:V30" si="1">IFERROR(U4/F4*100,0)/10000000</f>
-        <v>-0.81596000000000002</v>
+        <v>-1.2529600000000001</v>
       </c>
       <c r="AC4" s="133" t="s">
         <v>170</v>
@@ -6020,15 +6027,17 @@
       <c r="R5" s="147">
         <v>81831</v>
       </c>
-      <c r="S5" s="147"/>
+      <c r="S5" s="147">
+        <v>-92500</v>
+      </c>
       <c r="T5" s="174"/>
       <c r="U5" s="171">
         <f t="shared" si="0"/>
-        <v>168284</v>
+        <v>75784</v>
       </c>
       <c r="V5" s="149">
         <f t="shared" si="1"/>
-        <v>0.56094666666666659</v>
+        <v>0.2526133333333333</v>
       </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
@@ -6084,7 +6093,9 @@
       <c r="R6" s="147">
         <v>0</v>
       </c>
-      <c r="S6" s="147"/>
+      <c r="S6" s="147">
+        <v>0</v>
+      </c>
       <c r="T6" s="174"/>
       <c r="U6" s="171">
         <f t="shared" si="0"/>
@@ -6148,15 +6159,17 @@
       <c r="R7" s="147">
         <v>23300</v>
       </c>
-      <c r="S7" s="147"/>
+      <c r="S7" s="147">
+        <v>-85900</v>
+      </c>
       <c r="T7" s="174"/>
       <c r="U7" s="171">
         <f t="shared" si="0"/>
-        <v>105547</v>
+        <v>19647</v>
       </c>
       <c r="V7" s="149">
         <f t="shared" si="1"/>
-        <v>1.0554699999999999</v>
+        <v>0.19647000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6212,19 +6225,21 @@
       <c r="R8" s="147">
         <v>-30125</v>
       </c>
-      <c r="S8" s="147"/>
+      <c r="S8" s="147">
+        <v>-78630</v>
+      </c>
       <c r="T8" s="174"/>
       <c r="U8" s="171">
         <f t="shared" si="0"/>
-        <v>34234</v>
+        <v>-44396</v>
       </c>
       <c r="V8" s="149">
         <f t="shared" si="1"/>
-        <v>0.11411333333333334</v>
+        <v>-0.14798666666666666</v>
       </c>
       <c r="X8" s="5"/>
       <c r="Y8" s="134">
-        <v>13</v>
+        <v>-11170</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
@@ -6280,18 +6295,20 @@
       <c r="R9" s="147">
         <v>-63430</v>
       </c>
-      <c r="S9" s="147"/>
+      <c r="S9" s="147">
+        <v>-31200</v>
+      </c>
       <c r="T9" s="174"/>
       <c r="U9" s="171">
         <f t="shared" si="0"/>
-        <v>49903</v>
+        <v>18703</v>
       </c>
       <c r="V9" s="149">
         <f t="shared" si="1"/>
-        <v>0.33268666666666663</v>
+        <v>0.12468666666666665</v>
       </c>
       <c r="X9" s="134">
-        <v>32574</v>
+        <v>97890</v>
       </c>
       <c r="Y9" s="134"/>
     </row>
@@ -6346,22 +6363,24 @@
       <c r="R10" s="147">
         <v>-31500</v>
       </c>
-      <c r="S10" s="147"/>
+      <c r="S10" s="147">
+        <v>-900</v>
+      </c>
       <c r="T10" s="174"/>
       <c r="U10" s="171">
         <f t="shared" si="0"/>
-        <v>9337</v>
+        <v>8437</v>
       </c>
       <c r="V10" s="149">
         <f t="shared" si="1"/>
-        <v>0.15561666666666668</v>
+        <v>0.14061666666666667</v>
       </c>
       <c r="X10" s="134">
-        <v>32587</v>
+        <v>86719</v>
       </c>
       <c r="Y10" s="134">
         <f>(X10+X9)/10000000*13780</f>
-        <v>89.791858000000005</v>
+        <v>254.39120199999999</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
@@ -6417,15 +6436,17 @@
       <c r="R11" s="147">
         <v>0</v>
       </c>
-      <c r="S11" s="147"/>
+      <c r="S11" s="147">
+        <v>4326</v>
+      </c>
       <c r="T11" s="174"/>
       <c r="U11" s="171">
         <f t="shared" si="0"/>
-        <v>-764248</v>
+        <v>-759922</v>
       </c>
       <c r="V11" s="149">
         <f t="shared" si="1"/>
-        <v>-0.50949866666666666</v>
+        <v>-0.50661466666666666</v>
       </c>
       <c r="X11" s="134"/>
       <c r="Y11" s="134"/>
@@ -6483,15 +6504,17 @@
       <c r="R12" s="147">
         <v>-100</v>
       </c>
-      <c r="S12" s="147"/>
+      <c r="S12" s="147">
+        <v>-35135</v>
+      </c>
       <c r="T12" s="174"/>
       <c r="U12" s="171">
         <f t="shared" si="0"/>
-        <v>25206</v>
+        <v>-9929</v>
       </c>
       <c r="V12" s="149">
         <f t="shared" si="1"/>
-        <v>4.2009999999999999E-2</v>
+        <v>-1.6548333333333332E-2</v>
       </c>
       <c r="X12" s="134"/>
       <c r="Y12" s="134"/>
@@ -6549,7 +6572,9 @@
       <c r="R13" s="147">
         <v>2399</v>
       </c>
-      <c r="S13" s="147"/>
+      <c r="S13" s="147">
+        <v>0</v>
+      </c>
       <c r="T13" s="174"/>
       <c r="U13" s="171">
         <f t="shared" si="0"/>
@@ -6615,15 +6640,17 @@
       <c r="R14" s="147">
         <v>-10140</v>
       </c>
-      <c r="S14" s="147"/>
+      <c r="S14" s="147">
+        <v>-16054</v>
+      </c>
       <c r="T14" s="174"/>
       <c r="U14" s="171">
         <f t="shared" si="0"/>
-        <v>3762</v>
+        <v>-12292</v>
       </c>
       <c r="V14" s="149">
         <f t="shared" si="1"/>
-        <v>1.5048000000000001E-2</v>
+        <v>-4.9168000000000003E-2</v>
       </c>
       <c r="X14" s="134"/>
       <c r="Y14" s="134"/>
@@ -6681,27 +6708,29 @@
       <c r="R15" s="147">
         <v>-6220</v>
       </c>
-      <c r="S15" s="147"/>
+      <c r="S15" s="147">
+        <v>-17616</v>
+      </c>
       <c r="T15" s="174"/>
       <c r="U15" s="171">
         <f t="shared" si="0"/>
-        <v>6980</v>
+        <v>-10636</v>
       </c>
       <c r="V15" s="149">
         <f t="shared" si="1"/>
-        <v>3.1727272727272722E-2</v>
+        <v>-4.8345454545454539E-2</v>
       </c>
       <c r="X15" s="134"/>
       <c r="Y15" s="193">
         <f>Y8-Y10</f>
-        <v>-76.791858000000005</v>
+        <v>-11424.391202000001</v>
       </c>
       <c r="AB15" s="133">
         <v>116185</v>
       </c>
       <c r="AD15" s="133">
         <f>AB15+Y15</f>
-        <v>116108.208142</v>
+        <v>104760.608798</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.25">
@@ -6757,15 +6786,17 @@
       <c r="R16" s="147">
         <v>5959</v>
       </c>
-      <c r="S16" s="147"/>
+      <c r="S16" s="147">
+        <v>7570</v>
+      </c>
       <c r="T16" s="174"/>
       <c r="U16" s="171">
         <f t="shared" si="0"/>
-        <v>-25908</v>
+        <v>-18338</v>
       </c>
       <c r="V16" s="149">
         <f t="shared" si="1"/>
-        <v>-0.25907999999999998</v>
+        <v>-0.18337999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.25">
@@ -6821,15 +6852,17 @@
       <c r="R17" s="147">
         <v>0</v>
       </c>
-      <c r="S17" s="147"/>
+      <c r="S17" s="147">
+        <v>-22321</v>
+      </c>
       <c r="T17" s="174"/>
       <c r="U17" s="171">
         <f t="shared" si="0"/>
-        <v>9579</v>
+        <v>-12742</v>
       </c>
       <c r="V17" s="149">
         <f t="shared" si="1"/>
-        <v>3.8316000000000003E-2</v>
+        <v>-5.0967999999999999E-2</v>
       </c>
       <c r="AD17" s="133">
         <v>4000000</v>
@@ -6896,15 +6929,17 @@
       <c r="R18" s="147">
         <v>0</v>
       </c>
-      <c r="S18" s="147"/>
+      <c r="S18" s="147">
+        <v>-38652</v>
+      </c>
       <c r="T18" s="174"/>
       <c r="U18" s="171">
         <f t="shared" si="0"/>
-        <v>13543</v>
+        <v>-25109</v>
       </c>
       <c r="V18" s="149">
         <f t="shared" si="1"/>
-        <v>3.3857499999999999E-2</v>
+        <v>-6.2772499999999995E-2</v>
       </c>
       <c r="AE18" s="133">
         <f>AE17/12</f>
@@ -6964,15 +6999,17 @@
       <c r="R19" s="147">
         <v>-73400</v>
       </c>
-      <c r="S19" s="147"/>
+      <c r="S19" s="147">
+        <v>-81145</v>
+      </c>
       <c r="T19" s="174"/>
       <c r="U19" s="171">
         <f t="shared" si="0"/>
-        <v>-200398</v>
+        <v>-281543</v>
       </c>
       <c r="V19" s="149">
         <f t="shared" si="1"/>
-        <v>-1.3359866666666667</v>
+        <v>-1.8769533333333335</v>
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
@@ -7028,7 +7065,9 @@
       <c r="R20" s="147">
         <v>-52025</v>
       </c>
-      <c r="S20" s="147"/>
+      <c r="S20" s="147">
+        <v>0</v>
+      </c>
       <c r="T20" s="174"/>
       <c r="U20" s="171">
         <f t="shared" si="0"/>
@@ -7095,15 +7134,17 @@
       <c r="R21" s="147">
         <v>580</v>
       </c>
-      <c r="S21" s="147"/>
+      <c r="S21" s="147">
+        <v>-13500</v>
+      </c>
       <c r="T21" s="174"/>
       <c r="U21" s="171">
         <f t="shared" si="0"/>
-        <v>-19503</v>
+        <v>-33003</v>
       </c>
       <c r="V21" s="149">
         <f t="shared" si="1"/>
-        <v>-0.78012000000000004</v>
+        <v>-1.32012</v>
       </c>
       <c r="Z21" s="133">
         <v>30400</v>
@@ -7162,7 +7203,9 @@
       <c r="R22" s="147">
         <v>0</v>
       </c>
-      <c r="S22" s="147"/>
+      <c r="S22" s="147">
+        <v>0</v>
+      </c>
       <c r="T22" s="174"/>
       <c r="U22" s="171">
         <f t="shared" si="0"/>
@@ -7229,7 +7272,9 @@
       <c r="R23" s="147">
         <v>0</v>
       </c>
-      <c r="S23" s="147"/>
+      <c r="S23" s="147">
+        <v>0</v>
+      </c>
       <c r="T23" s="174"/>
       <c r="U23" s="171">
         <f t="shared" si="0"/>
@@ -7293,15 +7338,17 @@
       <c r="R24" s="147">
         <v>-32214</v>
       </c>
-      <c r="S24" s="147"/>
+      <c r="S24" s="147">
+        <v>9741</v>
+      </c>
       <c r="T24" s="174"/>
       <c r="U24" s="171">
         <f t="shared" si="0"/>
-        <v>-11535</v>
+        <v>-1794</v>
       </c>
       <c r="V24" s="149">
         <f t="shared" si="1"/>
-        <v>-0.10486363636363635</v>
+        <v>-1.6309090909090908E-2</v>
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
@@ -7357,15 +7404,17 @@
       <c r="R25" s="147">
         <v>48600</v>
       </c>
-      <c r="S25" s="147"/>
+      <c r="S25" s="147">
+        <v>181200</v>
+      </c>
       <c r="T25" s="174"/>
       <c r="U25" s="171">
         <f t="shared" si="0"/>
-        <v>-1448523</v>
+        <v>-1267323</v>
       </c>
       <c r="V25" s="149">
         <f t="shared" si="1"/>
-        <v>-6.2979260869565215</v>
+        <v>-5.5101000000000004</v>
       </c>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
@@ -7419,15 +7468,17 @@
       <c r="R26" s="147">
         <v>1700</v>
       </c>
-      <c r="S26" s="147"/>
+      <c r="S26" s="147">
+        <v>1785</v>
+      </c>
       <c r="T26" s="174"/>
       <c r="U26" s="171">
         <f t="shared" si="0"/>
-        <v>5794</v>
+        <v>7579</v>
       </c>
       <c r="V26" s="149">
         <f t="shared" si="1"/>
-        <v>0.28970000000000001</v>
+        <v>0.37895000000000001</v>
       </c>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
@@ -7483,15 +7534,17 @@
       <c r="R27" s="147">
         <v>0</v>
       </c>
-      <c r="S27" s="147"/>
+      <c r="S27" s="147">
+        <v>-65000</v>
+      </c>
       <c r="T27" s="174"/>
       <c r="U27" s="171">
         <f t="shared" si="0"/>
-        <v>34666</v>
+        <v>-30334</v>
       </c>
       <c r="V27" s="149">
         <f t="shared" si="1"/>
-        <v>6.9332000000000005E-2</v>
+        <v>-6.0668E-2</v>
       </c>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
@@ -7547,15 +7600,17 @@
       <c r="R28" s="147">
         <v>-481200</v>
       </c>
-      <c r="S28" s="147"/>
+      <c r="S28" s="147">
+        <v>-443700</v>
+      </c>
       <c r="T28" s="174"/>
       <c r="U28" s="171">
         <f t="shared" si="0"/>
-        <v>-1231866</v>
+        <v>-1675566</v>
       </c>
       <c r="V28" s="149">
         <f t="shared" si="1"/>
-        <v>-1.2318659999999999</v>
+        <v>-1.6755660000000001</v>
       </c>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
@@ -7611,15 +7666,17 @@
       <c r="R29" s="147">
         <v>0</v>
       </c>
-      <c r="S29" s="147"/>
+      <c r="S29" s="147">
+        <v>-33000</v>
+      </c>
       <c r="T29" s="174"/>
       <c r="U29" s="171">
         <f t="shared" si="0"/>
-        <v>-341989</v>
+        <v>-374989</v>
       </c>
       <c r="V29" s="149">
         <f t="shared" si="1"/>
-        <v>-0.68397799999999997</v>
+        <v>-0.74997800000000003</v>
       </c>
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
@@ -7675,15 +7732,17 @@
       <c r="R30" s="147">
         <v>-100709</v>
       </c>
-      <c r="S30" s="147"/>
+      <c r="S30" s="147">
+        <v>-184894</v>
+      </c>
       <c r="T30" s="174"/>
       <c r="U30" s="171">
         <f t="shared" si="0"/>
-        <v>65134</v>
+        <v>-119760</v>
       </c>
       <c r="V30" s="149">
         <f t="shared" si="1"/>
-        <v>0.13026799999999999</v>
+        <v>-0.23952000000000001</v>
       </c>
     </row>
     <row r="31" spans="1:33" x14ac:dyDescent="0.25">
@@ -7739,15 +7798,17 @@
       <c r="R31" s="147">
         <v>-55712</v>
       </c>
-      <c r="S31" s="147"/>
+      <c r="S31" s="147">
+        <v>-11425</v>
+      </c>
       <c r="T31" s="174"/>
       <c r="U31" s="171">
         <f t="shared" ref="U31:U56" si="2">SUM(H31:T31)</f>
-        <v>-186096</v>
+        <v>-197521</v>
       </c>
       <c r="V31" s="149">
         <f t="shared" ref="V31:V56" si="3">IFERROR(U31/F31*100,0)/10000000</f>
-        <v>-3.7219199999999999</v>
+        <v>-3.9504199999999998</v>
       </c>
     </row>
     <row r="32" spans="1:33" x14ac:dyDescent="0.25">
@@ -7803,15 +7864,17 @@
       <c r="R32" s="147">
         <v>-24900</v>
       </c>
-      <c r="S32" s="147"/>
+      <c r="S32" s="147">
+        <v>-6308</v>
+      </c>
       <c r="T32" s="174"/>
       <c r="U32" s="171">
         <f t="shared" si="2"/>
-        <v>115289</v>
+        <v>108981</v>
       </c>
       <c r="V32" s="149">
         <f t="shared" si="3"/>
-        <v>2.882225</v>
+        <v>2.7245249999999999</v>
       </c>
       <c r="Y32" s="134"/>
     </row>
@@ -7868,7 +7931,9 @@
       <c r="R33" s="147">
         <v>0</v>
       </c>
-      <c r="S33" s="147"/>
+      <c r="S33" s="147">
+        <v>0</v>
+      </c>
       <c r="T33" s="174"/>
       <c r="U33" s="171">
         <f t="shared" si="2"/>
@@ -7880,7 +7945,7 @@
       </c>
       <c r="X33" s="5"/>
       <c r="Y33" s="134">
-        <v>-97634</v>
+        <v>-23327</v>
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
@@ -7936,7 +8001,9 @@
       <c r="R34" s="147">
         <v>0</v>
       </c>
-      <c r="S34" s="147"/>
+      <c r="S34" s="147">
+        <v>0</v>
+      </c>
       <c r="T34" s="174"/>
       <c r="U34" s="171">
         <f t="shared" si="2"/>
@@ -8002,22 +8069,24 @@
       <c r="R35" s="147">
         <v>-14983</v>
       </c>
-      <c r="S35" s="147"/>
+      <c r="S35" s="147">
+        <v>-31590</v>
+      </c>
       <c r="T35" s="174"/>
       <c r="U35" s="171">
         <f t="shared" si="2"/>
-        <v>-131563</v>
+        <v>-163153</v>
       </c>
       <c r="V35" s="149">
         <f t="shared" si="3"/>
-        <v>-0.32890750000000002</v>
+        <v>-0.40788249999999998</v>
       </c>
       <c r="X35" s="134">
-        <v>1164469</v>
+        <v>3334436</v>
       </c>
       <c r="Y35" s="134">
         <f>(X36+X35)/10000000*13780</f>
-        <v>3074.7369120000003</v>
+        <v>9554.3078800000003</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
@@ -8073,18 +8142,20 @@
       <c r="R36" s="147">
         <v>17600</v>
       </c>
-      <c r="S36" s="147"/>
+      <c r="S36" s="147">
+        <v>30200</v>
+      </c>
       <c r="T36" s="174"/>
       <c r="U36" s="171">
         <f t="shared" si="2"/>
-        <v>-191279</v>
+        <v>-161079</v>
       </c>
       <c r="V36" s="149">
         <f t="shared" si="3"/>
-        <v>-1.91279</v>
+        <v>-1.6107899999999999</v>
       </c>
       <c r="X36" s="134">
-        <v>1066835</v>
+        <v>3599024</v>
       </c>
       <c r="Y36" s="134"/>
     </row>
@@ -8139,7 +8210,9 @@
       <c r="R37" s="147">
         <v>0</v>
       </c>
-      <c r="S37" s="147"/>
+      <c r="S37" s="147">
+        <v>0</v>
+      </c>
       <c r="T37" s="174"/>
       <c r="U37" s="171">
         <f t="shared" si="2"/>
@@ -8152,7 +8225,7 @@
       <c r="X37" s="134"/>
       <c r="Y37" s="134">
         <f>+Y33-Y35</f>
-        <v>-100708.73691199999</v>
+        <v>-32881.30788</v>
       </c>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.25">
@@ -8208,15 +8281,17 @@
       <c r="R38" s="147">
         <v>-5240</v>
       </c>
-      <c r="S38" s="147"/>
+      <c r="S38" s="147">
+        <v>52612</v>
+      </c>
       <c r="T38" s="174"/>
       <c r="U38" s="171">
         <f t="shared" si="2"/>
-        <v>-13195</v>
+        <v>39417</v>
       </c>
       <c r="V38" s="149">
         <f t="shared" si="3"/>
-        <v>-0.26390000000000002</v>
+        <v>0.78834000000000004</v>
       </c>
       <c r="X38" s="134"/>
       <c r="Y38" s="134"/>
@@ -8274,7 +8349,9 @@
       <c r="R39" s="147">
         <v>0</v>
       </c>
-      <c r="S39" s="147"/>
+      <c r="S39" s="147">
+        <v>0</v>
+      </c>
       <c r="T39" s="174"/>
       <c r="U39" s="171">
         <f t="shared" si="2"/>
@@ -8340,15 +8417,17 @@
       <c r="R40" s="147">
         <v>-83825</v>
       </c>
-      <c r="S40" s="147"/>
+      <c r="S40" s="147">
+        <v>-44514</v>
+      </c>
       <c r="T40" s="174"/>
       <c r="U40" s="171">
         <f t="shared" si="2"/>
-        <v>-27892</v>
+        <v>-72406</v>
       </c>
       <c r="V40" s="149">
         <f t="shared" si="3"/>
-        <v>-9.2973333333333338E-2</v>
+        <v>-0.24135333333333331</v>
       </c>
       <c r="X40" s="134"/>
       <c r="Y40" s="134"/>
@@ -8404,7 +8483,9 @@
       <c r="R41" s="147">
         <v>0</v>
       </c>
-      <c r="S41" s="147"/>
+      <c r="S41" s="147">
+        <v>0</v>
+      </c>
       <c r="T41" s="174"/>
       <c r="U41" s="171">
         <f t="shared" si="2"/>
@@ -8469,15 +8550,17 @@
       <c r="R42" s="147">
         <v>-15800</v>
       </c>
-      <c r="S42" s="147"/>
+      <c r="S42" s="147">
+        <v>-7355</v>
+      </c>
       <c r="T42" s="174"/>
       <c r="U42" s="171">
         <f t="shared" si="2"/>
-        <v>-6378</v>
+        <v>-13733</v>
       </c>
       <c r="V42" s="149">
         <f t="shared" si="3"/>
-        <v>-0.12756000000000001</v>
+        <v>-0.27466000000000002</v>
       </c>
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
@@ -8533,15 +8616,17 @@
       <c r="R43" s="147">
         <v>-13600</v>
       </c>
-      <c r="S43" s="147"/>
+      <c r="S43" s="147">
+        <v>25400</v>
+      </c>
       <c r="T43" s="174"/>
       <c r="U43" s="171">
         <f t="shared" si="2"/>
-        <v>-463353</v>
+        <v>-437953</v>
       </c>
       <c r="V43" s="149">
         <f t="shared" si="3"/>
-        <v>-4.6335300000000004</v>
+        <v>-4.3795299999999999</v>
       </c>
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
@@ -8595,15 +8680,17 @@
       <c r="R44" s="147">
         <v>-4699</v>
       </c>
-      <c r="S44" s="147"/>
+      <c r="S44" s="147">
+        <v>534</v>
+      </c>
       <c r="T44" s="174"/>
       <c r="U44" s="171">
         <f t="shared" si="2"/>
-        <v>7247</v>
+        <v>7781</v>
       </c>
       <c r="V44" s="149">
         <f t="shared" si="3"/>
-        <v>0.72470000000000001</v>
+        <v>0.77810000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
@@ -8659,15 +8746,17 @@
       <c r="R45" s="147">
         <v>-29500</v>
       </c>
-      <c r="S45" s="147"/>
+      <c r="S45" s="147">
+        <v>-42504</v>
+      </c>
       <c r="T45" s="174"/>
       <c r="U45" s="171">
         <f t="shared" si="2"/>
-        <v>-185625</v>
+        <v>-228129</v>
       </c>
       <c r="V45" s="149">
         <f t="shared" si="3"/>
-        <v>-0.46406249999999999</v>
+        <v>-0.57032249999999995</v>
       </c>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.25">
@@ -8723,7 +8812,9 @@
       <c r="R46" s="147">
         <v>0</v>
       </c>
-      <c r="S46" s="147"/>
+      <c r="S46" s="147">
+        <v>0</v>
+      </c>
       <c r="T46" s="174"/>
       <c r="U46" s="171">
         <f t="shared" si="2"/>
@@ -8787,15 +8878,17 @@
       <c r="R47" s="147">
         <v>-296157</v>
       </c>
-      <c r="S47" s="147"/>
+      <c r="S47" s="147">
+        <v>-211473</v>
+      </c>
       <c r="T47" s="174"/>
       <c r="U47" s="171">
         <f t="shared" si="2"/>
-        <v>376191</v>
+        <v>164718</v>
       </c>
       <c r="V47" s="149">
         <f t="shared" si="3"/>
-        <v>1.25397</v>
+        <v>0.54905999999999999</v>
       </c>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.25">
@@ -8849,15 +8942,17 @@
       <c r="R48" s="151">
         <v>54600</v>
       </c>
-      <c r="S48" s="151"/>
+      <c r="S48" s="151">
+        <v>219000</v>
+      </c>
       <c r="T48" s="174"/>
       <c r="U48" s="171">
         <f t="shared" si="2"/>
-        <v>-653336</v>
+        <v>-434336</v>
       </c>
       <c r="V48" s="149">
         <f t="shared" si="3"/>
-        <v>-0.65333600000000003</v>
+        <v>-0.434336</v>
       </c>
     </row>
     <row r="49" spans="1:26" x14ac:dyDescent="0.25">
@@ -8909,7 +9004,9 @@
       <c r="R49" s="151">
         <v>0</v>
       </c>
-      <c r="S49" s="151"/>
+      <c r="S49" s="151">
+        <v>0</v>
+      </c>
       <c r="T49" s="174"/>
       <c r="U49" s="171">
         <f t="shared" si="2"/>
@@ -8973,15 +9070,17 @@
       <c r="R50" s="151">
         <v>-100</v>
       </c>
-      <c r="S50" s="151"/>
+      <c r="S50" s="151">
+        <v>4098</v>
+      </c>
       <c r="T50" s="174"/>
       <c r="U50" s="171">
         <f t="shared" si="2"/>
-        <v>30570</v>
+        <v>34668</v>
       </c>
       <c r="V50" s="149">
         <f t="shared" si="3"/>
-        <v>0.61140000000000005</v>
+        <v>0.69335999999999998</v>
       </c>
     </row>
     <row r="51" spans="1:26" x14ac:dyDescent="0.25">
@@ -9037,15 +9136,17 @@
       <c r="R51" s="151">
         <v>-500</v>
       </c>
-      <c r="S51" s="151"/>
+      <c r="S51" s="151">
+        <v>36340</v>
+      </c>
       <c r="T51" s="174"/>
       <c r="U51" s="171">
         <f t="shared" si="2"/>
-        <v>-618213</v>
+        <v>-581873</v>
       </c>
       <c r="V51" s="149">
         <f t="shared" si="3"/>
-        <v>-0.95109692307692317</v>
+        <v>-0.89518923076923085</v>
       </c>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.25">
@@ -9101,7 +9202,9 @@
       <c r="R52" s="151">
         <v>0</v>
       </c>
-      <c r="S52" s="151"/>
+      <c r="S52" s="151">
+        <v>0</v>
+      </c>
       <c r="T52" s="174"/>
       <c r="U52" s="171">
         <f t="shared" si="2"/>
@@ -9165,15 +9268,17 @@
       <c r="R53" s="151">
         <v>0</v>
       </c>
-      <c r="S53" s="151"/>
+      <c r="S53" s="151">
+        <v>-42834</v>
+      </c>
       <c r="T53" s="174"/>
       <c r="U53" s="171">
         <f t="shared" si="2"/>
-        <v>-174516</v>
+        <v>-217350</v>
       </c>
       <c r="V53" s="149">
         <f t="shared" si="3"/>
-        <v>-0.58172000000000001</v>
+        <v>-0.72450000000000003</v>
       </c>
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.25">
@@ -9227,7 +9332,9 @@
       <c r="R54" s="151">
         <v>0</v>
       </c>
-      <c r="S54" s="151"/>
+      <c r="S54" s="151">
+        <v>0</v>
+      </c>
       <c r="T54" s="174"/>
       <c r="U54" s="171">
         <f t="shared" si="2"/>
@@ -9289,15 +9396,17 @@
       <c r="R55" s="151">
         <v>-13500</v>
       </c>
-      <c r="S55" s="151"/>
+      <c r="S55" s="151">
+        <v>14150</v>
+      </c>
       <c r="T55" s="174"/>
       <c r="U55" s="171">
         <f t="shared" si="2"/>
-        <v>8628</v>
+        <v>22778</v>
       </c>
       <c r="V55" s="149">
         <f t="shared" si="3"/>
-        <v>1.7256000000000001E-2</v>
+        <v>4.5556000000000006E-2</v>
       </c>
     </row>
     <row r="56" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -9354,7 +9463,7 @@
       </c>
       <c r="S56" s="254">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-1073044</v>
       </c>
       <c r="T56" s="254">
         <f>SUM(T4:T55)</f>
@@ -9362,7 +9471,7 @@
       </c>
       <c r="U56" s="254">
         <f t="shared" si="2"/>
-        <v>-6039129</v>
+        <v>-7112173</v>
       </c>
       <c r="V56" s="255">
         <f t="shared" si="3"/>
@@ -9446,15 +9555,17 @@
       <c r="R58" s="162">
         <v>0</v>
       </c>
-      <c r="S58" s="162"/>
+      <c r="S58" s="162">
+        <v>-101150</v>
+      </c>
       <c r="T58" s="246"/>
       <c r="U58" s="247">
         <f>SUM(H58:T58)</f>
-        <v>-715553</v>
+        <v>-816703</v>
       </c>
       <c r="V58" s="248">
         <f>IFERROR(U58/F58*100,0)/10000000</f>
-        <v>-2.3851766666666663</v>
+        <v>-2.7223433333333333</v>
       </c>
       <c r="Y58" s="134"/>
     </row>
@@ -9509,7 +9620,9 @@
       <c r="R59" s="162">
         <v>0</v>
       </c>
-      <c r="S59" s="162"/>
+      <c r="S59" s="162">
+        <v>0</v>
+      </c>
       <c r="T59" s="174"/>
       <c r="U59" s="171">
         <f>SUM(H59:T59)</f>
@@ -9575,7 +9688,7 @@
       </c>
       <c r="S60" s="170">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-101150</v>
       </c>
       <c r="T60" s="170">
         <f>SUM(T58:T59)</f>
@@ -9583,7 +9696,7 @@
       </c>
       <c r="U60" s="254">
         <f>SUM(H60:T60)</f>
-        <v>-628287</v>
+        <v>-729437</v>
       </c>
       <c r="V60" s="19"/>
       <c r="X60" s="5"/>
@@ -22776,19 +22889,19 @@
       </c>
       <c r="K4" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-40798</v>
+        <v>-62648</v>
       </c>
       <c r="L4" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.81596000000000002</v>
+        <v>-1.2529600000000001</v>
       </c>
       <c r="M4" s="71">
         <f t="shared" ref="M4:N62" si="0">G4+I4+K4</f>
-        <v>-67842</v>
+        <v>-89692</v>
       </c>
       <c r="N4" s="166">
         <f t="shared" si="0"/>
-        <v>-1.35684</v>
+        <v>-1.7938400000000001</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -22828,19 +22941,19 @@
       </c>
       <c r="K5" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>168284</v>
+        <v>75784</v>
       </c>
       <c r="L5" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.56094666666666659</v>
+        <v>0.2526133333333333</v>
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>-82687</v>
+        <v>-175187</v>
       </c>
       <c r="N5" s="166">
         <f t="shared" si="0"/>
-        <v>-0.27562333333333344</v>
+        <v>-0.58395666666666668</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -22932,19 +23045,19 @@
       </c>
       <c r="K7" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>105547</v>
+        <v>19647</v>
       </c>
       <c r="L7" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>1.0554699999999999</v>
+        <v>0.19647000000000001</v>
       </c>
       <c r="M7" s="71">
         <f t="shared" si="1"/>
-        <v>76557</v>
+        <v>-9343</v>
       </c>
       <c r="N7" s="166">
         <f t="shared" si="2"/>
-        <v>1.0554699999999999</v>
+        <v>0.19647000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -22984,19 +23097,19 @@
       </c>
       <c r="K8" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>34234</v>
+        <v>-44396</v>
       </c>
       <c r="L8" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.11411333333333334</v>
+        <v>-0.14798666666666666</v>
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>-420863</v>
+        <v>-499493</v>
       </c>
       <c r="N8" s="166">
         <f t="shared" si="0"/>
-        <v>-1.4028766666666668</v>
+        <v>-1.6649766666666668</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -23036,19 +23149,19 @@
       </c>
       <c r="K9" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>49903</v>
+        <v>18703</v>
       </c>
       <c r="L9" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.33268666666666663</v>
+        <v>0.12468666666666665</v>
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>-244233</v>
+        <v>-275433</v>
       </c>
       <c r="N9" s="166">
         <f t="shared" si="0"/>
-        <v>-1.6282200000000004</v>
+        <v>-1.8362200000000004</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -23088,19 +23201,19 @@
       </c>
       <c r="K10" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>9337</v>
+        <v>8437</v>
       </c>
       <c r="L10" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.15561666666666668</v>
+        <v>0.14061666666666667</v>
       </c>
       <c r="M10" s="71">
         <f t="shared" ref="M10" si="3">G10+I10+K10</f>
-        <v>-182912</v>
+        <v>-183812</v>
       </c>
       <c r="N10" s="166">
         <f t="shared" ref="N10" si="4">H10+J10+L10</f>
-        <v>-3.0485333333333338</v>
+        <v>-3.0635333333333334</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -23140,19 +23253,19 @@
       </c>
       <c r="K11" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-764248</v>
+        <v>-759922</v>
       </c>
       <c r="L11" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.50949866666666666</v>
+        <v>-0.50661466666666666</v>
       </c>
       <c r="M11" s="71">
         <f t="shared" si="0"/>
-        <v>203017</v>
+        <v>207343</v>
       </c>
       <c r="N11" s="166">
         <f t="shared" si="0"/>
-        <v>0.13534466666666678</v>
+        <v>0.13822866666666678</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -23192,19 +23305,19 @@
       </c>
       <c r="K12" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>25206</v>
+        <v>-9929</v>
       </c>
       <c r="L12" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>4.2009999999999999E-2</v>
+        <v>-1.6548333333333332E-2</v>
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>432986</v>
+        <v>397851</v>
       </c>
       <c r="N12" s="166">
         <f t="shared" si="0"/>
-        <v>0.72164333333333341</v>
+        <v>0.66308500000000015</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -23296,19 +23409,19 @@
       </c>
       <c r="K14" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>3762</v>
+        <v>-12292</v>
       </c>
       <c r="L14" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>1.5048000000000001E-2</v>
+        <v>-4.9168000000000003E-2</v>
       </c>
       <c r="M14" s="71">
         <f t="shared" si="0"/>
-        <v>48682</v>
+        <v>32628</v>
       </c>
       <c r="N14" s="166">
         <f t="shared" si="0"/>
-        <v>0.19472799999999996</v>
+        <v>0.13051199999999996</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -23400,19 +23513,19 @@
       </c>
       <c r="K16" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-25908</v>
+        <v>-18338</v>
       </c>
       <c r="L16" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.25907999999999998</v>
+        <v>-0.18337999999999999</v>
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>47499</v>
+        <v>55069</v>
       </c>
       <c r="N16" s="166">
         <f t="shared" si="0"/>
-        <v>0.47499000000000002</v>
+        <v>0.55069000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -23452,19 +23565,19 @@
       </c>
       <c r="K17" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>6980</v>
+        <v>-10636</v>
       </c>
       <c r="L17" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>3.1727272727272722E-2</v>
+        <v>-4.8345454545454539E-2</v>
       </c>
       <c r="M17" s="71">
         <f t="shared" ref="M17" si="5">G17+I17+K17</f>
-        <v>-80928</v>
+        <v>-98544</v>
       </c>
       <c r="N17" s="166">
         <f t="shared" ref="N17" si="6">H17+J17+L17</f>
-        <v>-0.36785454545454543</v>
+        <v>-0.44792727272727267</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -23504,19 +23617,19 @@
       </c>
       <c r="K18" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>9579</v>
+        <v>-12742</v>
       </c>
       <c r="L18" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>3.8316000000000003E-2</v>
+        <v>-5.0967999999999999E-2</v>
       </c>
       <c r="M18" s="71">
         <f t="shared" si="0"/>
-        <v>-54338</v>
+        <v>-76659</v>
       </c>
       <c r="N18" s="166">
         <f t="shared" si="0"/>
-        <v>-0.21735199999999999</v>
+        <v>-0.30663600000000002</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -23556,19 +23669,19 @@
       </c>
       <c r="K19" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>13543</v>
+        <v>-25109</v>
       </c>
       <c r="L19" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>3.3857499999999999E-2</v>
+        <v>-6.2772499999999995E-2</v>
       </c>
       <c r="M19" s="71">
         <f t="shared" si="0"/>
-        <v>280858</v>
+        <v>242206</v>
       </c>
       <c r="N19" s="166">
         <f t="shared" si="0"/>
-        <v>0.70214499999999991</v>
+        <v>0.60551499999999991</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -23660,19 +23773,19 @@
       </c>
       <c r="K21" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-19503</v>
+        <v>-33003</v>
       </c>
       <c r="L21" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.78012000000000004</v>
+        <v>-1.32012</v>
       </c>
       <c r="M21" s="71">
         <f t="shared" ref="M21:M22" si="7">G21+I21+K21</f>
-        <v>-63049</v>
+        <v>-76549</v>
       </c>
       <c r="N21" s="166">
         <f t="shared" ref="N21:N22" si="8">H21+J21+L21</f>
-        <v>-2.52196</v>
+        <v>-3.06196</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -23764,19 +23877,19 @@
       </c>
       <c r="K23" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-200398</v>
+        <v>-281543</v>
       </c>
       <c r="L23" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-1.3359866666666667</v>
+        <v>-1.8769533333333335</v>
       </c>
       <c r="M23" s="71">
         <f t="shared" si="0"/>
-        <v>-85385</v>
+        <v>-166530</v>
       </c>
       <c r="N23" s="166">
         <f t="shared" si="0"/>
-        <v>-0.56923333333333326</v>
+        <v>-1.1102000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -23868,19 +23981,19 @@
       </c>
       <c r="K25" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-11535</v>
+        <v>-1794</v>
       </c>
       <c r="L25" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.10486363636363635</v>
+        <v>-1.6309090909090908E-2</v>
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>193169</v>
+        <v>202910</v>
       </c>
       <c r="N25" s="166">
         <f t="shared" si="0"/>
-        <v>1.7560818181818176</v>
+        <v>1.8446363636363632</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -23920,19 +24033,19 @@
       </c>
       <c r="K26" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-1448523</v>
+        <v>-1267323</v>
       </c>
       <c r="L26" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-6.2979260869565215</v>
+        <v>-5.5101000000000004</v>
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>-1094462</v>
+        <v>-913262</v>
       </c>
       <c r="N26" s="166">
         <f t="shared" si="0"/>
-        <v>-4.7585304347826085</v>
+        <v>-3.9707043478260879</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -23970,19 +24083,19 @@
       </c>
       <c r="K27" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>5794</v>
+        <v>7579</v>
       </c>
       <c r="L27" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.28970000000000001</v>
+        <v>0.37895000000000001</v>
       </c>
       <c r="M27" s="71">
         <f t="shared" ref="M27" si="9">G27+I27+K27</f>
-        <v>-14502</v>
+        <v>-12717</v>
       </c>
       <c r="N27" s="166">
         <f t="shared" ref="N27" si="10">H27+J27+L27</f>
-        <v>-0.72509999999999986</v>
+        <v>-0.63584999999999992</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -24022,19 +24135,19 @@
       </c>
       <c r="K28" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>34666</v>
+        <v>-30334</v>
       </c>
       <c r="L28" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>6.9332000000000005E-2</v>
+        <v>-6.0668E-2</v>
       </c>
       <c r="M28" s="71">
         <f t="shared" si="0"/>
-        <v>-230252</v>
+        <v>-295252</v>
       </c>
       <c r="N28" s="166">
         <f t="shared" si="0"/>
-        <v>-0.46050399999999997</v>
+        <v>-0.59050399999999992</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -24074,19 +24187,19 @@
       </c>
       <c r="K29" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-1231866</v>
+        <v>-1675566</v>
       </c>
       <c r="L29" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-1.2318659999999999</v>
+        <v>-1.6755660000000001</v>
       </c>
       <c r="M29" s="71">
         <f t="shared" si="0"/>
-        <v>2235546</v>
+        <v>1791846</v>
       </c>
       <c r="N29" s="166">
         <f t="shared" si="0"/>
-        <v>2.2355460000000003</v>
+        <v>1.7918459999999998</v>
       </c>
       <c r="O29" s="131"/>
     </row>
@@ -24387,19 +24500,19 @@
       </c>
       <c r="K35" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-341989</v>
+        <v>-374989</v>
       </c>
       <c r="L35" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.68397799999999997</v>
+        <v>-0.74997800000000003</v>
       </c>
       <c r="M35" s="71">
         <f t="shared" si="0"/>
-        <v>357863</v>
+        <v>324863</v>
       </c>
       <c r="N35" s="166">
         <f t="shared" si="0"/>
-        <v>0.71572599999999986</v>
+        <v>0.6497259999999998</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -24439,19 +24552,19 @@
       </c>
       <c r="K36" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>65134</v>
+        <v>-119760</v>
       </c>
       <c r="L36" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.13026799999999999</v>
+        <v>-0.23952000000000001</v>
       </c>
       <c r="M36" s="71">
         <f t="shared" si="0"/>
-        <v>1092541</v>
+        <v>907647</v>
       </c>
       <c r="N36" s="166">
         <f t="shared" si="0"/>
-        <v>2.185082</v>
+        <v>1.815294</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -24491,19 +24604,19 @@
       </c>
       <c r="K37" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-186096</v>
+        <v>-197521</v>
       </c>
       <c r="L37" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-3.7219199999999999</v>
+        <v>-3.9504199999999998</v>
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>-265460</v>
+        <v>-276885</v>
       </c>
       <c r="N37" s="166">
         <f t="shared" si="0"/>
-        <v>-5.3091999999999997</v>
+        <v>-5.5377000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -24543,19 +24656,19 @@
       </c>
       <c r="K38" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>115289</v>
+        <v>108981</v>
       </c>
       <c r="L38" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>2.882225</v>
+        <v>2.7245249999999999</v>
       </c>
       <c r="M38" s="71">
         <f t="shared" si="0"/>
-        <v>49764</v>
+        <v>43456</v>
       </c>
       <c r="N38" s="166">
         <f t="shared" si="0"/>
-        <v>1.2441000000000002</v>
+        <v>1.0864</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -24699,19 +24812,19 @@
       </c>
       <c r="K41" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-131563</v>
+        <v>-163153</v>
       </c>
       <c r="L41" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.32890750000000002</v>
+        <v>-0.40788249999999998</v>
       </c>
       <c r="M41" s="71">
         <f t="shared" si="0"/>
-        <v>579373</v>
+        <v>547783</v>
       </c>
       <c r="N41" s="166">
         <f t="shared" si="0"/>
-        <v>1.4484325</v>
+        <v>1.3694575000000002</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -24751,19 +24864,19 @@
       </c>
       <c r="K42" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-191279</v>
+        <v>-161079</v>
       </c>
       <c r="L42" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-1.91279</v>
+        <v>-1.6107899999999999</v>
       </c>
       <c r="M42" s="71">
         <f t="shared" si="0"/>
-        <v>12353</v>
+        <v>42553</v>
       </c>
       <c r="N42" s="166">
         <f t="shared" si="0"/>
-        <v>0.12352999999999992</v>
+        <v>0.42552999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -24853,19 +24966,19 @@
       </c>
       <c r="K44" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-13195</v>
+        <v>39417</v>
       </c>
       <c r="L44" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.26390000000000002</v>
+        <v>0.78834000000000004</v>
       </c>
       <c r="M44" s="71">
         <f t="shared" si="0"/>
-        <v>-79578</v>
+        <v>-26966</v>
       </c>
       <c r="N44" s="166">
         <f t="shared" si="0"/>
-        <v>-1.5915599999999999</v>
+        <v>-0.5393199999999998</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -24905,19 +25018,19 @@
       </c>
       <c r="K45" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-27892</v>
+        <v>-72406</v>
       </c>
       <c r="L45" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-9.2973333333333338E-2</v>
+        <v>-0.24135333333333331</v>
       </c>
       <c r="M45" s="71">
         <f t="shared" si="0"/>
-        <v>-138684</v>
+        <v>-183198</v>
       </c>
       <c r="N45" s="166">
         <f t="shared" si="0"/>
-        <v>-0.46228000000000002</v>
+        <v>-0.61065999999999998</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -25111,19 +25224,19 @@
       </c>
       <c r="K49" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-6378</v>
+        <v>-13733</v>
       </c>
       <c r="L49" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.12756000000000001</v>
+        <v>-0.27466000000000002</v>
       </c>
       <c r="M49" s="71">
         <f t="shared" si="0"/>
-        <v>27950</v>
+        <v>20595</v>
       </c>
       <c r="N49" s="166">
         <f t="shared" si="0"/>
-        <v>0.2384</v>
+        <v>9.1299999999999992E-2</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -25163,19 +25276,19 @@
       </c>
       <c r="K50" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-463353</v>
+        <v>-437953</v>
       </c>
       <c r="L50" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-4.6335300000000004</v>
+        <v>-4.3795299999999999</v>
       </c>
       <c r="M50" s="71">
         <f t="shared" si="0"/>
-        <v>424021</v>
+        <v>449421</v>
       </c>
       <c r="N50" s="166">
         <f t="shared" si="0"/>
-        <v>4.2402099999999994</v>
+        <v>4.4942099999999998</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -25213,19 +25326,19 @@
       </c>
       <c r="K51" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>7247</v>
+        <v>7781</v>
       </c>
       <c r="L51" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.72470000000000001</v>
+        <v>0.77810000000000001</v>
       </c>
       <c r="M51" s="71">
         <f t="shared" ref="M51" si="17">G51+I51+K51</f>
-        <v>3701</v>
+        <v>4235</v>
       </c>
       <c r="N51" s="166">
         <f t="shared" ref="N51" si="18">H51+J51+L51</f>
-        <v>0.37009999999999998</v>
+        <v>0.42349999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -25265,19 +25378,19 @@
       </c>
       <c r="K52" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>376191</v>
+        <v>164718</v>
       </c>
       <c r="L52" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>1.25397</v>
+        <v>0.54905999999999999</v>
       </c>
       <c r="M52" s="71">
         <f t="shared" si="0"/>
-        <v>367458</v>
+        <v>155985</v>
       </c>
       <c r="N52" s="166">
         <f t="shared" si="0"/>
-        <v>1.2248600000000001</v>
+        <v>0.51995000000000002</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -25363,19 +25476,19 @@
       </c>
       <c r="K54" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-185625</v>
+        <v>-228129</v>
       </c>
       <c r="L54" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.46406249999999999</v>
+        <v>-0.57032249999999995</v>
       </c>
       <c r="M54" s="71">
         <f t="shared" si="0"/>
-        <v>289577</v>
+        <v>247073</v>
       </c>
       <c r="N54" s="166">
         <f t="shared" si="0"/>
-        <v>0.72394249999999993</v>
+        <v>0.61768250000000002</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -25465,19 +25578,19 @@
       </c>
       <c r="K56" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-653336</v>
+        <v>-434336</v>
       </c>
       <c r="L56" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.65333600000000003</v>
+        <v>-0.434336</v>
       </c>
       <c r="M56" s="71">
         <f t="shared" ref="M56" si="21">G56+I56+K56</f>
-        <v>-1688416</v>
+        <v>-1469416</v>
       </c>
       <c r="N56" s="166">
         <f t="shared" ref="N56" si="22">H56+J56+L56</f>
-        <v>-1.6885159999999999</v>
+        <v>-1.469516</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -25563,19 +25676,19 @@
       </c>
       <c r="K58" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>30570</v>
+        <v>34668</v>
       </c>
       <c r="L58" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>0.61140000000000005</v>
+        <v>0.69335999999999998</v>
       </c>
       <c r="M58" s="71">
         <f t="shared" si="0"/>
-        <v>-3725</v>
+        <v>373</v>
       </c>
       <c r="N58" s="166">
         <f t="shared" si="0"/>
-        <v>-7.44999999999999E-2</v>
+        <v>7.4600000000000222E-3</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
@@ -25615,19 +25728,19 @@
       </c>
       <c r="K59" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-618213</v>
+        <v>-581873</v>
       </c>
       <c r="L59" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.95109692307692317</v>
+        <v>-0.89518923076923085</v>
       </c>
       <c r="M59" s="71">
         <f t="shared" si="0"/>
-        <v>325731</v>
+        <v>362071</v>
       </c>
       <c r="N59" s="166">
         <f t="shared" si="0"/>
-        <v>1.3445140384615386</v>
+        <v>1.4004217307692308</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -25719,19 +25832,19 @@
       </c>
       <c r="K61" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-174516</v>
+        <v>-217350</v>
       </c>
       <c r="L61" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-0.58172000000000001</v>
+        <v>-0.72450000000000003</v>
       </c>
       <c r="M61" s="71">
         <f t="shared" si="0"/>
-        <v>529557</v>
+        <v>486723</v>
       </c>
       <c r="N61" s="166">
         <f t="shared" si="0"/>
-        <v>1.7651900000000003</v>
+        <v>1.6224100000000004</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
@@ -25871,19 +25984,19 @@
       </c>
       <c r="K64" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>8628</v>
+        <v>22778</v>
       </c>
       <c r="L64" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>1.7256000000000001E-2</v>
+        <v>4.5556000000000006E-2</v>
       </c>
       <c r="M64" s="71">
         <f t="shared" ref="M64" si="27">G64+I64+K64</f>
-        <v>498033</v>
+        <v>512183</v>
       </c>
       <c r="N64" s="166">
         <f t="shared" ref="N64" si="28">H64+J64+L64</f>
-        <v>0.99606600000000001</v>
+        <v>1.0243659999999999</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -25905,12 +26018,12 @@
       <c r="J65" s="100"/>
       <c r="K65" s="109">
         <f>SUM(K4:K62)</f>
-        <v>-6059497</v>
+        <v>-7146691</v>
       </c>
       <c r="L65" s="109"/>
       <c r="M65" s="154">
         <f>SUM(M4:M62)</f>
-        <v>5691550</v>
+        <v>4604356</v>
       </c>
       <c r="N65" s="235"/>
     </row>
@@ -25991,19 +26104,19 @@
       </c>
       <c r="K69" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-715553</v>
+        <v>-816703</v>
       </c>
       <c r="L69" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$ADW$124,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$DX$2,0),0),0)</f>
-        <v>-2.3851766666666663</v>
+        <v>-2.7223433333333333</v>
       </c>
       <c r="M69" s="153">
         <f t="shared" ref="M69:N69" si="29">G69+I69+K69</f>
-        <v>-29043</v>
+        <v>-130193</v>
       </c>
       <c r="N69" s="167">
         <f t="shared" si="29"/>
-        <v>-9.6809999999999174E-2</v>
+        <v>-0.43397666666666623</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -26069,12 +26182,12 @@
       <c r="J71" s="104"/>
       <c r="K71" s="93">
         <f>SUM(K69:K70)</f>
-        <v>-628287</v>
+        <v>-729437</v>
       </c>
       <c r="L71" s="113"/>
       <c r="M71" s="93">
         <f>SUM(M69:M70)</f>
-        <v>1227108</v>
+        <v>1125958</v>
       </c>
       <c r="N71" s="236"/>
     </row>
@@ -44806,11 +44919,11 @@
       <c r="O6" s="215"/>
       <c r="P6" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-67842</v>
+        <v>-89692</v>
       </c>
       <c r="Q6" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1.35684</v>
+        <v>-1.7938400000000001</v>
       </c>
       <c r="R6" s="159"/>
       <c r="S6" s="153">
@@ -44827,11 +44940,11 @@
       <c r="X6" s="132"/>
       <c r="Y6" s="154">
         <f t="shared" si="0"/>
-        <v>-116178</v>
+        <v>-138028</v>
       </c>
       <c r="Z6" s="168">
         <f t="shared" si="1"/>
-        <v>-2.3235600000000001</v>
+        <v>-2.7605599999999999</v>
       </c>
     </row>
     <row r="7" spans="1:26" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -44888,11 +45001,11 @@
       <c r="O7" s="215"/>
       <c r="P7" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-82687</v>
+        <v>-175187</v>
       </c>
       <c r="Q7" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.27562333333333344</v>
+        <v>-0.58395666666666668</v>
       </c>
       <c r="R7" s="159"/>
       <c r="S7" s="88">
@@ -44909,11 +45022,11 @@
       <c r="X7"/>
       <c r="Y7" s="154">
         <f t="shared" si="0"/>
-        <v>1251587</v>
+        <v>1159087</v>
       </c>
       <c r="Z7" s="168">
         <f t="shared" si="1"/>
-        <v>4.1719566666666665</v>
+        <v>3.8636233333333339</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45085,11 +45198,11 @@
       <c r="O10" s="215"/>
       <c r="P10" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-420863</v>
+        <v>-499493</v>
       </c>
       <c r="Q10" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1.4028766666666668</v>
+        <v>-1.6649766666666668</v>
       </c>
       <c r="R10" s="159"/>
       <c r="S10" s="88">
@@ -45105,11 +45218,11 @@
       <c r="W10" s="72"/>
       <c r="Y10" s="154">
         <f t="shared" si="0"/>
-        <v>-779772</v>
+        <v>-858402</v>
       </c>
       <c r="Z10" s="168">
         <f t="shared" si="1"/>
-        <v>-4.0435566666666674</v>
+        <v>-4.3056566666666667</v>
       </c>
     </row>
     <row r="11" spans="1:26" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45166,11 +45279,11 @@
       <c r="O11" s="215"/>
       <c r="P11" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-244233</v>
+        <v>-275433</v>
       </c>
       <c r="Q11" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1.6282200000000004</v>
+        <v>-1.8362200000000004</v>
       </c>
       <c r="R11" s="159"/>
       <c r="S11" s="153">
@@ -45186,11 +45299,11 @@
       <c r="W11" s="150"/>
       <c r="Y11" s="154">
         <f t="shared" si="0"/>
-        <v>-419195</v>
+        <v>-450395</v>
       </c>
       <c r="Z11" s="168">
         <f t="shared" si="1"/>
-        <v>-2.7946333333333335</v>
+        <v>-3.0026333333333337</v>
       </c>
     </row>
     <row r="12" spans="1:26" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45247,11 +45360,11 @@
       <c r="O12" s="215"/>
       <c r="P12" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-182912</v>
+        <v>-183812</v>
       </c>
       <c r="Q12" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-3.0485333333333338</v>
+        <v>-3.0635333333333334</v>
       </c>
       <c r="R12" s="159"/>
       <c r="S12" s="153">
@@ -45267,11 +45380,11 @@
       <c r="W12" s="150"/>
       <c r="Y12" s="154">
         <f t="shared" ref="Y12" si="10">M12+P12+S12+V12</f>
-        <v>-182912</v>
+        <v>-183812</v>
       </c>
       <c r="Z12" s="168">
         <f t="shared" ref="Z12" si="11">(N12+Q12+T12+W12)</f>
-        <v>-3.0485333333333338</v>
+        <v>-3.0635333333333334</v>
       </c>
     </row>
     <row r="13" spans="1:26" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45328,11 +45441,11 @@
       <c r="O13" s="215"/>
       <c r="P13" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>203017</v>
+        <v>207343</v>
       </c>
       <c r="Q13" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.13534466666666678</v>
+        <v>0.13822866666666678</v>
       </c>
       <c r="R13" s="159"/>
       <c r="S13" s="88">
@@ -45349,11 +45462,11 @@
       <c r="X13"/>
       <c r="Y13" s="154">
         <f t="shared" si="0"/>
-        <v>-1165182</v>
+        <v>-1160856</v>
       </c>
       <c r="Z13" s="168">
         <f t="shared" si="1"/>
-        <v>-0.77678799999999992</v>
+        <v>-0.77390399999999993</v>
       </c>
     </row>
     <row r="14" spans="1:26" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45737,11 +45850,11 @@
       <c r="O18" s="215"/>
       <c r="P18" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>432986</v>
+        <v>397851</v>
       </c>
       <c r="Q18" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.72164333333333341</v>
+        <v>0.66308500000000015</v>
       </c>
       <c r="R18" s="159"/>
       <c r="S18" s="88">
@@ -45757,11 +45870,11 @@
       <c r="W18" s="72"/>
       <c r="Y18" s="154">
         <f t="shared" si="0"/>
-        <v>237652</v>
+        <v>202517</v>
       </c>
       <c r="Z18" s="168">
         <f t="shared" si="1"/>
-        <v>-2.6959766666666667</v>
+        <v>-2.7545349999999997</v>
       </c>
     </row>
     <row r="19" spans="1:34" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -45989,11 +46102,11 @@
       <c r="O21" s="215"/>
       <c r="P21" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>48682</v>
+        <v>32628</v>
       </c>
       <c r="Q21" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.19472799999999996</v>
+        <v>0.13051199999999996</v>
       </c>
       <c r="R21" s="159"/>
       <c r="S21" s="88">
@@ -46009,11 +46122,11 @@
       <c r="W21" s="72"/>
       <c r="Y21" s="154">
         <f t="shared" si="0"/>
-        <v>-218734</v>
+        <v>-234788</v>
       </c>
       <c r="Z21" s="168">
         <f t="shared" si="1"/>
-        <v>-2.4794320000000001</v>
+        <v>-2.5436480000000001</v>
       </c>
     </row>
     <row r="22" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46070,11 +46183,11 @@
       <c r="O22" s="215"/>
       <c r="P22" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-80928</v>
+        <v>-98544</v>
       </c>
       <c r="Q22" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.36785454545454543</v>
+        <v>-0.44792727272727267</v>
       </c>
       <c r="R22" s="159"/>
       <c r="S22" s="88">
@@ -46090,11 +46203,11 @@
       <c r="W22" s="72"/>
       <c r="Y22" s="154">
         <f t="shared" si="0"/>
-        <v>-169828</v>
+        <v>-187444</v>
       </c>
       <c r="Z22" s="168">
         <f t="shared" si="1"/>
-        <v>-1.2568545454545454</v>
+        <v>-1.3369272727272727</v>
       </c>
     </row>
     <row r="23" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46232,11 +46345,11 @@
       <c r="O24" s="215"/>
       <c r="P24" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>47499</v>
+        <v>55069</v>
       </c>
       <c r="Q24" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.47499000000000002</v>
+        <v>0.55069000000000001</v>
       </c>
       <c r="R24" s="159"/>
       <c r="S24" s="88">
@@ -46252,11 +46365,11 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="154">
         <f t="shared" si="0"/>
-        <v>1762844</v>
+        <v>1770414</v>
       </c>
       <c r="Z24" s="168">
         <f t="shared" si="1"/>
-        <v>17.628439999999998</v>
+        <v>17.704139999999999</v>
       </c>
     </row>
     <row r="25" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46554,11 +46667,11 @@
       <c r="O28" s="215"/>
       <c r="P28" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-54338</v>
+        <v>-76659</v>
       </c>
       <c r="Q28" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.21735199999999999</v>
+        <v>-0.30663600000000002</v>
       </c>
       <c r="R28" s="159"/>
       <c r="S28" s="88">
@@ -46574,11 +46687,11 @@
       <c r="W28" s="72"/>
       <c r="Y28" s="154">
         <f t="shared" si="0"/>
-        <v>303875</v>
+        <v>281554</v>
       </c>
       <c r="Z28" s="168">
         <f t="shared" si="1"/>
-        <v>1.2155</v>
+        <v>1.1262159999999999</v>
       </c>
     </row>
     <row r="29" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46635,11 +46748,11 @@
       <c r="O29" s="215"/>
       <c r="P29" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>280858</v>
+        <v>242206</v>
       </c>
       <c r="Q29" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.70214499999999991</v>
+        <v>0.60551499999999991</v>
       </c>
       <c r="R29" s="159"/>
       <c r="S29" s="88">
@@ -46656,11 +46769,11 @@
       <c r="X29" s="1"/>
       <c r="Y29" s="154">
         <f t="shared" si="0"/>
-        <v>951321</v>
+        <v>912669</v>
       </c>
       <c r="Z29" s="168">
         <f t="shared" si="1"/>
-        <v>2.3783024999999998</v>
+        <v>2.2816725</v>
       </c>
     </row>
     <row r="30" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46888,11 +47001,11 @@
       <c r="O32" s="215"/>
       <c r="P32" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-85385</v>
+        <v>-166530</v>
       </c>
       <c r="Q32" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.56923333333333326</v>
+        <v>-1.1102000000000001</v>
       </c>
       <c r="R32" s="159"/>
       <c r="S32" s="88">
@@ -46909,11 +47022,11 @@
       <c r="X32"/>
       <c r="Y32" s="154">
         <f t="shared" si="0"/>
-        <v>-590454</v>
+        <v>-671599</v>
       </c>
       <c r="Z32" s="168">
         <f t="shared" si="1"/>
-        <v>-3.9363600000000005</v>
+        <v>-4.4773266666666673</v>
       </c>
     </row>
     <row r="33" spans="1:34" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47051,11 +47164,11 @@
       <c r="O34" s="215"/>
       <c r="P34" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>193169</v>
+        <v>202910</v>
       </c>
       <c r="Q34" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.7560818181818176</v>
+        <v>1.8446363636363632</v>
       </c>
       <c r="R34" s="159"/>
       <c r="S34" s="88">
@@ -47071,11 +47184,11 @@
       <c r="W34" s="72"/>
       <c r="Y34" s="154">
         <f t="shared" si="0"/>
-        <v>-125771</v>
+        <v>-116030</v>
       </c>
       <c r="Z34" s="168">
         <f t="shared" si="1"/>
-        <v>-1.1433727272727274</v>
+        <v>-1.0548181818181819</v>
       </c>
       <c r="AB34" s="1"/>
       <c r="AC34" s="1"/>
@@ -47220,11 +47333,11 @@
       <c r="O36" s="215"/>
       <c r="P36" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1094462</v>
+        <v>-913262</v>
       </c>
       <c r="Q36" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-4.7585304347826085</v>
+        <v>-3.9707043478260879</v>
       </c>
       <c r="R36" s="159"/>
       <c r="S36" s="88">
@@ -47240,11 +47353,11 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="154">
         <f t="shared" si="0"/>
-        <v>3066641</v>
+        <v>3247841</v>
       </c>
       <c r="Z36" s="168">
         <f t="shared" si="1"/>
-        <v>13.333221739130435</v>
+        <v>14.121047826086956</v>
       </c>
     </row>
     <row r="37" spans="1:34" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47299,11 +47412,11 @@
       <c r="O37" s="215"/>
       <c r="P37" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-14502</v>
+        <v>-12717</v>
       </c>
       <c r="Q37" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.72509999999999986</v>
+        <v>-0.63584999999999992</v>
       </c>
       <c r="R37" s="159"/>
       <c r="S37" s="153">
@@ -47319,11 +47432,11 @@
       <c r="W37" s="150"/>
       <c r="Y37" s="154">
         <f t="shared" ref="Y37" si="20">M37+P37+S37+V37</f>
-        <v>-14502</v>
+        <v>-12717</v>
       </c>
       <c r="Z37" s="168">
         <f t="shared" ref="Z37" si="21">(N37+Q37+T37+W37)</f>
-        <v>-0.72509999999999986</v>
+        <v>-0.63584999999999992</v>
       </c>
     </row>
     <row r="38" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47380,11 +47493,11 @@
       <c r="O38" s="215"/>
       <c r="P38" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-230252</v>
+        <v>-295252</v>
       </c>
       <c r="Q38" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.46050399999999997</v>
+        <v>-0.59050399999999992</v>
       </c>
       <c r="R38" s="159"/>
       <c r="S38" s="88">
@@ -47400,11 +47513,11 @@
       <c r="W38" s="72"/>
       <c r="Y38" s="154">
         <f t="shared" si="0"/>
-        <v>2836154</v>
+        <v>2771154</v>
       </c>
       <c r="Z38" s="168">
         <f t="shared" si="1"/>
-        <v>5.6723079999999992</v>
+        <v>5.5423079999999993</v>
       </c>
     </row>
     <row r="39" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47461,11 +47574,11 @@
       <c r="O39" s="215"/>
       <c r="P39" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>2235546</v>
+        <v>1791846</v>
       </c>
       <c r="Q39" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>2.2355460000000003</v>
+        <v>1.7918459999999998</v>
       </c>
       <c r="R39" s="159"/>
       <c r="S39" s="88">
@@ -47482,11 +47595,11 @@
       <c r="X39" s="132"/>
       <c r="Y39" s="154">
         <f t="shared" ref="Y39:Y74" si="22">M39+P39+S39+V39</f>
-        <v>5828952</v>
+        <v>5385252</v>
       </c>
       <c r="Z39" s="168">
         <f t="shared" ref="Z39:Z74" si="23">(N39+Q39+T39+W39)</f>
-        <v>5.828952000000001</v>
+        <v>5.3852520000000004</v>
       </c>
       <c r="AB39" s="131"/>
     </row>
@@ -47977,11 +48090,11 @@
       <c r="O45" s="215"/>
       <c r="P45" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>357863</v>
+        <v>324863</v>
       </c>
       <c r="Q45" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.71572599999999986</v>
+        <v>0.6497259999999998</v>
       </c>
       <c r="R45" s="159"/>
       <c r="S45" s="88">
@@ -47997,11 +48110,11 @@
       <c r="W45" s="72"/>
       <c r="Y45" s="154">
         <f t="shared" si="22"/>
-        <v>1575181</v>
+        <v>1542181</v>
       </c>
       <c r="Z45" s="168">
         <f t="shared" si="23"/>
-        <v>3.1503619999999994</v>
+        <v>3.0843619999999996</v>
       </c>
     </row>
     <row r="46" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -48058,11 +48171,11 @@
       <c r="O46" s="215"/>
       <c r="P46" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1092541</v>
+        <v>907647</v>
       </c>
       <c r="Q46" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>2.185082</v>
+        <v>1.815294</v>
       </c>
       <c r="R46" s="159"/>
       <c r="S46" s="88">
@@ -48079,11 +48192,11 @@
       <c r="X46" s="1"/>
       <c r="Y46" s="154">
         <f t="shared" si="22"/>
-        <v>1044803</v>
+        <v>859909</v>
       </c>
       <c r="Z46" s="168">
         <f t="shared" si="23"/>
-        <v>2.0896059999999999</v>
+        <v>1.7198179999999998</v>
       </c>
       <c r="AA46" s="1"/>
     </row>
@@ -48141,11 +48254,11 @@
       <c r="O47" s="215"/>
       <c r="P47" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-265460</v>
+        <v>-276885</v>
       </c>
       <c r="Q47" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-5.3091999999999997</v>
+        <v>-5.5377000000000001</v>
       </c>
       <c r="R47" s="159"/>
       <c r="S47" s="88">
@@ -48161,11 +48274,11 @@
       <c r="W47" s="72"/>
       <c r="Y47" s="154">
         <f t="shared" si="22"/>
-        <v>-148565</v>
+        <v>-159990</v>
       </c>
       <c r="Z47" s="168">
         <f t="shared" si="23"/>
-        <v>-2.9712999999999998</v>
+        <v>-3.1998000000000002</v>
       </c>
       <c r="AD47" s="1"/>
       <c r="AE47" s="1"/>
@@ -48310,11 +48423,11 @@
       <c r="O49" s="215"/>
       <c r="P49" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>49764</v>
+        <v>43456</v>
       </c>
       <c r="Q49" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.2441000000000002</v>
+        <v>1.0864</v>
       </c>
       <c r="R49" s="159"/>
       <c r="S49" s="88">
@@ -48330,11 +48443,11 @@
       <c r="W49" s="72"/>
       <c r="Y49" s="154">
         <f t="shared" si="22"/>
-        <v>37936</v>
+        <v>31628</v>
       </c>
       <c r="Z49" s="168">
         <f t="shared" si="23"/>
-        <v>0.94840000000000013</v>
+        <v>0.79069999999999996</v>
       </c>
       <c r="AD49"/>
       <c r="AE49"/>
@@ -48565,11 +48678,11 @@
       <c r="O52" s="215"/>
       <c r="P52" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>579373</v>
+        <v>547783</v>
       </c>
       <c r="Q52" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.4484325</v>
+        <v>1.3694575000000002</v>
       </c>
       <c r="R52" s="159"/>
       <c r="S52" s="88">
@@ -48585,11 +48698,11 @@
       <c r="W52" s="72"/>
       <c r="Y52" s="154">
         <f t="shared" si="22"/>
-        <v>179074</v>
+        <v>147484</v>
       </c>
       <c r="Z52" s="168">
         <f t="shared" si="23"/>
-        <v>0.44768499999999989</v>
+        <v>0.36871000000000009</v>
       </c>
     </row>
     <row r="53" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -48646,11 +48759,11 @@
       <c r="O53" s="215"/>
       <c r="P53" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>12353</v>
+        <v>42553</v>
       </c>
       <c r="Q53" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.12352999999999992</v>
+        <v>0.42552999999999996</v>
       </c>
       <c r="R53" s="159"/>
       <c r="S53" s="88">
@@ -48666,11 +48779,11 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="154">
         <f t="shared" si="22"/>
-        <v>758146</v>
+        <v>788346</v>
       </c>
       <c r="Z53" s="168">
         <f t="shared" si="23"/>
-        <v>7.5814600000000008</v>
+        <v>7.8834600000000012</v>
       </c>
     </row>
     <row r="54" spans="1:34" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -48808,11 +48921,11 @@
       <c r="O55" s="215"/>
       <c r="P55" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-79578</v>
+        <v>-26966</v>
       </c>
       <c r="Q55" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1.5915599999999999</v>
+        <v>-0.5393199999999998</v>
       </c>
       <c r="R55" s="159"/>
       <c r="S55" s="153">
@@ -48829,11 +48942,11 @@
       <c r="X55" s="132"/>
       <c r="Y55" s="154">
         <f t="shared" si="22"/>
-        <v>-325356</v>
+        <v>-272744</v>
       </c>
       <c r="Z55" s="168">
         <f t="shared" si="23"/>
-        <v>-6.5071200000000005</v>
+        <v>-5.4548800000000002</v>
       </c>
       <c r="AA55" s="132"/>
     </row>
@@ -48891,11 +49004,11 @@
       <c r="O56" s="215"/>
       <c r="P56" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-138684</v>
+        <v>-183198</v>
       </c>
       <c r="Q56" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-0.46228000000000002</v>
+        <v>-0.61065999999999998</v>
       </c>
       <c r="R56" s="159"/>
       <c r="S56" s="88">
@@ -48911,11 +49024,11 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="154">
         <f t="shared" si="22"/>
-        <v>-4837659</v>
+        <v>-4882173</v>
       </c>
       <c r="Z56" s="168">
         <f t="shared" si="23"/>
-        <v>-16.125530000000005</v>
+        <v>-16.273910000000004</v>
       </c>
       <c r="AB56" s="132"/>
       <c r="AC56" s="132"/>
@@ -49145,11 +49258,11 @@
       <c r="O59" s="215"/>
       <c r="P59" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>27950</v>
+        <v>20595</v>
       </c>
       <c r="Q59" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.2384</v>
+        <v>9.1299999999999992E-2</v>
       </c>
       <c r="R59" s="159"/>
       <c r="S59" s="88">
@@ -49166,11 +49279,11 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="154">
         <f t="shared" si="22"/>
-        <v>64673</v>
+        <v>57318</v>
       </c>
       <c r="Z59" s="168">
         <f t="shared" si="23"/>
-        <v>0.56723333333333326</v>
+        <v>0.4201333333333333</v>
       </c>
       <c r="AB59" s="1"/>
       <c r="AC59" s="1"/>
@@ -49234,11 +49347,11 @@
       <c r="O60" s="215"/>
       <c r="P60" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>424021</v>
+        <v>449421</v>
       </c>
       <c r="Q60" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>4.2402099999999994</v>
+        <v>4.4942099999999998</v>
       </c>
       <c r="R60" s="159"/>
       <c r="S60" s="88">
@@ -49254,11 +49367,11 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="154">
         <f t="shared" si="22"/>
-        <v>3974090</v>
+        <v>3999490</v>
       </c>
       <c r="Z60" s="168">
         <f t="shared" si="23"/>
-        <v>39.740899999999996</v>
+        <v>39.994900000000001</v>
       </c>
       <c r="AB60" s="132"/>
       <c r="AC60" s="132"/>
@@ -49320,11 +49433,11 @@
       <c r="O61" s="215"/>
       <c r="P61" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>3701</v>
+        <v>4235</v>
       </c>
       <c r="Q61" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.37009999999999998</v>
+        <v>0.42349999999999999</v>
       </c>
       <c r="R61" s="159"/>
       <c r="S61" s="153">
@@ -49340,11 +49453,11 @@
       <c r="W61" s="150"/>
       <c r="Y61" s="154">
         <f t="shared" ref="Y61" si="37">M61+P61+S61+V61</f>
-        <v>3701</v>
+        <v>4235</v>
       </c>
       <c r="Z61" s="168">
         <f t="shared" ref="Z61" si="38">(N61+Q61+T61+W61)</f>
-        <v>0.37009999999999998</v>
+        <v>0.42349999999999999</v>
       </c>
     </row>
     <row r="62" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -49401,11 +49514,11 @@
       <c r="O62" s="215"/>
       <c r="P62" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>367458</v>
+        <v>155985</v>
       </c>
       <c r="Q62" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.2248600000000001</v>
+        <v>0.51995000000000002</v>
       </c>
       <c r="R62" s="159"/>
       <c r="S62" s="88">
@@ -49421,11 +49534,11 @@
       <c r="W62" s="72"/>
       <c r="Y62" s="154">
         <f t="shared" si="22"/>
-        <v>1040307</v>
+        <v>828834</v>
       </c>
       <c r="Z62" s="168">
         <f t="shared" si="23"/>
-        <v>3.4676899999999997</v>
+        <v>2.7627799999999998</v>
       </c>
       <c r="AB62" s="1"/>
       <c r="AC62" s="1"/>
@@ -49489,11 +49602,11 @@
       <c r="O63" s="215"/>
       <c r="P63" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>289577</v>
+        <v>247073</v>
       </c>
       <c r="Q63" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.72394249999999993</v>
+        <v>0.61768250000000002</v>
       </c>
       <c r="R63" s="159"/>
       <c r="S63" s="88">
@@ -49509,11 +49622,11 @@
       <c r="W63" s="72"/>
       <c r="Y63" s="154">
         <f t="shared" si="22"/>
-        <v>964577</v>
+        <v>922073</v>
       </c>
       <c r="Z63" s="168">
         <f t="shared" si="23"/>
-        <v>2.4114424999999997</v>
+        <v>2.3051824999999999</v>
       </c>
     </row>
     <row r="64" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -49814,11 +49927,11 @@
       <c r="O67" s="215"/>
       <c r="P67" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1688416</v>
+        <v>-1469416</v>
       </c>
       <c r="Q67" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1.6885159999999999</v>
+        <v>-1.469516</v>
       </c>
       <c r="R67" s="159"/>
       <c r="S67" s="153">
@@ -49834,11 +49947,11 @@
       <c r="W67" s="150"/>
       <c r="Y67" s="154">
         <f t="shared" ref="Y67" si="43">M67+P67+S67+V67</f>
-        <v>-1688416</v>
+        <v>-1469416</v>
       </c>
       <c r="Z67" s="168">
         <f t="shared" ref="Z67" si="44">(N67+Q67+T67+W67)</f>
-        <v>-1.6885159999999999</v>
+        <v>-1.469516</v>
       </c>
     </row>
     <row r="68" spans="1:26" s="132" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -49952,11 +50065,11 @@
       <c r="O69" s="215"/>
       <c r="P69" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-3725</v>
+        <v>373</v>
       </c>
       <c r="Q69" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-7.44999999999999E-2</v>
+        <v>7.4600000000000222E-3</v>
       </c>
       <c r="R69" s="159"/>
       <c r="S69" s="153">
@@ -49972,11 +50085,11 @@
       <c r="W69" s="150"/>
       <c r="Y69" s="154">
         <f t="shared" si="22"/>
-        <v>-50379</v>
+        <v>-46281</v>
       </c>
       <c r="Z69" s="168">
         <f t="shared" si="23"/>
-        <v>-1.0075799999999999</v>
+        <v>-0.92562</v>
       </c>
     </row>
     <row r="70" spans="1:26" x14ac:dyDescent="0.25">
@@ -50033,11 +50146,11 @@
       <c r="O70" s="215"/>
       <c r="P70" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>325731</v>
+        <v>362071</v>
       </c>
       <c r="Q70" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.3445140384615386</v>
+        <v>1.4004217307692308</v>
       </c>
       <c r="R70" s="159"/>
       <c r="S70" s="153">
@@ -50053,11 +50166,11 @@
       <c r="W70" s="150"/>
       <c r="Y70" s="154">
         <f t="shared" si="22"/>
-        <v>-82221</v>
+        <v>-45881</v>
       </c>
       <c r="Z70" s="168">
         <f t="shared" si="23"/>
-        <v>0.32463403846153849</v>
+        <v>0.3805417307692307</v>
       </c>
     </row>
     <row r="71" spans="1:26" x14ac:dyDescent="0.25">
@@ -50276,11 +50389,11 @@
       <c r="O73" s="215"/>
       <c r="P73" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>529557</v>
+        <v>486723</v>
       </c>
       <c r="Q73" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>1.7651900000000003</v>
+        <v>1.6224100000000004</v>
       </c>
       <c r="R73" s="159"/>
       <c r="S73" s="88">
@@ -50296,11 +50409,11 @@
       <c r="W73" s="72"/>
       <c r="Y73" s="154">
         <f t="shared" si="22"/>
-        <v>362175</v>
+        <v>319341</v>
       </c>
       <c r="Z73" s="168">
         <f t="shared" si="23"/>
-        <v>1.2072500000000002</v>
+        <v>1.0644700000000005</v>
       </c>
     </row>
     <row r="74" spans="1:26" x14ac:dyDescent="0.25">
@@ -50515,11 +50628,11 @@
       <c r="O76" s="215"/>
       <c r="P76" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>498033</v>
+        <v>512183</v>
       </c>
       <c r="Q76" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>0.99606600000000001</v>
+        <v>1.0243659999999999</v>
       </c>
       <c r="R76" s="159"/>
       <c r="S76" s="153">
@@ -50535,11 +50648,11 @@
       <c r="W76" s="150"/>
       <c r="Y76" s="154">
         <f t="shared" si="53"/>
-        <v>498033</v>
+        <v>512183</v>
       </c>
       <c r="Z76" s="168">
         <f t="shared" si="54"/>
-        <v>0.99606600000000001</v>
+        <v>1.0243659999999999</v>
       </c>
     </row>
     <row r="77" spans="1:26" x14ac:dyDescent="0.25">
@@ -50572,7 +50685,7 @@
       <c r="O77" s="122"/>
       <c r="P77" s="109">
         <f>SUM(P4:P74)</f>
-        <v>5739364</v>
+        <v>4751570</v>
       </c>
       <c r="Q77" s="122"/>
       <c r="R77" s="122"/>
@@ -50583,7 +50696,7 @@
       <c r="W77" s="50"/>
       <c r="Y77" s="154">
         <f>SUM(Y4:Y76)</f>
-        <v>25686497</v>
+        <v>24712853</v>
       </c>
       <c r="Z77" s="161"/>
     </row>
@@ -50879,11 +50992,11 @@
       <c r="O82" s="167"/>
       <c r="P82" s="153">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-29043</v>
+        <v>-130193</v>
       </c>
       <c r="Q82" s="155">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-9.6809999999999174E-2</v>
+        <v>-0.43397666666666623</v>
       </c>
       <c r="R82" s="159"/>
       <c r="S82" s="153">
@@ -50900,11 +51013,11 @@
       <c r="X82" s="132"/>
       <c r="Y82" s="52">
         <f t="shared" si="56"/>
-        <v>182457</v>
+        <v>81307</v>
       </c>
       <c r="Z82" s="53">
         <f t="shared" si="56"/>
-        <v>-9.6809999999999174E-2</v>
+        <v>-0.43397666666666623</v>
       </c>
       <c r="AA82" s="132"/>
     </row>
@@ -51014,7 +51127,7 @@
       <c r="O84" s="123"/>
       <c r="P84" s="112">
         <f>SUM(P80:P83)</f>
-        <v>1227108</v>
+        <v>1125958</v>
       </c>
       <c r="Q84" s="123"/>
       <c r="R84" s="123"/>

</xml_diff>

<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Fri 10/09/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3236" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3237" uniqueCount="332">
   <si>
     <t>Sudeep</t>
   </si>
@@ -1020,6 +1020,9 @@
   </si>
   <si>
     <t>DEC ROI</t>
+  </si>
+  <si>
+    <t>P3445</t>
   </si>
 </sst>
 </file>
@@ -6740,15 +6743,17 @@
       <c r="K4" s="157">
         <v>29052</v>
       </c>
-      <c r="L4" s="157"/>
+      <c r="L4" s="157">
+        <v>42300</v>
+      </c>
       <c r="M4" s="210"/>
       <c r="N4" s="170">
         <f t="shared" ref="N4:N35" si="0">SUM(H4:M4)</f>
-        <v>44320</v>
+        <v>86620</v>
       </c>
       <c r="O4" s="148">
         <f t="shared" ref="O4:O35" si="1">IFERROR(N4/F4*100,0)/10000000</f>
-        <v>0.88639999999999997</v>
+        <v>1.7323999999999999</v>
       </c>
       <c r="V4" s="132" t="s">
         <v>170</v>
@@ -6789,15 +6794,17 @@
       <c r="K5" s="146">
         <v>94938</v>
       </c>
-      <c r="L5" s="146"/>
+      <c r="L5" s="146">
+        <v>96755</v>
+      </c>
       <c r="M5" s="173"/>
       <c r="N5" s="170">
         <f t="shared" si="0"/>
-        <v>94140</v>
+        <v>190895</v>
       </c>
       <c r="O5" s="148">
         <f t="shared" si="1"/>
-        <v>0.31380000000000002</v>
+        <v>0.63631666666666664</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
@@ -6832,15 +6839,17 @@
       <c r="K6" s="146">
         <v>50440</v>
       </c>
-      <c r="L6" s="146"/>
+      <c r="L6" s="146">
+        <v>44170</v>
+      </c>
       <c r="M6" s="173"/>
       <c r="N6" s="170">
         <f t="shared" si="0"/>
-        <v>27367</v>
+        <v>71537</v>
       </c>
       <c r="O6" s="148">
         <f t="shared" si="1"/>
-        <v>0.27367000000000002</v>
+        <v>0.71536999999999995</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6875,15 +6884,17 @@
       <c r="K7" s="146">
         <v>-140210</v>
       </c>
-      <c r="L7" s="146"/>
+      <c r="L7" s="146">
+        <v>-117400</v>
+      </c>
       <c r="M7" s="173"/>
       <c r="N7" s="170">
         <f t="shared" si="0"/>
-        <v>-207210</v>
+        <v>-324610</v>
       </c>
       <c r="O7" s="148">
         <f t="shared" si="1"/>
-        <v>-0.69069999999999998</v>
+        <v>-1.0820333333333332</v>
       </c>
       <c r="Q7" s="5"/>
       <c r="R7" s="133">
@@ -6922,15 +6933,17 @@
       <c r="K8" s="146">
         <v>18290</v>
       </c>
-      <c r="L8" s="146"/>
+      <c r="L8" s="146">
+        <v>11000</v>
+      </c>
       <c r="M8" s="173"/>
       <c r="N8" s="170">
         <f t="shared" si="0"/>
-        <v>108340</v>
+        <v>119340</v>
       </c>
       <c r="O8" s="148">
         <f t="shared" si="1"/>
-        <v>0.72226666666666672</v>
+        <v>0.79559999999999997</v>
       </c>
       <c r="Q8" s="133">
         <v>468159</v>
@@ -6967,15 +6980,17 @@
       <c r="K9" s="146">
         <v>4948</v>
       </c>
-      <c r="L9" s="146"/>
+      <c r="L9" s="146">
+        <v>25000</v>
+      </c>
       <c r="M9" s="173"/>
       <c r="N9" s="170">
         <f t="shared" si="0"/>
-        <v>42214</v>
+        <v>67214</v>
       </c>
       <c r="O9" s="148">
         <f t="shared" si="1"/>
-        <v>0.70356666666666667</v>
+        <v>1.1202333333333334</v>
       </c>
       <c r="Q9" s="133">
         <v>453904</v>
@@ -7017,7 +7032,9 @@
       <c r="K10" s="146">
         <v>13730</v>
       </c>
-      <c r="L10" s="146"/>
+      <c r="L10" s="146">
+        <v>0</v>
+      </c>
       <c r="M10" s="173"/>
       <c r="N10" s="170">
         <f t="shared" si="0"/>
@@ -7062,15 +7079,17 @@
       <c r="K11" s="146">
         <v>0</v>
       </c>
-      <c r="L11" s="146"/>
+      <c r="L11" s="146">
+        <v>55700</v>
+      </c>
       <c r="M11" s="173"/>
       <c r="N11" s="170">
         <f t="shared" si="0"/>
-        <v>170431</v>
+        <v>226131</v>
       </c>
       <c r="O11" s="148">
         <f t="shared" si="1"/>
-        <v>0.2840516666666667</v>
+        <v>0.37688500000000003</v>
       </c>
       <c r="Q11" s="133"/>
       <c r="R11" s="133"/>
@@ -7107,15 +7126,17 @@
       <c r="K12" s="146">
         <v>-1616</v>
       </c>
-      <c r="L12" s="146"/>
+      <c r="L12" s="146">
+        <v>-2953</v>
+      </c>
       <c r="M12" s="173"/>
       <c r="N12" s="170">
         <f t="shared" si="0"/>
-        <v>-1938</v>
+        <v>-4891</v>
       </c>
       <c r="O12" s="148">
         <f t="shared" si="1"/>
-        <v>-1.9380000000000001E-2</v>
+        <v>-4.8910000000000002E-2</v>
       </c>
       <c r="Q12" s="133"/>
       <c r="R12" s="133"/>
@@ -7152,15 +7173,17 @@
       <c r="K13" s="146">
         <v>0</v>
       </c>
-      <c r="L13" s="146"/>
+      <c r="L13" s="146">
+        <v>22700</v>
+      </c>
       <c r="M13" s="173"/>
       <c r="N13" s="170">
         <f t="shared" si="0"/>
-        <v>68353</v>
+        <v>91053</v>
       </c>
       <c r="O13" s="148">
         <f t="shared" si="1"/>
-        <v>0.27341199999999999</v>
+        <v>0.36421199999999998</v>
       </c>
       <c r="Q13" s="133"/>
       <c r="R13" s="133"/>
@@ -7197,15 +7220,17 @@
       <c r="K14" s="146">
         <v>0</v>
       </c>
-      <c r="L14" s="146"/>
+      <c r="L14" s="146">
+        <v>30900</v>
+      </c>
       <c r="M14" s="173"/>
       <c r="N14" s="170">
         <f t="shared" si="0"/>
-        <v>77903</v>
+        <v>108803</v>
       </c>
       <c r="O14" s="148">
         <f t="shared" si="1"/>
-        <v>0.35410454545454545</v>
+        <v>0.49455909090909089</v>
       </c>
       <c r="Q14" s="133"/>
       <c r="R14" s="192">
@@ -7252,15 +7277,17 @@
       <c r="K15" s="146">
         <v>-6218</v>
       </c>
-      <c r="L15" s="146"/>
+      <c r="L15" s="146">
+        <v>-30200</v>
+      </c>
       <c r="M15" s="173"/>
       <c r="N15" s="170">
         <f t="shared" si="0"/>
-        <v>14282</v>
+        <v>-15918</v>
       </c>
       <c r="O15" s="148">
         <f t="shared" si="1"/>
-        <v>0.14282</v>
+        <v>-0.15917999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
@@ -7295,7 +7322,9 @@
       <c r="K16" s="146">
         <v>0</v>
       </c>
-      <c r="L16" s="146"/>
+      <c r="L16" s="146">
+        <v>0</v>
+      </c>
       <c r="M16" s="173"/>
       <c r="N16" s="170">
         <f t="shared" si="0"/>
@@ -7349,7 +7378,9 @@
       <c r="K17" s="146">
         <v>0</v>
       </c>
-      <c r="L17" s="146"/>
+      <c r="L17" s="146">
+        <v>0</v>
+      </c>
       <c r="M17" s="173"/>
       <c r="N17" s="170">
         <f t="shared" si="0"/>
@@ -7396,15 +7427,17 @@
       <c r="K18" s="146">
         <v>-95099</v>
       </c>
-      <c r="L18" s="146"/>
+      <c r="L18" s="146">
+        <v>141000</v>
+      </c>
       <c r="M18" s="173"/>
       <c r="N18" s="170">
         <f t="shared" si="0"/>
-        <v>-50285</v>
+        <v>90715</v>
       </c>
       <c r="O18" s="148">
         <f t="shared" si="1"/>
-        <v>-0.33523333333333333</v>
+        <v>0.60476666666666656</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
@@ -7439,7 +7472,9 @@
       <c r="K19" s="146">
         <v>0</v>
       </c>
-      <c r="L19" s="146"/>
+      <c r="L19" s="146">
+        <v>0</v>
+      </c>
       <c r="M19" s="173"/>
       <c r="N19" s="170">
         <f t="shared" si="0"/>
@@ -7485,15 +7520,17 @@
       <c r="K20" s="146">
         <v>7212</v>
       </c>
-      <c r="L20" s="146"/>
+      <c r="L20" s="146">
+        <v>-17400</v>
+      </c>
       <c r="M20" s="173"/>
       <c r="N20" s="170">
         <f t="shared" si="0"/>
-        <v>-68242</v>
+        <v>-85642</v>
       </c>
       <c r="O20" s="148">
         <f t="shared" si="1"/>
-        <v>-2.7296800000000001</v>
+        <v>-3.4256799999999998</v>
       </c>
       <c r="S20" s="132">
         <v>-52140</v>
@@ -7531,7 +7568,9 @@
       <c r="K21" s="146">
         <v>0</v>
       </c>
-      <c r="L21" s="146"/>
+      <c r="L21" s="146">
+        <v>0</v>
+      </c>
       <c r="M21" s="173"/>
       <c r="N21" s="170">
         <f t="shared" si="0"/>
@@ -7577,7 +7616,9 @@
       <c r="K22" s="146">
         <v>0</v>
       </c>
-      <c r="L22" s="146"/>
+      <c r="L22" s="146">
+        <v>0</v>
+      </c>
       <c r="M22" s="173"/>
       <c r="N22" s="170">
         <f t="shared" si="0"/>
@@ -7620,15 +7661,17 @@
       <c r="K23" s="146">
         <v>38700</v>
       </c>
-      <c r="L23" s="146"/>
+      <c r="L23" s="146">
+        <v>-1623</v>
+      </c>
       <c r="M23" s="173"/>
       <c r="N23" s="170">
         <f t="shared" si="0"/>
-        <v>28323</v>
+        <v>26700</v>
       </c>
       <c r="O23" s="148">
         <f t="shared" si="1"/>
-        <v>0.25748181818181815</v>
+        <v>0.24272727272727271</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
@@ -7663,15 +7706,17 @@
       <c r="K24" s="146">
         <v>-128600</v>
       </c>
-      <c r="L24" s="146"/>
+      <c r="L24" s="146">
+        <v>-381800</v>
+      </c>
       <c r="M24" s="173"/>
       <c r="N24" s="170">
         <f t="shared" si="0"/>
-        <v>-61800</v>
+        <v>-443600</v>
       </c>
       <c r="O24" s="148">
         <f t="shared" si="1"/>
-        <v>-0.26869565217391306</v>
+        <v>-1.9286956521739134</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
@@ -7704,15 +7749,17 @@
       <c r="K25" s="146">
         <v>-2835</v>
       </c>
-      <c r="L25" s="146"/>
+      <c r="L25" s="146">
+        <v>10900</v>
+      </c>
       <c r="M25" s="173"/>
       <c r="N25" s="170">
         <f t="shared" si="0"/>
-        <v>-109</v>
+        <v>10791</v>
       </c>
       <c r="O25" s="148">
         <f t="shared" si="1"/>
-        <v>-5.45E-3</v>
+        <v>0.53954999999999997</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
@@ -7747,7 +7794,9 @@
       <c r="K26" s="146">
         <v>0</v>
       </c>
-      <c r="L26" s="146"/>
+      <c r="L26" s="146">
+        <v>0</v>
+      </c>
       <c r="M26" s="173"/>
       <c r="N26" s="170">
         <f t="shared" si="0"/>
@@ -7790,15 +7839,17 @@
       <c r="K27" s="146">
         <v>302380</v>
       </c>
-      <c r="L27" s="146"/>
+      <c r="L27" s="146">
+        <v>55800</v>
+      </c>
       <c r="M27" s="173"/>
       <c r="N27" s="170">
         <f t="shared" si="0"/>
-        <v>412715</v>
+        <v>468515</v>
       </c>
       <c r="O27" s="148">
         <f t="shared" si="1"/>
-        <v>0.412715</v>
+        <v>0.46851500000000001</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
@@ -7833,15 +7884,17 @@
       <c r="K28" s="146">
         <v>0</v>
       </c>
-      <c r="L28" s="146"/>
+      <c r="L28" s="146">
+        <v>155700</v>
+      </c>
       <c r="M28" s="173"/>
       <c r="N28" s="170">
         <f t="shared" si="0"/>
-        <v>401130</v>
+        <v>556830</v>
       </c>
       <c r="O28" s="148">
         <f t="shared" si="1"/>
-        <v>0.80225999999999997</v>
+        <v>1.1136600000000001</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.25">
@@ -7876,15 +7929,17 @@
       <c r="K29" s="146">
         <v>2600</v>
       </c>
-      <c r="L29" s="146"/>
+      <c r="L29" s="146">
+        <v>44000</v>
+      </c>
       <c r="M29" s="173"/>
       <c r="N29" s="170">
         <f t="shared" si="0"/>
-        <v>-108150</v>
+        <v>-64150</v>
       </c>
       <c r="O29" s="148">
         <f t="shared" si="1"/>
-        <v>-0.21629999999999999</v>
+        <v>-0.1283</v>
       </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
@@ -7919,15 +7974,17 @@
       <c r="K30" s="146">
         <v>-7694</v>
       </c>
-      <c r="L30" s="146"/>
+      <c r="L30" s="146">
+        <v>34100</v>
+      </c>
       <c r="M30" s="173"/>
       <c r="N30" s="170">
         <f t="shared" si="0"/>
-        <v>3799</v>
+        <v>37899</v>
       </c>
       <c r="O30" s="148">
         <f t="shared" si="1"/>
-        <v>7.5980000000000006E-2</v>
+        <v>0.75797999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
@@ -7962,15 +8019,17 @@
       <c r="K31" s="146">
         <v>1293</v>
       </c>
-      <c r="L31" s="146"/>
+      <c r="L31" s="146">
+        <v>33700</v>
+      </c>
       <c r="M31" s="173"/>
       <c r="N31" s="170">
         <f t="shared" si="0"/>
-        <v>81468</v>
+        <v>115168</v>
       </c>
       <c r="O31" s="148">
         <f t="shared" si="1"/>
-        <v>2.0367000000000002</v>
+        <v>2.8792</v>
       </c>
       <c r="R31" s="133"/>
     </row>
@@ -8006,15 +8065,17 @@
       <c r="K32" s="146">
         <v>-98197</v>
       </c>
-      <c r="L32" s="146"/>
+      <c r="L32" s="146">
+        <v>149600</v>
+      </c>
       <c r="M32" s="173"/>
       <c r="N32" s="170">
         <f t="shared" si="0"/>
-        <v>-147529</v>
+        <v>2071</v>
       </c>
       <c r="O32" s="148">
         <f t="shared" si="1"/>
-        <v>-0.3688225</v>
+        <v>5.1774999999999998E-3</v>
       </c>
       <c r="Q32" s="5"/>
       <c r="R32" s="133">
@@ -8053,15 +8114,17 @@
       <c r="K33" s="146">
         <v>-13148</v>
       </c>
-      <c r="L33" s="146"/>
+      <c r="L33" s="146">
+        <v>-107400</v>
+      </c>
       <c r="M33" s="173"/>
       <c r="N33" s="170">
         <f t="shared" si="0"/>
-        <v>9674</v>
+        <v>-97726</v>
       </c>
       <c r="O33" s="148">
         <f t="shared" si="1"/>
-        <v>9.6740000000000007E-2</v>
+        <v>-0.97726000000000002</v>
       </c>
       <c r="Q33" s="5"/>
       <c r="R33" s="133"/>
@@ -8096,7 +8159,9 @@
       <c r="K34" s="146">
         <v>0</v>
       </c>
-      <c r="L34" s="146"/>
+      <c r="L34" s="146">
+        <v>0</v>
+      </c>
       <c r="M34" s="173"/>
       <c r="N34" s="170">
         <f t="shared" si="0"/>
@@ -8146,15 +8211,17 @@
       <c r="K35" s="146">
         <v>-15524</v>
       </c>
-      <c r="L35" s="146"/>
+      <c r="L35" s="146">
+        <v>23400</v>
+      </c>
       <c r="M35" s="173"/>
       <c r="N35" s="170">
         <f t="shared" si="0"/>
-        <v>-8895</v>
+        <v>14505</v>
       </c>
       <c r="O35" s="148">
         <f t="shared" si="1"/>
-        <v>-0.1779</v>
+        <v>0.29010000000000002</v>
       </c>
       <c r="Q35" s="133">
         <v>604754</v>
@@ -8193,15 +8260,17 @@
       <c r="K36" s="146">
         <v>79524</v>
       </c>
-      <c r="L36" s="146"/>
+      <c r="L36" s="146">
+        <v>-8546</v>
+      </c>
       <c r="M36" s="173"/>
       <c r="N36" s="170">
         <f t="shared" ref="N36:N67" si="2">SUM(H36:M36)</f>
-        <v>183624</v>
+        <v>175078</v>
       </c>
       <c r="O36" s="148">
         <f t="shared" ref="O36:O67" si="3">IFERROR(N36/F36*100,0)/10000000</f>
-        <v>0.61207999999999996</v>
+        <v>0.58359333333333341</v>
       </c>
       <c r="Q36" s="133"/>
       <c r="R36" s="133">
@@ -8239,15 +8308,17 @@
       <c r="K37" s="146">
         <v>-19285</v>
       </c>
-      <c r="L37" s="146"/>
+      <c r="L37" s="146">
+        <v>59000</v>
+      </c>
       <c r="M37" s="173"/>
       <c r="N37" s="170">
         <f t="shared" si="2"/>
-        <v>6368</v>
+        <v>65368</v>
       </c>
       <c r="O37" s="148">
         <f t="shared" si="3"/>
-        <v>0.63680000000000003</v>
+        <v>6.5368000000000004</v>
       </c>
       <c r="Q37" s="133"/>
       <c r="R37" s="133"/>
@@ -8284,15 +8355,17 @@
       <c r="K38" s="146">
         <v>-16500</v>
       </c>
-      <c r="L38" s="146"/>
+      <c r="L38" s="146">
+        <v>26900</v>
+      </c>
       <c r="M38" s="173"/>
       <c r="N38" s="170">
         <f t="shared" si="2"/>
-        <v>3300</v>
+        <v>30200</v>
       </c>
       <c r="O38" s="148">
         <f t="shared" si="3"/>
-        <v>6.6000000000000003E-2</v>
+        <v>0.60399999999999998</v>
       </c>
       <c r="Q38" s="133"/>
       <c r="R38" s="133"/>
@@ -8329,15 +8402,17 @@
       <c r="K39" s="146">
         <v>-85245</v>
       </c>
-      <c r="L39" s="146"/>
+      <c r="L39" s="146">
+        <v>-484000</v>
+      </c>
       <c r="M39" s="173"/>
       <c r="N39" s="170">
         <f t="shared" si="2"/>
-        <v>-171229</v>
+        <v>-655229</v>
       </c>
       <c r="O39" s="148">
         <f t="shared" si="3"/>
-        <v>-1.7122900000000001</v>
+        <v>-6.5522900000000002</v>
       </c>
       <c r="Q39" s="133"/>
       <c r="R39" s="133"/>
@@ -8372,15 +8447,17 @@
       <c r="K40" s="146">
         <v>-21500</v>
       </c>
-      <c r="L40" s="146"/>
+      <c r="L40" s="146">
+        <v>18000</v>
+      </c>
       <c r="M40" s="173"/>
       <c r="N40" s="170">
         <f t="shared" si="2"/>
-        <v>-17235</v>
+        <v>765</v>
       </c>
       <c r="O40" s="148">
         <f t="shared" si="3"/>
-        <v>-1.7235</v>
+        <v>7.6499999999999999E-2</v>
       </c>
       <c r="Q40" s="133"/>
     </row>
@@ -8416,15 +8493,17 @@
       <c r="K41" s="146">
         <v>0</v>
       </c>
-      <c r="L41" s="146"/>
+      <c r="L41" s="146">
+        <v>52100</v>
+      </c>
       <c r="M41" s="173"/>
       <c r="N41" s="170">
         <f t="shared" si="2"/>
-        <v>2920</v>
+        <v>55020</v>
       </c>
       <c r="O41" s="148">
         <f t="shared" si="3"/>
-        <v>7.3000000000000001E-3</v>
+        <v>0.13755000000000001</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
@@ -8459,7 +8538,9 @@
       <c r="K42" s="146">
         <v>0</v>
       </c>
-      <c r="L42" s="146"/>
+      <c r="L42" s="146">
+        <v>0</v>
+      </c>
       <c r="M42" s="173"/>
       <c r="N42" s="170">
         <f t="shared" si="2"/>
@@ -8502,15 +8583,17 @@
       <c r="K43" s="146">
         <v>-135130</v>
       </c>
-      <c r="L43" s="146"/>
+      <c r="L43" s="146">
+        <v>290000</v>
+      </c>
       <c r="M43" s="173"/>
       <c r="N43" s="170">
         <f t="shared" si="2"/>
-        <v>33128</v>
+        <v>323128</v>
       </c>
       <c r="O43" s="148">
         <f t="shared" si="3"/>
-        <v>0.11042666666666665</v>
+        <v>1.0770933333333332</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -8543,15 +8626,17 @@
       <c r="K44" s="150">
         <v>63150</v>
       </c>
-      <c r="L44" s="150"/>
+      <c r="L44" s="150">
+        <v>-461500</v>
+      </c>
       <c r="M44" s="173"/>
       <c r="N44" s="170">
         <f t="shared" si="2"/>
-        <v>206750</v>
+        <v>-254750</v>
       </c>
       <c r="O44" s="148">
         <f t="shared" si="3"/>
-        <v>0.20674999999999999</v>
+        <v>-0.25474999999999998</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -8582,7 +8667,9 @@
       <c r="K45" s="150">
         <v>0</v>
       </c>
-      <c r="L45" s="150"/>
+      <c r="L45" s="150">
+        <v>0</v>
+      </c>
       <c r="M45" s="173"/>
       <c r="N45" s="170">
         <f t="shared" si="2"/>
@@ -8625,15 +8712,17 @@
       <c r="K46" s="150">
         <v>30076</v>
       </c>
-      <c r="L46" s="150"/>
+      <c r="L46" s="150">
+        <v>-25200</v>
+      </c>
       <c r="M46" s="173"/>
       <c r="N46" s="170">
         <f t="shared" si="2"/>
-        <v>65485</v>
+        <v>40285</v>
       </c>
       <c r="O46" s="148">
         <f t="shared" si="3"/>
-        <v>1.3097000000000001</v>
+        <v>0.80569999999999997</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -8668,15 +8757,17 @@
       <c r="K47" s="150">
         <v>0</v>
       </c>
-      <c r="L47" s="150"/>
+      <c r="L47" s="150">
+        <v>53400</v>
+      </c>
       <c r="M47" s="173"/>
       <c r="N47" s="170">
         <f t="shared" si="2"/>
-        <v>306496</v>
+        <v>359896</v>
       </c>
       <c r="O47" s="148">
         <f t="shared" si="3"/>
-        <v>0.4715323076923077</v>
+        <v>0.55368615384615383</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
@@ -8711,7 +8802,9 @@
       <c r="K48" s="150">
         <v>0</v>
       </c>
-      <c r="L48" s="150"/>
+      <c r="L48" s="150">
+        <v>0</v>
+      </c>
       <c r="M48" s="173"/>
       <c r="N48" s="170">
         <f t="shared" si="2"/>
@@ -8754,19 +8847,23 @@
       <c r="K49" s="150">
         <v>0</v>
       </c>
-      <c r="L49" s="150"/>
+      <c r="L49" s="150">
+        <v>96100</v>
+      </c>
       <c r="M49" s="173"/>
       <c r="N49" s="170">
         <f t="shared" si="2"/>
-        <v>56120</v>
+        <v>152220</v>
       </c>
       <c r="O49" s="148">
         <f t="shared" si="3"/>
-        <v>0.18706666666666669</v>
+        <v>0.50739999999999996</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A50" s="59"/>
+      <c r="A50" s="59" t="s">
+        <v>331</v>
+      </c>
       <c r="B50" s="59" t="s">
         <v>286</v>
       </c>
@@ -8795,15 +8892,17 @@
       <c r="K50" s="150">
         <v>520</v>
       </c>
-      <c r="L50" s="150"/>
+      <c r="L50" s="150">
+        <v>-800</v>
+      </c>
       <c r="M50" s="173"/>
       <c r="N50" s="170">
         <f t="shared" si="2"/>
-        <v>570</v>
+        <v>-230</v>
       </c>
       <c r="O50" s="148">
         <f t="shared" si="3"/>
-        <v>5.7000000000000002E-3</v>
+        <v>-2.3E-3</v>
       </c>
     </row>
     <row r="51" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8838,15 +8937,17 @@
       <c r="K51" s="150">
         <v>17309</v>
       </c>
-      <c r="L51" s="150"/>
+      <c r="L51" s="150">
+        <v>26900</v>
+      </c>
       <c r="M51" s="173"/>
       <c r="N51" s="170">
         <f t="shared" si="2"/>
-        <v>100956</v>
+        <v>127856</v>
       </c>
       <c r="O51" s="148">
         <f t="shared" si="3"/>
-        <v>0.20191200000000001</v>
+        <v>0.25571199999999999</v>
       </c>
     </row>
     <row r="52" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8875,7 +8976,7 @@
       </c>
       <c r="L52" s="253">
         <f>SUM(L4:L51)</f>
-        <v>0</v>
+        <v>-39697</v>
       </c>
       <c r="M52" s="253">
         <f>SUM(M4:M51)</f>
@@ -8883,7 +8984,7 @@
       </c>
       <c r="N52" s="253">
         <f t="shared" si="2"/>
-        <v>1252672</v>
+        <v>1212975</v>
       </c>
       <c r="O52" s="254">
         <f t="shared" si="3"/>
@@ -8939,15 +9040,17 @@
       <c r="K54" s="161">
         <v>15600</v>
       </c>
-      <c r="L54" s="161"/>
+      <c r="L54" s="161">
+        <v>149000</v>
+      </c>
       <c r="M54" s="245"/>
       <c r="N54" s="246">
         <f>SUM(H54:M54)</f>
-        <v>151126</v>
+        <v>300126</v>
       </c>
       <c r="O54" s="247">
         <f>IFERROR(N54/F54*100,0)/10000000</f>
-        <v>0.50375333333333339</v>
+        <v>1.0004200000000001</v>
       </c>
     </row>
     <row r="55" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8980,7 +9083,9 @@
       <c r="K55" s="161">
         <v>0</v>
       </c>
-      <c r="L55" s="161"/>
+      <c r="L55" s="161">
+        <v>0</v>
+      </c>
       <c r="M55" s="173"/>
       <c r="N55" s="170">
         <f>SUM(H55:M55)</f>
@@ -9017,7 +9122,7 @@
       </c>
       <c r="L56" s="169">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>149000</v>
       </c>
       <c r="M56" s="169">
         <f>SUM(M54:M55)</f>
@@ -9025,7 +9130,7 @@
       </c>
       <c r="N56" s="256">
         <f>SUM(H56:M56)</f>
-        <v>249126</v>
+        <v>398126</v>
       </c>
       <c r="O56" s="172"/>
     </row>
@@ -9502,7 +9607,7 @@
       <c r="R6" s="158"/>
       <c r="S6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>44320</v>
+        <v>86620</v>
       </c>
       <c r="T6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9514,7 +9619,7 @@
       <c r="X6" s="131"/>
       <c r="Y6" s="153">
         <f t="shared" si="0"/>
-        <v>-508154</v>
+        <v>-465854</v>
       </c>
       <c r="Z6" s="167">
         <f t="shared" si="1"/>
@@ -9584,7 +9689,7 @@
       <c r="R7" s="158"/>
       <c r="S7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>94140</v>
+        <v>190895</v>
       </c>
       <c r="T7" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9596,7 +9701,7 @@
       <c r="X7"/>
       <c r="Y7" s="153">
         <f t="shared" si="0"/>
-        <v>1336354</v>
+        <v>1433109</v>
       </c>
       <c r="Z7" s="167">
         <f t="shared" si="1"/>
@@ -9720,7 +9825,7 @@
       <c r="R9" s="158"/>
       <c r="S9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>27367</v>
+        <v>71537</v>
       </c>
       <c r="T9" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9731,7 +9836,7 @@
       <c r="W9" s="149"/>
       <c r="Y9" s="153">
         <f t="shared" ref="Y9" si="6">M9+P9+S9+V9</f>
-        <v>-109019</v>
+        <v>-64849</v>
       </c>
       <c r="Z9" s="167">
         <f t="shared" ref="Z9" si="7">(N9+Q9+T9+W9)</f>
@@ -9801,7 +9906,7 @@
       <c r="R10" s="158"/>
       <c r="S10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-207210</v>
+        <v>-324610</v>
       </c>
       <c r="T10" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9812,7 +9917,7 @@
       <c r="W10" s="72"/>
       <c r="Y10" s="153">
         <f t="shared" si="0"/>
-        <v>-1383277</v>
+        <v>-1500677</v>
       </c>
       <c r="Z10" s="167">
         <f t="shared" si="1"/>
@@ -9882,7 +9987,7 @@
       <c r="R11" s="158"/>
       <c r="S11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>108340</v>
+        <v>119340</v>
       </c>
       <c r="T11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9893,7 +9998,7 @@
       <c r="W11" s="149"/>
       <c r="Y11" s="153">
         <f t="shared" si="0"/>
-        <v>-293535</v>
+        <v>-282535</v>
       </c>
       <c r="Z11" s="167">
         <f t="shared" si="1"/>
@@ -9963,7 +10068,7 @@
       <c r="R12" s="158"/>
       <c r="S12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>42214</v>
+        <v>67214</v>
       </c>
       <c r="T12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -9974,7 +10079,7 @@
       <c r="W12" s="149"/>
       <c r="Y12" s="153">
         <f t="shared" ref="Y12" si="12">M12+P12+S12+V12</f>
-        <v>-47715</v>
+        <v>-22715</v>
       </c>
       <c r="Z12" s="167">
         <f t="shared" ref="Z12" si="13">(N12+Q12+T12+W12)</f>
@@ -10453,7 +10558,7 @@
       <c r="R18" s="158"/>
       <c r="S18" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>170431</v>
+        <v>226131</v>
       </c>
       <c r="T18" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10464,7 +10569,7 @@
       <c r="W18" s="72"/>
       <c r="Y18" s="153">
         <f t="shared" si="0"/>
-        <v>370483</v>
+        <v>426183</v>
       </c>
       <c r="Z18" s="167">
         <f t="shared" si="1"/>
@@ -10534,7 +10639,7 @@
       <c r="R19" s="158"/>
       <c r="S19" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1938</v>
+        <v>-4891</v>
       </c>
       <c r="T19" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10545,7 +10650,7 @@
       <c r="W19" s="149"/>
       <c r="Y19" s="153">
         <f t="shared" si="0"/>
-        <v>637</v>
+        <v>-2316</v>
       </c>
       <c r="Z19" s="167">
         <f t="shared" si="1"/>
@@ -10705,7 +10810,7 @@
       <c r="R21" s="158"/>
       <c r="S21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>68353</v>
+        <v>91053</v>
       </c>
       <c r="T21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10716,7 +10821,7 @@
       <c r="W21" s="72"/>
       <c r="Y21" s="153">
         <f t="shared" si="0"/>
-        <v>-182829</v>
+        <v>-160129</v>
       </c>
       <c r="Z21" s="167">
         <f t="shared" si="1"/>
@@ -10786,7 +10891,7 @@
       <c r="R22" s="158"/>
       <c r="S22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>77903</v>
+        <v>108803</v>
       </c>
       <c r="T22" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10797,7 +10902,7 @@
       <c r="W22" s="72"/>
       <c r="Y22" s="153">
         <f t="shared" si="0"/>
-        <v>-125720</v>
+        <v>-94820</v>
       </c>
       <c r="Z22" s="167">
         <f t="shared" si="1"/>
@@ -10948,7 +11053,7 @@
       <c r="R24" s="158"/>
       <c r="S24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>14282</v>
+        <v>-15918</v>
       </c>
       <c r="T24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10959,7 +11064,7 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="153">
         <f t="shared" si="0"/>
-        <v>1760463</v>
+        <v>1730263</v>
       </c>
       <c r="Z24" s="167">
         <f t="shared" si="1"/>
@@ -11604,7 +11709,7 @@
       <c r="R32" s="158"/>
       <c r="S32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-50285</v>
+        <v>90715</v>
       </c>
       <c r="T32" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11616,7 +11721,7 @@
       <c r="X32"/>
       <c r="Y32" s="153">
         <f t="shared" si="0"/>
-        <v>-536290</v>
+        <v>-395290</v>
       </c>
       <c r="Z32" s="167">
         <f t="shared" si="1"/>
@@ -11767,7 +11872,7 @@
       <c r="R34" s="158"/>
       <c r="S34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>28323</v>
+        <v>26700</v>
       </c>
       <c r="T34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11778,7 +11883,7 @@
       <c r="W34" s="72"/>
       <c r="Y34" s="153">
         <f t="shared" si="0"/>
-        <v>-119304</v>
+        <v>-120927</v>
       </c>
       <c r="Z34" s="167">
         <f t="shared" si="1"/>
@@ -11936,7 +12041,7 @@
       <c r="R36" s="158"/>
       <c r="S36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-61800</v>
+        <v>-443600</v>
       </c>
       <c r="T36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11947,7 +12052,7 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="153">
         <f t="shared" si="0"/>
-        <v>2840826</v>
+        <v>2459026</v>
       </c>
       <c r="Z36" s="167">
         <f t="shared" si="1"/>
@@ -12015,7 +12120,7 @@
       <c r="R37" s="158"/>
       <c r="S37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-109</v>
+        <v>10791</v>
       </c>
       <c r="T37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12026,7 +12131,7 @@
       <c r="W37" s="149"/>
       <c r="Y37" s="153">
         <f t="shared" ref="Y37" si="22">M37+P37+S37+V37</f>
-        <v>-43775</v>
+        <v>-32875</v>
       </c>
       <c r="Z37" s="167">
         <f t="shared" ref="Z37" si="23">(N37+Q37+T37+W37)</f>
@@ -12177,7 +12282,7 @@
       <c r="R39" s="158"/>
       <c r="S39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>412715</v>
+        <v>468515</v>
       </c>
       <c r="T39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12189,7 +12294,7 @@
       <c r="X39" s="131"/>
       <c r="Y39" s="153">
         <f t="shared" ref="Y39:Y74" si="24">M39+P39+S39+V39</f>
-        <v>5693462</v>
+        <v>5749262</v>
       </c>
       <c r="Z39" s="167">
         <f t="shared" ref="Z39:Z74" si="25">(N39+Q39+T39+W39)</f>
@@ -12693,7 +12798,7 @@
       <c r="R45" s="158"/>
       <c r="S45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>401130</v>
+        <v>556830</v>
       </c>
       <c r="T45" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12704,7 +12809,7 @@
       <c r="W45" s="72"/>
       <c r="Y45" s="153">
         <f t="shared" si="24"/>
-        <v>1502008</v>
+        <v>1657708</v>
       </c>
       <c r="Z45" s="167">
         <f t="shared" si="25"/>
@@ -12774,7 +12879,7 @@
       <c r="R46" s="158"/>
       <c r="S46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-108150</v>
+        <v>-64150</v>
       </c>
       <c r="T46" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12786,7 +12891,7 @@
       <c r="X46" s="1"/>
       <c r="Y46" s="153">
         <f t="shared" si="24"/>
-        <v>664721</v>
+        <v>708721</v>
       </c>
       <c r="Z46" s="167">
         <f t="shared" si="25"/>
@@ -12852,12 +12957,12 @@
       </c>
       <c r="Q47" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q2'!$A$4:$ABW$124,MATCH('FY-(26-27)Q1'!$P$2:$Q$2,'FY-(26-27)Q2'!$A$2:$BX$2,0),0),0)</f>
-        <v>-3.9188999999999998</v>
+        <v>-1.9594499999999999</v>
       </c>
       <c r="R47" s="158"/>
       <c r="S47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>3799</v>
+        <v>37899</v>
       </c>
       <c r="T47" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12868,11 +12973,11 @@
       <c r="W47" s="72"/>
       <c r="Y47" s="153">
         <f t="shared" si="24"/>
-        <v>-75251</v>
+        <v>-41151</v>
       </c>
       <c r="Z47" s="167">
         <f t="shared" si="25"/>
-        <v>-1.581</v>
+        <v>0.37844999999999995</v>
       </c>
       <c r="AD47" s="1"/>
       <c r="AE47" s="1"/>
@@ -13026,7 +13131,7 @@
       <c r="R49" s="158"/>
       <c r="S49" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>81468</v>
+        <v>115168</v>
       </c>
       <c r="T49" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13037,7 +13142,7 @@
       <c r="W49" s="72"/>
       <c r="Y49" s="153">
         <f t="shared" si="24"/>
-        <v>149733</v>
+        <v>183433</v>
       </c>
       <c r="Z49" s="167">
         <f t="shared" si="25"/>
@@ -13281,7 +13386,7 @@
       <c r="R52" s="158"/>
       <c r="S52" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-147529</v>
+        <v>2071</v>
       </c>
       <c r="T52" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13292,7 +13397,7 @@
       <c r="W52" s="72"/>
       <c r="Y52" s="153">
         <f t="shared" si="24"/>
-        <v>47532</v>
+        <v>197132</v>
       </c>
       <c r="Z52" s="167">
         <f t="shared" si="25"/>
@@ -13362,7 +13467,7 @@
       <c r="R53" s="158"/>
       <c r="S53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>9674</v>
+        <v>-97726</v>
       </c>
       <c r="T53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13373,7 +13478,7 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="153">
         <f t="shared" si="24"/>
-        <v>669923</v>
+        <v>562523</v>
       </c>
       <c r="Z53" s="167">
         <f t="shared" si="25"/>
@@ -13524,7 +13629,7 @@
       <c r="R55" s="158"/>
       <c r="S55" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-8895</v>
+        <v>14505</v>
       </c>
       <c r="T55" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13536,7 +13641,7 @@
       <c r="X55" s="131"/>
       <c r="Y55" s="153">
         <f t="shared" si="24"/>
-        <v>-282920</v>
+        <v>-259520</v>
       </c>
       <c r="Z55" s="167">
         <f t="shared" si="25"/>
@@ -13607,7 +13712,7 @@
       <c r="R56" s="158"/>
       <c r="S56" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>183624</v>
+        <v>175078</v>
       </c>
       <c r="T56" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13618,7 +13723,7 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="153">
         <f t="shared" si="24"/>
-        <v>-4470711</v>
+        <v>-4479257</v>
       </c>
       <c r="Z56" s="167">
         <f t="shared" si="25"/>
@@ -13861,7 +13966,7 @@
       <c r="R59" s="158"/>
       <c r="S59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>3300</v>
+        <v>30200</v>
       </c>
       <c r="T59" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13873,7 +13978,7 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="153">
         <f t="shared" si="24"/>
-        <v>35991</v>
+        <v>62891</v>
       </c>
       <c r="Z59" s="167">
         <f t="shared" si="25"/>
@@ -13950,7 +14055,7 @@
       <c r="R60" s="158"/>
       <c r="S60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-171229</v>
+        <v>-655229</v>
       </c>
       <c r="T60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13961,7 +14066,7 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="153">
         <f t="shared" si="24"/>
-        <v>3508386</v>
+        <v>3024386</v>
       </c>
       <c r="Z60" s="167">
         <f t="shared" si="25"/>
@@ -14036,7 +14141,7 @@
       <c r="R61" s="158"/>
       <c r="S61" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-17235</v>
+        <v>765</v>
       </c>
       <c r="T61" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14047,7 +14152,7 @@
       <c r="W61" s="149"/>
       <c r="Y61" s="153">
         <f t="shared" ref="Y61" si="39">M61+P61+S61+V61</f>
-        <v>-3944</v>
+        <v>14056</v>
       </c>
       <c r="Z61" s="167">
         <f t="shared" ref="Z61" si="40">(N61+Q61+T61+W61)</f>
@@ -14117,7 +14222,7 @@
       <c r="R62" s="158"/>
       <c r="S62" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>33128</v>
+        <v>323128</v>
       </c>
       <c r="T62" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14128,7 +14233,7 @@
       <c r="W62" s="72"/>
       <c r="Y62" s="153">
         <f t="shared" si="24"/>
-        <v>876229</v>
+        <v>1166229</v>
       </c>
       <c r="Z62" s="167">
         <f t="shared" si="25"/>
@@ -14205,7 +14310,7 @@
       <c r="R63" s="158"/>
       <c r="S63" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>2920</v>
+        <v>55020</v>
       </c>
       <c r="T63" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14216,7 +14321,7 @@
       <c r="W63" s="72"/>
       <c r="Y63" s="153">
         <f t="shared" si="24"/>
-        <v>967793</v>
+        <v>1019893</v>
       </c>
       <c r="Z63" s="167">
         <f t="shared" si="25"/>
@@ -14530,7 +14635,7 @@
       <c r="R67" s="158"/>
       <c r="S67" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>206750</v>
+        <v>-254750</v>
       </c>
       <c r="T67" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14541,7 +14646,7 @@
       <c r="W67" s="149"/>
       <c r="Y67" s="153">
         <f t="shared" ref="Y67" si="45">M67+P67+S67+V67</f>
-        <v>-756079</v>
+        <v>-1217579</v>
       </c>
       <c r="Z67" s="167">
         <f t="shared" ref="Z67" si="46">(N67+Q67+T67+W67)</f>
@@ -14668,7 +14773,7 @@
       <c r="R69" s="158"/>
       <c r="S69" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>65485</v>
+        <v>40285</v>
       </c>
       <c r="T69" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14679,7 +14784,7 @@
       <c r="W69" s="149"/>
       <c r="Y69" s="153">
         <f t="shared" si="24"/>
-        <v>-4400</v>
+        <v>-29600</v>
       </c>
       <c r="Z69" s="167">
         <f t="shared" si="25"/>
@@ -14749,7 +14854,7 @@
       <c r="R70" s="158"/>
       <c r="S70" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>306496</v>
+        <v>359896</v>
       </c>
       <c r="T70" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14760,7 +14865,7 @@
       <c r="W70" s="149"/>
       <c r="Y70" s="153">
         <f t="shared" si="24"/>
-        <v>-54335</v>
+        <v>-935</v>
       </c>
       <c r="Z70" s="167">
         <f t="shared" si="25"/>
@@ -14992,7 +15097,7 @@
       <c r="R73" s="158"/>
       <c r="S73" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>56120</v>
+        <v>152220</v>
       </c>
       <c r="T73" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15003,7 +15108,7 @@
       <c r="W73" s="72"/>
       <c r="Y73" s="153">
         <f t="shared" si="24"/>
-        <v>428424</v>
+        <v>524524</v>
       </c>
       <c r="Z73" s="167">
         <f t="shared" si="25"/>
@@ -15231,7 +15336,7 @@
       <c r="R76" s="158"/>
       <c r="S76" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>100956</v>
+        <v>127856</v>
       </c>
       <c r="T76" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$123,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15242,7 +15347,7 @@
       <c r="W76" s="149"/>
       <c r="Y76" s="153">
         <f t="shared" si="55"/>
-        <v>591809</v>
+        <v>618709</v>
       </c>
       <c r="Z76" s="167">
         <f t="shared" si="56"/>
@@ -15285,7 +15390,7 @@
       <c r="R77" s="122"/>
       <c r="S77" s="109">
         <f>SUM(S4:S74)</f>
-        <v>1213020</v>
+        <v>1105623</v>
       </c>
       <c r="T77" s="122"/>
       <c r="U77" s="122"/>
@@ -15293,7 +15398,7 @@
       <c r="W77" s="50"/>
       <c r="Y77" s="153">
         <f>SUM(Y4:Y76)</f>
-        <v>24695192</v>
+        <v>24614695</v>
       </c>
       <c r="Z77" s="160"/>
     </row>
@@ -17076,11 +17181,11 @@
       </c>
       <c r="G4" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>44320</v>
+        <v>86620</v>
       </c>
       <c r="H4" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.88639999999999997</v>
+        <v>1.7323999999999999</v>
       </c>
       <c r="I4" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17100,11 +17205,11 @@
       </c>
       <c r="M4" s="71">
         <f t="shared" ref="M4:N58" si="0">G4+I4+K4</f>
-        <v>44320</v>
+        <v>86620</v>
       </c>
       <c r="N4" s="165">
         <f t="shared" si="0"/>
-        <v>0.88639999999999997</v>
+        <v>1.7323999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -17128,11 +17233,11 @@
       </c>
       <c r="G5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>94140</v>
+        <v>190895</v>
       </c>
       <c r="H5" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.31380000000000002</v>
+        <v>0.63631666666666664</v>
       </c>
       <c r="I5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17152,11 +17257,11 @@
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>94140</v>
+        <v>190895</v>
       </c>
       <c r="N5" s="165">
         <f t="shared" si="0"/>
-        <v>0.31380000000000002</v>
+        <v>0.63631666666666664</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -17180,11 +17285,11 @@
       </c>
       <c r="G6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>27367</v>
+        <v>71537</v>
       </c>
       <c r="H6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.27367000000000002</v>
+        <v>0.71536999999999995</v>
       </c>
       <c r="I6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17204,11 +17309,11 @@
       </c>
       <c r="M6" s="71">
         <f t="shared" si="0"/>
-        <v>27367</v>
+        <v>71537</v>
       </c>
       <c r="N6" s="165">
         <f t="shared" si="0"/>
-        <v>0.27367000000000002</v>
+        <v>0.71536999999999995</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -17232,11 +17337,11 @@
       </c>
       <c r="G7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-207210</v>
+        <v>-324610</v>
       </c>
       <c r="H7" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.69069999999999998</v>
+        <v>-1.0820333333333332</v>
       </c>
       <c r="I7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17256,11 +17361,11 @@
       </c>
       <c r="M7" s="71">
         <f t="shared" si="0"/>
-        <v>-207210</v>
+        <v>-324610</v>
       </c>
       <c r="N7" s="165">
         <f t="shared" si="0"/>
-        <v>-0.69069999999999998</v>
+        <v>-1.0820333333333332</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -17284,11 +17389,11 @@
       </c>
       <c r="G8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>108340</v>
+        <v>119340</v>
       </c>
       <c r="H8" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.72226666666666672</v>
+        <v>0.79559999999999997</v>
       </c>
       <c r="I8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17308,11 +17413,11 @@
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>108340</v>
+        <v>119340</v>
       </c>
       <c r="N8" s="165">
         <f t="shared" si="0"/>
-        <v>0.72226666666666672</v>
+        <v>0.79559999999999997</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -17336,11 +17441,11 @@
       </c>
       <c r="G9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>42214</v>
+        <v>67214</v>
       </c>
       <c r="H9" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.70356666666666667</v>
+        <v>1.1202333333333334</v>
       </c>
       <c r="I9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17360,11 +17465,11 @@
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>42214</v>
+        <v>67214</v>
       </c>
       <c r="N9" s="165">
         <f t="shared" si="0"/>
-        <v>0.70356666666666667</v>
+        <v>1.1202333333333334</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -17440,11 +17545,11 @@
       </c>
       <c r="G11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>170431</v>
+        <v>226131</v>
       </c>
       <c r="H11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.2840516666666667</v>
+        <v>0.37688500000000003</v>
       </c>
       <c r="I11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17464,11 +17569,11 @@
       </c>
       <c r="M11" s="71">
         <f t="shared" si="0"/>
-        <v>170431</v>
+        <v>226131</v>
       </c>
       <c r="N11" s="165">
         <f t="shared" si="0"/>
-        <v>0.2840516666666667</v>
+        <v>0.37688500000000003</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -17492,11 +17597,11 @@
       </c>
       <c r="G12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-1938</v>
+        <v>-4891</v>
       </c>
       <c r="H12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-1.9380000000000001E-2</v>
+        <v>-4.8910000000000002E-2</v>
       </c>
       <c r="I12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17516,11 +17621,11 @@
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>-1938</v>
+        <v>-4891</v>
       </c>
       <c r="N12" s="165">
         <f t="shared" si="0"/>
-        <v>-1.9380000000000001E-2</v>
+        <v>-4.8910000000000002E-2</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -17544,11 +17649,11 @@
       </c>
       <c r="G13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>68353</v>
+        <v>91053</v>
       </c>
       <c r="H13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.27341199999999999</v>
+        <v>0.36421199999999998</v>
       </c>
       <c r="I13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17568,11 +17673,11 @@
       </c>
       <c r="M13" s="71">
         <f t="shared" si="0"/>
-        <v>68353</v>
+        <v>91053</v>
       </c>
       <c r="N13" s="165">
         <f t="shared" si="0"/>
-        <v>0.27341199999999999</v>
+        <v>0.36421199999999998</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -17648,11 +17753,11 @@
       </c>
       <c r="G15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>14282</v>
+        <v>-15918</v>
       </c>
       <c r="H15" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.14282</v>
+        <v>-0.15917999999999999</v>
       </c>
       <c r="I15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17672,11 +17777,11 @@
       </c>
       <c r="M15" s="71">
         <f t="shared" si="0"/>
-        <v>14282</v>
+        <v>-15918</v>
       </c>
       <c r="N15" s="165">
         <f t="shared" si="0"/>
-        <v>0.14282</v>
+        <v>-0.15917999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -17700,11 +17805,11 @@
       </c>
       <c r="G16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>77903</v>
+        <v>108803</v>
       </c>
       <c r="H16" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.35410454545454545</v>
+        <v>0.49455909090909089</v>
       </c>
       <c r="I16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17724,11 +17829,11 @@
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>77903</v>
+        <v>108803</v>
       </c>
       <c r="N16" s="165">
         <f t="shared" si="0"/>
-        <v>0.35410454545454545</v>
+        <v>0.49455909090909089</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -17908,11 +18013,11 @@
       </c>
       <c r="G20" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-68242</v>
+        <v>-85642</v>
       </c>
       <c r="H20" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-2.7296800000000001</v>
+        <v>-3.4256799999999998</v>
       </c>
       <c r="I20" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -17932,11 +18037,11 @@
       </c>
       <c r="M20" s="71">
         <f t="shared" si="0"/>
-        <v>-68242</v>
+        <v>-85642</v>
       </c>
       <c r="N20" s="165">
         <f t="shared" si="0"/>
-        <v>-2.7296800000000001</v>
+        <v>-3.4256799999999998</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -18012,11 +18117,11 @@
       </c>
       <c r="G22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-50285</v>
+        <v>90715</v>
       </c>
       <c r="H22" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.33523333333333333</v>
+        <v>0.60476666666666656</v>
       </c>
       <c r="I22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18036,11 +18141,11 @@
       </c>
       <c r="M22" s="71">
         <f t="shared" si="0"/>
-        <v>-50285</v>
+        <v>90715</v>
       </c>
       <c r="N22" s="165">
         <f t="shared" si="0"/>
-        <v>-0.33523333333333333</v>
+        <v>0.60476666666666656</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -18116,11 +18221,11 @@
       </c>
       <c r="G24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>28323</v>
+        <v>26700</v>
       </c>
       <c r="H24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.25748181818181815</v>
+        <v>0.24272727272727271</v>
       </c>
       <c r="I24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18140,11 +18245,11 @@
       </c>
       <c r="M24" s="71">
         <f t="shared" si="0"/>
-        <v>28323</v>
+        <v>26700</v>
       </c>
       <c r="N24" s="165">
         <f t="shared" si="0"/>
-        <v>0.25748181818181815</v>
+        <v>0.24272727272727271</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -18168,11 +18273,11 @@
       </c>
       <c r="G25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-61800</v>
+        <v>-443600</v>
       </c>
       <c r="H25" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.26869565217391306</v>
+        <v>-1.9286956521739134</v>
       </c>
       <c r="I25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18192,11 +18297,11 @@
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>-61800</v>
+        <v>-443600</v>
       </c>
       <c r="N25" s="165">
         <f t="shared" si="0"/>
-        <v>-0.26869565217391306</v>
+        <v>-1.9286956521739134</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -18218,11 +18323,11 @@
       </c>
       <c r="G26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-109</v>
+        <v>10791</v>
       </c>
       <c r="H26" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-5.45E-3</v>
+        <v>0.53954999999999997</v>
       </c>
       <c r="I26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18242,11 +18347,11 @@
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>-109</v>
+        <v>10791</v>
       </c>
       <c r="N26" s="165">
         <f t="shared" si="0"/>
-        <v>-5.45E-3</v>
+        <v>0.53954999999999997</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -18322,11 +18427,11 @@
       </c>
       <c r="G28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>412715</v>
+        <v>468515</v>
       </c>
       <c r="H28" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.412715</v>
+        <v>0.46851500000000001</v>
       </c>
       <c r="I28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18346,11 +18451,11 @@
       </c>
       <c r="M28" s="71">
         <f t="shared" si="0"/>
-        <v>412715</v>
+        <v>468515</v>
       </c>
       <c r="N28" s="165">
         <f t="shared" si="0"/>
-        <v>0.412715</v>
+        <v>0.46851500000000001</v>
       </c>
       <c r="O28" s="130"/>
     </row>
@@ -18635,11 +18740,11 @@
       </c>
       <c r="G34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>401130</v>
+        <v>556830</v>
       </c>
       <c r="H34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.80225999999999997</v>
+        <v>1.1136600000000001</v>
       </c>
       <c r="I34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18659,11 +18764,11 @@
       </c>
       <c r="M34" s="71">
         <f t="shared" si="0"/>
-        <v>401130</v>
+        <v>556830</v>
       </c>
       <c r="N34" s="165">
         <f t="shared" si="0"/>
-        <v>0.80225999999999997</v>
+        <v>1.1136600000000001</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -18687,11 +18792,11 @@
       </c>
       <c r="G35" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-108150</v>
+        <v>-64150</v>
       </c>
       <c r="H35" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.21629999999999999</v>
+        <v>-0.1283</v>
       </c>
       <c r="I35" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18711,11 +18816,11 @@
       </c>
       <c r="M35" s="71">
         <f t="shared" si="0"/>
-        <v>-108150</v>
+        <v>-64150</v>
       </c>
       <c r="N35" s="165">
         <f t="shared" si="0"/>
-        <v>-0.21629999999999999</v>
+        <v>-0.1283</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -18739,11 +18844,11 @@
       </c>
       <c r="G36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>3799</v>
+        <v>37899</v>
       </c>
       <c r="H36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>7.5980000000000006E-2</v>
+        <v>0.75797999999999999</v>
       </c>
       <c r="I36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18763,11 +18868,11 @@
       </c>
       <c r="M36" s="71">
         <f t="shared" si="0"/>
-        <v>3799</v>
+        <v>37899</v>
       </c>
       <c r="N36" s="165">
         <f t="shared" si="0"/>
-        <v>7.5980000000000006E-2</v>
+        <v>0.75797999999999999</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -18791,11 +18896,11 @@
       </c>
       <c r="G37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>81468</v>
+        <v>115168</v>
       </c>
       <c r="H37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>2.0367000000000002</v>
+        <v>2.8792</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18815,11 +18920,11 @@
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>81468</v>
+        <v>115168</v>
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>2.0367000000000002</v>
+        <v>2.8792</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -18843,11 +18948,11 @@
       </c>
       <c r="G38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-147529</v>
+        <v>2071</v>
       </c>
       <c r="H38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.3688225</v>
+        <v>5.1774999999999998E-3</v>
       </c>
       <c r="I38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18867,11 +18972,11 @@
       </c>
       <c r="M38" s="71">
         <f t="shared" si="0"/>
-        <v>-147529</v>
+        <v>2071</v>
       </c>
       <c r="N38" s="165">
         <f t="shared" si="0"/>
-        <v>-0.3688225</v>
+        <v>5.1774999999999998E-3</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -18895,11 +19000,11 @@
       </c>
       <c r="G39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>9674</v>
+        <v>-97726</v>
       </c>
       <c r="H39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>9.6740000000000007E-2</v>
+        <v>-0.97726000000000002</v>
       </c>
       <c r="I39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18919,11 +19024,11 @@
       </c>
       <c r="M39" s="71">
         <f t="shared" si="0"/>
-        <v>9674</v>
+        <v>-97726</v>
       </c>
       <c r="N39" s="165">
         <f t="shared" si="0"/>
-        <v>9.6740000000000007E-2</v>
+        <v>-0.97726000000000002</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -18997,11 +19102,11 @@
       </c>
       <c r="G41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-8895</v>
+        <v>14505</v>
       </c>
       <c r="H41" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-0.1779</v>
+        <v>0.29010000000000002</v>
       </c>
       <c r="I41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19021,11 +19126,11 @@
       </c>
       <c r="M41" s="71">
         <f t="shared" si="0"/>
-        <v>-8895</v>
+        <v>14505</v>
       </c>
       <c r="N41" s="165">
         <f t="shared" si="0"/>
-        <v>-0.1779</v>
+        <v>0.29010000000000002</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -19049,11 +19154,11 @@
       </c>
       <c r="G42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>183624</v>
+        <v>175078</v>
       </c>
       <c r="H42" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.61207999999999996</v>
+        <v>0.58359333333333341</v>
       </c>
       <c r="I42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19073,11 +19178,11 @@
       </c>
       <c r="M42" s="71">
         <f t="shared" si="0"/>
-        <v>183624</v>
+        <v>175078</v>
       </c>
       <c r="N42" s="165">
         <f t="shared" si="0"/>
-        <v>0.61207999999999996</v>
+        <v>0.58359333333333341</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -19151,11 +19256,11 @@
       </c>
       <c r="G44" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>6368</v>
+        <v>65368</v>
       </c>
       <c r="H44" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.63680000000000003</v>
+        <v>6.5368000000000004</v>
       </c>
       <c r="I44" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19175,11 +19280,11 @@
       </c>
       <c r="M44" s="71">
         <f t="shared" si="0"/>
-        <v>6368</v>
+        <v>65368</v>
       </c>
       <c r="N44" s="165">
         <f t="shared" si="0"/>
-        <v>0.63680000000000003</v>
+        <v>6.5368000000000004</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -19203,11 +19308,11 @@
       </c>
       <c r="G45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>3300</v>
+        <v>30200</v>
       </c>
       <c r="H45" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>6.6000000000000003E-2</v>
+        <v>0.60399999999999998</v>
       </c>
       <c r="I45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19227,11 +19332,11 @@
       </c>
       <c r="M45" s="71">
         <f t="shared" si="0"/>
-        <v>3300</v>
+        <v>30200</v>
       </c>
       <c r="N45" s="165">
         <f t="shared" si="0"/>
-        <v>6.6000000000000003E-2</v>
+        <v>0.60399999999999998</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -19255,11 +19360,11 @@
       </c>
       <c r="G46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-171229</v>
+        <v>-655229</v>
       </c>
       <c r="H46" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-1.7122900000000001</v>
+        <v>-6.5522900000000002</v>
       </c>
       <c r="I46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19279,11 +19384,11 @@
       </c>
       <c r="M46" s="71">
         <f t="shared" si="0"/>
-        <v>-171229</v>
+        <v>-655229</v>
       </c>
       <c r="N46" s="165">
         <f t="shared" si="0"/>
-        <v>-1.7122900000000001</v>
+        <v>-6.5522900000000002</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -19305,11 +19410,11 @@
       </c>
       <c r="G47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-17235</v>
+        <v>765</v>
       </c>
       <c r="H47" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>-1.7235</v>
+        <v>7.6499999999999999E-2</v>
       </c>
       <c r="I47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19329,11 +19434,11 @@
       </c>
       <c r="M47" s="71">
         <f t="shared" si="0"/>
-        <v>-17235</v>
+        <v>765</v>
       </c>
       <c r="N47" s="165">
         <f t="shared" si="0"/>
-        <v>-1.7235</v>
+        <v>7.6499999999999999E-2</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -19357,11 +19462,11 @@
       </c>
       <c r="G48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>33128</v>
+        <v>323128</v>
       </c>
       <c r="H48" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.11042666666666665</v>
+        <v>1.0770933333333332</v>
       </c>
       <c r="I48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19381,11 +19486,11 @@
       </c>
       <c r="M48" s="71">
         <f t="shared" si="0"/>
-        <v>33128</v>
+        <v>323128</v>
       </c>
       <c r="N48" s="165">
         <f t="shared" si="0"/>
-        <v>0.11042666666666665</v>
+        <v>1.0770933333333332</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -19455,11 +19560,11 @@
       </c>
       <c r="G50" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>2920</v>
+        <v>55020</v>
       </c>
       <c r="H50" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>7.3000000000000001E-3</v>
+        <v>0.13755000000000001</v>
       </c>
       <c r="I50" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19479,11 +19584,11 @@
       </c>
       <c r="M50" s="71">
         <f t="shared" si="0"/>
-        <v>2920</v>
+        <v>55020</v>
       </c>
       <c r="N50" s="165">
         <f t="shared" si="0"/>
-        <v>7.3000000000000001E-3</v>
+        <v>0.13755000000000001</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -19557,11 +19662,11 @@
       </c>
       <c r="G52" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>206750</v>
+        <v>-254750</v>
       </c>
       <c r="H52" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.20674999999999999</v>
+        <v>-0.25474999999999998</v>
       </c>
       <c r="I52" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19581,11 +19686,11 @@
       </c>
       <c r="M52" s="71">
         <f t="shared" si="0"/>
-        <v>206750</v>
+        <v>-254750</v>
       </c>
       <c r="N52" s="165">
         <f t="shared" si="0"/>
-        <v>0.20674999999999999</v>
+        <v>-0.25474999999999998</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -19655,11 +19760,11 @@
       </c>
       <c r="G54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>65485</v>
+        <v>40285</v>
       </c>
       <c r="H54" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>1.3097000000000001</v>
+        <v>0.80569999999999997</v>
       </c>
       <c r="I54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19679,11 +19784,11 @@
       </c>
       <c r="M54" s="71">
         <f t="shared" si="0"/>
-        <v>65485</v>
+        <v>40285</v>
       </c>
       <c r="N54" s="165">
         <f t="shared" si="0"/>
-        <v>1.3097000000000001</v>
+        <v>0.80569999999999997</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -19707,11 +19812,11 @@
       </c>
       <c r="G55" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>306496</v>
+        <v>359896</v>
       </c>
       <c r="H55" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.4715323076923077</v>
+        <v>0.55368615384615383</v>
       </c>
       <c r="I55" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19731,11 +19836,11 @@
       </c>
       <c r="M55" s="71">
         <f t="shared" si="0"/>
-        <v>306496</v>
+        <v>359896</v>
       </c>
       <c r="N55" s="165">
         <f t="shared" si="0"/>
-        <v>0.4715323076923077</v>
+        <v>0.55368615384615383</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
@@ -19811,11 +19916,11 @@
       </c>
       <c r="G57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>56120</v>
+        <v>152220</v>
       </c>
       <c r="H57" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.18706666666666669</v>
+        <v>0.50739999999999996</v>
       </c>
       <c r="I57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19835,11 +19940,11 @@
       </c>
       <c r="M57" s="71">
         <f t="shared" si="0"/>
-        <v>56120</v>
+        <v>152220</v>
       </c>
       <c r="N57" s="165">
         <f t="shared" si="0"/>
-        <v>0.18706666666666669</v>
+        <v>0.50739999999999996</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -19967,11 +20072,11 @@
       </c>
       <c r="G60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>100956</v>
+        <v>127856</v>
       </c>
       <c r="H60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.20191200000000001</v>
+        <v>0.25571199999999999</v>
       </c>
       <c r="I60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19991,11 +20096,11 @@
       </c>
       <c r="M60" s="71">
         <f t="shared" si="1"/>
-        <v>100956</v>
+        <v>127856</v>
       </c>
       <c r="N60" s="165">
         <f t="shared" si="1"/>
-        <v>0.20191200000000001</v>
+        <v>0.25571199999999999</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
@@ -20007,7 +20112,7 @@
       <c r="F61" s="233"/>
       <c r="G61" s="230">
         <f>SUM(G4:G58)</f>
-        <v>1151146</v>
+        <v>1085349</v>
       </c>
       <c r="H61" s="90"/>
       <c r="I61" s="99">
@@ -20022,7 +20127,7 @@
       <c r="L61" s="109"/>
       <c r="M61" s="153">
         <f>SUM(M4:M58)</f>
-        <v>1151146</v>
+        <v>1085349</v>
       </c>
       <c r="N61" s="234"/>
     </row>
@@ -20087,11 +20192,11 @@
       <c r="F65" s="206"/>
       <c r="G65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>151126</v>
+        <v>300126</v>
       </c>
       <c r="H65" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'OCT-2026'!$A$4:$ACW$116,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$CX$2,0),0),0)</f>
-        <v>0.50375333333333339</v>
+        <v>1.0004200000000001</v>
       </c>
       <c r="I65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$122,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20111,11 +20216,11 @@
       </c>
       <c r="M65" s="152">
         <f t="shared" ref="M65:N66" si="2">G65+I65+K65</f>
-        <v>151126</v>
+        <v>300126</v>
       </c>
       <c r="N65" s="166">
         <f t="shared" si="2"/>
-        <v>0.50375333333333339</v>
+        <v>1.0004200000000001</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
@@ -20171,7 +20276,7 @@
     <row r="67" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G67" s="93">
         <f>SUM(G65:G66)</f>
-        <v>249126</v>
+        <v>398126</v>
       </c>
       <c r="H67" s="94"/>
       <c r="I67" s="93">
@@ -20186,7 +20291,7 @@
       <c r="L67" s="113"/>
       <c r="M67" s="93">
         <f>SUM(M65:M66)</f>
-        <v>249126</v>
+        <v>398126</v>
       </c>
       <c r="N67" s="235"/>
     </row>
@@ -23422,7 +23527,7 @@
         <v>256</v>
       </c>
       <c r="F31" s="118">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G31" s="196"/>
       <c r="H31" s="146">
@@ -23494,7 +23599,7 @@
       </c>
       <c r="AD31" s="148">
         <f t="shared" ref="AD31:AD57" si="3">IFERROR(AC31/F31*100,0)/10000000</f>
-        <v>-2.33162</v>
+        <v>-1.16581</v>
       </c>
     </row>
     <row r="32" spans="1:41" x14ac:dyDescent="0.25">
@@ -29650,7 +29755,7 @@
         <v>256</v>
       </c>
       <c r="F38" s="118">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G38" s="196"/>
       <c r="H38" s="146">
@@ -29722,7 +29827,7 @@
       </c>
       <c r="AD38" s="148">
         <f t="shared" si="1"/>
-        <v>-1.28678</v>
+        <v>-0.64339000000000002</v>
       </c>
     </row>
     <row r="39" spans="1:39" x14ac:dyDescent="0.25">
@@ -36163,7 +36268,7 @@
         <v>256</v>
       </c>
       <c r="F35" s="118">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G35" s="196"/>
       <c r="H35" s="146">
@@ -36241,7 +36346,7 @@
       </c>
       <c r="AF35" s="148">
         <f t="shared" si="1"/>
-        <v>-0.30049999999999999</v>
+        <v>-0.15024999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:35" x14ac:dyDescent="0.25">
@@ -41082,7 +41187,7 @@
       </c>
       <c r="H37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'JULY-2026'!$A$4:$ACS$118,MATCH('FY-(26-27)Q2'!$G$2:$H$2,'JULY-2026'!$A$2:$CT$2,0),0),0)</f>
-        <v>-0.30049999999999999</v>
+        <v>-0.15024999999999999</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'AUG-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q2'!$I$2:$J$2,'AUG-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -41090,7 +41195,7 @@
       </c>
       <c r="J37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'AUG-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q2'!$I$2:$J$2,'AUG-2026'!$A$2:$DM$2,0),0),0)</f>
-        <v>-1.28678</v>
+        <v>-0.64339000000000002</v>
       </c>
       <c r="K37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$AEE$125,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$EF$2,0),0),0)</f>
@@ -41098,7 +41203,7 @@
       </c>
       <c r="L37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$126,'SEP-2026'!$A$4:$AEE$125,MATCH('FY-(26-27)Q2'!$K$2:$L$2,'SEP-2026'!$A$2:$EF$2,0),0),0)</f>
-        <v>-2.33162</v>
+        <v>-1.16581</v>
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
@@ -41106,7 +41211,7 @@
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>-3.9188999999999998</v>
+        <v>-1.9594499999999999</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Mon 10/19/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3210" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="342">
   <si>
     <t>Sudeep</t>
   </si>
@@ -1042,6 +1042,18 @@
   <si>
     <t>ATS_1513</t>
   </si>
+  <si>
+    <t>Prateek Amardev</t>
+  </si>
+  <si>
+    <t>Arti Bisht</t>
+  </si>
+  <si>
+    <t>P3159</t>
+  </si>
+  <si>
+    <t>DK SIR_A</t>
+  </si>
 </sst>
 </file>
 
@@ -1769,7 +1781,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="257">
+  <cellXfs count="259">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2373,6 +2385,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -6595,7 +6611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF67"/>
+  <dimension ref="A1:AG69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="132" customWidth="1" outlineLevel="1"/>
@@ -6607,19 +6623,19 @@
     <col min="7" max="7" width="1.7109375" style="132" customWidth="1"/>
     <col min="8" max="17" width="13.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="18" max="18" width="13.42578125" style="132" customWidth="1" collapsed="1"/>
-    <col min="19" max="19" width="11.28515625" style="132" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="21" max="21" width="10.7109375" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="22" width="9.140625" style="132" collapsed="1"/>
-    <col min="23" max="27" width="9.140625" style="132"/>
-    <col min="28" max="28" width="14.140625" style="132" customWidth="1"/>
-    <col min="29" max="29" width="12" style="132" customWidth="1"/>
-    <col min="30" max="30" width="15.85546875" style="132" customWidth="1"/>
-    <col min="31" max="16384" width="9.140625" style="132"/>
+    <col min="19" max="19" width="13.42578125" style="132" customWidth="1"/>
+    <col min="20" max="20" width="11.28515625" style="132" customWidth="1"/>
+    <col min="21" max="21" width="10.42578125" style="132" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="10.7109375" style="132" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="28" width="9.140625" style="132"/>
+    <col min="29" max="29" width="14.140625" style="132" customWidth="1"/>
+    <col min="30" max="30" width="12" style="132" customWidth="1"/>
+    <col min="31" max="31" width="15.85546875" style="132" customWidth="1"/>
+    <col min="32" max="16384" width="9.140625" style="132"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G2" s="220"/>
       <c r="H2" s="255">
         <v>46296</v>
@@ -6654,15 +6670,18 @@
       <c r="R2" s="255">
         <v>46311</v>
       </c>
-      <c r="S2" s="182"/>
-      <c r="T2" s="183" t="s">
+      <c r="S2" s="255">
+        <v>46314</v>
+      </c>
+      <c r="T2" s="182"/>
+      <c r="U2" s="183" t="s">
         <v>325</v>
       </c>
-      <c r="U2" s="184" t="s">
+      <c r="V2" s="184" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="185" t="s">
         <v>54</v>
       </c>
@@ -6715,17 +6734,20 @@
       <c r="R3" s="178" t="s">
         <v>235</v>
       </c>
-      <c r="S3" s="179"/>
-      <c r="T3" s="188"/>
-      <c r="U3" s="179"/>
-      <c r="AB3" s="132" t="s">
+      <c r="S3" s="178" t="s">
+        <v>234</v>
+      </c>
+      <c r="T3" s="179"/>
+      <c r="U3" s="188"/>
+      <c r="V3" s="179"/>
+      <c r="AC3" s="132" t="s">
         <v>198</v>
       </c>
-      <c r="AC3" s="132">
+      <c r="AD3" s="132">
         <v>13780</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="141" t="s">
         <v>216</v>
       </c>
@@ -6778,23 +6800,26 @@
       <c r="R4" s="157">
         <v>-3015</v>
       </c>
-      <c r="S4" s="210"/>
-      <c r="T4" s="170">
-        <f t="shared" ref="T4:T37" si="0">SUM(H4:S4)</f>
-        <v>121236</v>
-      </c>
-      <c r="U4" s="148">
-        <f t="shared" ref="U4:U37" si="1">IFERROR(T4/F4*100,0)/10000000</f>
-        <v>2.4247200000000002</v>
-      </c>
-      <c r="AB4" s="132" t="s">
+      <c r="S4" s="157">
+        <v>-4789</v>
+      </c>
+      <c r="T4" s="210"/>
+      <c r="U4" s="170">
+        <f t="shared" ref="U4:U37" si="0">SUM(H4:T4)</f>
+        <v>116447</v>
+      </c>
+      <c r="V4" s="148">
+        <f t="shared" ref="V4:V37" si="1">IFERROR(U4/F4*100,0)/10000000</f>
+        <v>2.3289399999999998</v>
+      </c>
+      <c r="AC4" s="132" t="s">
         <v>170</v>
       </c>
-      <c r="AC4" s="132">
+      <c r="AD4" s="132">
         <v>2865</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="141" t="s">
         <v>30</v>
       </c>
@@ -6847,17 +6872,20 @@
       <c r="R5" s="146">
         <v>95575</v>
       </c>
-      <c r="S5" s="173"/>
-      <c r="T5" s="170">
+      <c r="S5" s="146">
+        <v>57336</v>
+      </c>
+      <c r="T5" s="173"/>
+      <c r="U5" s="170">
         <f t="shared" si="0"/>
-        <v>469496</v>
-      </c>
-      <c r="U5" s="148">
+        <v>526832</v>
+      </c>
+      <c r="V5" s="148">
         <f t="shared" si="1"/>
-        <v>1.5649866666666665</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+        <v>1.7561066666666665</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="141" t="s">
         <v>323</v>
       </c>
@@ -6910,17 +6938,20 @@
       <c r="R6" s="146">
         <v>68940</v>
       </c>
-      <c r="S6" s="173"/>
-      <c r="T6" s="170">
+      <c r="S6" s="146">
+        <v>93200</v>
+      </c>
+      <c r="T6" s="173"/>
+      <c r="U6" s="170">
         <f t="shared" si="0"/>
-        <v>316777</v>
-      </c>
-      <c r="U6" s="148">
+        <v>409977</v>
+      </c>
+      <c r="V6" s="148">
         <f t="shared" si="1"/>
-        <v>3.16777</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.0997700000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="141" t="s">
         <v>134</v>
       </c>
@@ -6973,21 +7004,24 @@
       <c r="R7" s="146">
         <v>-95555</v>
       </c>
-      <c r="S7" s="173"/>
-      <c r="T7" s="170">
+      <c r="S7" s="146">
+        <v>71500</v>
+      </c>
+      <c r="T7" s="173"/>
+      <c r="U7" s="170">
         <f t="shared" si="0"/>
-        <v>-100437</v>
-      </c>
-      <c r="U7" s="148">
+        <v>-28937</v>
+      </c>
+      <c r="V7" s="148">
         <f t="shared" si="1"/>
-        <v>-0.33478999999999998</v>
-      </c>
-      <c r="W7" s="5"/>
-      <c r="X7" s="133">
-        <v>13586</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+        <v>-9.6456666666666663E-2</v>
+      </c>
+      <c r="X7" s="5"/>
+      <c r="Y7" s="133">
+        <v>224282</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="141" t="s">
         <v>217</v>
       </c>
@@ -7040,21 +7074,24 @@
       <c r="R8" s="146">
         <v>36368</v>
       </c>
-      <c r="S8" s="173"/>
-      <c r="T8" s="170">
+      <c r="S8" s="146">
+        <v>-78711</v>
+      </c>
+      <c r="T8" s="173"/>
+      <c r="U8" s="170">
         <f t="shared" si="0"/>
-        <v>300980</v>
-      </c>
-      <c r="U8" s="148">
+        <v>222269</v>
+      </c>
+      <c r="V8" s="148">
         <f t="shared" si="1"/>
-        <v>2.0065333333333335</v>
-      </c>
-      <c r="W8" s="133">
-        <v>288489</v>
-      </c>
-      <c r="X8" s="133"/>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+        <v>1.4817933333333333</v>
+      </c>
+      <c r="X8" s="133">
+        <v>1735771</v>
+      </c>
+      <c r="Y8" s="133"/>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" s="141" t="s">
         <v>313</v>
       </c>
@@ -7105,24 +7142,27 @@
       <c r="R9" s="146">
         <v>10900</v>
       </c>
-      <c r="S9" s="173"/>
-      <c r="T9" s="170">
+      <c r="S9" s="146">
+        <v>60900</v>
+      </c>
+      <c r="T9" s="173"/>
+      <c r="U9" s="170">
         <f t="shared" si="0"/>
-        <v>107224</v>
-      </c>
-      <c r="U9" s="148">
+        <v>168124</v>
+      </c>
+      <c r="V9" s="148">
         <f t="shared" si="1"/>
-        <v>1.7870666666666668</v>
-      </c>
-      <c r="W9" s="133">
-        <v>302058</v>
+        <v>2.8020666666666667</v>
       </c>
       <c r="X9" s="133">
-        <f>(W9+W8)/10000000*13780</f>
-        <v>813.77376600000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+        <v>1960153</v>
+      </c>
+      <c r="Y9" s="133">
+        <f>(X9+X8)/10000000*13780</f>
+        <v>5092.9832719999995</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="142" t="s">
         <v>35</v>
       </c>
@@ -7175,19 +7215,22 @@
       <c r="R10" s="146">
         <v>1160</v>
       </c>
-      <c r="S10" s="173"/>
-      <c r="T10" s="170">
+      <c r="S10" s="146">
+        <v>47501</v>
+      </c>
+      <c r="T10" s="173"/>
+      <c r="U10" s="170">
         <f t="shared" si="0"/>
-        <v>-136160</v>
-      </c>
-      <c r="U10" s="148">
+        <v>-88659</v>
+      </c>
+      <c r="V10" s="148">
         <f t="shared" si="1"/>
-        <v>-9.0773333333333331E-2</v>
-      </c>
-      <c r="W10" s="133"/>
+        <v>-5.9105999999999999E-2</v>
+      </c>
       <c r="X10" s="133"/>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="Y10" s="133"/>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="142" t="s">
         <v>137</v>
       </c>
@@ -7240,19 +7283,22 @@
       <c r="R11" s="146">
         <v>32041</v>
       </c>
-      <c r="S11" s="173"/>
-      <c r="T11" s="170">
+      <c r="S11" s="146">
+        <v>-270400</v>
+      </c>
+      <c r="T11" s="173"/>
+      <c r="U11" s="170">
         <f t="shared" si="0"/>
-        <v>643754</v>
-      </c>
-      <c r="U11" s="148">
+        <v>373354</v>
+      </c>
+      <c r="V11" s="148">
         <f t="shared" si="1"/>
-        <v>1.0729233333333332</v>
-      </c>
-      <c r="W11" s="133"/>
+        <v>0.62225666666666657</v>
+      </c>
       <c r="X11" s="133"/>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="Y11" s="133"/>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="142" t="s">
         <v>42</v>
       </c>
@@ -7305,19 +7351,22 @@
       <c r="R12" s="146">
         <v>2072</v>
       </c>
-      <c r="S12" s="173"/>
-      <c r="T12" s="170">
+      <c r="S12" s="146">
+        <v>-1965</v>
+      </c>
+      <c r="T12" s="173"/>
+      <c r="U12" s="170">
         <f t="shared" si="0"/>
-        <v>-2608</v>
-      </c>
-      <c r="U12" s="148">
+        <v>-4573</v>
+      </c>
+      <c r="V12" s="148">
         <f t="shared" si="1"/>
-        <v>-2.6079999999999999E-2</v>
-      </c>
-      <c r="W12" s="133"/>
+        <v>-4.573E-2</v>
+      </c>
       <c r="X12" s="133"/>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="Y12" s="133"/>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="141" t="s">
         <v>212</v>
       </c>
@@ -7370,19 +7419,22 @@
       <c r="R13" s="146">
         <v>-39105</v>
       </c>
-      <c r="S13" s="173"/>
-      <c r="T13" s="170">
+      <c r="S13" s="146">
+        <v>-15290</v>
+      </c>
+      <c r="T13" s="173"/>
+      <c r="U13" s="170">
         <f t="shared" si="0"/>
-        <v>116171</v>
-      </c>
-      <c r="U13" s="148">
+        <v>100881</v>
+      </c>
+      <c r="V13" s="148">
         <f t="shared" si="1"/>
-        <v>0.46468399999999999</v>
-      </c>
-      <c r="W13" s="133"/>
+        <v>0.40352399999999999</v>
+      </c>
       <c r="X13" s="133"/>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="Y13" s="133"/>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="141" t="s">
         <v>51</v>
       </c>
@@ -7435,29 +7487,32 @@
       <c r="R14" s="146">
         <v>-48238</v>
       </c>
-      <c r="S14" s="173"/>
-      <c r="T14" s="170">
+      <c r="S14" s="146">
+        <v>-9374</v>
+      </c>
+      <c r="T14" s="173"/>
+      <c r="U14" s="170">
         <f t="shared" si="0"/>
-        <v>127541</v>
-      </c>
-      <c r="U14" s="148">
+        <v>118167</v>
+      </c>
+      <c r="V14" s="148">
         <f t="shared" si="1"/>
-        <v>0.57973181818181818</v>
-      </c>
-      <c r="W14" s="133"/>
-      <c r="X14" s="192">
-        <f>X7-X9</f>
-        <v>12772.226234</v>
-      </c>
-      <c r="AA14" s="132">
+        <v>0.53712272727272725</v>
+      </c>
+      <c r="X14" s="133"/>
+      <c r="Y14" s="192">
+        <f>Y7-Y9</f>
+        <v>219189.01672799999</v>
+      </c>
+      <c r="AB14" s="132">
         <v>116185</v>
       </c>
-      <c r="AC14" s="132">
-        <f>AA14+X14</f>
-        <v>128957.226234</v>
-      </c>
-    </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AD14" s="132">
+        <f>AB14+Y14</f>
+        <v>335374.01672800002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="141" t="s">
         <v>43</v>
       </c>
@@ -7510,17 +7565,20 @@
       <c r="R15" s="146">
         <v>14300</v>
       </c>
-      <c r="S15" s="173"/>
-      <c r="T15" s="170">
+      <c r="S15" s="146">
+        <v>-13384</v>
+      </c>
+      <c r="T15" s="173"/>
+      <c r="U15" s="170">
         <f t="shared" si="0"/>
-        <v>24274</v>
-      </c>
-      <c r="U15" s="148">
+        <v>10890</v>
+      </c>
+      <c r="V15" s="148">
         <f t="shared" si="1"/>
-        <v>0.24274000000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+        <v>0.1089</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" s="141" t="s">
         <v>24</v>
       </c>
@@ -7573,28 +7631,31 @@
       <c r="R16" s="146">
         <v>62711</v>
       </c>
-      <c r="S16" s="173"/>
-      <c r="T16" s="170">
+      <c r="S16" s="146">
+        <v>230600</v>
+      </c>
+      <c r="T16" s="173"/>
+      <c r="U16" s="170">
         <f t="shared" si="0"/>
-        <v>76475</v>
-      </c>
-      <c r="U16" s="148">
+        <v>307075</v>
+      </c>
+      <c r="V16" s="148">
         <f t="shared" si="1"/>
-        <v>0.30590000000000001</v>
-      </c>
-      <c r="AC16" s="132">
+        <v>1.2282999999999999</v>
+      </c>
+      <c r="AD16" s="132">
         <v>4000000</v>
       </c>
-      <c r="AD16" s="132">
-        <f>AC16*7/100</f>
+      <c r="AE16" s="132">
+        <f>AD16*7/100</f>
         <v>280000</v>
       </c>
-      <c r="AF16" s="132">
+      <c r="AG16" s="132">
         <f>15*12</f>
         <v>180</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="141" t="s">
         <v>23</v>
       </c>
@@ -7647,21 +7708,24 @@
       <c r="R17" s="146">
         <v>33838</v>
       </c>
-      <c r="S17" s="173"/>
-      <c r="T17" s="170">
+      <c r="S17" s="146">
+        <v>157000</v>
+      </c>
+      <c r="T17" s="173"/>
+      <c r="U17" s="170">
         <f t="shared" si="0"/>
-        <v>83439</v>
-      </c>
-      <c r="U17" s="148">
+        <v>240439</v>
+      </c>
+      <c r="V17" s="148">
         <f t="shared" si="1"/>
-        <v>0.20859749999999999</v>
-      </c>
-      <c r="AD17" s="132">
-        <f>AD16/12</f>
+        <v>0.60109749999999995</v>
+      </c>
+      <c r="AE17" s="132">
+        <f>AE16/12</f>
         <v>23333.333333333332</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="141" t="s">
         <v>165</v>
       </c>
@@ -7714,17 +7778,20 @@
       <c r="R18" s="146">
         <v>31800</v>
       </c>
-      <c r="S18" s="173"/>
-      <c r="T18" s="170">
+      <c r="S18" s="146">
+        <v>17210</v>
+      </c>
+      <c r="T18" s="173"/>
+      <c r="U18" s="170">
         <f t="shared" si="0"/>
-        <v>482273</v>
-      </c>
-      <c r="U18" s="148">
+        <v>499483</v>
+      </c>
+      <c r="V18" s="148">
         <f t="shared" si="1"/>
-        <v>3.2151533333333333</v>
-      </c>
-    </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+        <v>3.3298866666666669</v>
+      </c>
+    </row>
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="141" t="s">
         <v>110</v>
       </c>
@@ -7777,20 +7844,23 @@
       <c r="R19" s="146">
         <v>0</v>
       </c>
-      <c r="S19" s="173"/>
-      <c r="T19" s="170">
+      <c r="S19" s="146">
+        <v>0</v>
+      </c>
+      <c r="T19" s="173"/>
+      <c r="U19" s="170">
         <f t="shared" si="0"/>
         <v>-150688</v>
       </c>
-      <c r="U19" s="148">
+      <c r="V19" s="148">
         <f t="shared" si="1"/>
         <v>-1.3698909090909093</v>
       </c>
-      <c r="Y19" s="132">
+      <c r="Z19" s="132">
         <v>54000</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="141" t="s">
         <v>319</v>
       </c>
@@ -7843,20 +7913,23 @@
       <c r="R20" s="146">
         <v>0</v>
       </c>
-      <c r="S20" s="173"/>
-      <c r="T20" s="170">
+      <c r="S20" s="146">
+        <v>0</v>
+      </c>
+      <c r="T20" s="173"/>
+      <c r="U20" s="170">
         <f t="shared" si="0"/>
         <v>-107972</v>
       </c>
-      <c r="U20" s="148">
+      <c r="V20" s="148">
         <f t="shared" si="1"/>
         <v>-4.3188800000000001</v>
       </c>
-      <c r="Y20" s="132">
+      <c r="Z20" s="132">
         <v>11100</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="141" t="s">
         <v>316</v>
       </c>
@@ -7909,20 +7982,23 @@
       <c r="R21" s="146">
         <v>0</v>
       </c>
-      <c r="S21" s="173"/>
-      <c r="T21" s="170">
+      <c r="S21" s="146">
+        <v>0</v>
+      </c>
+      <c r="T21" s="173"/>
+      <c r="U21" s="170">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="U21" s="148">
+      <c r="V21" s="148">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Y21" s="132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="Z21" s="132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="141" t="s">
         <v>317</v>
       </c>
@@ -7975,21 +8051,24 @@
       <c r="R22" s="146">
         <v>0</v>
       </c>
-      <c r="S22" s="173"/>
-      <c r="T22" s="170">
+      <c r="S22" s="146">
+        <v>0</v>
+      </c>
+      <c r="T22" s="173"/>
+      <c r="U22" s="170">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="U22" s="148">
+      <c r="V22" s="148">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Y22" s="132">
-        <f>SUM(Y19:Y21)</f>
+      <c r="Z22" s="132">
+        <f>SUM(Z19:Z21)</f>
         <v>65100</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="141" t="s">
         <v>32</v>
       </c>
@@ -8042,17 +8121,20 @@
       <c r="R23" s="146">
         <v>12772</v>
       </c>
-      <c r="S23" s="173"/>
-      <c r="T23" s="170">
+      <c r="S23" s="146">
+        <v>-40307</v>
+      </c>
+      <c r="T23" s="173"/>
+      <c r="U23" s="170">
         <f t="shared" si="0"/>
-        <v>16051</v>
-      </c>
-      <c r="U23" s="148">
+        <v>-24256</v>
+      </c>
+      <c r="V23" s="148">
         <f t="shared" si="1"/>
-        <v>0.14591818181818181</v>
-      </c>
-    </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+        <v>-0.22050909090909088</v>
+      </c>
+    </row>
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="141" t="s">
         <v>97</v>
       </c>
@@ -8105,17 +8187,20 @@
       <c r="R24" s="146">
         <v>18400</v>
       </c>
-      <c r="S24" s="173"/>
-      <c r="T24" s="170">
+      <c r="S24" s="146">
+        <v>-154667</v>
+      </c>
+      <c r="T24" s="173"/>
+      <c r="U24" s="170">
         <f t="shared" si="0"/>
-        <v>-4207</v>
-      </c>
-      <c r="U24" s="148">
+        <v>-158874</v>
+      </c>
+      <c r="V24" s="148">
         <f t="shared" si="1"/>
-        <v>-1.8291304347826085E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+        <v>-0.6907565217391306</v>
+      </c>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="141" t="s">
         <v>335</v>
       </c>
@@ -8152,17 +8237,20 @@
       <c r="R25" s="146">
         <v>-10395</v>
       </c>
-      <c r="S25" s="173"/>
-      <c r="T25" s="170">
-        <f t="shared" ref="T25" si="2">SUM(H25:S25)</f>
-        <v>44179</v>
-      </c>
-      <c r="U25" s="148">
-        <f t="shared" ref="U25" si="3">IFERROR(T25/F25*100,0)/10000000</f>
-        <v>2.2089500000000002</v>
-      </c>
-    </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="S25" s="146">
+        <v>-4185</v>
+      </c>
+      <c r="T25" s="173"/>
+      <c r="U25" s="170">
+        <f t="shared" ref="U25" si="2">SUM(H25:T25)</f>
+        <v>39994</v>
+      </c>
+      <c r="V25" s="148">
+        <f t="shared" ref="V25" si="3">IFERROR(U25/F25*100,0)/10000000</f>
+        <v>1.9997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="141" t="s">
         <v>302</v>
       </c>
@@ -8213,17 +8301,20 @@
       <c r="R26" s="146">
         <v>-19506</v>
       </c>
-      <c r="S26" s="173"/>
-      <c r="T26" s="170">
+      <c r="S26" s="146">
+        <v>-11119</v>
+      </c>
+      <c r="T26" s="173"/>
+      <c r="U26" s="170">
         <f t="shared" si="0"/>
-        <v>-3157</v>
-      </c>
-      <c r="U26" s="148">
+        <v>-14276</v>
+      </c>
+      <c r="V26" s="148">
         <f t="shared" si="1"/>
-        <v>-0.15784999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+        <v>-0.71379999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="141" t="s">
         <v>29</v>
       </c>
@@ -8276,17 +8367,20 @@
       <c r="R27" s="146">
         <v>140100</v>
       </c>
-      <c r="S27" s="173"/>
-      <c r="T27" s="170">
+      <c r="S27" s="146">
+        <v>103000</v>
+      </c>
+      <c r="T27" s="173"/>
+      <c r="U27" s="170">
         <f t="shared" si="0"/>
-        <v>107300</v>
-      </c>
-      <c r="U27" s="148">
+        <v>210300</v>
+      </c>
+      <c r="V27" s="148">
         <f t="shared" si="1"/>
-        <v>0.21460000000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0.42059999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="141" t="s">
         <v>28</v>
       </c>
@@ -8339,17 +8433,20 @@
       <c r="R28" s="146">
         <v>40700</v>
       </c>
-      <c r="S28" s="173"/>
-      <c r="T28" s="170">
+      <c r="S28" s="146">
+        <v>-648400</v>
+      </c>
+      <c r="T28" s="173"/>
+      <c r="U28" s="170">
         <f t="shared" si="0"/>
-        <v>1216859</v>
-      </c>
-      <c r="U28" s="148">
+        <v>568459</v>
+      </c>
+      <c r="V28" s="148">
         <f t="shared" si="1"/>
-        <v>1.2168589999999999</v>
-      </c>
-    </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+        <v>0.56845900000000005</v>
+      </c>
+    </row>
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" s="141" t="s">
         <v>332</v>
       </c>
@@ -8398,17 +8495,20 @@
       <c r="R29" s="146">
         <v>30700</v>
       </c>
-      <c r="S29" s="173"/>
-      <c r="T29" s="170">
-        <f t="shared" ref="T29" si="4">SUM(H29:S29)</f>
-        <v>74309</v>
-      </c>
-      <c r="U29" s="148">
-        <f t="shared" ref="U29" si="5">IFERROR(T29/F29*100,0)/10000000</f>
-        <v>1.4861800000000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="S29" s="146">
+        <v>-27300</v>
+      </c>
+      <c r="T29" s="173"/>
+      <c r="U29" s="170">
+        <f t="shared" ref="U29" si="4">SUM(H29:T29)</f>
+        <v>47009</v>
+      </c>
+      <c r="V29" s="148">
+        <f t="shared" ref="V29" si="5">IFERROR(U29/F29*100,0)/10000000</f>
+        <v>0.94018000000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" s="141" t="s">
         <v>65</v>
       </c>
@@ -8461,17 +8561,20 @@
       <c r="R30" s="146">
         <v>0</v>
       </c>
-      <c r="S30" s="173"/>
-      <c r="T30" s="170">
+      <c r="S30" s="146">
+        <v>219189</v>
+      </c>
+      <c r="T30" s="173"/>
+      <c r="U30" s="170">
         <f t="shared" si="0"/>
-        <v>621985</v>
-      </c>
-      <c r="U30" s="148">
+        <v>841174</v>
+      </c>
+      <c r="V30" s="148">
         <f t="shared" si="1"/>
-        <v>1.24397</v>
-      </c>
-    </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+        <v>1.682348</v>
+      </c>
+    </row>
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31" s="140" t="s">
         <v>34</v>
       </c>
@@ -8524,17 +8627,20 @@
       <c r="R31" s="146">
         <v>37102</v>
       </c>
-      <c r="S31" s="173"/>
-      <c r="T31" s="170">
+      <c r="S31" s="146">
+        <v>0</v>
+      </c>
+      <c r="T31" s="173"/>
+      <c r="U31" s="170">
         <f t="shared" si="0"/>
         <v>140133</v>
       </c>
-      <c r="U31" s="148">
+      <c r="V31" s="148">
         <f t="shared" si="1"/>
         <v>0.28026600000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" s="140" t="s">
         <v>131</v>
       </c>
@@ -8587,17 +8693,20 @@
       <c r="R32" s="146">
         <v>22950</v>
       </c>
-      <c r="S32" s="173"/>
-      <c r="T32" s="170">
+      <c r="S32" s="146">
+        <v>-78603</v>
+      </c>
+      <c r="T32" s="173"/>
+      <c r="U32" s="170">
         <f t="shared" si="0"/>
-        <v>139658</v>
-      </c>
-      <c r="U32" s="148">
+        <v>61055</v>
+      </c>
+      <c r="V32" s="148">
         <f t="shared" si="1"/>
-        <v>2.7931599999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+        <v>1.2211000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" s="43" t="s">
         <v>67</v>
       </c>
@@ -8650,18 +8759,21 @@
       <c r="R33" s="146">
         <v>30400</v>
       </c>
-      <c r="S33" s="173"/>
-      <c r="T33" s="170">
+      <c r="S33" s="146">
+        <v>39761</v>
+      </c>
+      <c r="T33" s="173"/>
+      <c r="U33" s="170">
         <f t="shared" si="0"/>
-        <v>201245</v>
-      </c>
-      <c r="U33" s="148">
+        <v>241006</v>
+      </c>
+      <c r="V33" s="148">
         <f t="shared" si="1"/>
-        <v>5.0311250000000003</v>
-      </c>
-      <c r="X33" s="133"/>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+        <v>6.02515</v>
+      </c>
+      <c r="Y33" s="133"/>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" s="141" t="s">
         <v>31</v>
       </c>
@@ -8714,21 +8826,24 @@
       <c r="R34" s="146">
         <v>-53800</v>
       </c>
-      <c r="S34" s="173"/>
-      <c r="T34" s="170">
+      <c r="S34" s="146">
+        <v>50100</v>
+      </c>
+      <c r="T34" s="173"/>
+      <c r="U34" s="170">
         <f t="shared" si="0"/>
-        <v>163505</v>
-      </c>
-      <c r="U34" s="148">
+        <v>213605</v>
+      </c>
+      <c r="V34" s="148">
         <f t="shared" si="1"/>
-        <v>0.40876249999999997</v>
-      </c>
-      <c r="W34" s="5"/>
-      <c r="X34" s="133">
-        <v>942</v>
-      </c>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+        <v>0.5340125</v>
+      </c>
+      <c r="X34" s="5"/>
+      <c r="Y34" s="133">
+        <v>-43296</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" s="141" t="s">
         <v>104</v>
       </c>
@@ -8781,19 +8896,22 @@
       <c r="R35" s="146">
         <v>26400</v>
       </c>
-      <c r="S35" s="173"/>
-      <c r="T35" s="170">
+      <c r="S35" s="146">
+        <v>-56804</v>
+      </c>
+      <c r="T35" s="173"/>
+      <c r="U35" s="170">
         <f t="shared" si="0"/>
-        <v>6239</v>
-      </c>
-      <c r="U35" s="148">
+        <v>-50565</v>
+      </c>
+      <c r="V35" s="148">
         <f t="shared" si="1"/>
-        <v>6.2390000000000001E-2</v>
-      </c>
-      <c r="W35" s="5"/>
-      <c r="X35" s="133"/>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+        <v>-0.50565000000000004</v>
+      </c>
+      <c r="X35" s="5"/>
+      <c r="Y35" s="133"/>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" s="141" t="s">
         <v>314</v>
       </c>
@@ -8844,24 +8962,27 @@
       <c r="R36" s="146">
         <v>0</v>
       </c>
-      <c r="S36" s="173"/>
-      <c r="T36" s="170">
+      <c r="S36" s="146">
+        <v>0</v>
+      </c>
+      <c r="T36" s="173"/>
+      <c r="U36" s="170">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="U36" s="148">
+      <c r="V36" s="148">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="W36" s="133">
-        <v>23331</v>
-      </c>
       <c r="X36" s="133">
-        <f>(W37+W36)/10000000*13780</f>
-        <v>65.599689999999995</v>
-      </c>
-    </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+        <v>1968047</v>
+      </c>
+      <c r="Y36" s="133">
+        <f>(X37+X36)/10000000*13780</f>
+        <v>5364.2742660000004</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" s="141" t="s">
         <v>229</v>
       </c>
@@ -8914,21 +9035,24 @@
       <c r="R37" s="146">
         <v>192</v>
       </c>
-      <c r="S37" s="173"/>
-      <c r="T37" s="170">
+      <c r="S37" s="146">
+        <v>-5600</v>
+      </c>
+      <c r="T37" s="173"/>
+      <c r="U37" s="170">
         <f t="shared" si="0"/>
-        <v>-27574</v>
-      </c>
-      <c r="U37" s="148">
+        <v>-33174</v>
+      </c>
+      <c r="V37" s="148">
         <f t="shared" si="1"/>
-        <v>-0.55147999999999997</v>
-      </c>
-      <c r="W37" s="133">
-        <v>24274</v>
-      </c>
-      <c r="X37" s="133"/>
-    </row>
-    <row r="38" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>-0.66347999999999996</v>
+      </c>
+      <c r="X37" s="133">
+        <v>1924750</v>
+      </c>
+      <c r="Y37" s="133"/>
+    </row>
+    <row r="38" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="141" t="s">
         <v>45</v>
       </c>
@@ -8981,22 +9105,25 @@
       <c r="R38" s="146">
         <v>-11174</v>
       </c>
-      <c r="S38" s="173"/>
-      <c r="T38" s="170">
-        <f t="shared" ref="T38:T54" si="6">SUM(H38:S38)</f>
-        <v>647499</v>
-      </c>
-      <c r="U38" s="148">
-        <f t="shared" ref="U38:U54" si="7">IFERROR(T38/F38*100,0)/10000000</f>
-        <v>2.1583299999999999</v>
-      </c>
-      <c r="W38" s="133"/>
-      <c r="X38" s="133">
-        <f>+X34-X36</f>
-        <v>876.40030999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S38" s="146">
+        <v>223000</v>
+      </c>
+      <c r="T38" s="173"/>
+      <c r="U38" s="170">
+        <f t="shared" ref="U38:U54" si="6">SUM(H38:T38)</f>
+        <v>870499</v>
+      </c>
+      <c r="V38" s="148">
+        <f t="shared" ref="V38:V54" si="7">IFERROR(U38/F38*100,0)/10000000</f>
+        <v>2.901663333333333</v>
+      </c>
+      <c r="X38" s="133"/>
+      <c r="Y38" s="133">
+        <f>+Y34-Y36</f>
+        <v>-48660.274266</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="141" t="s">
         <v>292</v>
       </c>
@@ -9047,19 +9174,22 @@
       <c r="R39" s="146">
         <v>-72104</v>
       </c>
-      <c r="S39" s="173"/>
-      <c r="T39" s="170">
+      <c r="S39" s="146">
+        <v>32900</v>
+      </c>
+      <c r="T39" s="173"/>
+      <c r="U39" s="170">
         <f t="shared" si="6"/>
-        <v>-39672</v>
-      </c>
-      <c r="U39" s="148">
+        <v>-6772</v>
+      </c>
+      <c r="V39" s="148">
         <f t="shared" si="7"/>
-        <v>-3.9672000000000001</v>
-      </c>
-      <c r="W39" s="133"/>
+        <v>-0.67720000000000002</v>
+      </c>
       <c r="X39" s="133"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y39" s="133"/>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40" s="141" t="s">
         <v>132</v>
       </c>
@@ -9112,19 +9242,22 @@
       <c r="R40" s="146">
         <v>1932</v>
       </c>
-      <c r="S40" s="173"/>
-      <c r="T40" s="170">
+      <c r="S40" s="146">
+        <v>0</v>
+      </c>
+      <c r="T40" s="173"/>
+      <c r="U40" s="170">
         <f t="shared" si="6"/>
         <v>27311</v>
       </c>
-      <c r="U40" s="148">
+      <c r="V40" s="148">
         <f t="shared" si="7"/>
         <v>0.54622000000000004</v>
       </c>
-      <c r="W40" s="133"/>
       <c r="X40" s="133"/>
-    </row>
-    <row r="41" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y40" s="133"/>
+    </row>
+    <row r="41" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="141" t="s">
         <v>48</v>
       </c>
@@ -9177,19 +9310,22 @@
       <c r="R41" s="146">
         <v>60000</v>
       </c>
-      <c r="S41" s="173"/>
-      <c r="T41" s="170">
+      <c r="S41" s="146">
+        <v>-71974</v>
+      </c>
+      <c r="T41" s="173"/>
+      <c r="U41" s="170">
         <f t="shared" si="6"/>
-        <v>-901416</v>
-      </c>
-      <c r="U41" s="148">
+        <v>-973390</v>
+      </c>
+      <c r="V41" s="148">
         <f t="shared" si="7"/>
-        <v>-9.0141600000000004</v>
-      </c>
-      <c r="W41" s="133"/>
+        <v>-9.7339000000000002</v>
+      </c>
       <c r="X41" s="133"/>
-    </row>
-    <row r="42" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y41" s="133"/>
+    </row>
+    <row r="42" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="141" t="s">
         <v>336</v>
       </c>
@@ -9228,19 +9364,22 @@
       <c r="R42" s="146">
         <v>136800</v>
       </c>
-      <c r="S42" s="173"/>
-      <c r="T42" s="170">
-        <f t="shared" ref="T42" si="8">SUM(H42:S42)</f>
-        <v>412452</v>
-      </c>
-      <c r="U42" s="148">
-        <f t="shared" ref="U42" si="9">IFERROR(T42/F42*100,0)/10000000</f>
-        <v>8.2490400000000008</v>
-      </c>
-      <c r="W42" s="133"/>
+      <c r="S42" s="146">
+        <v>-41019</v>
+      </c>
+      <c r="T42" s="173"/>
+      <c r="U42" s="170">
+        <f t="shared" ref="U42" si="8">SUM(H42:T42)</f>
+        <v>371433</v>
+      </c>
+      <c r="V42" s="148">
+        <f t="shared" ref="V42" si="9">IFERROR(U42/F42*100,0)/10000000</f>
+        <v>7.4286599999999998</v>
+      </c>
       <c r="X42" s="133"/>
-    </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y42" s="133"/>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43" s="141" t="s">
         <v>301</v>
       </c>
@@ -9291,18 +9430,21 @@
       <c r="R43" s="146">
         <v>-1908</v>
       </c>
-      <c r="S43" s="173"/>
-      <c r="T43" s="170">
+      <c r="S43" s="146">
+        <v>14500</v>
+      </c>
+      <c r="T43" s="173"/>
+      <c r="U43" s="170">
         <f t="shared" si="6"/>
-        <v>-33711</v>
-      </c>
-      <c r="U43" s="148">
+        <v>-19211</v>
+      </c>
+      <c r="V43" s="148">
         <f t="shared" si="7"/>
-        <v>-3.3711000000000002</v>
-      </c>
-      <c r="W43" s="133"/>
-    </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+        <v>-1.9211</v>
+      </c>
+      <c r="X43" s="133"/>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" s="142" t="s">
         <v>168</v>
       </c>
@@ -9355,17 +9497,20 @@
       <c r="R44" s="146">
         <v>0</v>
       </c>
-      <c r="S44" s="173"/>
-      <c r="T44" s="170">
+      <c r="S44" s="146">
+        <v>0</v>
+      </c>
+      <c r="T44" s="173"/>
+      <c r="U44" s="170">
         <f t="shared" si="6"/>
         <v>112320</v>
       </c>
-      <c r="U44" s="148">
+      <c r="V44" s="148">
         <f t="shared" si="7"/>
         <v>0.28079999999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" s="142" t="s">
         <v>202</v>
       </c>
@@ -9418,17 +9563,20 @@
       <c r="R45" s="146">
         <v>3058</v>
       </c>
-      <c r="S45" s="173"/>
-      <c r="T45" s="170">
+      <c r="S45" s="146">
+        <v>-116345</v>
+      </c>
+      <c r="T45" s="173"/>
+      <c r="U45" s="170">
         <f t="shared" si="6"/>
-        <v>167758</v>
-      </c>
-      <c r="U45" s="148">
+        <v>51413</v>
+      </c>
+      <c r="V45" s="148">
         <f t="shared" si="7"/>
-        <v>0.41939500000000002</v>
-      </c>
-    </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+        <v>0.12853249999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46" s="142" t="s">
         <v>33</v>
       </c>
@@ -9481,17 +9629,20 @@
       <c r="R46" s="146">
         <v>96778</v>
       </c>
-      <c r="S46" s="173"/>
-      <c r="T46" s="170">
+      <c r="S46" s="146">
+        <v>206116</v>
+      </c>
+      <c r="T46" s="173"/>
+      <c r="U46" s="170">
         <f t="shared" si="6"/>
-        <v>898923</v>
-      </c>
-      <c r="U46" s="148">
+        <v>1105039</v>
+      </c>
+      <c r="V46" s="148">
         <f t="shared" si="7"/>
-        <v>2.99641</v>
-      </c>
-    </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+        <v>3.6834633333333326</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47" s="59" t="s">
         <v>306</v>
       </c>
@@ -9542,17 +9693,20 @@
       <c r="R47" s="150">
         <v>390000</v>
       </c>
-      <c r="S47" s="173"/>
-      <c r="T47" s="170">
+      <c r="S47" s="150">
+        <v>-749200</v>
+      </c>
+      <c r="T47" s="173"/>
+      <c r="U47" s="170">
         <f t="shared" si="6"/>
-        <v>-1334350</v>
-      </c>
-      <c r="U47" s="148">
+        <v>-2083550</v>
+      </c>
+      <c r="V47" s="148">
         <f t="shared" si="7"/>
-        <v>-1.3343499999999999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+        <v>-2.0835499999999998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48" s="59" t="s">
         <v>197</v>
       </c>
@@ -9605,17 +9759,20 @@
       <c r="R48" s="150">
         <v>876</v>
       </c>
-      <c r="S48" s="173"/>
-      <c r="T48" s="170">
+      <c r="S48" s="150">
+        <v>0</v>
+      </c>
+      <c r="T48" s="173"/>
+      <c r="U48" s="170">
         <f t="shared" si="6"/>
         <v>64488</v>
       </c>
-      <c r="U48" s="148">
+      <c r="V48" s="148">
         <f t="shared" si="7"/>
         <v>1.28976</v>
       </c>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" s="59" t="s">
         <v>213</v>
       </c>
@@ -9668,17 +9825,20 @@
       <c r="R49" s="150">
         <v>0</v>
       </c>
-      <c r="S49" s="173"/>
-      <c r="T49" s="170">
+      <c r="S49" s="150">
+        <v>-48660</v>
+      </c>
+      <c r="T49" s="173"/>
+      <c r="U49" s="170">
         <f t="shared" si="6"/>
-        <v>418303</v>
-      </c>
-      <c r="U49" s="148">
+        <v>369643</v>
+      </c>
+      <c r="V49" s="148">
         <f t="shared" si="7"/>
-        <v>0.643543076923077</v>
-      </c>
-    </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.56868153846153835</v>
+      </c>
+    </row>
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" s="59" t="s">
         <v>214</v>
       </c>
@@ -9731,17 +9891,20 @@
       <c r="R50" s="150">
         <v>0</v>
       </c>
-      <c r="S50" s="173"/>
-      <c r="T50" s="170">
+      <c r="S50" s="150">
+        <v>0</v>
+      </c>
+      <c r="T50" s="173"/>
+      <c r="U50" s="170">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="U50" s="148">
+      <c r="V50" s="148">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" s="59" t="s">
         <v>49</v>
       </c>
@@ -9794,17 +9957,20 @@
       <c r="R51" s="150">
         <v>0</v>
       </c>
-      <c r="S51" s="173"/>
-      <c r="T51" s="170">
+      <c r="S51" s="150">
+        <v>27140</v>
+      </c>
+      <c r="T51" s="173"/>
+      <c r="U51" s="170">
         <f t="shared" si="6"/>
-        <v>284547</v>
-      </c>
-      <c r="U51" s="148">
+        <v>311687</v>
+      </c>
+      <c r="V51" s="148">
         <f t="shared" si="7"/>
-        <v>0.94849000000000006</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+        <v>1.0389566666666668</v>
+      </c>
+    </row>
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" s="59" t="s">
         <v>331</v>
       </c>
@@ -9857,17 +10023,20 @@
       <c r="R52" s="150">
         <v>-3721</v>
       </c>
-      <c r="S52" s="173"/>
-      <c r="T52" s="170">
+      <c r="S52" s="150">
+        <v>13135</v>
+      </c>
+      <c r="T52" s="173"/>
+      <c r="U52" s="170">
         <f t="shared" si="6"/>
-        <v>874</v>
-      </c>
-      <c r="U52" s="148">
+        <v>14009</v>
+      </c>
+      <c r="V52" s="148">
         <f t="shared" si="7"/>
-        <v>8.7399999999999995E-3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.14008999999999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="59" t="s">
         <v>288</v>
       </c>
@@ -9920,17 +10089,20 @@
       <c r="R53" s="150">
         <v>-16377</v>
       </c>
-      <c r="S53" s="173"/>
-      <c r="T53" s="170">
+      <c r="S53" s="150">
+        <v>165250</v>
+      </c>
+      <c r="T53" s="173"/>
+      <c r="U53" s="170">
         <f t="shared" si="6"/>
-        <v>600079</v>
-      </c>
-      <c r="U53" s="148">
+        <v>765329</v>
+      </c>
+      <c r="V53" s="148">
         <f t="shared" si="7"/>
-        <v>0.60007900000000003</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.76532899999999993</v>
+      </c>
+    </row>
+    <row r="54" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="24"/>
       <c r="B54" s="25"/>
       <c r="C54" s="26"/>
@@ -9939,7 +10111,7 @@
       <c r="F54" s="115"/>
       <c r="G54" s="16"/>
       <c r="H54" s="253">
-        <f t="shared" ref="H54:R54" si="10">SUM(H4:H53)</f>
+        <f t="shared" ref="H54:S54" si="10">SUM(H4:H53)</f>
         <v>38252</v>
       </c>
       <c r="I54" s="253">
@@ -9983,19 +10155,23 @@
         <v>1063967</v>
       </c>
       <c r="S54" s="253">
-        <f>SUM(S4:S53)</f>
-        <v>0</v>
+        <f t="shared" si="10"/>
+        <v>-618758</v>
       </c>
       <c r="T54" s="253">
+        <f>SUM(T4:T53)</f>
+        <v>0</v>
+      </c>
+      <c r="U54" s="253">
         <f t="shared" si="6"/>
-        <v>6393705</v>
-      </c>
-      <c r="U54" s="254">
+        <v>5774947</v>
+      </c>
+      <c r="V54" s="254">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="249"/>
       <c r="B55" s="249"/>
       <c r="C55" s="249"/>
@@ -10016,9 +10192,10 @@
       <c r="R55" s="249"/>
       <c r="S55" s="249"/>
       <c r="T55" s="249"/>
-      <c r="U55" s="251"/>
-    </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U55" s="249"/>
+      <c r="V55" s="251"/>
+    </row>
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" s="201" t="s">
         <v>241</v>
       </c>
@@ -10071,17 +10248,20 @@
       <c r="R56" s="161">
         <v>789</v>
       </c>
-      <c r="S56" s="245"/>
-      <c r="T56" s="246">
-        <f>SUM(H56:S56)</f>
-        <v>-35230</v>
-      </c>
-      <c r="U56" s="247">
-        <f>IFERROR(T56/F56*100,0)/10000000</f>
-        <v>-0.11743333333333335</v>
-      </c>
-    </row>
-    <row r="57" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S56" s="161">
+        <v>34900</v>
+      </c>
+      <c r="T56" s="245"/>
+      <c r="U56" s="246">
+        <f>SUM(H56:T56)</f>
+        <v>-330</v>
+      </c>
+      <c r="V56" s="247">
+        <f>IFERROR(U56/F56*100,0)/10000000</f>
+        <v>-1.1000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" s="201" t="s">
         <v>273</v>
       </c>
@@ -10132,186 +10312,263 @@
       <c r="R57" s="161">
         <v>0</v>
       </c>
-      <c r="S57" s="173"/>
-      <c r="T57" s="170">
-        <f>SUM(H57:S57)</f>
-        <v>-218465</v>
-      </c>
-      <c r="U57" s="148">
-        <f>IFERROR(T57/F57*100,0)/10000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:25" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="199"/>
-      <c r="B58" s="16"/>
-      <c r="C58" s="16"/>
-      <c r="D58" s="16"/>
-      <c r="E58" s="16"/>
-      <c r="F58" s="74"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="169">
-        <f t="shared" ref="H58:R58" si="11">SUM(H56:H57)</f>
+      <c r="S57" s="161">
+        <v>-19129</v>
+      </c>
+      <c r="T57" s="173"/>
+      <c r="U57" s="170">
+        <f>SUM(H57:T57)</f>
+        <v>-237594</v>
+      </c>
+      <c r="V57" s="148">
+        <f>IFERROR(U57/F57*100,0)/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A58" s="201"/>
+      <c r="B58" s="202" t="s">
+        <v>338</v>
+      </c>
+      <c r="C58" s="202" t="s">
+        <v>57</v>
+      </c>
+      <c r="D58" s="202" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58" s="202" t="s">
+        <v>256</v>
+      </c>
+      <c r="F58" s="203"/>
+      <c r="G58" s="204"/>
+      <c r="H58" s="161"/>
+      <c r="I58" s="161"/>
+      <c r="J58" s="161"/>
+      <c r="K58" s="161"/>
+      <c r="L58" s="161"/>
+      <c r="M58" s="161"/>
+      <c r="N58" s="161"/>
+      <c r="O58" s="161"/>
+      <c r="P58" s="161"/>
+      <c r="Q58" s="161"/>
+      <c r="R58" s="161"/>
+      <c r="S58" s="161">
+        <v>0</v>
+      </c>
+      <c r="T58" s="161"/>
+      <c r="U58" s="257"/>
+      <c r="V58" s="258"/>
+    </row>
+    <row r="59" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="201" t="s">
+        <v>340</v>
+      </c>
+      <c r="B59" s="202" t="s">
+        <v>339</v>
+      </c>
+      <c r="C59" s="202" t="s">
+        <v>57</v>
+      </c>
+      <c r="D59" s="202" t="s">
+        <v>87</v>
+      </c>
+      <c r="E59" s="202" t="s">
+        <v>256</v>
+      </c>
+      <c r="F59" s="203"/>
+      <c r="G59" s="204"/>
+      <c r="H59" s="161"/>
+      <c r="I59" s="161"/>
+      <c r="J59" s="161"/>
+      <c r="K59" s="161"/>
+      <c r="L59" s="161"/>
+      <c r="M59" s="161"/>
+      <c r="N59" s="161"/>
+      <c r="O59" s="161"/>
+      <c r="P59" s="161"/>
+      <c r="Q59" s="161"/>
+      <c r="R59" s="161"/>
+      <c r="S59" s="161">
+        <v>-58780</v>
+      </c>
+      <c r="T59" s="161"/>
+      <c r="U59" s="257"/>
+      <c r="V59" s="258"/>
+    </row>
+    <row r="60" spans="1:26" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="199"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="74"/>
+      <c r="G60" s="17"/>
+      <c r="H60" s="169">
+        <f t="shared" ref="H60:S60" si="11">SUM(H56:H57)</f>
         <v>5771</v>
       </c>
-      <c r="I58" s="169">
+      <c r="I60" s="169">
         <f t="shared" si="11"/>
         <v>-81800</v>
       </c>
-      <c r="J58" s="169">
+      <c r="J60" s="169">
         <f t="shared" si="11"/>
         <v>309555</v>
       </c>
-      <c r="K58" s="169">
+      <c r="K60" s="169">
         <f t="shared" si="11"/>
         <v>15600</v>
       </c>
-      <c r="L58" s="169">
+      <c r="L60" s="169">
         <f t="shared" si="11"/>
         <v>149000</v>
       </c>
-      <c r="M58" s="169">
+      <c r="M60" s="169">
         <f t="shared" si="11"/>
         <v>-9023</v>
       </c>
-      <c r="N58" s="169">
+      <c r="N60" s="169">
         <f t="shared" si="11"/>
         <v>-50</v>
       </c>
-      <c r="O58" s="169">
+      <c r="O60" s="169">
         <f t="shared" si="11"/>
         <v>-458665</v>
       </c>
-      <c r="P58" s="169">
+      <c r="P60" s="169">
         <f t="shared" si="11"/>
         <v>-608</v>
       </c>
-      <c r="Q58" s="169">
+      <c r="Q60" s="169">
         <f t="shared" si="11"/>
         <v>-184264</v>
       </c>
-      <c r="R58" s="169">
+      <c r="R60" s="169">
         <f t="shared" si="11"/>
         <v>789</v>
       </c>
-      <c r="S58" s="169">
-        <f>SUM(S56:S57)</f>
-        <v>0</v>
-      </c>
-      <c r="T58" s="256">
-        <f>SUM(H58:S58)</f>
-        <v>-253695</v>
-      </c>
-      <c r="U58" s="172"/>
-    </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="X59" s="133"/>
-    </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W60" s="133"/>
-    </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W61" s="5"/>
-      <c r="X61" s="133"/>
-      <c r="Y61" s="236"/>
-    </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W62" s="133"/>
+      <c r="S60" s="169">
+        <f t="shared" si="11"/>
+        <v>15771</v>
+      </c>
+      <c r="T60" s="169">
+        <f>SUM(T56:T57)</f>
+        <v>0</v>
+      </c>
+      <c r="U60" s="256">
+        <f>SUM(H60:T60)</f>
+        <v>-237924</v>
+      </c>
+      <c r="V60" s="172"/>
+    </row>
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y61" s="133"/>
+    </row>
+    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X62" s="133"/>
-      <c r="Y62" s="236"/>
-    </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W63" s="133"/>
-      <c r="X63" s="133"/>
-      <c r="Y63" s="236"/>
-    </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W64" s="133"/>
+    </row>
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="X63" s="5"/>
+      <c r="Y63" s="133"/>
+      <c r="Z63" s="236"/>
+    </row>
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X64" s="133"/>
-      <c r="Y64" s="236"/>
-    </row>
-    <row r="65" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W65" s="133"/>
+      <c r="Y64" s="133"/>
+      <c r="Z64" s="236"/>
+    </row>
+    <row r="65" spans="24:26" x14ac:dyDescent="0.25">
       <c r="X65" s="133"/>
-      <c r="Y65" s="236"/>
-    </row>
-    <row r="66" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W66" s="133"/>
-      <c r="X66" s="236"/>
-      <c r="Y66" s="236"/>
-    </row>
-    <row r="67" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W67" s="236"/>
-      <c r="X67" s="236"/>
-      <c r="Y67" s="236"/>
+      <c r="Y65" s="133"/>
+      <c r="Z65" s="236"/>
+    </row>
+    <row r="66" spans="24:26" x14ac:dyDescent="0.25">
+      <c r="X66" s="133"/>
+      <c r="Y66" s="133"/>
+      <c r="Z66" s="236"/>
+    </row>
+    <row r="67" spans="24:26" x14ac:dyDescent="0.25">
+      <c r="X67" s="133"/>
+      <c r="Y67" s="133"/>
+      <c r="Z67" s="236"/>
+    </row>
+    <row r="68" spans="24:26" x14ac:dyDescent="0.25">
+      <c r="X68" s="133"/>
+      <c r="Y68" s="236"/>
+      <c r="Z68" s="236"/>
+    </row>
+    <row r="69" spans="24:26" x14ac:dyDescent="0.25">
+      <c r="X69" s="236"/>
+      <c r="Y69" s="236"/>
+      <c r="Z69" s="236"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2 A3:G3 U54:U55 U58 U10:U20 T10:T21 H2:U3 A36:T36 A37:S37 G38:S38 T5:U9 T27:U28 T37:T39 U38 U30:U34 T30:T35 A4:S35 A56:U57 T41:U42 T23:U25 T44:U53 A39:S54 A58:S58">
+  <conditionalFormatting sqref="G2 A3:G3 V54:V55 V60 V10:V20 U10:U21 H2:V3 A36:U36 A37:T37 G38:T38 U5:V9 U27:V28 U37:U39 V38 V30:V34 U30:U35 A4:T35 U41:V42 U23:V25 U44:V53 A39:T54 A60:T60 A56:V59">
     <cfRule type="expression" dxfId="554" priority="18">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U35">
+  <conditionalFormatting sqref="V35">
     <cfRule type="expression" dxfId="553" priority="17">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T4:U4">
+  <conditionalFormatting sqref="U4:V4">
     <cfRule type="expression" dxfId="552" priority="15">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U37">
+  <conditionalFormatting sqref="V37">
     <cfRule type="expression" dxfId="551" priority="14">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U21">
+  <conditionalFormatting sqref="V21">
     <cfRule type="expression" dxfId="550" priority="13">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T54">
+  <conditionalFormatting sqref="U54">
     <cfRule type="expression" dxfId="549" priority="12">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U39">
+  <conditionalFormatting sqref="V39">
     <cfRule type="expression" dxfId="548" priority="11">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T26:U26">
+  <conditionalFormatting sqref="U26:V26">
     <cfRule type="expression" dxfId="547" priority="10">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T43:U43">
+  <conditionalFormatting sqref="U43:V43">
     <cfRule type="expression" dxfId="546" priority="8">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T58">
+  <conditionalFormatting sqref="U60">
     <cfRule type="expression" dxfId="545" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T40:U40">
+  <conditionalFormatting sqref="U40:V40">
     <cfRule type="expression" dxfId="544" priority="6">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T22">
+  <conditionalFormatting sqref="U22">
     <cfRule type="expression" dxfId="543" priority="5">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U22">
+  <conditionalFormatting sqref="V22">
     <cfRule type="expression" dxfId="542" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U36">
+  <conditionalFormatting sqref="V36">
     <cfRule type="expression" dxfId="541" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -10321,7 +10578,7 @@
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T29:U29">
+  <conditionalFormatting sqref="U29:V29">
     <cfRule type="expression" dxfId="539" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -10682,7 +10939,7 @@
       <c r="R6" s="158"/>
       <c r="S6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>121236</v>
+        <v>116447</v>
       </c>
       <c r="T6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10694,7 +10951,7 @@
       <c r="X6" s="131"/>
       <c r="Y6" s="153">
         <f t="shared" si="0"/>
-        <v>-431238</v>
+        <v>-436027</v>
       </c>
       <c r="Z6" s="167">
         <f t="shared" si="1"/>
@@ -10764,7 +11021,7 @@
       <c r="R7" s="158"/>
       <c r="S7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>469496</v>
+        <v>526832</v>
       </c>
       <c r="T7" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10776,7 +11033,7 @@
       <c r="X7"/>
       <c r="Y7" s="153">
         <f t="shared" si="0"/>
-        <v>1711710</v>
+        <v>1769046</v>
       </c>
       <c r="Z7" s="167">
         <f t="shared" si="1"/>
@@ -10900,7 +11157,7 @@
       <c r="R9" s="158"/>
       <c r="S9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>316777</v>
+        <v>409977</v>
       </c>
       <c r="T9" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10911,7 +11168,7 @@
       <c r="W9" s="149"/>
       <c r="Y9" s="153">
         <f t="shared" ref="Y9" si="6">M9+P9+S9+V9</f>
-        <v>180391</v>
+        <v>273591</v>
       </c>
       <c r="Z9" s="167">
         <f t="shared" ref="Z9" si="7">(N9+Q9+T9+W9)</f>
@@ -10981,7 +11238,7 @@
       <c r="R10" s="158"/>
       <c r="S10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-100437</v>
+        <v>-28937</v>
       </c>
       <c r="T10" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -10992,7 +11249,7 @@
       <c r="W10" s="72"/>
       <c r="Y10" s="153">
         <f t="shared" si="0"/>
-        <v>-1276504</v>
+        <v>-1205004</v>
       </c>
       <c r="Z10" s="167">
         <f t="shared" si="1"/>
@@ -11062,7 +11319,7 @@
       <c r="R11" s="158"/>
       <c r="S11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>300980</v>
+        <v>222269</v>
       </c>
       <c r="T11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11073,7 +11330,7 @@
       <c r="W11" s="149"/>
       <c r="Y11" s="153">
         <f t="shared" si="0"/>
-        <v>-100895</v>
+        <v>-179606</v>
       </c>
       <c r="Z11" s="167">
         <f t="shared" si="1"/>
@@ -11143,7 +11400,7 @@
       <c r="R12" s="158"/>
       <c r="S12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>107224</v>
+        <v>168124</v>
       </c>
       <c r="T12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11154,7 +11411,7 @@
       <c r="W12" s="149"/>
       <c r="Y12" s="153">
         <f t="shared" ref="Y12" si="12">M12+P12+S12+V12</f>
-        <v>17295</v>
+        <v>78195</v>
       </c>
       <c r="Z12" s="167">
         <f t="shared" ref="Z12" si="13">(N12+Q12+T12+W12)</f>
@@ -11224,7 +11481,7 @@
       <c r="R13" s="158"/>
       <c r="S13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-136160</v>
+        <v>-88659</v>
       </c>
       <c r="T13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11236,7 +11493,7 @@
       <c r="X13"/>
       <c r="Y13" s="153">
         <f t="shared" si="0"/>
-        <v>-1120428</v>
+        <v>-1072927</v>
       </c>
       <c r="Z13" s="167">
         <f t="shared" si="1"/>
@@ -11633,7 +11890,7 @@
       <c r="R18" s="158"/>
       <c r="S18" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>643754</v>
+        <v>373354</v>
       </c>
       <c r="T18" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11644,7 +11901,7 @@
       <c r="W18" s="72"/>
       <c r="Y18" s="153">
         <f t="shared" si="0"/>
-        <v>843806</v>
+        <v>573406</v>
       </c>
       <c r="Z18" s="167">
         <f t="shared" si="1"/>
@@ -11714,7 +11971,7 @@
       <c r="R19" s="158"/>
       <c r="S19" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-2608</v>
+        <v>-4573</v>
       </c>
       <c r="T19" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11725,7 +11982,7 @@
       <c r="W19" s="149"/>
       <c r="Y19" s="153">
         <f t="shared" si="0"/>
-        <v>-33</v>
+        <v>-1998</v>
       </c>
       <c r="Z19" s="167">
         <f t="shared" si="1"/>
@@ -11885,7 +12142,7 @@
       <c r="R21" s="158"/>
       <c r="S21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>116171</v>
+        <v>100881</v>
       </c>
       <c r="T21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11896,7 +12153,7 @@
       <c r="W21" s="72"/>
       <c r="Y21" s="153">
         <f t="shared" si="0"/>
-        <v>-135011</v>
+        <v>-150301</v>
       </c>
       <c r="Z21" s="167">
         <f t="shared" si="1"/>
@@ -11966,7 +12223,7 @@
       <c r="R22" s="158"/>
       <c r="S22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>127541</v>
+        <v>118167</v>
       </c>
       <c r="T22" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11977,7 +12234,7 @@
       <c r="W22" s="72"/>
       <c r="Y22" s="153">
         <f t="shared" si="0"/>
-        <v>-76082</v>
+        <v>-85456</v>
       </c>
       <c r="Z22" s="167">
         <f t="shared" si="1"/>
@@ -12128,7 +12385,7 @@
       <c r="R24" s="158"/>
       <c r="S24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>24274</v>
+        <v>10890</v>
       </c>
       <c r="T24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12139,7 +12396,7 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="153">
         <f t="shared" si="0"/>
-        <v>1770455</v>
+        <v>1757071</v>
       </c>
       <c r="Z24" s="167">
         <f t="shared" si="1"/>
@@ -12450,7 +12707,7 @@
       <c r="R28" s="158"/>
       <c r="S28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>76475</v>
+        <v>307075</v>
       </c>
       <c r="T28" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12461,7 +12718,7 @@
       <c r="W28" s="72"/>
       <c r="Y28" s="153">
         <f t="shared" si="0"/>
-        <v>454743</v>
+        <v>685343</v>
       </c>
       <c r="Z28" s="167">
         <f t="shared" si="1"/>
@@ -12531,7 +12788,7 @@
       <c r="R29" s="158"/>
       <c r="S29" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>83439</v>
+        <v>240439</v>
       </c>
       <c r="T29" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12543,7 +12800,7 @@
       <c r="X29" s="1"/>
       <c r="Y29" s="153">
         <f t="shared" si="0"/>
-        <v>962892</v>
+        <v>1119892</v>
       </c>
       <c r="Z29" s="167">
         <f t="shared" si="1"/>
@@ -12784,7 +13041,7 @@
       <c r="R32" s="158"/>
       <c r="S32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>482273</v>
+        <v>499483</v>
       </c>
       <c r="T32" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12796,7 +13053,7 @@
       <c r="X32"/>
       <c r="Y32" s="153">
         <f t="shared" si="0"/>
-        <v>-3732</v>
+        <v>13478</v>
       </c>
       <c r="Z32" s="167">
         <f t="shared" si="1"/>
@@ -12947,7 +13204,7 @@
       <c r="R34" s="158"/>
       <c r="S34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>16051</v>
+        <v>-24256</v>
       </c>
       <c r="T34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12958,7 +13215,7 @@
       <c r="W34" s="72"/>
       <c r="Y34" s="153">
         <f t="shared" si="0"/>
-        <v>-131576</v>
+        <v>-171883</v>
       </c>
       <c r="Z34" s="167">
         <f t="shared" si="1"/>
@@ -13116,7 +13373,7 @@
       <c r="R36" s="158"/>
       <c r="S36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-4207</v>
+        <v>-158874</v>
       </c>
       <c r="T36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13127,7 +13384,7 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="153">
         <f t="shared" si="0"/>
-        <v>2898419</v>
+        <v>2743752</v>
       </c>
       <c r="Z36" s="167">
         <f t="shared" si="1"/>
@@ -13195,7 +13452,7 @@
       <c r="R37" s="158"/>
       <c r="S37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-3157</v>
+        <v>-14276</v>
       </c>
       <c r="T37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13206,7 +13463,7 @@
       <c r="W37" s="149"/>
       <c r="Y37" s="153">
         <f t="shared" ref="Y37" si="22">M37+P37+S37+V37</f>
-        <v>-46823</v>
+        <v>-57942</v>
       </c>
       <c r="Z37" s="167">
         <f t="shared" ref="Z37" si="23">(N37+Q37+T37+W37)</f>
@@ -13276,7 +13533,7 @@
       <c r="R38" s="158"/>
       <c r="S38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>107300</v>
+        <v>210300</v>
       </c>
       <c r="T38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13287,7 +13544,7 @@
       <c r="W38" s="72"/>
       <c r="Y38" s="153">
         <f t="shared" si="0"/>
-        <v>2648354</v>
+        <v>2751354</v>
       </c>
       <c r="Z38" s="167">
         <f t="shared" si="1"/>
@@ -13357,7 +13614,7 @@
       <c r="R39" s="158"/>
       <c r="S39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>1216859</v>
+        <v>568459</v>
       </c>
       <c r="T39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13369,7 +13626,7 @@
       <c r="X39" s="131"/>
       <c r="Y39" s="153">
         <f t="shared" ref="Y39:Y74" si="24">M39+P39+S39+V39</f>
-        <v>6497606</v>
+        <v>5849206</v>
       </c>
       <c r="Z39" s="167">
         <f t="shared" ref="Z39:Z74" si="25">(N39+Q39+T39+W39)</f>
@@ -13873,7 +14130,7 @@
       <c r="R45" s="158"/>
       <c r="S45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>621985</v>
+        <v>841174</v>
       </c>
       <c r="T45" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13884,7 +14141,7 @@
       <c r="W45" s="72"/>
       <c r="Y45" s="153">
         <f t="shared" si="24"/>
-        <v>1722863</v>
+        <v>1942052</v>
       </c>
       <c r="Z45" s="167">
         <f t="shared" si="25"/>
@@ -14037,7 +14294,7 @@
       <c r="R47" s="158"/>
       <c r="S47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>139658</v>
+        <v>61055</v>
       </c>
       <c r="T47" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14048,7 +14305,7 @@
       <c r="W47" s="72"/>
       <c r="Y47" s="153">
         <f t="shared" si="24"/>
-        <v>60608</v>
+        <v>-17995</v>
       </c>
       <c r="Z47" s="167">
         <f t="shared" si="25"/>
@@ -14206,7 +14463,7 @@
       <c r="R49" s="158"/>
       <c r="S49" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>201245</v>
+        <v>241006</v>
       </c>
       <c r="T49" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14217,7 +14474,7 @@
       <c r="W49" s="72"/>
       <c r="Y49" s="153">
         <f t="shared" si="24"/>
-        <v>269510</v>
+        <v>309271</v>
       </c>
       <c r="Z49" s="167">
         <f t="shared" si="25"/>
@@ -14461,7 +14718,7 @@
       <c r="R52" s="158"/>
       <c r="S52" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>163505</v>
+        <v>213605</v>
       </c>
       <c r="T52" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14472,7 +14729,7 @@
       <c r="W52" s="72"/>
       <c r="Y52" s="153">
         <f t="shared" si="24"/>
-        <v>358566</v>
+        <v>408666</v>
       </c>
       <c r="Z52" s="167">
         <f t="shared" si="25"/>
@@ -14542,7 +14799,7 @@
       <c r="R53" s="158"/>
       <c r="S53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>6239</v>
+        <v>-50565</v>
       </c>
       <c r="T53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14553,7 +14810,7 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="153">
         <f t="shared" si="24"/>
-        <v>666488</v>
+        <v>609684</v>
       </c>
       <c r="Z53" s="167">
         <f t="shared" si="25"/>
@@ -14704,7 +14961,7 @@
       <c r="R55" s="158"/>
       <c r="S55" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-27574</v>
+        <v>-33174</v>
       </c>
       <c r="T55" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14716,7 +14973,7 @@
       <c r="X55" s="131"/>
       <c r="Y55" s="153">
         <f t="shared" si="24"/>
-        <v>-301599</v>
+        <v>-307199</v>
       </c>
       <c r="Z55" s="167">
         <f t="shared" si="25"/>
@@ -14787,7 +15044,7 @@
       <c r="R56" s="158"/>
       <c r="S56" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>647499</v>
+        <v>870499</v>
       </c>
       <c r="T56" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14798,7 +15055,7 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="153">
         <f t="shared" si="24"/>
-        <v>-4006836</v>
+        <v>-3783836</v>
       </c>
       <c r="Z56" s="167">
         <f t="shared" si="25"/>
@@ -15130,7 +15387,7 @@
       <c r="R60" s="158"/>
       <c r="S60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-901416</v>
+        <v>-973390</v>
       </c>
       <c r="T60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15141,7 +15398,7 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="153">
         <f t="shared" si="24"/>
-        <v>2778199</v>
+        <v>2706225</v>
       </c>
       <c r="Z60" s="167">
         <f t="shared" si="25"/>
@@ -15216,7 +15473,7 @@
       <c r="R61" s="158"/>
       <c r="S61" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-33711</v>
+        <v>-19211</v>
       </c>
       <c r="T61" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15227,7 +15484,7 @@
       <c r="W61" s="149"/>
       <c r="Y61" s="153">
         <f t="shared" ref="Y61" si="39">M61+P61+S61+V61</f>
-        <v>-20420</v>
+        <v>-5920</v>
       </c>
       <c r="Z61" s="167">
         <f t="shared" ref="Z61" si="40">(N61+Q61+T61+W61)</f>
@@ -15297,7 +15554,7 @@
       <c r="R62" s="158"/>
       <c r="S62" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>898923</v>
+        <v>1105039</v>
       </c>
       <c r="T62" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15308,7 +15565,7 @@
       <c r="W62" s="72"/>
       <c r="Y62" s="153">
         <f t="shared" si="24"/>
-        <v>1742024</v>
+        <v>1948140</v>
       </c>
       <c r="Z62" s="167">
         <f t="shared" si="25"/>
@@ -15548,7 +15805,7 @@
       <c r="R65" s="158"/>
       <c r="S65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>167758</v>
+        <v>51413</v>
       </c>
       <c r="T65" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15560,7 +15817,7 @@
       <c r="X65" s="131"/>
       <c r="Y65" s="153">
         <f t="shared" si="24"/>
-        <v>950539</v>
+        <v>834194</v>
       </c>
       <c r="Z65" s="167">
         <f t="shared" si="25"/>
@@ -15710,7 +15967,7 @@
       <c r="R67" s="158"/>
       <c r="S67" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1334350</v>
+        <v>-2083550</v>
       </c>
       <c r="T67" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15721,7 +15978,7 @@
       <c r="W67" s="149"/>
       <c r="Y67" s="153">
         <f t="shared" ref="Y67" si="45">M67+P67+S67+V67</f>
-        <v>-2297179</v>
+        <v>-3046379</v>
       </c>
       <c r="Z67" s="167">
         <f t="shared" ref="Z67" si="46">(N67+Q67+T67+W67)</f>
@@ -15929,7 +16186,7 @@
       <c r="R70" s="158"/>
       <c r="S70" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>418303</v>
+        <v>369643</v>
       </c>
       <c r="T70" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15940,7 +16197,7 @@
       <c r="W70" s="149"/>
       <c r="Y70" s="153">
         <f t="shared" si="24"/>
-        <v>57472</v>
+        <v>8812</v>
       </c>
       <c r="Z70" s="167">
         <f t="shared" si="25"/>
@@ -16172,7 +16429,7 @@
       <c r="R73" s="158"/>
       <c r="S73" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>284547</v>
+        <v>311687</v>
       </c>
       <c r="T73" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16183,7 +16440,7 @@
       <c r="W73" s="72"/>
       <c r="Y73" s="153">
         <f t="shared" si="24"/>
-        <v>656851</v>
+        <v>683991</v>
       </c>
       <c r="Z73" s="167">
         <f t="shared" si="25"/>
@@ -16411,7 +16668,7 @@
       <c r="R76" s="158"/>
       <c r="S76" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>600079</v>
+        <v>765329</v>
       </c>
       <c r="T76" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$139,'FY-(26-27)Q3'!$A$4:$ABW$115,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16422,7 +16679,7 @@
       <c r="W76" s="149"/>
       <c r="Y76" s="153">
         <f t="shared" si="55"/>
-        <v>1090932</v>
+        <v>1256182</v>
       </c>
       <c r="Z76" s="167">
         <f t="shared" si="56"/>
@@ -16465,7 +16722,7 @@
       <c r="R77" s="122"/>
       <c r="S77" s="109">
         <f>SUM(S4:S74)</f>
-        <v>5409456</v>
+        <v>4651917</v>
       </c>
       <c r="T77" s="122"/>
       <c r="U77" s="122"/>
@@ -16473,7 +16730,7 @@
       <c r="W77" s="50"/>
       <c r="Y77" s="153">
         <f>SUM(Y4:Y76)</f>
-        <v>29390751</v>
+        <v>28798462</v>
       </c>
       <c r="Z77" s="160"/>
     </row>
@@ -18255,12 +18512,12 @@
         <v>0.5</v>
       </c>
       <c r="G4" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>121236</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>116447</v>
       </c>
       <c r="H4" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>2.4247200000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>2.3289399999999998</v>
       </c>
       <c r="I4" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18280,11 +18537,11 @@
       </c>
       <c r="M4" s="71">
         <f t="shared" ref="M4:N50" si="0">G4+I4+K4</f>
-        <v>121236</v>
+        <v>116447</v>
       </c>
       <c r="N4" s="165">
         <f t="shared" si="0"/>
-        <v>2.4247200000000002</v>
+        <v>2.3289399999999998</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -18307,12 +18564,12 @@
         <v>3.5</v>
       </c>
       <c r="G5" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>469496</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>526832</v>
       </c>
       <c r="H5" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.5649866666666665</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.7561066666666665</v>
       </c>
       <c r="I5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18332,11 +18589,11 @@
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>469496</v>
+        <v>526832</v>
       </c>
       <c r="N5" s="165">
         <f t="shared" si="0"/>
-        <v>1.5649866666666665</v>
+        <v>1.7561066666666665</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -18359,12 +18616,12 @@
         <v>1</v>
       </c>
       <c r="G6" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>316777</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>409977</v>
       </c>
       <c r="H6" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>3.16777</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>4.0997700000000004</v>
       </c>
       <c r="I6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18384,11 +18641,11 @@
       </c>
       <c r="M6" s="71">
         <f t="shared" si="0"/>
-        <v>316777</v>
+        <v>409977</v>
       </c>
       <c r="N6" s="165">
         <f t="shared" si="0"/>
-        <v>3.16777</v>
+        <v>4.0997700000000004</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -18411,12 +18668,12 @@
         <v>3</v>
       </c>
       <c r="G7" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-100437</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-28937</v>
       </c>
       <c r="H7" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-0.33478999999999998</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-9.6456666666666663E-2</v>
       </c>
       <c r="I7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18436,11 +18693,11 @@
       </c>
       <c r="M7" s="71">
         <f t="shared" si="0"/>
-        <v>-100437</v>
+        <v>-28937</v>
       </c>
       <c r="N7" s="165">
         <f t="shared" si="0"/>
-        <v>-0.33478999999999998</v>
+        <v>-9.6456666666666663E-2</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -18463,12 +18720,12 @@
         <v>1.5</v>
       </c>
       <c r="G8" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>300980</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>222269</v>
       </c>
       <c r="H8" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>2.0065333333333335</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.4817933333333333</v>
       </c>
       <c r="I8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18488,11 +18745,11 @@
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>300980</v>
+        <v>222269</v>
       </c>
       <c r="N8" s="165">
         <f t="shared" si="0"/>
-        <v>2.0065333333333335</v>
+        <v>1.4817933333333333</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -18515,12 +18772,12 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>107224</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>168124</v>
       </c>
       <c r="H9" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.7870666666666668</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>2.8020666666666667</v>
       </c>
       <c r="I9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18540,11 +18797,11 @@
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>107224</v>
+        <v>168124</v>
       </c>
       <c r="N9" s="165">
         <f t="shared" si="0"/>
-        <v>1.7870666666666668</v>
+        <v>2.8020666666666667</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -18567,12 +18824,12 @@
         <v>15</v>
       </c>
       <c r="G10" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-136160</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-88659</v>
       </c>
       <c r="H10" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-9.0773333333333331E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-5.9105999999999999E-2</v>
       </c>
       <c r="I10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18592,11 +18849,11 @@
       </c>
       <c r="M10" s="71">
         <f t="shared" si="0"/>
-        <v>-136160</v>
+        <v>-88659</v>
       </c>
       <c r="N10" s="165">
         <f t="shared" si="0"/>
-        <v>-9.0773333333333331E-2</v>
+        <v>-5.9105999999999999E-2</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -18619,12 +18876,12 @@
         <v>6</v>
       </c>
       <c r="G11" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>643754</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>373354</v>
       </c>
       <c r="H11" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.0729233333333332</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.62225666666666657</v>
       </c>
       <c r="I11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18644,11 +18901,11 @@
       </c>
       <c r="M11" s="71">
         <f t="shared" si="0"/>
-        <v>643754</v>
+        <v>373354</v>
       </c>
       <c r="N11" s="165">
         <f t="shared" si="0"/>
-        <v>1.0729233333333332</v>
+        <v>0.62225666666666657</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -18671,12 +18928,12 @@
         <v>1</v>
       </c>
       <c r="G12" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-2608</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-4573</v>
       </c>
       <c r="H12" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-2.6079999999999999E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-4.573E-2</v>
       </c>
       <c r="I12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18696,11 +18953,11 @@
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>-2608</v>
+        <v>-4573</v>
       </c>
       <c r="N12" s="165">
         <f t="shared" si="0"/>
-        <v>-2.6079999999999999E-2</v>
+        <v>-4.573E-2</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -18723,12 +18980,12 @@
         <v>1</v>
       </c>
       <c r="G13" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>116171</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>100881</v>
       </c>
       <c r="H13" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.46468399999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.40352399999999999</v>
       </c>
       <c r="I13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18748,11 +19005,11 @@
       </c>
       <c r="M13" s="71">
         <f t="shared" si="0"/>
-        <v>116171</v>
+        <v>100881</v>
       </c>
       <c r="N13" s="165">
         <f t="shared" si="0"/>
-        <v>0.46468399999999999</v>
+        <v>0.40352399999999999</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -18775,12 +19032,12 @@
         <v>1</v>
       </c>
       <c r="G14" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>24274</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>10890</v>
       </c>
       <c r="H14" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.24274000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.1089</v>
       </c>
       <c r="I14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18800,11 +19057,11 @@
       </c>
       <c r="M14" s="71">
         <f t="shared" si="0"/>
-        <v>24274</v>
+        <v>10890</v>
       </c>
       <c r="N14" s="165">
         <f t="shared" si="0"/>
-        <v>0.24274000000000001</v>
+        <v>0.1089</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -18827,12 +19084,12 @@
         <v>0.2</v>
       </c>
       <c r="G15" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>127541</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>118167</v>
       </c>
       <c r="H15" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.57973181818181818</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.53712272727272725</v>
       </c>
       <c r="I15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18852,11 +19109,11 @@
       </c>
       <c r="M15" s="71">
         <f t="shared" si="0"/>
-        <v>127541</v>
+        <v>118167</v>
       </c>
       <c r="N15" s="165">
         <f t="shared" si="0"/>
-        <v>0.57973181818181818</v>
+        <v>0.53712272727272725</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -18879,12 +19136,12 @@
         <v>2.5</v>
       </c>
       <c r="G16" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>76475</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>307075</v>
       </c>
       <c r="H16" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.30590000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.2282999999999999</v>
       </c>
       <c r="I16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18904,11 +19161,11 @@
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>76475</v>
+        <v>307075</v>
       </c>
       <c r="N16" s="165">
         <f t="shared" si="0"/>
-        <v>0.30590000000000001</v>
+        <v>1.2282999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -18931,12 +19188,12 @@
         <v>4</v>
       </c>
       <c r="G17" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>83439</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>240439</v>
       </c>
       <c r="H17" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.20859749999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.60109749999999995</v>
       </c>
       <c r="I17" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -18956,11 +19213,11 @@
       </c>
       <c r="M17" s="71">
         <f t="shared" si="0"/>
-        <v>83439</v>
+        <v>240439</v>
       </c>
       <c r="N17" s="165">
         <f t="shared" si="0"/>
-        <v>0.20859749999999999</v>
+        <v>0.60109749999999995</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -18983,11 +19240,11 @@
         <v>0.25</v>
       </c>
       <c r="G18" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>-150688</v>
       </c>
       <c r="H18" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>-1.3698909090909093</v>
       </c>
       <c r="I18" s="152">
@@ -19035,11 +19292,11 @@
         <v>0.25</v>
       </c>
       <c r="G19" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>-107972</v>
       </c>
       <c r="H19" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>-4.3188800000000001</v>
       </c>
       <c r="I19" s="152">
@@ -19087,11 +19344,11 @@
         <v>2</v>
       </c>
       <c r="G20" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="152">
@@ -19139,12 +19396,12 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>482273</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>499483</v>
       </c>
       <c r="H21" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>3.2151533333333333</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>3.3298866666666669</v>
       </c>
       <c r="I21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19164,11 +19421,11 @@
       </c>
       <c r="M21" s="71">
         <f t="shared" si="0"/>
-        <v>482273</v>
+        <v>499483</v>
       </c>
       <c r="N21" s="165">
         <f t="shared" si="0"/>
-        <v>3.2151533333333333</v>
+        <v>3.3298866666666669</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -19191,12 +19448,12 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="G22" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>16051</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-24256</v>
       </c>
       <c r="H22" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.14591818181818181</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.22050909090909088</v>
       </c>
       <c r="I22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19216,11 +19473,11 @@
       </c>
       <c r="M22" s="71">
         <f t="shared" si="0"/>
-        <v>16051</v>
+        <v>-24256</v>
       </c>
       <c r="N22" s="165">
         <f t="shared" si="0"/>
-        <v>0.14591818181818181</v>
+        <v>-0.22050909090909088</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -19243,12 +19500,12 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G23" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-4207</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-158874</v>
       </c>
       <c r="H23" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-1.8291304347826085E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.6907565217391306</v>
       </c>
       <c r="I23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19268,11 +19525,11 @@
       </c>
       <c r="M23" s="71">
         <f t="shared" si="0"/>
-        <v>-4207</v>
+        <v>-158874</v>
       </c>
       <c r="N23" s="165">
         <f t="shared" si="0"/>
-        <v>-1.8291304347826085E-2</v>
+        <v>-0.6907565217391306</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -19293,12 +19550,12 @@
         <v>0.2</v>
       </c>
       <c r="G24" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-3157</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-14276</v>
       </c>
       <c r="H24" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-0.15784999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.71379999999999999</v>
       </c>
       <c r="I24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19318,11 +19575,11 @@
       </c>
       <c r="M24" s="71">
         <f t="shared" si="0"/>
-        <v>-3157</v>
+        <v>-14276</v>
       </c>
       <c r="N24" s="165">
         <f t="shared" si="0"/>
-        <v>-0.15784999999999999</v>
+        <v>-0.71379999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -19345,12 +19602,12 @@
         <v>5</v>
       </c>
       <c r="G25" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>107300</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>210300</v>
       </c>
       <c r="H25" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.21460000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.42059999999999997</v>
       </c>
       <c r="I25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19370,11 +19627,11 @@
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>107300</v>
+        <v>210300</v>
       </c>
       <c r="N25" s="165">
         <f t="shared" si="0"/>
-        <v>0.21460000000000001</v>
+        <v>0.42059999999999997</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -19397,12 +19654,12 @@
         <v>10</v>
       </c>
       <c r="G26" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1216859</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>568459</v>
       </c>
       <c r="H26" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.2168589999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.56845900000000005</v>
       </c>
       <c r="I26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19422,11 +19679,11 @@
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>1216859</v>
+        <v>568459</v>
       </c>
       <c r="N26" s="165">
         <f t="shared" si="0"/>
-        <v>1.2168589999999999</v>
+        <v>0.56845900000000005</v>
       </c>
       <c r="O26" s="130"/>
     </row>
@@ -19448,12 +19705,12 @@
         <v>1</v>
       </c>
       <c r="G27" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>74309</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>47009</v>
       </c>
       <c r="H27" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.4861800000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.94018000000000002</v>
       </c>
       <c r="I27" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19473,11 +19730,11 @@
       </c>
       <c r="M27" s="71">
         <f t="shared" ref="M27" si="1">G27+I27+K27</f>
-        <v>74309</v>
+        <v>47009</v>
       </c>
       <c r="N27" s="165">
         <f t="shared" ref="N27" si="2">H27+J27+L27</f>
-        <v>1.4861800000000001</v>
+        <v>0.94018000000000002</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -19500,12 +19757,12 @@
         <v>5</v>
       </c>
       <c r="G28" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>621985</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>841174</v>
       </c>
       <c r="H28" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>1.24397</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.682348</v>
       </c>
       <c r="I28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19525,11 +19782,11 @@
       </c>
       <c r="M28" s="71">
         <f t="shared" si="0"/>
-        <v>621985</v>
+        <v>841174</v>
       </c>
       <c r="N28" s="165">
         <f t="shared" si="0"/>
-        <v>1.24397</v>
+        <v>1.682348</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -19552,11 +19809,11 @@
         <v>5</v>
       </c>
       <c r="G29" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>140133</v>
       </c>
       <c r="H29" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0.28026600000000002</v>
       </c>
       <c r="I29" s="152">
@@ -19604,12 +19861,12 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>139658</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>61055</v>
       </c>
       <c r="H30" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>2.7931599999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.2211000000000001</v>
       </c>
       <c r="I30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19629,11 +19886,11 @@
       </c>
       <c r="M30" s="71">
         <f t="shared" si="0"/>
-        <v>139658</v>
+        <v>61055</v>
       </c>
       <c r="N30" s="165">
         <f t="shared" si="0"/>
-        <v>2.7931599999999999</v>
+        <v>1.2211000000000001</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -19656,12 +19913,12 @@
         <v>0.4</v>
       </c>
       <c r="G31" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>201245</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>241006</v>
       </c>
       <c r="H31" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>5.0311250000000003</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>6.02515</v>
       </c>
       <c r="I31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19681,11 +19938,11 @@
       </c>
       <c r="M31" s="71">
         <f t="shared" si="0"/>
-        <v>201245</v>
+        <v>241006</v>
       </c>
       <c r="N31" s="165">
         <f t="shared" si="0"/>
-        <v>5.0311250000000003</v>
+        <v>6.02515</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -19708,12 +19965,12 @@
         <v>4</v>
       </c>
       <c r="G32" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>163505</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>213605</v>
       </c>
       <c r="H32" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.40876249999999997</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.5340125</v>
       </c>
       <c r="I32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19733,11 +19990,11 @@
       </c>
       <c r="M32" s="71">
         <f t="shared" si="0"/>
-        <v>163505</v>
+        <v>213605</v>
       </c>
       <c r="N32" s="165">
         <f t="shared" si="0"/>
-        <v>0.40876249999999997</v>
+        <v>0.5340125</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -19760,12 +20017,12 @@
         <v>1</v>
       </c>
       <c r="G33" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>6239</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-50565</v>
       </c>
       <c r="H33" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>6.2390000000000001E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.50565000000000004</v>
       </c>
       <c r="I33" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19785,11 +20042,11 @@
       </c>
       <c r="M33" s="71">
         <f t="shared" si="0"/>
-        <v>6239</v>
+        <v>-50565</v>
       </c>
       <c r="N33" s="165">
         <f t="shared" si="0"/>
-        <v>6.2390000000000001E-2</v>
+        <v>-0.50565000000000004</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -19810,11 +20067,11 @@
       </c>
       <c r="F34" s="155"/>
       <c r="G34" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H34" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I34" s="152">
@@ -19862,12 +20119,12 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-27574</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-33174</v>
       </c>
       <c r="H35" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-0.55147999999999997</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.66347999999999996</v>
       </c>
       <c r="I35" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19887,11 +20144,11 @@
       </c>
       <c r="M35" s="71">
         <f t="shared" si="0"/>
-        <v>-27574</v>
+        <v>-33174</v>
       </c>
       <c r="N35" s="165">
         <f t="shared" si="0"/>
-        <v>-0.55147999999999997</v>
+        <v>-0.66347999999999996</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -19914,12 +20171,12 @@
         <v>1</v>
       </c>
       <c r="G36" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>647499</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>870499</v>
       </c>
       <c r="H36" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>2.1583299999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>2.901663333333333</v>
       </c>
       <c r="I36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19939,11 +20196,11 @@
       </c>
       <c r="M36" s="71">
         <f t="shared" si="0"/>
-        <v>647499</v>
+        <v>870499</v>
       </c>
       <c r="N36" s="165">
         <f t="shared" si="0"/>
-        <v>2.1583299999999999</v>
+        <v>2.901663333333333</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -19964,12 +20221,12 @@
         <v>0.1</v>
       </c>
       <c r="G37" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-39672</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-6772</v>
       </c>
       <c r="H37" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-3.9672000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-0.67720000000000002</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19989,11 +20246,11 @@
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>-39672</v>
+        <v>-6772</v>
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>-3.9672000000000001</v>
+        <v>-0.67720000000000002</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -20016,11 +20273,11 @@
         <v>1</v>
       </c>
       <c r="G38" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>27311</v>
       </c>
       <c r="H38" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0.54622000000000004</v>
       </c>
       <c r="I38" s="152">
@@ -20068,12 +20325,12 @@
         <v>1</v>
       </c>
       <c r="G39" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-901416</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-973390</v>
       </c>
       <c r="H39" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-9.0141600000000004</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-9.7339000000000002</v>
       </c>
       <c r="I39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20093,11 +20350,11 @@
       </c>
       <c r="M39" s="71">
         <f t="shared" si="0"/>
-        <v>-901416</v>
+        <v>-973390</v>
       </c>
       <c r="N39" s="165">
         <f t="shared" si="0"/>
-        <v>-9.0141600000000004</v>
+        <v>-9.7339000000000002</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -20118,12 +20375,12 @@
         <v>0.1</v>
       </c>
       <c r="G40" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-33711</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-19211</v>
       </c>
       <c r="H40" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-3.3711000000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-1.9211</v>
       </c>
       <c r="I40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20143,11 +20400,11 @@
       </c>
       <c r="M40" s="71">
         <f t="shared" si="0"/>
-        <v>-33711</v>
+        <v>-19211</v>
       </c>
       <c r="N40" s="165">
         <f t="shared" si="0"/>
-        <v>-3.3711000000000002</v>
+        <v>-1.9211</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -20170,12 +20427,12 @@
         <v>1</v>
       </c>
       <c r="G41" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>898923</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1105039</v>
       </c>
       <c r="H41" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>2.99641</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>3.6834633333333326</v>
       </c>
       <c r="I41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20195,11 +20452,11 @@
       </c>
       <c r="M41" s="71">
         <f t="shared" si="0"/>
-        <v>898923</v>
+        <v>1105039</v>
       </c>
       <c r="N41" s="165">
         <f t="shared" si="0"/>
-        <v>2.99641</v>
+        <v>3.6834633333333326</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -20216,11 +20473,11 @@
         <v>1</v>
       </c>
       <c r="G42" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H42" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I42" s="152">
@@ -20268,11 +20525,11 @@
         <v>4</v>
       </c>
       <c r="G43" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>112320</v>
       </c>
       <c r="H43" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0.28079999999999999</v>
       </c>
       <c r="I43" s="152">
@@ -20320,12 +20577,12 @@
         <v>4</v>
       </c>
       <c r="G44" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>167758</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>51413</v>
       </c>
       <c r="H44" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.41939500000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.12853249999999999</v>
       </c>
       <c r="I44" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20345,11 +20602,11 @@
       </c>
       <c r="M44" s="71">
         <f t="shared" si="0"/>
-        <v>167758</v>
+        <v>51413</v>
       </c>
       <c r="N44" s="165">
         <f t="shared" si="0"/>
-        <v>0.41939500000000002</v>
+        <v>0.12853249999999999</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -20370,12 +20627,12 @@
         <v>0.1</v>
       </c>
       <c r="G45" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-1334350</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-2083550</v>
       </c>
       <c r="H45" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-1.3343499999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-2.0835499999999998</v>
       </c>
       <c r="I45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20395,11 +20652,11 @@
       </c>
       <c r="M45" s="71">
         <f t="shared" si="0"/>
-        <v>-1334350</v>
+        <v>-2083550</v>
       </c>
       <c r="N45" s="165">
         <f t="shared" si="0"/>
-        <v>-1.3343499999999999</v>
+        <v>-2.0835499999999998</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -20416,11 +20673,11 @@
       </c>
       <c r="F46" s="114"/>
       <c r="G46" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H46" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I46" s="152">
@@ -20468,11 +20725,11 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>64488</v>
       </c>
       <c r="H47" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>1.28976</v>
       </c>
       <c r="I47" s="152">
@@ -20520,12 +20777,12 @@
         <v>5</v>
       </c>
       <c r="G48" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>418303</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>369643</v>
       </c>
       <c r="H48" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.643543076923077</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.56868153846153835</v>
       </c>
       <c r="I48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20545,11 +20802,11 @@
       </c>
       <c r="M48" s="71">
         <f t="shared" si="0"/>
-        <v>418303</v>
+        <v>369643</v>
       </c>
       <c r="N48" s="165">
         <f t="shared" si="0"/>
-        <v>0.643543076923077</v>
+        <v>0.56868153846153835</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -20572,11 +20829,11 @@
         <v>1</v>
       </c>
       <c r="G49" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H49" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I49" s="152">
@@ -20624,12 +20881,12 @@
         <v>2.5</v>
       </c>
       <c r="G50" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>284547</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>311687</v>
       </c>
       <c r="H50" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.94849000000000006</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>1.0389566666666668</v>
       </c>
       <c r="I50" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20649,11 +20906,11 @@
       </c>
       <c r="M50" s="71">
         <f t="shared" si="0"/>
-        <v>284547</v>
+        <v>311687</v>
       </c>
       <c r="N50" s="165">
         <f t="shared" si="0"/>
-        <v>0.94849000000000006</v>
+        <v>1.0389566666666668</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -20676,11 +20933,11 @@
         <v>0.25</v>
       </c>
       <c r="G51" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I51" s="152">
@@ -20728,12 +20985,12 @@
         <v>5</v>
       </c>
       <c r="G52" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>600079</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>765329</v>
       </c>
       <c r="H52" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>0.60007900000000003</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>0.76532899999999993</v>
       </c>
       <c r="I52" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20753,11 +21010,11 @@
       </c>
       <c r="M52" s="71">
         <f t="shared" si="3"/>
-        <v>600079</v>
+        <v>765329</v>
       </c>
       <c r="N52" s="165">
         <f t="shared" si="3"/>
-        <v>0.60007900000000003</v>
+        <v>0.76532899999999993</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -20769,7 +21026,7 @@
       <c r="F53" s="233"/>
       <c r="G53" s="230">
         <f>SUM(G4:G50)</f>
-        <v>5336121</v>
+        <v>4584182</v>
       </c>
       <c r="H53" s="90"/>
       <c r="I53" s="99">
@@ -20784,7 +21041,7 @@
       <c r="L53" s="109"/>
       <c r="M53" s="153">
         <f>SUM(M4:M50)</f>
-        <v>5336121</v>
+        <v>4584182</v>
       </c>
       <c r="N53" s="234"/>
     </row>
@@ -20848,12 +21105,12 @@
       <c r="E57" s="208"/>
       <c r="F57" s="206"/>
       <c r="G57" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-35230</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-330</v>
       </c>
       <c r="H57" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-0.11743333333333335</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-1.1000000000000001E-3</v>
       </c>
       <c r="I57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$114,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20873,11 +21130,11 @@
       </c>
       <c r="M57" s="152">
         <f t="shared" ref="M57:N58" si="4">G57+I57+K57</f>
-        <v>-35230</v>
+        <v>-330</v>
       </c>
       <c r="N57" s="166">
         <f t="shared" si="4"/>
-        <v>-0.11743333333333335</v>
+        <v>-1.1000000000000001E-3</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -20898,11 +21155,11 @@
       </c>
       <c r="F58" s="237"/>
       <c r="G58" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
-        <v>-218465</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
+        <v>-237594</v>
       </c>
       <c r="H58" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADC$118,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DD$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$114,'OCT-2026'!$A$4:$ADD$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DE$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I58" s="152">
@@ -20923,7 +21180,7 @@
       </c>
       <c r="M58" s="152">
         <f t="shared" si="4"/>
-        <v>-218465</v>
+        <v>-237594</v>
       </c>
       <c r="N58" s="166">
         <f t="shared" si="4"/>
@@ -20933,7 +21190,7 @@
     <row r="59" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G59" s="93">
         <f>SUM(G57:G58)</f>
-        <v>-253695</v>
+        <v>-237924</v>
       </c>
       <c r="H59" s="94"/>
       <c r="I59" s="93">
@@ -20948,7 +21205,7 @@
       <c r="L59" s="113"/>
       <c r="M59" s="93">
         <f>SUM(M57:M58)</f>
-        <v>-253695</v>
+        <v>-237924</v>
       </c>
       <c r="N59" s="235"/>
     </row>
@@ -40126,7 +40383,7 @@
         <v>30</v>
       </c>
       <c r="B5" s="140" t="s">
-        <v>309</v>
+        <v>341</v>
       </c>
       <c r="C5" s="140" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Mon 10/26/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3255" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3256" uniqueCount="346">
   <si>
     <t>Sudeep</t>
   </si>
@@ -6505,7 +6505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ69"/>
+  <dimension ref="A1:AK69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="132" customWidth="1" outlineLevel="1"/>
@@ -6517,20 +6517,19 @@
     <col min="7" max="7" width="1.7109375" style="132" customWidth="1"/>
     <col min="8" max="17" width="13.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="18" max="18" width="13.42578125" style="132" customWidth="1" collapsed="1"/>
-    <col min="19" max="22" width="13.42578125" style="132" customWidth="1"/>
-    <col min="23" max="23" width="11.28515625" style="132" customWidth="1"/>
-    <col min="24" max="24" width="10.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="10.7109375" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="9.140625" style="132" collapsed="1"/>
-    <col min="27" max="31" width="9.140625" style="132"/>
-    <col min="32" max="32" width="14.140625" style="132" customWidth="1"/>
-    <col min="33" max="33" width="12" style="132" customWidth="1"/>
-    <col min="34" max="34" width="15.85546875" style="132" customWidth="1"/>
-    <col min="35" max="16384" width="9.140625" style="132"/>
+    <col min="19" max="23" width="13.42578125" style="132" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" style="132" customWidth="1"/>
+    <col min="25" max="25" width="10.42578125" style="132" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="10.7109375" style="132" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="32" width="9.140625" style="132"/>
+    <col min="33" max="33" width="14.140625" style="132" customWidth="1"/>
+    <col min="34" max="34" width="12" style="132" customWidth="1"/>
+    <col min="35" max="35" width="15.85546875" style="132" customWidth="1"/>
+    <col min="36" max="16384" width="9.140625" style="132"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G2" s="220"/>
       <c r="H2" s="255">
         <v>46296</v>
@@ -6577,15 +6576,18 @@
       <c r="V2" s="255">
         <v>46318</v>
       </c>
-      <c r="W2" s="182"/>
-      <c r="X2" s="183" t="s">
+      <c r="W2" s="255">
+        <v>46321</v>
+      </c>
+      <c r="X2" s="182"/>
+      <c r="Y2" s="183" t="s">
         <v>325</v>
       </c>
-      <c r="Y2" s="184" t="s">
+      <c r="Z2" s="184" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="185" t="s">
         <v>54</v>
       </c>
@@ -6650,17 +6652,20 @@
       <c r="V3" s="178" t="s">
         <v>235</v>
       </c>
-      <c r="W3" s="179"/>
-      <c r="X3" s="188"/>
-      <c r="Y3" s="179"/>
-      <c r="AF3" s="132" t="s">
+      <c r="W3" s="178" t="s">
+        <v>234</v>
+      </c>
+      <c r="X3" s="179"/>
+      <c r="Y3" s="188"/>
+      <c r="Z3" s="179"/>
+      <c r="AG3" s="132" t="s">
         <v>198</v>
       </c>
-      <c r="AG3" s="132">
+      <c r="AH3" s="132">
         <v>13780</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="141" t="s">
         <v>216</v>
       </c>
@@ -6725,23 +6730,26 @@
       <c r="V4" s="157">
         <v>7452</v>
       </c>
-      <c r="W4" s="210"/>
-      <c r="X4" s="170">
-        <f t="shared" ref="X4" si="0">SUM(H4:W4)</f>
-        <v>129765</v>
-      </c>
-      <c r="Y4" s="148">
-        <f t="shared" ref="Y4" si="1">IFERROR(X4/F4*100,0)/10000000</f>
-        <v>2.5952999999999999</v>
-      </c>
-      <c r="AF4" s="132" t="s">
+      <c r="W4" s="157">
+        <v>-6562</v>
+      </c>
+      <c r="X4" s="210"/>
+      <c r="Y4" s="170">
+        <f t="shared" ref="Y4" si="0">SUM(H4:X4)</f>
+        <v>123203</v>
+      </c>
+      <c r="Z4" s="148">
+        <f t="shared" ref="Z4" si="1">IFERROR(Y4/F4*100,0)/10000000</f>
+        <v>2.4640599999999999</v>
+      </c>
+      <c r="AG4" s="132" t="s">
         <v>170</v>
       </c>
-      <c r="AG4" s="132">
+      <c r="AH4" s="132">
         <v>2865</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="141" t="s">
         <v>343</v>
       </c>
@@ -6806,17 +6814,20 @@
       <c r="V5" s="146">
         <v>106000</v>
       </c>
-      <c r="W5" s="173"/>
-      <c r="X5" s="170">
-        <f t="shared" ref="X5:X53" si="2">SUM(H5:W5)</f>
-        <v>438873</v>
-      </c>
-      <c r="Y5" s="148">
-        <f t="shared" ref="Y5:Y53" si="3">IFERROR(X5/F5*100,0)/10000000</f>
-        <v>1.4629099999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="W5" s="146">
+        <v>-57900</v>
+      </c>
+      <c r="X5" s="173"/>
+      <c r="Y5" s="170">
+        <f t="shared" ref="Y5:Y53" si="2">SUM(H5:X5)</f>
+        <v>380973</v>
+      </c>
+      <c r="Z5" s="148">
+        <f t="shared" ref="Z5:Z53" si="3">IFERROR(Y5/F5*100,0)/10000000</f>
+        <v>1.2699100000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="141" t="s">
         <v>344</v>
       </c>
@@ -6881,17 +6892,20 @@
       <c r="V6" s="146">
         <v>-61600</v>
       </c>
-      <c r="W6" s="173"/>
-      <c r="X6" s="170">
+      <c r="W6" s="146">
+        <v>-169055</v>
+      </c>
+      <c r="X6" s="173"/>
+      <c r="Y6" s="170">
         <f t="shared" si="2"/>
-        <v>421142</v>
-      </c>
-      <c r="Y6" s="148">
+        <v>252087</v>
+      </c>
+      <c r="Z6" s="148">
         <f t="shared" si="3"/>
-        <v>4.2114200000000004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2.5208699999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="141" t="s">
         <v>134</v>
       </c>
@@ -6956,21 +6970,24 @@
       <c r="V7" s="146">
         <v>-37900</v>
       </c>
-      <c r="W7" s="173"/>
-      <c r="X7" s="170">
+      <c r="W7" s="146">
+        <v>92400</v>
+      </c>
+      <c r="X7" s="173"/>
+      <c r="Y7" s="170">
         <f t="shared" si="2"/>
-        <v>-100760</v>
-      </c>
-      <c r="Y7" s="148">
+        <v>-8360</v>
+      </c>
+      <c r="Z7" s="148">
         <f t="shared" si="3"/>
-        <v>-0.33586666666666665</v>
-      </c>
-      <c r="AA7" s="5"/>
-      <c r="AB7" s="133">
-        <v>3861</v>
-      </c>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+        <v>-2.7866666666666661E-2</v>
+      </c>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="133">
+        <v>5037</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="141" t="s">
         <v>217</v>
       </c>
@@ -7035,21 +7052,24 @@
       <c r="V8" s="146">
         <v>0</v>
       </c>
-      <c r="W8" s="173"/>
-      <c r="X8" s="170">
+      <c r="W8" s="146">
+        <v>-16364</v>
+      </c>
+      <c r="X8" s="173"/>
+      <c r="Y8" s="170">
         <f t="shared" si="2"/>
-        <v>272350</v>
-      </c>
-      <c r="Y8" s="148">
+        <v>255986</v>
+      </c>
+      <c r="Z8" s="148">
         <f t="shared" si="3"/>
-        <v>1.8156666666666663</v>
-      </c>
-      <c r="AA8" s="133">
-        <v>7319</v>
-      </c>
-      <c r="AB8" s="133"/>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+        <v>1.7065733333333335</v>
+      </c>
+      <c r="AB8" s="133">
+        <v>20085</v>
+      </c>
+      <c r="AC8" s="133"/>
+    </row>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="141" t="s">
         <v>313</v>
       </c>
@@ -7112,24 +7132,27 @@
       <c r="V9" s="146">
         <v>0</v>
       </c>
-      <c r="W9" s="173"/>
-      <c r="X9" s="170">
+      <c r="W9" s="146">
+        <v>50600</v>
+      </c>
+      <c r="X9" s="173"/>
+      <c r="Y9" s="170">
         <f t="shared" si="2"/>
-        <v>162827</v>
-      </c>
-      <c r="Y9" s="148">
+        <v>213427</v>
+      </c>
+      <c r="Z9" s="148">
         <f t="shared" si="3"/>
-        <v>2.7137833333333337</v>
-      </c>
-      <c r="AA9" s="133">
-        <v>11180</v>
+        <v>3.5571166666666674</v>
       </c>
       <c r="AB9" s="133">
-        <f>(AA9+AA8)/10000000*13780</f>
-        <v>25.491622</v>
-      </c>
-    </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+        <v>25122</v>
+      </c>
+      <c r="AC9" s="133">
+        <f>(AB9+AB8)/10000000*13780</f>
+        <v>62.295245999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="142" t="s">
         <v>35</v>
       </c>
@@ -7194,19 +7217,22 @@
       <c r="V10" s="146">
         <v>0</v>
       </c>
-      <c r="W10" s="173"/>
-      <c r="X10" s="170">
+      <c r="W10" s="146">
+        <v>0</v>
+      </c>
+      <c r="X10" s="173"/>
+      <c r="Y10" s="170">
         <f t="shared" si="2"/>
         <v>-87379</v>
       </c>
-      <c r="Y10" s="148">
+      <c r="Z10" s="148">
         <f t="shared" si="3"/>
         <v>-5.8252666666666661E-2</v>
       </c>
-      <c r="AA10" s="133"/>
       <c r="AB10" s="133"/>
-    </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AC10" s="133"/>
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="142" t="s">
         <v>137</v>
       </c>
@@ -7271,19 +7297,22 @@
       <c r="V11" s="146">
         <v>0</v>
       </c>
-      <c r="W11" s="173"/>
-      <c r="X11" s="170">
+      <c r="W11" s="146">
+        <v>12420</v>
+      </c>
+      <c r="X11" s="173"/>
+      <c r="Y11" s="170">
         <f t="shared" si="2"/>
-        <v>373354</v>
-      </c>
-      <c r="Y11" s="148">
+        <v>385774</v>
+      </c>
+      <c r="Z11" s="148">
         <f t="shared" si="3"/>
-        <v>0.62225666666666657</v>
-      </c>
-      <c r="AA11" s="133"/>
+        <v>0.64295666666666662</v>
+      </c>
       <c r="AB11" s="133"/>
-    </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AC11" s="133"/>
+    </row>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="142" t="s">
         <v>42</v>
       </c>
@@ -7348,19 +7377,22 @@
       <c r="V12" s="146">
         <v>-3576</v>
       </c>
-      <c r="W12" s="173"/>
-      <c r="X12" s="170">
+      <c r="W12" s="146">
+        <v>1111</v>
+      </c>
+      <c r="X12" s="173"/>
+      <c r="Y12" s="170">
         <f t="shared" si="2"/>
-        <v>-13646</v>
-      </c>
-      <c r="Y12" s="148">
+        <v>-12535</v>
+      </c>
+      <c r="Z12" s="148">
         <f t="shared" si="3"/>
-        <v>-0.13646</v>
-      </c>
-      <c r="AA12" s="133"/>
+        <v>-0.12534999999999999</v>
+      </c>
       <c r="AB12" s="133"/>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AC12" s="133"/>
+    </row>
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="141" t="s">
         <v>212</v>
       </c>
@@ -7425,19 +7457,22 @@
       <c r="V13" s="146">
         <v>24090</v>
       </c>
-      <c r="W13" s="173"/>
-      <c r="X13" s="170">
+      <c r="W13" s="146">
+        <v>-40457</v>
+      </c>
+      <c r="X13" s="173"/>
+      <c r="Y13" s="170">
         <f t="shared" si="2"/>
-        <v>146992</v>
-      </c>
-      <c r="Y13" s="148">
+        <v>106535</v>
+      </c>
+      <c r="Z13" s="148">
         <f t="shared" si="3"/>
-        <v>0.58796800000000005</v>
-      </c>
-      <c r="AA13" s="133"/>
+        <v>0.42614000000000002</v>
+      </c>
       <c r="AB13" s="133"/>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AC13" s="133"/>
+    </row>
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="141" t="s">
         <v>51</v>
       </c>
@@ -7502,29 +7537,32 @@
       <c r="V14" s="146">
         <v>31125</v>
       </c>
-      <c r="W14" s="173"/>
-      <c r="X14" s="170">
+      <c r="W14" s="146">
+        <v>-37218</v>
+      </c>
+      <c r="X14" s="173"/>
+      <c r="Y14" s="170">
         <f t="shared" si="2"/>
-        <v>176336</v>
-      </c>
-      <c r="Y14" s="148">
+        <v>139118</v>
+      </c>
+      <c r="Z14" s="148">
         <f t="shared" si="3"/>
-        <v>0.80152727272727264</v>
-      </c>
-      <c r="AA14" s="133"/>
-      <c r="AB14" s="192">
-        <f>AB7-AB9</f>
-        <v>3835.508378</v>
-      </c>
-      <c r="AE14" s="132">
-        <v>-4955</v>
-      </c>
-      <c r="AG14" s="132">
-        <f>AE14+AB14</f>
-        <v>-1119.491622</v>
-      </c>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+        <v>0.63235454545454539</v>
+      </c>
+      <c r="AB14" s="133"/>
+      <c r="AC14" s="192">
+        <f>AC7-AC9</f>
+        <v>4974.7047540000003</v>
+      </c>
+      <c r="AF14" s="132">
+        <v>-13200</v>
+      </c>
+      <c r="AH14" s="132">
+        <f>AF14+AC14</f>
+        <v>-8225.2952459999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="141" t="s">
         <v>43</v>
       </c>
@@ -7589,17 +7627,20 @@
       <c r="V15" s="146">
         <v>-27445</v>
       </c>
-      <c r="W15" s="173"/>
-      <c r="X15" s="170">
+      <c r="W15" s="146">
+        <v>17900</v>
+      </c>
+      <c r="X15" s="173"/>
+      <c r="Y15" s="170">
         <f t="shared" si="2"/>
-        <v>-48533</v>
-      </c>
-      <c r="Y15" s="148">
+        <v>-30633</v>
+      </c>
+      <c r="Z15" s="148">
         <f t="shared" si="3"/>
-        <v>-0.48532999999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+        <v>-0.30632999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A16" s="141" t="s">
         <v>24</v>
       </c>
@@ -7664,28 +7705,31 @@
       <c r="V16" s="146">
         <v>50000</v>
       </c>
-      <c r="W16" s="173"/>
-      <c r="X16" s="170">
+      <c r="W16" s="146">
+        <v>30270</v>
+      </c>
+      <c r="X16" s="173"/>
+      <c r="Y16" s="170">
         <f t="shared" si="2"/>
-        <v>398598</v>
-      </c>
-      <c r="Y16" s="148">
+        <v>428868</v>
+      </c>
+      <c r="Z16" s="148">
         <f t="shared" si="3"/>
-        <v>1.5943920000000003</v>
-      </c>
-      <c r="AG16" s="132">
+        <v>1.7154720000000001</v>
+      </c>
+      <c r="AH16" s="132">
         <v>4000000</v>
       </c>
-      <c r="AH16" s="132">
-        <f>AG16*7/100</f>
+      <c r="AI16" s="132">
+        <f>AH16*7/100</f>
         <v>280000</v>
       </c>
-      <c r="AJ16" s="132">
+      <c r="AK16" s="132">
         <f>15*12</f>
         <v>180</v>
       </c>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17" s="141" t="s">
         <v>23</v>
       </c>
@@ -7750,21 +7794,24 @@
       <c r="V17" s="146">
         <v>410000</v>
       </c>
-      <c r="W17" s="173"/>
-      <c r="X17" s="170">
+      <c r="W17" s="146">
+        <v>168000</v>
+      </c>
+      <c r="X17" s="173"/>
+      <c r="Y17" s="170">
         <f t="shared" si="2"/>
-        <v>569424</v>
-      </c>
-      <c r="Y17" s="148">
+        <v>737424</v>
+      </c>
+      <c r="Z17" s="148">
         <f t="shared" si="3"/>
-        <v>1.4235599999999999</v>
-      </c>
-      <c r="AH17" s="132">
-        <f>AH16/12</f>
+        <v>1.8435600000000001</v>
+      </c>
+      <c r="AI17" s="132">
+        <f>AI16/12</f>
         <v>23333.333333333332</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18" s="141" t="s">
         <v>165</v>
       </c>
@@ -7829,17 +7876,20 @@
       <c r="V18" s="146">
         <v>113500</v>
       </c>
-      <c r="W18" s="173"/>
-      <c r="X18" s="170">
+      <c r="W18" s="146">
+        <v>39300</v>
+      </c>
+      <c r="X18" s="173"/>
+      <c r="Y18" s="170">
         <f t="shared" si="2"/>
-        <v>680036</v>
-      </c>
-      <c r="Y18" s="148">
+        <v>719336</v>
+      </c>
+      <c r="Z18" s="148">
         <f t="shared" si="3"/>
-        <v>4.533573333333333</v>
-      </c>
-    </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+        <v>4.7955733333333326</v>
+      </c>
+    </row>
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19" s="141" t="s">
         <v>110</v>
       </c>
@@ -7904,20 +7954,23 @@
       <c r="V19" s="146">
         <v>0</v>
       </c>
-      <c r="W19" s="173"/>
-      <c r="X19" s="170">
+      <c r="W19" s="146">
+        <v>0</v>
+      </c>
+      <c r="X19" s="173"/>
+      <c r="Y19" s="170">
         <f t="shared" si="2"/>
         <v>-150688</v>
       </c>
-      <c r="Y19" s="148">
+      <c r="Z19" s="148">
         <f t="shared" si="3"/>
         <v>-1.3698909090909093</v>
       </c>
-      <c r="AC19" s="132">
+      <c r="AD19" s="132">
         <v>54000</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20" s="141" t="s">
         <v>319</v>
       </c>
@@ -7982,20 +8035,23 @@
       <c r="V20" s="146">
         <v>0</v>
       </c>
-      <c r="W20" s="173"/>
-      <c r="X20" s="170">
+      <c r="W20" s="146">
+        <v>0</v>
+      </c>
+      <c r="X20" s="173"/>
+      <c r="Y20" s="170">
         <f t="shared" si="2"/>
         <v>-110972</v>
       </c>
-      <c r="Y20" s="148">
+      <c r="Z20" s="148">
         <f t="shared" si="3"/>
         <v>-4.4388800000000002</v>
       </c>
-      <c r="AC20" s="132">
+      <c r="AD20" s="132">
         <v>11100</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" s="141" t="s">
         <v>316</v>
       </c>
@@ -8060,20 +8116,23 @@
       <c r="V21" s="146">
         <v>0</v>
       </c>
-      <c r="W21" s="173"/>
-      <c r="X21" s="170">
+      <c r="W21" s="146">
+        <v>0</v>
+      </c>
+      <c r="X21" s="173"/>
+      <c r="Y21" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Y21" s="148">
+      <c r="Z21" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AC21" s="132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AD21" s="132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22" s="141" t="s">
         <v>317</v>
       </c>
@@ -8138,21 +8197,24 @@
       <c r="V22" s="146">
         <v>0</v>
       </c>
-      <c r="W22" s="173"/>
-      <c r="X22" s="170">
+      <c r="W22" s="146">
+        <v>0</v>
+      </c>
+      <c r="X22" s="173"/>
+      <c r="Y22" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Y22" s="148">
+      <c r="Z22" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AC22" s="132">
-        <f>SUM(AC19:AC21)</f>
+      <c r="AD22" s="132">
+        <f>SUM(AD19:AD21)</f>
         <v>65100</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" s="141" t="s">
         <v>32</v>
       </c>
@@ -8217,17 +8279,20 @@
       <c r="V23" s="146">
         <v>-200</v>
       </c>
-      <c r="W23" s="173"/>
-      <c r="X23" s="170">
+      <c r="W23" s="146">
+        <v>54387</v>
+      </c>
+      <c r="X23" s="173"/>
+      <c r="Y23" s="170">
         <f t="shared" si="2"/>
-        <v>-75904</v>
-      </c>
-      <c r="Y23" s="148">
+        <v>-21517</v>
+      </c>
+      <c r="Z23" s="148">
         <f t="shared" si="3"/>
-        <v>-0.69003636363636345</v>
-      </c>
-    </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+        <v>-0.19560909090909087</v>
+      </c>
+    </row>
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24" s="141" t="s">
         <v>97</v>
       </c>
@@ -8292,17 +8357,20 @@
       <c r="V24" s="146">
         <v>-303200</v>
       </c>
-      <c r="W24" s="173"/>
-      <c r="X24" s="170">
+      <c r="W24" s="146">
+        <v>77900</v>
+      </c>
+      <c r="X24" s="173"/>
+      <c r="Y24" s="170">
         <f t="shared" si="2"/>
-        <v>-777579</v>
-      </c>
-      <c r="Y24" s="148">
+        <v>-699679</v>
+      </c>
+      <c r="Z24" s="148">
         <f t="shared" si="3"/>
-        <v>-3.3807782608695658</v>
-      </c>
-    </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+        <v>-3.0420826086956523</v>
+      </c>
+    </row>
+    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A25" s="141" t="s">
         <v>335</v>
       </c>
@@ -8353,17 +8421,20 @@
       <c r="V25" s="146">
         <v>-13000</v>
       </c>
-      <c r="W25" s="173"/>
-      <c r="X25" s="170">
+      <c r="W25" s="146">
+        <v>71400</v>
+      </c>
+      <c r="X25" s="173"/>
+      <c r="Y25" s="170">
         <f t="shared" si="2"/>
-        <v>29671</v>
-      </c>
-      <c r="Y25" s="148">
+        <v>101071</v>
+      </c>
+      <c r="Z25" s="148">
         <f t="shared" si="3"/>
-        <v>1.4835499999999999</v>
-      </c>
-    </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+        <v>5.0535500000000004</v>
+      </c>
+    </row>
+    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A26" s="141" t="s">
         <v>302</v>
       </c>
@@ -8426,17 +8497,20 @@
       <c r="V26" s="146">
         <v>-4293</v>
       </c>
-      <c r="W26" s="173"/>
-      <c r="X26" s="170">
+      <c r="W26" s="146">
+        <v>-18145</v>
+      </c>
+      <c r="X26" s="173"/>
+      <c r="Y26" s="170">
         <f t="shared" si="2"/>
-        <v>-27659</v>
-      </c>
-      <c r="Y26" s="148">
+        <v>-45804</v>
+      </c>
+      <c r="Z26" s="148">
         <f t="shared" si="3"/>
-        <v>-0.55318000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+        <v>-0.91608000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27" s="141" t="s">
         <v>29</v>
       </c>
@@ -8501,17 +8575,20 @@
       <c r="V27" s="146">
         <v>691000</v>
       </c>
-      <c r="W27" s="173"/>
-      <c r="X27" s="170">
+      <c r="W27" s="146">
+        <v>397000</v>
+      </c>
+      <c r="X27" s="173"/>
+      <c r="Y27" s="170">
         <f t="shared" si="2"/>
-        <v>1893800</v>
-      </c>
-      <c r="Y27" s="148">
+        <v>2290800</v>
+      </c>
+      <c r="Z27" s="148">
         <f t="shared" si="3"/>
-        <v>3.7875999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+        <v>4.5815999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A28" s="141" t="s">
         <v>28</v>
       </c>
@@ -8576,17 +8653,20 @@
       <c r="V28" s="146">
         <v>0</v>
       </c>
-      <c r="W28" s="173"/>
-      <c r="X28" s="170">
+      <c r="W28" s="146">
+        <v>-162700</v>
+      </c>
+      <c r="X28" s="173"/>
+      <c r="Y28" s="170">
         <f t="shared" si="2"/>
-        <v>388591</v>
-      </c>
-      <c r="Y28" s="148">
+        <v>225891</v>
+      </c>
+      <c r="Z28" s="148">
         <f t="shared" si="3"/>
-        <v>0.38859100000000002</v>
-      </c>
-    </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
+        <v>0.22589100000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A29" s="141" t="s">
         <v>332</v>
       </c>
@@ -8647,17 +8727,20 @@
       <c r="V29" s="146">
         <v>-13700</v>
       </c>
-      <c r="W29" s="173"/>
-      <c r="X29" s="170">
+      <c r="W29" s="146">
+        <v>-28900</v>
+      </c>
+      <c r="X29" s="173"/>
+      <c r="Y29" s="170">
         <f t="shared" si="2"/>
-        <v>24820</v>
-      </c>
-      <c r="Y29" s="148">
+        <v>-4080</v>
+      </c>
+      <c r="Z29" s="148">
         <f t="shared" si="3"/>
-        <v>0.49640000000000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
+        <v>-8.1600000000000006E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A30" s="141" t="s">
         <v>65</v>
       </c>
@@ -8722,17 +8805,20 @@
       <c r="V30" s="146">
         <v>0</v>
       </c>
-      <c r="W30" s="173"/>
-      <c r="X30" s="170">
+      <c r="W30" s="146">
+        <v>0</v>
+      </c>
+      <c r="X30" s="173"/>
+      <c r="Y30" s="170">
         <f t="shared" si="2"/>
         <v>841174</v>
       </c>
-      <c r="Y30" s="148">
+      <c r="Z30" s="148">
         <f t="shared" si="3"/>
         <v>1.682348</v>
       </c>
     </row>
-    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A31" s="140" t="s">
         <v>34</v>
       </c>
@@ -8797,17 +8883,20 @@
       <c r="V31" s="146">
         <v>0</v>
       </c>
-      <c r="W31" s="173"/>
-      <c r="X31" s="170">
+      <c r="W31" s="146">
+        <v>0</v>
+      </c>
+      <c r="X31" s="173"/>
+      <c r="Y31" s="170">
         <f t="shared" si="2"/>
         <v>140133</v>
       </c>
-      <c r="Y31" s="148">
+      <c r="Z31" s="148">
         <f t="shared" si="3"/>
         <v>0.28026600000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A32" s="140" t="s">
         <v>131</v>
       </c>
@@ -8872,17 +8961,20 @@
       <c r="V32" s="146">
         <v>-43208</v>
       </c>
-      <c r="W32" s="173"/>
-      <c r="X32" s="170">
+      <c r="W32" s="146">
+        <v>4974</v>
+      </c>
+      <c r="X32" s="173"/>
+      <c r="Y32" s="170">
         <f t="shared" si="2"/>
-        <v>65192</v>
-      </c>
-      <c r="Y32" s="148">
+        <v>70166</v>
+      </c>
+      <c r="Z32" s="148">
         <f t="shared" si="3"/>
-        <v>1.3038400000000001</v>
-      </c>
-    </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.25">
+        <v>1.4033199999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="43" t="s">
         <v>67</v>
       </c>
@@ -8947,18 +9039,21 @@
       <c r="V33" s="146">
         <v>33000</v>
       </c>
-      <c r="W33" s="173"/>
-      <c r="X33" s="170">
+      <c r="W33" s="146">
+        <v>38495</v>
+      </c>
+      <c r="X33" s="173"/>
+      <c r="Y33" s="170">
         <f t="shared" si="2"/>
-        <v>301842</v>
-      </c>
-      <c r="Y33" s="148">
+        <v>340337</v>
+      </c>
+      <c r="Z33" s="148">
         <f t="shared" si="3"/>
-        <v>7.5460500000000001</v>
-      </c>
-      <c r="AB33" s="133"/>
-    </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
+        <v>8.5084250000000008</v>
+      </c>
+      <c r="AC33" s="133"/>
+    </row>
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A34" s="141" t="s">
         <v>31</v>
       </c>
@@ -9023,21 +9118,24 @@
       <c r="V34" s="146">
         <v>44000</v>
       </c>
-      <c r="W34" s="173"/>
-      <c r="X34" s="170">
+      <c r="W34" s="146">
+        <v>16600</v>
+      </c>
+      <c r="X34" s="173"/>
+      <c r="Y34" s="170">
         <f t="shared" si="2"/>
-        <v>354905</v>
-      </c>
-      <c r="Y34" s="148">
+        <v>371505</v>
+      </c>
+      <c r="Z34" s="148">
         <f t="shared" si="3"/>
-        <v>0.88726249999999995</v>
-      </c>
-      <c r="AA34" s="5"/>
-      <c r="AB34" s="133">
-        <v>3981</v>
-      </c>
-    </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.25">
+        <v>0.92876250000000005</v>
+      </c>
+      <c r="AB34" s="5"/>
+      <c r="AC34" s="133">
+        <v>46634</v>
+      </c>
+    </row>
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A35" s="141" t="s">
         <v>104</v>
       </c>
@@ -9102,19 +9200,22 @@
       <c r="V35" s="146">
         <v>-111976</v>
       </c>
-      <c r="W35" s="173"/>
-      <c r="X35" s="170">
+      <c r="W35" s="146">
+        <v>41600</v>
+      </c>
+      <c r="X35" s="173"/>
+      <c r="Y35" s="170">
         <f t="shared" si="2"/>
-        <v>-138965</v>
-      </c>
-      <c r="Y35" s="148">
+        <v>-97365</v>
+      </c>
+      <c r="Z35" s="148">
         <f t="shared" si="3"/>
-        <v>-1.3896500000000001</v>
-      </c>
-      <c r="AA35" s="5"/>
-      <c r="AB35" s="133"/>
-    </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.25">
+        <v>-0.97365000000000002</v>
+      </c>
+      <c r="AB35" s="5"/>
+      <c r="AC35" s="133"/>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A36" s="141" t="s">
         <v>314</v>
       </c>
@@ -9177,24 +9278,27 @@
       <c r="V36" s="146">
         <v>0</v>
       </c>
-      <c r="W36" s="173"/>
-      <c r="X36" s="170">
+      <c r="W36" s="146">
+        <v>0</v>
+      </c>
+      <c r="X36" s="173"/>
+      <c r="Y36" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Y36" s="148">
+      <c r="Z36" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AA36" s="133">
-        <v>1047315</v>
-      </c>
       <c r="AB36" s="133">
-        <f>(AA37+AA36)/10000000*13780</f>
-        <v>2891.8873359999998</v>
-      </c>
-    </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.25">
+        <v>233083</v>
+      </c>
+      <c r="AC36" s="133">
+        <f>(AB37+AB36)/10000000*13780</f>
+        <v>706.63839999999993</v>
+      </c>
+    </row>
+    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A37" s="141" t="s">
         <v>229</v>
       </c>
@@ -9259,21 +9363,24 @@
       <c r="V37" s="146">
         <v>3835</v>
       </c>
-      <c r="W37" s="173"/>
-      <c r="X37" s="170">
+      <c r="W37" s="146">
+        <v>-6562</v>
+      </c>
+      <c r="X37" s="173"/>
+      <c r="Y37" s="170">
         <f t="shared" si="2"/>
-        <v>-17765</v>
-      </c>
-      <c r="Y37" s="148">
+        <v>-24327</v>
+      </c>
+      <c r="Z37" s="148">
         <f t="shared" si="3"/>
-        <v>-0.3553</v>
-      </c>
-      <c r="AA37" s="133">
-        <v>1051297</v>
-      </c>
-      <c r="AB37" s="133"/>
-    </row>
-    <row r="38" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>-0.48653999999999997</v>
+      </c>
+      <c r="AB37" s="133">
+        <v>279717</v>
+      </c>
+      <c r="AC37" s="133"/>
+    </row>
+    <row r="38" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="141" t="s">
         <v>45</v>
       </c>
@@ -9338,22 +9445,25 @@
       <c r="V38" s="146">
         <v>-42428</v>
       </c>
-      <c r="W38" s="173"/>
-      <c r="X38" s="170">
+      <c r="W38" s="146">
+        <v>-219600</v>
+      </c>
+      <c r="X38" s="173"/>
+      <c r="Y38" s="170">
         <f t="shared" si="2"/>
-        <v>948171</v>
-      </c>
-      <c r="Y38" s="148">
+        <v>728571</v>
+      </c>
+      <c r="Z38" s="148">
         <f t="shared" si="3"/>
-        <v>3.1605699999999999</v>
-      </c>
-      <c r="AA38" s="133"/>
-      <c r="AB38" s="133">
-        <f>+AB34-AB36</f>
-        <v>1089.1126640000002</v>
-      </c>
-    </row>
-    <row r="39" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2.4285700000000001</v>
+      </c>
+      <c r="AB38" s="133"/>
+      <c r="AC38" s="133">
+        <f>+AC34-AC36</f>
+        <v>45927.361599999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="141" t="s">
         <v>292</v>
       </c>
@@ -9416,19 +9526,22 @@
       <c r="V39" s="146">
         <v>1089</v>
       </c>
-      <c r="W39" s="173"/>
-      <c r="X39" s="170">
+      <c r="W39" s="146">
+        <v>15022</v>
+      </c>
+      <c r="X39" s="173"/>
+      <c r="Y39" s="170">
         <f t="shared" si="2"/>
-        <v>-88014</v>
-      </c>
-      <c r="Y39" s="148">
+        <v>-72992</v>
+      </c>
+      <c r="Z39" s="148">
         <f t="shared" si="3"/>
-        <v>-8.8013999999999992</v>
-      </c>
-      <c r="AA39" s="133"/>
+        <v>-7.2991999999999999</v>
+      </c>
       <c r="AB39" s="133"/>
-    </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC39" s="133"/>
+    </row>
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="141" t="s">
         <v>132</v>
       </c>
@@ -9493,19 +9606,22 @@
       <c r="V40" s="146">
         <v>16400</v>
       </c>
-      <c r="W40" s="173"/>
-      <c r="X40" s="170">
+      <c r="W40" s="146">
+        <v>12700</v>
+      </c>
+      <c r="X40" s="173"/>
+      <c r="Y40" s="170">
         <f t="shared" si="2"/>
-        <v>68041</v>
-      </c>
-      <c r="Y40" s="148">
+        <v>80741</v>
+      </c>
+      <c r="Z40" s="148">
         <f t="shared" si="3"/>
-        <v>1.3608199999999999</v>
-      </c>
-      <c r="AA40" s="133"/>
+        <v>1.6148199999999999</v>
+      </c>
       <c r="AB40" s="133"/>
-    </row>
-    <row r="41" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AC40" s="133"/>
+    </row>
+    <row r="41" spans="1:29" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="141" t="s">
         <v>48</v>
       </c>
@@ -9570,19 +9686,22 @@
       <c r="V41" s="146">
         <v>-6386</v>
       </c>
-      <c r="W41" s="173"/>
-      <c r="X41" s="170">
+      <c r="W41" s="146">
+        <v>119000</v>
+      </c>
+      <c r="X41" s="173"/>
+      <c r="Y41" s="170">
         <f t="shared" si="2"/>
-        <v>-1082743</v>
-      </c>
-      <c r="Y41" s="148">
+        <v>-963743</v>
+      </c>
+      <c r="Z41" s="148">
         <f t="shared" si="3"/>
-        <v>-10.82743</v>
-      </c>
-      <c r="AA41" s="133"/>
+        <v>-9.6374300000000002</v>
+      </c>
       <c r="AB41" s="133"/>
-    </row>
-    <row r="42" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AC41" s="133"/>
+    </row>
+    <row r="42" spans="1:29" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="141" t="s">
         <v>336</v>
       </c>
@@ -9633,19 +9752,22 @@
       <c r="V42" s="146">
         <v>-23900</v>
       </c>
-      <c r="W42" s="173"/>
-      <c r="X42" s="170">
+      <c r="W42" s="146">
+        <v>136200</v>
+      </c>
+      <c r="X42" s="173"/>
+      <c r="Y42" s="170">
         <f t="shared" si="2"/>
-        <v>359790</v>
-      </c>
-      <c r="Y42" s="148">
+        <v>495990</v>
+      </c>
+      <c r="Z42" s="148">
         <f t="shared" si="3"/>
-        <v>7.1958000000000002</v>
-      </c>
-      <c r="AA42" s="133"/>
+        <v>9.9198000000000004</v>
+      </c>
       <c r="AB42" s="133"/>
-    </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC42" s="133"/>
+    </row>
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A43" s="141" t="s">
         <v>301</v>
       </c>
@@ -9708,18 +9830,21 @@
       <c r="V43" s="146">
         <v>-5756</v>
       </c>
-      <c r="W43" s="173"/>
-      <c r="X43" s="170">
+      <c r="W43" s="146">
+        <v>18400</v>
+      </c>
+      <c r="X43" s="173"/>
+      <c r="Y43" s="170">
         <f t="shared" si="2"/>
-        <v>-51613</v>
-      </c>
-      <c r="Y43" s="148">
+        <v>-33213</v>
+      </c>
+      <c r="Z43" s="148">
         <f t="shared" si="3"/>
-        <v>-1.03226</v>
-      </c>
-      <c r="AA43" s="133"/>
-    </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.25">
+        <v>-0.66425999999999996</v>
+      </c>
+      <c r="AB43" s="133"/>
+    </row>
+    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A44" s="142" t="s">
         <v>168</v>
       </c>
@@ -9784,17 +9909,20 @@
       <c r="V44" s="146">
         <v>0</v>
       </c>
-      <c r="W44" s="173"/>
-      <c r="X44" s="170">
+      <c r="W44" s="146">
+        <v>0</v>
+      </c>
+      <c r="X44" s="173"/>
+      <c r="Y44" s="170">
         <f t="shared" si="2"/>
         <v>80210</v>
       </c>
-      <c r="Y44" s="148">
+      <c r="Z44" s="148">
         <f t="shared" si="3"/>
         <v>0.20052500000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A45" s="142" t="s">
         <v>202</v>
       </c>
@@ -9859,17 +9987,20 @@
       <c r="V45" s="146">
         <v>-3152</v>
       </c>
-      <c r="W45" s="173"/>
-      <c r="X45" s="170">
+      <c r="W45" s="146">
+        <v>-39900</v>
+      </c>
+      <c r="X45" s="173"/>
+      <c r="Y45" s="170">
         <f t="shared" si="2"/>
-        <v>48261</v>
-      </c>
-      <c r="Y45" s="148">
+        <v>8361</v>
+      </c>
+      <c r="Z45" s="148">
         <f t="shared" si="3"/>
-        <v>0.1206525</v>
-      </c>
-    </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.25">
+        <v>2.0902500000000001E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A46" s="142" t="s">
         <v>33</v>
       </c>
@@ -9934,17 +10065,20 @@
       <c r="V46" s="146">
         <v>0</v>
       </c>
-      <c r="W46" s="173"/>
-      <c r="X46" s="170">
+      <c r="W46" s="146">
+        <v>0</v>
+      </c>
+      <c r="X46" s="173"/>
+      <c r="Y46" s="170">
         <f t="shared" si="2"/>
         <v>1105039</v>
       </c>
-      <c r="Y46" s="148">
+      <c r="Z46" s="148">
         <f t="shared" si="3"/>
         <v>3.6834633333333326</v>
       </c>
     </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A47" s="59" t="s">
         <v>306</v>
       </c>
@@ -10007,17 +10141,20 @@
       <c r="V47" s="150">
         <v>-57500</v>
       </c>
-      <c r="W47" s="173"/>
-      <c r="X47" s="170">
+      <c r="W47" s="150">
+        <v>-181800</v>
+      </c>
+      <c r="X47" s="173"/>
+      <c r="Y47" s="170">
         <f t="shared" si="2"/>
-        <v>-2950940</v>
-      </c>
-      <c r="Y47" s="148">
+        <v>-3132740</v>
+      </c>
+      <c r="Z47" s="148">
         <f t="shared" si="3"/>
-        <v>-2.9509400000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
+        <v>-3.1327400000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A48" s="59" t="s">
         <v>197</v>
       </c>
@@ -10082,17 +10219,20 @@
       <c r="V48" s="150">
         <v>0</v>
       </c>
-      <c r="W48" s="173"/>
-      <c r="X48" s="170">
+      <c r="W48" s="150">
+        <v>45927</v>
+      </c>
+      <c r="X48" s="173"/>
+      <c r="Y48" s="170">
         <f t="shared" si="2"/>
-        <v>15532</v>
-      </c>
-      <c r="Y48" s="148">
+        <v>61459</v>
+      </c>
+      <c r="Z48" s="148">
         <f t="shared" si="3"/>
-        <v>0.31064000000000003</v>
-      </c>
-    </row>
-    <row r="49" spans="1:29" x14ac:dyDescent="0.25">
+        <v>1.2291799999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="59" t="s">
         <v>213</v>
       </c>
@@ -10157,17 +10297,20 @@
       <c r="V49" s="150">
         <v>0</v>
       </c>
-      <c r="W49" s="173"/>
-      <c r="X49" s="170">
+      <c r="W49" s="150">
+        <v>0</v>
+      </c>
+      <c r="X49" s="173"/>
+      <c r="Y49" s="170">
         <f t="shared" si="2"/>
         <v>369643</v>
       </c>
-      <c r="Y49" s="148">
+      <c r="Z49" s="148">
         <f t="shared" si="3"/>
         <v>0.56868153846153835</v>
       </c>
     </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59" t="s">
         <v>214</v>
       </c>
@@ -10232,17 +10375,20 @@
       <c r="V50" s="150">
         <v>0</v>
       </c>
-      <c r="W50" s="173"/>
-      <c r="X50" s="170">
+      <c r="W50" s="150">
+        <v>0</v>
+      </c>
+      <c r="X50" s="173"/>
+      <c r="Y50" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Y50" s="148">
+      <c r="Z50" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="59" t="s">
         <v>49</v>
       </c>
@@ -10307,17 +10453,20 @@
       <c r="V51" s="150">
         <v>0</v>
       </c>
-      <c r="W51" s="173"/>
-      <c r="X51" s="170">
+      <c r="W51" s="150">
+        <v>0</v>
+      </c>
+      <c r="X51" s="173"/>
+      <c r="Y51" s="170">
         <f t="shared" si="2"/>
         <v>311687</v>
       </c>
-      <c r="Y51" s="148">
+      <c r="Z51" s="148">
         <f t="shared" si="3"/>
         <v>1.0389566666666668</v>
       </c>
     </row>
-    <row r="52" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="59" t="s">
         <v>331</v>
       </c>
@@ -10382,17 +10531,20 @@
       <c r="V52" s="150">
         <v>0</v>
       </c>
-      <c r="W52" s="173"/>
-      <c r="X52" s="170">
+      <c r="W52" s="150">
+        <v>13000</v>
+      </c>
+      <c r="X52" s="173"/>
+      <c r="Y52" s="170">
         <f t="shared" si="2"/>
-        <v>17634</v>
-      </c>
-      <c r="Y52" s="148">
+        <v>30634</v>
+      </c>
+      <c r="Z52" s="148">
         <f t="shared" si="3"/>
-        <v>0.17634</v>
-      </c>
-    </row>
-    <row r="53" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.30634</v>
+      </c>
+    </row>
+    <row r="53" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="59" t="s">
         <v>288</v>
       </c>
@@ -10457,17 +10609,20 @@
       <c r="V53" s="150">
         <v>-11500</v>
       </c>
-      <c r="W53" s="173"/>
-      <c r="X53" s="170">
+      <c r="W53" s="150">
+        <v>94734</v>
+      </c>
+      <c r="X53" s="173"/>
+      <c r="Y53" s="170">
         <f t="shared" si="2"/>
-        <v>786589</v>
-      </c>
-      <c r="Y53" s="148">
+        <v>881323</v>
+      </c>
+      <c r="Z53" s="148">
         <f t="shared" si="3"/>
-        <v>0.78658899999999987</v>
-      </c>
-    </row>
-    <row r="54" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.88132299999999997</v>
+      </c>
+    </row>
+    <row r="54" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="24"/>
       <c r="B54" s="25"/>
       <c r="C54" s="26"/>
@@ -10476,7 +10631,7 @@
       <c r="F54" s="115"/>
       <c r="G54" s="16"/>
       <c r="H54" s="253">
-        <f t="shared" ref="H54:V54" si="4">SUM(H4:H53)</f>
+        <f t="shared" ref="H54:W54" si="4">SUM(H4:H53)</f>
         <v>38252</v>
       </c>
       <c r="I54" s="253">
@@ -10536,19 +10691,23 @@
         <v>760771</v>
       </c>
       <c r="W54" s="253">
-        <f>SUM(W4:W53)</f>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>584177</v>
       </c>
       <c r="X54" s="253">
-        <f>SUM(H54:W54)</f>
-        <v>6197262</v>
-      </c>
-      <c r="Y54" s="254">
-        <f t="shared" ref="Y54" si="5">IFERROR(X54/F54*100,0)/10000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <f>SUM(X4:X53)</f>
+        <v>0</v>
+      </c>
+      <c r="Y54" s="253">
+        <f>SUM(H54:X54)</f>
+        <v>6781439</v>
+      </c>
+      <c r="Z54" s="254">
+        <f t="shared" ref="Z54" si="5">IFERROR(Y54/F54*100,0)/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="249"/>
       <c r="B55" s="249"/>
       <c r="C55" s="249"/>
@@ -10573,9 +10732,10 @@
       <c r="V55" s="249"/>
       <c r="W55" s="249"/>
       <c r="X55" s="249"/>
-      <c r="Y55" s="251"/>
-    </row>
-    <row r="56" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="Y55" s="249"/>
+      <c r="Z55" s="251"/>
+    </row>
+    <row r="56" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="201" t="s">
         <v>241</v>
       </c>
@@ -10640,17 +10800,20 @@
       <c r="V56" s="161">
         <v>550</v>
       </c>
-      <c r="W56" s="245"/>
-      <c r="X56" s="246">
-        <f>SUM(H56:W56)</f>
+      <c r="W56" s="161">
+        <v>0</v>
+      </c>
+      <c r="X56" s="245"/>
+      <c r="Y56" s="246">
+        <f>SUM(H56:X56)</f>
         <v>28620</v>
       </c>
-      <c r="Y56" s="247">
-        <f>IFERROR(X56/F56*100,0)/10000000</f>
+      <c r="Z56" s="247">
+        <f>IFERROR(Y56/F56*100,0)/10000000</f>
         <v>9.5399999999999999E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="201" t="s">
         <v>273</v>
       </c>
@@ -10713,17 +10876,20 @@
       <c r="V57" s="161">
         <v>0</v>
       </c>
-      <c r="W57" s="173"/>
-      <c r="X57" s="170">
-        <f>SUM(H57:W57)</f>
-        <v>-237594</v>
-      </c>
-      <c r="Y57" s="148">
-        <f>IFERROR(X57/F57*100,0)/10000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="W57" s="161">
+        <v>24300</v>
+      </c>
+      <c r="X57" s="173"/>
+      <c r="Y57" s="170">
+        <f>SUM(H57:X57)</f>
+        <v>-213294</v>
+      </c>
+      <c r="Z57" s="148">
+        <f>IFERROR(Y57/F57*100,0)/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="201"/>
       <c r="B58" s="202" t="s">
         <v>338</v>
@@ -10762,11 +10928,14 @@
       <c r="V58" s="161">
         <v>0</v>
       </c>
-      <c r="W58" s="161"/>
-      <c r="X58" s="257"/>
-      <c r="Y58" s="258"/>
-    </row>
-    <row r="59" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="W58" s="161">
+        <v>0</v>
+      </c>
+      <c r="X58" s="161"/>
+      <c r="Y58" s="257"/>
+      <c r="Z58" s="258"/>
+    </row>
+    <row r="59" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="201" t="s">
         <v>340</v>
       </c>
@@ -10807,11 +10976,14 @@
       <c r="V59" s="161">
         <v>3939</v>
       </c>
-      <c r="W59" s="161"/>
-      <c r="X59" s="257"/>
-      <c r="Y59" s="258"/>
-    </row>
-    <row r="60" spans="1:29" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="W59" s="161">
+        <v>1600</v>
+      </c>
+      <c r="X59" s="161"/>
+      <c r="Y59" s="257"/>
+      <c r="Z59" s="258"/>
+    </row>
+    <row r="60" spans="1:30" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="199"/>
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
@@ -10880,73 +11052,77 @@
         <v>4489</v>
       </c>
       <c r="W60" s="169">
-        <f>SUM(W56:W57)</f>
-        <v>0</v>
-      </c>
-      <c r="X60" s="256">
-        <f>SUM(H60:W60)</f>
-        <v>-314816</v>
-      </c>
-      <c r="Y60" s="172"/>
-    </row>
-    <row r="61" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="AB61" s="133"/>
-    </row>
-    <row r="62" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="AA62" s="133"/>
-    </row>
-    <row r="63" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="AA63" s="5"/>
-      <c r="AB63" s="133"/>
-      <c r="AC63" s="236"/>
-    </row>
-    <row r="64" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="AA64" s="133"/>
+        <f>SUM(W56:W59)</f>
+        <v>25900</v>
+      </c>
+      <c r="X60" s="169">
+        <f>SUM(X56:X57)</f>
+        <v>0</v>
+      </c>
+      <c r="Y60" s="256">
+        <f>SUM(H60:X60)</f>
+        <v>-288916</v>
+      </c>
+      <c r="Z60" s="172"/>
+    </row>
+    <row r="61" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AC61" s="133"/>
+    </row>
+    <row r="62" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AB62" s="133"/>
+    </row>
+    <row r="63" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AB63" s="5"/>
+      <c r="AC63" s="133"/>
+      <c r="AD63" s="236"/>
+    </row>
+    <row r="64" spans="1:30" x14ac:dyDescent="0.25">
       <c r="AB64" s="133"/>
-      <c r="AC64" s="236"/>
-    </row>
-    <row r="65" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA65" s="133"/>
+      <c r="AC64" s="133"/>
+      <c r="AD64" s="236"/>
+    </row>
+    <row r="65" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB65" s="133"/>
-      <c r="AC65" s="236"/>
-    </row>
-    <row r="66" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA66" s="133"/>
+      <c r="AC65" s="133"/>
+      <c r="AD65" s="236"/>
+    </row>
+    <row r="66" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB66" s="133"/>
-      <c r="AC66" s="236"/>
-    </row>
-    <row r="67" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA67" s="133"/>
+      <c r="AC66" s="133"/>
+      <c r="AD66" s="236"/>
+    </row>
+    <row r="67" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB67" s="133"/>
-      <c r="AC67" s="236"/>
-    </row>
-    <row r="68" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA68" s="133"/>
-      <c r="AB68" s="236"/>
+      <c r="AC67" s="133"/>
+      <c r="AD67" s="236"/>
+    </row>
+    <row r="68" spans="28:30" x14ac:dyDescent="0.25">
+      <c r="AB68" s="133"/>
       <c r="AC68" s="236"/>
-    </row>
-    <row r="69" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA69" s="236"/>
+      <c r="AD68" s="236"/>
+    </row>
+    <row r="69" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB69" s="236"/>
       <c r="AC69" s="236"/>
+      <c r="AD69" s="236"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2 A3:G3 Y54:Y55 Y60 H2:Y3 G38:W38 A4:W37 A56:Y59 A39:W54 A60:W60">
+  <conditionalFormatting sqref="G2 A3:G3 Z54:Z55 Z60 H2:Z3 G38:X38 A4:X37 A56:Z59 A39:X54 A60:X60">
     <cfRule type="expression" dxfId="537" priority="18">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X4:Y53">
+  <conditionalFormatting sqref="Y4:Z53">
     <cfRule type="expression" dxfId="536" priority="15">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X54">
+  <conditionalFormatting sqref="Y54">
     <cfRule type="expression" dxfId="535" priority="12">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X60">
+  <conditionalFormatting sqref="Y60">
     <cfRule type="expression" dxfId="534" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -11313,7 +11489,7 @@
       <c r="R6" s="158"/>
       <c r="S6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>129765</v>
+        <v>123203</v>
       </c>
       <c r="T6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11325,7 +11501,7 @@
       <c r="X6" s="131"/>
       <c r="Y6" s="153">
         <f t="shared" si="4"/>
-        <v>-422709</v>
+        <v>-429271</v>
       </c>
       <c r="Z6" s="167">
         <f t="shared" si="5"/>
@@ -11618,7 +11794,7 @@
       <c r="R10" s="158"/>
       <c r="S10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>438873</v>
+        <v>380973</v>
       </c>
       <c r="T10" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11629,7 +11805,7 @@
       <c r="W10" s="149"/>
       <c r="Y10" s="153">
         <f t="shared" ref="Y10:Y11" si="8">M10+P10+S10+V10</f>
-        <v>438873</v>
+        <v>380973</v>
       </c>
       <c r="Z10" s="167">
         <f t="shared" ref="Z10:Z11" si="9">(N10+Q10+T10+W10)</f>
@@ -11681,7 +11857,7 @@
       <c r="R11" s="158"/>
       <c r="S11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>421142</v>
+        <v>252087</v>
       </c>
       <c r="T11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11692,7 +11868,7 @@
       <c r="W11" s="149"/>
       <c r="Y11" s="153">
         <f t="shared" si="8"/>
-        <v>421142</v>
+        <v>252087</v>
       </c>
       <c r="Z11" s="167">
         <f t="shared" si="9"/>
@@ -11762,7 +11938,7 @@
       <c r="R12" s="158"/>
       <c r="S12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-100760</v>
+        <v>-8360</v>
       </c>
       <c r="T12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11773,7 +11949,7 @@
       <c r="W12" s="72"/>
       <c r="Y12" s="153">
         <f t="shared" si="4"/>
-        <v>-1276827</v>
+        <v>-1184427</v>
       </c>
       <c r="Z12" s="167">
         <f t="shared" si="5"/>
@@ -11843,7 +12019,7 @@
       <c r="R13" s="158"/>
       <c r="S13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>272350</v>
+        <v>255986</v>
       </c>
       <c r="T13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11854,7 +12030,7 @@
       <c r="W13" s="149"/>
       <c r="Y13" s="153">
         <f t="shared" si="4"/>
-        <v>-129525</v>
+        <v>-145889</v>
       </c>
       <c r="Z13" s="167">
         <f t="shared" si="5"/>
@@ -11924,7 +12100,7 @@
       <c r="R14" s="158"/>
       <c r="S14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>162827</v>
+        <v>213427</v>
       </c>
       <c r="T14" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11935,7 +12111,7 @@
       <c r="W14" s="149"/>
       <c r="Y14" s="153">
         <f t="shared" si="4"/>
-        <v>72898</v>
+        <v>123498</v>
       </c>
       <c r="Z14" s="167">
         <f t="shared" si="5"/>
@@ -12414,7 +12590,7 @@
       <c r="R20" s="158"/>
       <c r="S20" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>373354</v>
+        <v>385774</v>
       </c>
       <c r="T20" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12425,7 +12601,7 @@
       <c r="W20" s="72"/>
       <c r="Y20" s="153">
         <f t="shared" si="4"/>
-        <v>573406</v>
+        <v>585826</v>
       </c>
       <c r="Z20" s="167">
         <f t="shared" si="5"/>
@@ -12495,7 +12671,7 @@
       <c r="R21" s="158"/>
       <c r="S21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-13646</v>
+        <v>-12535</v>
       </c>
       <c r="T21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12506,7 +12682,7 @@
       <c r="W21" s="149"/>
       <c r="Y21" s="153">
         <f t="shared" si="4"/>
-        <v>-11071</v>
+        <v>-9960</v>
       </c>
       <c r="Z21" s="167">
         <f t="shared" si="5"/>
@@ -12666,7 +12842,7 @@
       <c r="R23" s="158"/>
       <c r="S23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>146992</v>
+        <v>106535</v>
       </c>
       <c r="T23" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12677,7 +12853,7 @@
       <c r="W23" s="72"/>
       <c r="Y23" s="153">
         <f t="shared" si="4"/>
-        <v>-104190</v>
+        <v>-144647</v>
       </c>
       <c r="Z23" s="167">
         <f t="shared" si="5"/>
@@ -12747,7 +12923,7 @@
       <c r="R24" s="158"/>
       <c r="S24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>176336</v>
+        <v>139118</v>
       </c>
       <c r="T24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12758,7 +12934,7 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="153">
         <f t="shared" si="4"/>
-        <v>-27287</v>
+        <v>-64505</v>
       </c>
       <c r="Z24" s="167">
         <f t="shared" si="5"/>
@@ -12909,7 +13085,7 @@
       <c r="R26" s="158"/>
       <c r="S26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-48533</v>
+        <v>-30633</v>
       </c>
       <c r="T26" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12920,7 +13096,7 @@
       <c r="W26" s="72"/>
       <c r="Y26" s="153">
         <f t="shared" si="4"/>
-        <v>1697648</v>
+        <v>1715548</v>
       </c>
       <c r="Z26" s="167">
         <f t="shared" si="5"/>
@@ -13231,7 +13407,7 @@
       <c r="R30" s="158"/>
       <c r="S30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>398598</v>
+        <v>428868</v>
       </c>
       <c r="T30" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13242,7 +13418,7 @@
       <c r="W30" s="72"/>
       <c r="Y30" s="153">
         <f t="shared" si="4"/>
-        <v>776866</v>
+        <v>807136</v>
       </c>
       <c r="Z30" s="167">
         <f t="shared" si="5"/>
@@ -13312,7 +13488,7 @@
       <c r="R31" s="158"/>
       <c r="S31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>569424</v>
+        <v>737424</v>
       </c>
       <c r="T31" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13324,7 +13500,7 @@
       <c r="X31" s="1"/>
       <c r="Y31" s="153">
         <f t="shared" si="4"/>
-        <v>1448877</v>
+        <v>1616877</v>
       </c>
       <c r="Z31" s="167">
         <f t="shared" si="5"/>
@@ -13565,7 +13741,7 @@
       <c r="R34" s="158"/>
       <c r="S34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>680036</v>
+        <v>719336</v>
       </c>
       <c r="T34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13577,7 +13753,7 @@
       <c r="X34"/>
       <c r="Y34" s="153">
         <f t="shared" si="4"/>
-        <v>194031</v>
+        <v>233331</v>
       </c>
       <c r="Z34" s="167">
         <f t="shared" si="5"/>
@@ -13728,7 +13904,7 @@
       <c r="R36" s="158"/>
       <c r="S36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-75904</v>
+        <v>-21517</v>
       </c>
       <c r="T36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13739,7 +13915,7 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="153">
         <f t="shared" si="4"/>
-        <v>-223531</v>
+        <v>-169144</v>
       </c>
       <c r="Z36" s="167">
         <f t="shared" si="5"/>
@@ -13897,7 +14073,7 @@
       <c r="R38" s="158"/>
       <c r="S38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-777579</v>
+        <v>-699679</v>
       </c>
       <c r="T38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13908,7 +14084,7 @@
       <c r="W38" s="72"/>
       <c r="Y38" s="153">
         <f t="shared" si="4"/>
-        <v>2125047</v>
+        <v>2202947</v>
       </c>
       <c r="Z38" s="167">
         <f t="shared" si="5"/>
@@ -13976,7 +14152,7 @@
       <c r="R39" s="158"/>
       <c r="S39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>29671</v>
+        <v>101071</v>
       </c>
       <c r="T39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13987,7 +14163,7 @@
       <c r="W39" s="149"/>
       <c r="Y39" s="153">
         <f t="shared" si="4"/>
-        <v>29671</v>
+        <v>101071</v>
       </c>
       <c r="Z39" s="167">
         <f t="shared" si="5"/>
@@ -14055,7 +14231,7 @@
       <c r="R40" s="158"/>
       <c r="S40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-27659</v>
+        <v>-45804</v>
       </c>
       <c r="T40" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14066,7 +14242,7 @@
       <c r="W40" s="149"/>
       <c r="Y40" s="153">
         <f t="shared" si="4"/>
-        <v>-71325</v>
+        <v>-89470</v>
       </c>
       <c r="Z40" s="167">
         <f t="shared" si="5"/>
@@ -14136,7 +14312,7 @@
       <c r="R41" s="158"/>
       <c r="S41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>1893800</v>
+        <v>2290800</v>
       </c>
       <c r="T41" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14147,7 +14323,7 @@
       <c r="W41" s="72"/>
       <c r="Y41" s="153">
         <f t="shared" si="4"/>
-        <v>4434854</v>
+        <v>4831854</v>
       </c>
       <c r="Z41" s="167">
         <f t="shared" si="5"/>
@@ -14217,7 +14393,7 @@
       <c r="R42" s="158"/>
       <c r="S42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>388591</v>
+        <v>225891</v>
       </c>
       <c r="T42" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14229,7 +14405,7 @@
       <c r="X42" s="131"/>
       <c r="Y42" s="153">
         <f t="shared" si="4"/>
-        <v>5669338</v>
+        <v>5506638</v>
       </c>
       <c r="Z42" s="167">
         <f t="shared" si="5"/>
@@ -14731,7 +14907,7 @@
       <c r="R48" s="158"/>
       <c r="S48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>24820</v>
+        <v>-4080</v>
       </c>
       <c r="T48" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14742,7 +14918,7 @@
       <c r="W48" s="149"/>
       <c r="Y48" s="153">
         <f t="shared" si="4"/>
-        <v>24820</v>
+        <v>-4080</v>
       </c>
       <c r="Z48" s="167">
         <f t="shared" si="5"/>
@@ -14976,7 +15152,7 @@
       <c r="R51" s="158"/>
       <c r="S51" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>65192</v>
+        <v>70166</v>
       </c>
       <c r="T51" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14987,7 +15163,7 @@
       <c r="W51" s="72"/>
       <c r="Y51" s="153">
         <f t="shared" si="4"/>
-        <v>-13858</v>
+        <v>-8884</v>
       </c>
       <c r="Z51" s="167">
         <f t="shared" si="5"/>
@@ -15145,7 +15321,7 @@
       <c r="R53" s="158"/>
       <c r="S53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>301842</v>
+        <v>340337</v>
       </c>
       <c r="T53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15156,7 +15332,7 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="153">
         <f t="shared" si="4"/>
-        <v>370107</v>
+        <v>408602</v>
       </c>
       <c r="Z53" s="167">
         <f t="shared" si="5"/>
@@ -15400,7 +15576,7 @@
       <c r="R56" s="158"/>
       <c r="S56" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>354905</v>
+        <v>371505</v>
       </c>
       <c r="T56" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15411,7 +15587,7 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="153">
         <f t="shared" si="4"/>
-        <v>549966</v>
+        <v>566566</v>
       </c>
       <c r="Z56" s="167">
         <f t="shared" si="5"/>
@@ -15481,7 +15657,7 @@
       <c r="R57" s="158"/>
       <c r="S57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-138965</v>
+        <v>-97365</v>
       </c>
       <c r="T57" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15492,7 +15668,7 @@
       <c r="W57" s="72"/>
       <c r="Y57" s="153">
         <f t="shared" si="4"/>
-        <v>521284</v>
+        <v>562884</v>
       </c>
       <c r="Z57" s="167">
         <f t="shared" si="5"/>
@@ -15643,7 +15819,7 @@
       <c r="R59" s="158"/>
       <c r="S59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-17765</v>
+        <v>-24327</v>
       </c>
       <c r="T59" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15655,7 +15831,7 @@
       <c r="X59" s="131"/>
       <c r="Y59" s="153">
         <f t="shared" si="4"/>
-        <v>-291790</v>
+        <v>-298352</v>
       </c>
       <c r="Z59" s="167">
         <f t="shared" si="5"/>
@@ -15726,7 +15902,7 @@
       <c r="R60" s="158"/>
       <c r="S60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>948171</v>
+        <v>728571</v>
       </c>
       <c r="T60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15737,7 +15913,7 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="153">
         <f t="shared" si="4"/>
-        <v>-3706164</v>
+        <v>-3925764</v>
       </c>
       <c r="Z60" s="167">
         <f t="shared" si="5"/>
@@ -15978,7 +16154,7 @@
       <c r="R63" s="158"/>
       <c r="S63" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-88014</v>
+        <v>-72992</v>
       </c>
       <c r="T63" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15989,7 +16165,7 @@
       <c r="W63" s="149"/>
       <c r="Y63" s="153">
         <f t="shared" si="4"/>
-        <v>-108135</v>
+        <v>-93113</v>
       </c>
       <c r="Z63" s="167">
         <f t="shared" si="5"/>
@@ -16059,7 +16235,7 @@
       <c r="R64" s="158"/>
       <c r="S64" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>68041</v>
+        <v>80741</v>
       </c>
       <c r="T64" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16071,7 +16247,7 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="153">
         <f t="shared" si="4"/>
-        <v>100732</v>
+        <v>113432</v>
       </c>
       <c r="Z64" s="167">
         <f t="shared" si="5"/>
@@ -16148,7 +16324,7 @@
       <c r="R65" s="158"/>
       <c r="S65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1082743</v>
+        <v>-963743</v>
       </c>
       <c r="T65" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16159,7 +16335,7 @@
       <c r="W65" s="72"/>
       <c r="Y65" s="153">
         <f t="shared" si="4"/>
-        <v>2596872</v>
+        <v>2715872</v>
       </c>
       <c r="Z65" s="167">
         <f t="shared" si="5"/>
@@ -16236,7 +16412,7 @@
       <c r="R66" s="158"/>
       <c r="S66" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>359790</v>
+        <v>495990</v>
       </c>
       <c r="T66" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16247,7 +16423,7 @@
       <c r="W66" s="149"/>
       <c r="Y66" s="153">
         <f t="shared" si="4"/>
-        <v>359790</v>
+        <v>495990</v>
       </c>
       <c r="Z66" s="167">
         <f t="shared" si="5"/>
@@ -16315,7 +16491,7 @@
       <c r="R67" s="158"/>
       <c r="S67" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-51613</v>
+        <v>-33213</v>
       </c>
       <c r="T67" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16326,7 +16502,7 @@
       <c r="W67" s="149"/>
       <c r="Y67" s="153">
         <f t="shared" si="4"/>
-        <v>-38322</v>
+        <v>-19922</v>
       </c>
       <c r="Z67" s="167">
         <f t="shared" si="5"/>
@@ -16647,7 +16823,7 @@
       <c r="R71" s="158"/>
       <c r="S71" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>48261</v>
+        <v>8361</v>
       </c>
       <c r="T71" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16659,7 +16835,7 @@
       <c r="X71" s="131"/>
       <c r="Y71" s="153">
         <f t="shared" ref="Y71:Y81" si="12">M71+P71+S71+V71</f>
-        <v>831042</v>
+        <v>791142</v>
       </c>
       <c r="Z71" s="167">
         <f t="shared" ref="Z71:Z81" si="13">(N71+Q71+T71+W71)</f>
@@ -16809,7 +16985,7 @@
       <c r="R73" s="158"/>
       <c r="S73" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-2950940</v>
+        <v>-3132740</v>
       </c>
       <c r="T73" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16820,7 +16996,7 @@
       <c r="W73" s="149"/>
       <c r="Y73" s="153">
         <f t="shared" si="12"/>
-        <v>-3913769</v>
+        <v>-4095569</v>
       </c>
       <c r="Z73" s="167">
         <f t="shared" si="13"/>
@@ -16965,7 +17141,7 @@
       <c r="R75" s="158"/>
       <c r="S75" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>15532</v>
+        <v>61459</v>
       </c>
       <c r="T75" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16976,7 +17152,7 @@
       <c r="W75" s="149"/>
       <c r="Y75" s="153">
         <f t="shared" si="12"/>
-        <v>-54353</v>
+        <v>-8426</v>
       </c>
       <c r="Z75" s="167">
         <f t="shared" si="13"/>
@@ -17368,7 +17544,7 @@
       <c r="R80" s="158"/>
       <c r="S80" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>17634</v>
+        <v>30634</v>
       </c>
       <c r="T80" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17379,7 +17555,7 @@
       <c r="W80" s="149"/>
       <c r="Y80" s="153">
         <f t="shared" si="12"/>
-        <v>17634</v>
+        <v>30634</v>
       </c>
       <c r="Z80" s="167">
         <f t="shared" si="13"/>
@@ -17447,7 +17623,7 @@
       <c r="R81" s="158"/>
       <c r="S81" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>786589</v>
+        <v>881323</v>
       </c>
       <c r="T81" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17458,7 +17634,7 @@
       <c r="W81" s="149"/>
       <c r="Y81" s="153">
         <f t="shared" si="12"/>
-        <v>1277442</v>
+        <v>1372176</v>
       </c>
       <c r="Z81" s="167">
         <f t="shared" si="13"/>
@@ -17501,7 +17677,7 @@
       <c r="R82" s="122"/>
       <c r="S82" s="153">
         <f>SUM(S4:S81)</f>
-        <v>6308234</v>
+        <v>6892411</v>
       </c>
       <c r="T82" s="122"/>
       <c r="U82" s="122"/>
@@ -17509,7 +17685,7 @@
       <c r="W82" s="50"/>
       <c r="Y82" s="153">
         <f>SUM(Y4:Y81)</f>
-        <v>29577764</v>
+        <v>30161941</v>
       </c>
       <c r="Z82" s="160"/>
     </row>
@@ -19246,12 +19422,12 @@
         <v>0.5</v>
       </c>
       <c r="G4" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>129765</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>123203</v>
       </c>
       <c r="H4" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>2.5952999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>2.4640599999999999</v>
       </c>
       <c r="I4" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19271,11 +19447,11 @@
       </c>
       <c r="M4" s="71">
         <f t="shared" ref="M4:N52" si="0">G4+I4+K4</f>
-        <v>129765</v>
+        <v>123203</v>
       </c>
       <c r="N4" s="165">
         <f t="shared" si="0"/>
-        <v>2.5952999999999999</v>
+        <v>2.4640599999999999</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -19298,12 +19474,12 @@
         <v>3.5</v>
       </c>
       <c r="G5" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>438873</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>380973</v>
       </c>
       <c r="H5" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.4629099999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.2699100000000001</v>
       </c>
       <c r="I5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19323,11 +19499,11 @@
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>438873</v>
+        <v>380973</v>
       </c>
       <c r="N5" s="165">
         <f t="shared" si="0"/>
-        <v>1.4629099999999999</v>
+        <v>1.2699100000000001</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -19350,12 +19526,12 @@
         <v>1</v>
       </c>
       <c r="G6" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>421142</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>252087</v>
       </c>
       <c r="H6" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>4.2114200000000004</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>2.5208699999999999</v>
       </c>
       <c r="I6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19375,11 +19551,11 @@
       </c>
       <c r="M6" s="71">
         <f t="shared" si="0"/>
-        <v>421142</v>
+        <v>252087</v>
       </c>
       <c r="N6" s="165">
         <f t="shared" si="0"/>
-        <v>4.2114200000000004</v>
+        <v>2.5208699999999999</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -19402,12 +19578,12 @@
         <v>3</v>
       </c>
       <c r="G7" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-100760</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-8360</v>
       </c>
       <c r="H7" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.33586666666666665</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-2.7866666666666661E-2</v>
       </c>
       <c r="I7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19427,11 +19603,11 @@
       </c>
       <c r="M7" s="71">
         <f t="shared" si="0"/>
-        <v>-100760</v>
+        <v>-8360</v>
       </c>
       <c r="N7" s="165">
         <f t="shared" si="0"/>
-        <v>-0.33586666666666665</v>
+        <v>-2.7866666666666661E-2</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -19454,12 +19630,12 @@
         <v>1.5</v>
       </c>
       <c r="G8" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>272350</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>255986</v>
       </c>
       <c r="H8" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.8156666666666663</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.7065733333333335</v>
       </c>
       <c r="I8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19479,11 +19655,11 @@
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>272350</v>
+        <v>255986</v>
       </c>
       <c r="N8" s="165">
         <f t="shared" si="0"/>
-        <v>1.8156666666666663</v>
+        <v>1.7065733333333335</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -19506,12 +19682,12 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>162827</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>213427</v>
       </c>
       <c r="H9" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>2.7137833333333337</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>3.5571166666666674</v>
       </c>
       <c r="I9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19531,11 +19707,11 @@
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>162827</v>
+        <v>213427</v>
       </c>
       <c r="N9" s="165">
         <f t="shared" si="0"/>
-        <v>2.7137833333333337</v>
+        <v>3.5571166666666674</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -19558,11 +19734,11 @@
         <v>15</v>
       </c>
       <c r="G10" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-87379</v>
       </c>
       <c r="H10" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-5.8252666666666661E-2</v>
       </c>
       <c r="I10" s="152">
@@ -19610,12 +19786,12 @@
         <v>6</v>
       </c>
       <c r="G11" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>373354</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>385774</v>
       </c>
       <c r="H11" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.62225666666666657</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.64295666666666662</v>
       </c>
       <c r="I11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19635,11 +19811,11 @@
       </c>
       <c r="M11" s="71">
         <f t="shared" si="0"/>
-        <v>373354</v>
+        <v>385774</v>
       </c>
       <c r="N11" s="165">
         <f t="shared" si="0"/>
-        <v>0.62225666666666657</v>
+        <v>0.64295666666666662</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -19662,12 +19838,12 @@
         <v>1</v>
       </c>
       <c r="G12" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-13646</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-12535</v>
       </c>
       <c r="H12" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.13646</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.12534999999999999</v>
       </c>
       <c r="I12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19687,11 +19863,11 @@
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>-13646</v>
+        <v>-12535</v>
       </c>
       <c r="N12" s="165">
         <f t="shared" si="0"/>
-        <v>-0.13646</v>
+        <v>-0.12534999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -19714,12 +19890,12 @@
         <v>1</v>
       </c>
       <c r="G13" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>146992</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>106535</v>
       </c>
       <c r="H13" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.58796800000000005</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.42614000000000002</v>
       </c>
       <c r="I13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19739,11 +19915,11 @@
       </c>
       <c r="M13" s="71">
         <f t="shared" si="0"/>
-        <v>146992</v>
+        <v>106535</v>
       </c>
       <c r="N13" s="165">
         <f t="shared" si="0"/>
-        <v>0.58796800000000005</v>
+        <v>0.42614000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -19766,12 +19942,12 @@
         <v>1</v>
       </c>
       <c r="G14" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-48533</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-30633</v>
       </c>
       <c r="H14" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.48532999999999998</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.30632999999999999</v>
       </c>
       <c r="I14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19791,11 +19967,11 @@
       </c>
       <c r="M14" s="71">
         <f t="shared" si="0"/>
-        <v>-48533</v>
+        <v>-30633</v>
       </c>
       <c r="N14" s="165">
         <f t="shared" si="0"/>
-        <v>-0.48532999999999998</v>
+        <v>-0.30632999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -19818,12 +19994,12 @@
         <v>0.2</v>
       </c>
       <c r="G15" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>176336</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>139118</v>
       </c>
       <c r="H15" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.80152727272727264</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.63235454545454539</v>
       </c>
       <c r="I15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19843,11 +20019,11 @@
       </c>
       <c r="M15" s="71">
         <f t="shared" si="0"/>
-        <v>176336</v>
+        <v>139118</v>
       </c>
       <c r="N15" s="165">
         <f t="shared" si="0"/>
-        <v>0.80152727272727264</v>
+        <v>0.63235454545454539</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -19870,12 +20046,12 @@
         <v>2.5</v>
       </c>
       <c r="G16" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>398598</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>428868</v>
       </c>
       <c r="H16" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.5943920000000003</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.7154720000000001</v>
       </c>
       <c r="I16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19895,11 +20071,11 @@
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>398598</v>
+        <v>428868</v>
       </c>
       <c r="N16" s="165">
         <f t="shared" si="0"/>
-        <v>1.5943920000000003</v>
+        <v>1.7154720000000001</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -19922,12 +20098,12 @@
         <v>4</v>
       </c>
       <c r="G17" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>569424</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>737424</v>
       </c>
       <c r="H17" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.4235599999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.8435600000000001</v>
       </c>
       <c r="I17" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19947,11 +20123,11 @@
       </c>
       <c r="M17" s="71">
         <f t="shared" si="0"/>
-        <v>569424</v>
+        <v>737424</v>
       </c>
       <c r="N17" s="165">
         <f t="shared" si="0"/>
-        <v>1.4235599999999999</v>
+        <v>1.8435600000000001</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -19974,11 +20150,11 @@
         <v>0.25</v>
       </c>
       <c r="G18" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-150688</v>
       </c>
       <c r="H18" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-1.3698909090909093</v>
       </c>
       <c r="I18" s="152">
@@ -20026,11 +20202,11 @@
         <v>0.25</v>
       </c>
       <c r="G19" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-110972</v>
       </c>
       <c r="H19" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>-4.4388800000000002</v>
       </c>
       <c r="I19" s="152">
@@ -20078,11 +20254,11 @@
         <v>2</v>
       </c>
       <c r="G20" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="152">
@@ -20130,12 +20306,12 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>680036</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>719336</v>
       </c>
       <c r="H21" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>4.533573333333333</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>4.7955733333333326</v>
       </c>
       <c r="I21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20155,11 +20331,11 @@
       </c>
       <c r="M21" s="71">
         <f t="shared" si="0"/>
-        <v>680036</v>
+        <v>719336</v>
       </c>
       <c r="N21" s="165">
         <f t="shared" si="0"/>
-        <v>4.533573333333333</v>
+        <v>4.7955733333333326</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -20182,12 +20358,12 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="G22" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-75904</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-21517</v>
       </c>
       <c r="H22" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.69003636363636345</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.19560909090909087</v>
       </c>
       <c r="I22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20207,11 +20383,11 @@
       </c>
       <c r="M22" s="71">
         <f t="shared" si="0"/>
-        <v>-75904</v>
+        <v>-21517</v>
       </c>
       <c r="N22" s="165">
         <f t="shared" si="0"/>
-        <v>-0.69003636363636345</v>
+        <v>-0.19560909090909087</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -20234,12 +20410,12 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G23" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-777579</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-699679</v>
       </c>
       <c r="H23" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-3.3807782608695658</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-3.0420826086956523</v>
       </c>
       <c r="I23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20259,11 +20435,11 @@
       </c>
       <c r="M23" s="71">
         <f t="shared" si="0"/>
-        <v>-777579</v>
+        <v>-699679</v>
       </c>
       <c r="N23" s="165">
         <f t="shared" si="0"/>
-        <v>-3.3807782608695658</v>
+        <v>-3.0420826086956523</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -20284,12 +20460,12 @@
         <v>0.2</v>
       </c>
       <c r="G24" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>29671</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>101071</v>
       </c>
       <c r="H24" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.4835499999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>5.0535500000000004</v>
       </c>
       <c r="I24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20309,11 +20485,11 @@
       </c>
       <c r="M24" s="71">
         <f t="shared" ref="M24" si="1">G24+I24+K24</f>
-        <v>29671</v>
+        <v>101071</v>
       </c>
       <c r="N24" s="165">
         <f t="shared" ref="N24" si="2">H24+J24+L24</f>
-        <v>1.4835499999999999</v>
+        <v>5.0535500000000004</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -20334,12 +20510,12 @@
         <v>0.2</v>
       </c>
       <c r="G25" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-27659</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-45804</v>
       </c>
       <c r="H25" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.55318000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.91608000000000001</v>
       </c>
       <c r="I25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20359,11 +20535,11 @@
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>-27659</v>
+        <v>-45804</v>
       </c>
       <c r="N25" s="165">
         <f t="shared" si="0"/>
-        <v>-0.55318000000000001</v>
+        <v>-0.91608000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -20386,12 +20562,12 @@
         <v>5</v>
       </c>
       <c r="G26" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1893800</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>2290800</v>
       </c>
       <c r="H26" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>3.7875999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>4.5815999999999999</v>
       </c>
       <c r="I26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20411,11 +20587,11 @@
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>1893800</v>
+        <v>2290800</v>
       </c>
       <c r="N26" s="165">
         <f t="shared" si="0"/>
-        <v>3.7875999999999999</v>
+        <v>4.5815999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -20438,12 +20614,12 @@
         <v>10</v>
       </c>
       <c r="G27" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>388591</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>225891</v>
       </c>
       <c r="H27" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.38859100000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.22589100000000001</v>
       </c>
       <c r="I27" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20463,11 +20639,11 @@
       </c>
       <c r="M27" s="71">
         <f t="shared" si="0"/>
-        <v>388591</v>
+        <v>225891</v>
       </c>
       <c r="N27" s="165">
         <f t="shared" si="0"/>
-        <v>0.38859100000000002</v>
+        <v>0.22589100000000001</v>
       </c>
       <c r="O27" s="130"/>
     </row>
@@ -20489,12 +20665,12 @@
         <v>1</v>
       </c>
       <c r="G28" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>24820</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-4080</v>
       </c>
       <c r="H28" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.49640000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-8.1600000000000006E-2</v>
       </c>
       <c r="I28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20514,11 +20690,11 @@
       </c>
       <c r="M28" s="71">
         <f t="shared" ref="M28" si="3">G28+I28+K28</f>
-        <v>24820</v>
+        <v>-4080</v>
       </c>
       <c r="N28" s="165">
         <f t="shared" ref="N28" si="4">H28+J28+L28</f>
-        <v>0.49640000000000001</v>
+        <v>-8.1600000000000006E-2</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -20541,11 +20717,11 @@
         <v>5</v>
       </c>
       <c r="G29" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>841174</v>
       </c>
       <c r="H29" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>1.682348</v>
       </c>
       <c r="I29" s="152">
@@ -20593,11 +20769,11 @@
         <v>5</v>
       </c>
       <c r="G30" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>140133</v>
       </c>
       <c r="H30" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0.28026600000000002</v>
       </c>
       <c r="I30" s="152">
@@ -20645,12 +20821,12 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>65192</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>70166</v>
       </c>
       <c r="H31" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.3038400000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.4033199999999999</v>
       </c>
       <c r="I31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20670,11 +20846,11 @@
       </c>
       <c r="M31" s="71">
         <f t="shared" si="0"/>
-        <v>65192</v>
+        <v>70166</v>
       </c>
       <c r="N31" s="165">
         <f t="shared" si="0"/>
-        <v>1.3038400000000001</v>
+        <v>1.4033199999999999</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -20697,12 +20873,12 @@
         <v>0.4</v>
       </c>
       <c r="G32" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>301842</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>340337</v>
       </c>
       <c r="H32" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>7.5460500000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>8.5084250000000008</v>
       </c>
       <c r="I32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20722,11 +20898,11 @@
       </c>
       <c r="M32" s="71">
         <f t="shared" si="0"/>
-        <v>301842</v>
+        <v>340337</v>
       </c>
       <c r="N32" s="165">
         <f t="shared" si="0"/>
-        <v>7.5460500000000001</v>
+        <v>8.5084250000000008</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -20749,12 +20925,12 @@
         <v>4</v>
       </c>
       <c r="G33" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>354905</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>371505</v>
       </c>
       <c r="H33" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.88726249999999995</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.92876250000000005</v>
       </c>
       <c r="I33" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20774,11 +20950,11 @@
       </c>
       <c r="M33" s="71">
         <f t="shared" si="0"/>
-        <v>354905</v>
+        <v>371505</v>
       </c>
       <c r="N33" s="165">
         <f t="shared" si="0"/>
-        <v>0.88726249999999995</v>
+        <v>0.92876250000000005</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -20801,12 +20977,12 @@
         <v>1</v>
       </c>
       <c r="G34" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-138965</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-97365</v>
       </c>
       <c r="H34" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-1.3896500000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.97365000000000002</v>
       </c>
       <c r="I34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20826,11 +21002,11 @@
       </c>
       <c r="M34" s="71">
         <f t="shared" si="0"/>
-        <v>-138965</v>
+        <v>-97365</v>
       </c>
       <c r="N34" s="165">
         <f t="shared" si="0"/>
-        <v>-1.3896500000000001</v>
+        <v>-0.97365000000000002</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -20851,11 +21027,11 @@
       </c>
       <c r="F35" s="155"/>
       <c r="G35" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H35" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I35" s="152">
@@ -20903,12 +21079,12 @@
         <v>0.5</v>
       </c>
       <c r="G36" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-17765</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-24327</v>
       </c>
       <c r="H36" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-0.3553</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.48653999999999997</v>
       </c>
       <c r="I36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20928,11 +21104,11 @@
       </c>
       <c r="M36" s="71">
         <f t="shared" si="0"/>
-        <v>-17765</v>
+        <v>-24327</v>
       </c>
       <c r="N36" s="165">
         <f t="shared" si="0"/>
-        <v>-0.3553</v>
+        <v>-0.48653999999999997</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -20955,12 +21131,12 @@
         <v>1</v>
       </c>
       <c r="G37" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>948171</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>728571</v>
       </c>
       <c r="H37" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>3.1605699999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>2.4285700000000001</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20980,11 +21156,11 @@
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>948171</v>
+        <v>728571</v>
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>3.1605699999999999</v>
+        <v>2.4285700000000001</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -21005,12 +21181,12 @@
         <v>0.1</v>
       </c>
       <c r="G38" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-88014</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-72992</v>
       </c>
       <c r="H38" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-8.8013999999999992</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-7.2991999999999999</v>
       </c>
       <c r="I38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21030,11 +21206,11 @@
       </c>
       <c r="M38" s="71">
         <f t="shared" si="0"/>
-        <v>-88014</v>
+        <v>-72992</v>
       </c>
       <c r="N38" s="165">
         <f t="shared" si="0"/>
-        <v>-8.8013999999999992</v>
+        <v>-7.2991999999999999</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -21057,12 +21233,12 @@
         <v>1</v>
       </c>
       <c r="G39" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>68041</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>80741</v>
       </c>
       <c r="H39" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>1.3608199999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.6148199999999999</v>
       </c>
       <c r="I39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21082,11 +21258,11 @@
       </c>
       <c r="M39" s="71">
         <f t="shared" si="0"/>
-        <v>68041</v>
+        <v>80741</v>
       </c>
       <c r="N39" s="165">
         <f t="shared" si="0"/>
-        <v>1.3608199999999999</v>
+        <v>1.6148199999999999</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -21109,12 +21285,12 @@
         <v>1</v>
       </c>
       <c r="G40" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-1082743</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-963743</v>
       </c>
       <c r="H40" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-10.82743</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-9.6374300000000002</v>
       </c>
       <c r="I40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21134,11 +21310,11 @@
       </c>
       <c r="M40" s="71">
         <f t="shared" si="0"/>
-        <v>-1082743</v>
+        <v>-963743</v>
       </c>
       <c r="N40" s="165">
         <f t="shared" si="0"/>
-        <v>-10.82743</v>
+        <v>-9.6374300000000002</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -21161,12 +21337,12 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>359790</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>495990</v>
       </c>
       <c r="H41" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>7.1958000000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>9.9198000000000004</v>
       </c>
       <c r="I41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21186,11 +21362,11 @@
       </c>
       <c r="M41" s="71">
         <f t="shared" ref="M41" si="5">G41+I41+K41</f>
-        <v>359790</v>
+        <v>495990</v>
       </c>
       <c r="N41" s="165">
         <f t="shared" ref="N41" si="6">H41+J41+L41</f>
-        <v>7.1958000000000002</v>
+        <v>9.9198000000000004</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -21211,12 +21387,12 @@
         <v>0.1</v>
       </c>
       <c r="G42" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-51613</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-33213</v>
       </c>
       <c r="H42" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-1.03226</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-0.66425999999999996</v>
       </c>
       <c r="I42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21236,11 +21412,11 @@
       </c>
       <c r="M42" s="71">
         <f t="shared" si="0"/>
-        <v>-51613</v>
+        <v>-33213</v>
       </c>
       <c r="N42" s="165">
         <f t="shared" si="0"/>
-        <v>-1.03226</v>
+        <v>-0.66425999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -21263,11 +21439,11 @@
         <v>1</v>
       </c>
       <c r="G43" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>1105039</v>
       </c>
       <c r="H43" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>3.6834633333333326</v>
       </c>
       <c r="I43" s="152">
@@ -21309,11 +21485,11 @@
         <v>1</v>
       </c>
       <c r="G44" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H44" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I44" s="152">
@@ -21361,11 +21537,11 @@
         <v>4</v>
       </c>
       <c r="G45" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>80210</v>
       </c>
       <c r="H45" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0.20052500000000001</v>
       </c>
       <c r="I45" s="152">
@@ -21413,12 +21589,12 @@
         <v>4</v>
       </c>
       <c r="G46" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>48261</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>8361</v>
       </c>
       <c r="H46" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.1206525</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>2.0902500000000001E-2</v>
       </c>
       <c r="I46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21438,11 +21614,11 @@
       </c>
       <c r="M46" s="71">
         <f t="shared" si="0"/>
-        <v>48261</v>
+        <v>8361</v>
       </c>
       <c r="N46" s="165">
         <f t="shared" si="0"/>
-        <v>0.1206525</v>
+        <v>2.0902500000000001E-2</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -21463,12 +21639,12 @@
         <v>0.1</v>
       </c>
       <c r="G47" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-2950940</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-3132740</v>
       </c>
       <c r="H47" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-2.9509400000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-3.1327400000000001</v>
       </c>
       <c r="I47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21488,11 +21664,11 @@
       </c>
       <c r="M47" s="71">
         <f t="shared" si="0"/>
-        <v>-2950940</v>
+        <v>-3132740</v>
       </c>
       <c r="N47" s="165">
         <f t="shared" si="0"/>
-        <v>-2.9509400000000001</v>
+        <v>-3.1327400000000001</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -21509,11 +21685,11 @@
       </c>
       <c r="F48" s="114"/>
       <c r="G48" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I48" s="152">
@@ -21561,12 +21737,12 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>15532</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>61459</v>
       </c>
       <c r="H49" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.31064000000000003</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>1.2291799999999999</v>
       </c>
       <c r="I49" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21586,11 +21762,11 @@
       </c>
       <c r="M49" s="71">
         <f t="shared" si="0"/>
-        <v>15532</v>
+        <v>61459</v>
       </c>
       <c r="N49" s="165">
         <f t="shared" si="0"/>
-        <v>0.31064000000000003</v>
+        <v>1.2291799999999999</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -21613,11 +21789,11 @@
         <v>5</v>
       </c>
       <c r="G50" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>369643</v>
       </c>
       <c r="H50" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0.56868153846153835</v>
       </c>
       <c r="I50" s="152">
@@ -21665,11 +21841,11 @@
         <v>1</v>
       </c>
       <c r="G51" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I51" s="152">
@@ -21717,11 +21893,11 @@
         <v>2.5</v>
       </c>
       <c r="G52" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>311687</v>
       </c>
       <c r="H52" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>1.0389566666666668</v>
       </c>
       <c r="I52" s="152">
@@ -21769,12 +21945,12 @@
         <v>0.25</v>
       </c>
       <c r="G53" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>17634</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>30634</v>
       </c>
       <c r="H53" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.17634</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.30634</v>
       </c>
       <c r="I53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21794,11 +21970,11 @@
       </c>
       <c r="M53" s="71">
         <f t="shared" ref="M53:N54" si="7">G53+I53+K53</f>
-        <v>17634</v>
+        <v>30634</v>
       </c>
       <c r="N53" s="165">
         <f t="shared" si="7"/>
-        <v>0.17634</v>
+        <v>0.30634</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -21821,12 +21997,12 @@
         <v>5</v>
       </c>
       <c r="G54" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>786589</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>881323</v>
       </c>
       <c r="H54" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>0.78658899999999987</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>0.88132299999999997</v>
       </c>
       <c r="I54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21846,11 +22022,11 @@
       </c>
       <c r="M54" s="71">
         <f t="shared" si="7"/>
-        <v>786589</v>
+        <v>881323</v>
       </c>
       <c r="N54" s="165">
         <f t="shared" si="7"/>
-        <v>0.78658899999999987</v>
+        <v>0.88132299999999997</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -21862,7 +22038,7 @@
       <c r="F55" s="233"/>
       <c r="G55" s="230">
         <f>SUM(G4:G54)</f>
-        <v>6197262</v>
+        <v>6781439</v>
       </c>
       <c r="H55" s="90"/>
       <c r="I55" s="230">
@@ -21877,7 +22053,7 @@
       <c r="L55" s="109"/>
       <c r="M55" s="230">
         <f>SUM(M4:M54)</f>
-        <v>6197262</v>
+        <v>6781439</v>
       </c>
       <c r="N55" s="234"/>
     </row>
@@ -21941,11 +22117,11 @@
       <c r="E59" s="208"/>
       <c r="F59" s="206"/>
       <c r="G59" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>28620</v>
       </c>
       <c r="H59" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>9.5399999999999999E-2</v>
       </c>
       <c r="I59" s="152">
@@ -21991,11 +22167,11 @@
       </c>
       <c r="F60" s="237"/>
       <c r="G60" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
-        <v>-237594</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <v>-213294</v>
       </c>
       <c r="H60" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADG$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DH$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I60" s="152">
@@ -22016,7 +22192,7 @@
       </c>
       <c r="M60" s="152">
         <f t="shared" si="8"/>
-        <v>-237594</v>
+        <v>-213294</v>
       </c>
       <c r="N60" s="166">
         <f t="shared" si="8"/>
@@ -22026,7 +22202,7 @@
     <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G61" s="93">
         <f>SUM(G59:G60)</f>
-        <v>-208974</v>
+        <v>-184674</v>
       </c>
       <c r="H61" s="94"/>
       <c r="I61" s="93">
@@ -22041,7 +22217,7 @@
       <c r="L61" s="113"/>
       <c r="M61" s="93">
         <f>SUM(M59:M60)</f>
-        <v>-208974</v>
+        <v>-184674</v>
       </c>
       <c r="N61" s="235"/>
     </row>

</xml_diff>

<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Tue 10/27/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3256" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3257" uniqueCount="346">
   <si>
     <t>Sudeep</t>
   </si>
@@ -1793,7 +1793,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="259">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2397,7 +2397,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2407,7 +2406,14 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="538">
+  <dxfs count="539">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -6505,7 +6511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AK69"/>
+  <dimension ref="A1:AL69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="132" customWidth="1" outlineLevel="1"/>
@@ -6517,19 +6523,20 @@
     <col min="7" max="7" width="1.7109375" style="132" customWidth="1"/>
     <col min="8" max="17" width="13.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="18" max="18" width="13.42578125" style="132" customWidth="1" collapsed="1"/>
-    <col min="19" max="23" width="13.42578125" style="132" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" style="132" customWidth="1"/>
-    <col min="25" max="25" width="10.42578125" style="132" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="10.7109375" style="132" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="32" width="9.140625" style="132"/>
-    <col min="33" max="33" width="14.140625" style="132" customWidth="1"/>
-    <col min="34" max="34" width="12" style="132" customWidth="1"/>
-    <col min="35" max="35" width="15.85546875" style="132" customWidth="1"/>
-    <col min="36" max="16384" width="9.140625" style="132"/>
+    <col min="19" max="24" width="13.42578125" style="132" customWidth="1"/>
+    <col min="25" max="25" width="11.28515625" style="132" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="10.7109375" style="132" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="9.140625" style="132" collapsed="1"/>
+    <col min="29" max="33" width="9.140625" style="132"/>
+    <col min="34" max="34" width="14.140625" style="132" customWidth="1"/>
+    <col min="35" max="35" width="12" style="132" customWidth="1"/>
+    <col min="36" max="36" width="15.85546875" style="132" customWidth="1"/>
+    <col min="37" max="16384" width="9.140625" style="132"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:38" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G2" s="220"/>
       <c r="H2" s="255">
         <v>46296</v>
@@ -6579,15 +6586,18 @@
       <c r="W2" s="255">
         <v>46321</v>
       </c>
-      <c r="X2" s="182"/>
-      <c r="Y2" s="183" t="s">
+      <c r="X2" s="255">
+        <v>46322</v>
+      </c>
+      <c r="Y2" s="182"/>
+      <c r="Z2" s="183" t="s">
         <v>325</v>
       </c>
-      <c r="Z2" s="184" t="s">
+      <c r="AA2" s="184" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A3" s="185" t="s">
         <v>54</v>
       </c>
@@ -6655,17 +6665,20 @@
       <c r="W3" s="178" t="s">
         <v>234</v>
       </c>
-      <c r="X3" s="179"/>
-      <c r="Y3" s="188"/>
-      <c r="Z3" s="179"/>
-      <c r="AG3" s="132" t="s">
+      <c r="X3" s="178" t="s">
+        <v>233</v>
+      </c>
+      <c r="Y3" s="179"/>
+      <c r="Z3" s="188"/>
+      <c r="AA3" s="179"/>
+      <c r="AH3" s="132" t="s">
         <v>198</v>
       </c>
-      <c r="AH3" s="132">
+      <c r="AI3" s="132">
         <v>13780</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A4" s="141" t="s">
         <v>216</v>
       </c>
@@ -6733,23 +6746,26 @@
       <c r="W4" s="157">
         <v>-6562</v>
       </c>
-      <c r="X4" s="210"/>
-      <c r="Y4" s="170">
-        <f t="shared" ref="Y4" si="0">SUM(H4:X4)</f>
-        <v>123203</v>
-      </c>
-      <c r="Z4" s="148">
-        <f t="shared" ref="Z4" si="1">IFERROR(Y4/F4*100,0)/10000000</f>
-        <v>2.4640599999999999</v>
-      </c>
-      <c r="AG4" s="132" t="s">
+      <c r="X4" s="157">
+        <v>-11883</v>
+      </c>
+      <c r="Y4" s="210"/>
+      <c r="Z4" s="170">
+        <f t="shared" ref="Z4" si="0">SUM(H4:Y4)</f>
+        <v>111320</v>
+      </c>
+      <c r="AA4" s="148">
+        <f t="shared" ref="AA4" si="1">IFERROR(Z4/F4*100,0)/10000000</f>
+        <v>2.2263999999999999</v>
+      </c>
+      <c r="AH4" s="132" t="s">
         <v>170</v>
       </c>
-      <c r="AH4" s="132">
+      <c r="AI4" s="132">
         <v>2865</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A5" s="141" t="s">
         <v>343</v>
       </c>
@@ -6817,17 +6833,20 @@
       <c r="W5" s="146">
         <v>-57900</v>
       </c>
-      <c r="X5" s="173"/>
-      <c r="Y5" s="170">
-        <f t="shared" ref="Y5:Y53" si="2">SUM(H5:X5)</f>
-        <v>380973</v>
-      </c>
-      <c r="Z5" s="148">
-        <f t="shared" ref="Z5:Z53" si="3">IFERROR(Y5/F5*100,0)/10000000</f>
-        <v>1.2699100000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="X5" s="146">
+        <v>-95500</v>
+      </c>
+      <c r="Y5" s="173"/>
+      <c r="Z5" s="170">
+        <f t="shared" ref="Z5:Z53" si="2">SUM(H5:Y5)</f>
+        <v>285473</v>
+      </c>
+      <c r="AA5" s="148">
+        <f t="shared" ref="AA5:AA53" si="3">IFERROR(Z5/F5*100,0)/10000000</f>
+        <v>0.95157666666666674</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A6" s="141" t="s">
         <v>344</v>
       </c>
@@ -6895,17 +6914,20 @@
       <c r="W6" s="146">
         <v>-169055</v>
       </c>
-      <c r="X6" s="173"/>
-      <c r="Y6" s="170">
+      <c r="X6" s="146">
+        <v>76500</v>
+      </c>
+      <c r="Y6" s="173"/>
+      <c r="Z6" s="170">
         <f t="shared" si="2"/>
-        <v>252087</v>
-      </c>
-      <c r="Z6" s="148">
+        <v>328587</v>
+      </c>
+      <c r="AA6" s="148">
         <f t="shared" si="3"/>
-        <v>2.5208699999999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.2858700000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:38" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="141" t="s">
         <v>134</v>
       </c>
@@ -6973,21 +6995,24 @@
       <c r="W7" s="146">
         <v>92400</v>
       </c>
-      <c r="X7" s="173"/>
-      <c r="Y7" s="170">
+      <c r="X7" s="146">
+        <v>121200</v>
+      </c>
+      <c r="Y7" s="173"/>
+      <c r="Z7" s="170">
         <f t="shared" si="2"/>
-        <v>-8360</v>
-      </c>
-      <c r="Z7" s="148">
+        <v>112840</v>
+      </c>
+      <c r="AA7" s="148">
         <f t="shared" si="3"/>
-        <v>-2.7866666666666661E-2</v>
-      </c>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="133">
-        <v>5037</v>
-      </c>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
+        <v>0.37613333333333338</v>
+      </c>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="133">
+        <v>-17173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A8" s="141" t="s">
         <v>217</v>
       </c>
@@ -7055,21 +7080,24 @@
       <c r="W8" s="146">
         <v>-16364</v>
       </c>
-      <c r="X8" s="173"/>
-      <c r="Y8" s="170">
+      <c r="X8" s="146">
+        <v>10700</v>
+      </c>
+      <c r="Y8" s="173"/>
+      <c r="Z8" s="170">
         <f t="shared" si="2"/>
-        <v>255986</v>
-      </c>
-      <c r="Z8" s="148">
+        <v>266686</v>
+      </c>
+      <c r="AA8" s="148">
         <f t="shared" si="3"/>
-        <v>1.7065733333333335</v>
-      </c>
-      <c r="AB8" s="133">
-        <v>20085</v>
-      </c>
-      <c r="AC8" s="133"/>
-    </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
+        <v>1.7779066666666665</v>
+      </c>
+      <c r="AC8" s="133">
+        <v>244627</v>
+      </c>
+      <c r="AD8" s="133"/>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A9" s="141" t="s">
         <v>313</v>
       </c>
@@ -7135,24 +7163,27 @@
       <c r="W9" s="146">
         <v>50600</v>
       </c>
-      <c r="X9" s="173"/>
-      <c r="Y9" s="170">
+      <c r="X9" s="146">
+        <v>62800</v>
+      </c>
+      <c r="Y9" s="173"/>
+      <c r="Z9" s="170">
         <f t="shared" si="2"/>
-        <v>213427</v>
-      </c>
-      <c r="Z9" s="148">
+        <v>276227</v>
+      </c>
+      <c r="AA9" s="148">
         <f t="shared" si="3"/>
-        <v>3.5571166666666674</v>
-      </c>
-      <c r="AB9" s="133">
-        <v>25122</v>
+        <v>4.6037833333333333</v>
       </c>
       <c r="AC9" s="133">
-        <f>(AB9+AB8)/10000000*13780</f>
-        <v>62.295245999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
+        <v>229732</v>
+      </c>
+      <c r="AD9" s="133">
+        <f>(AC9+AC8)/10000000*13780</f>
+        <v>653.66670199999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A10" s="142" t="s">
         <v>35</v>
       </c>
@@ -7220,19 +7251,22 @@
       <c r="W10" s="146">
         <v>0</v>
       </c>
-      <c r="X10" s="173"/>
-      <c r="Y10" s="170">
+      <c r="X10" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="173"/>
+      <c r="Z10" s="170">
         <f t="shared" si="2"/>
         <v>-87379</v>
       </c>
-      <c r="Z10" s="148">
+      <c r="AA10" s="148">
         <f t="shared" si="3"/>
         <v>-5.8252666666666661E-2</v>
       </c>
-      <c r="AB10" s="133"/>
       <c r="AC10" s="133"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="AD10" s="133"/>
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A11" s="142" t="s">
         <v>137</v>
       </c>
@@ -7300,19 +7334,22 @@
       <c r="W11" s="146">
         <v>12420</v>
       </c>
-      <c r="X11" s="173"/>
-      <c r="Y11" s="170">
+      <c r="X11" s="146">
+        <v>-114575</v>
+      </c>
+      <c r="Y11" s="173"/>
+      <c r="Z11" s="170">
         <f t="shared" si="2"/>
-        <v>385774</v>
-      </c>
-      <c r="Z11" s="148">
+        <v>271199</v>
+      </c>
+      <c r="AA11" s="148">
         <f t="shared" si="3"/>
-        <v>0.64295666666666662</v>
-      </c>
-      <c r="AB11" s="133"/>
+        <v>0.45199833333333339</v>
+      </c>
       <c r="AC11" s="133"/>
-    </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="AD11" s="133"/>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A12" s="142" t="s">
         <v>42</v>
       </c>
@@ -7380,19 +7417,22 @@
       <c r="W12" s="146">
         <v>1111</v>
       </c>
-      <c r="X12" s="173"/>
-      <c r="Y12" s="170">
+      <c r="X12" s="146">
+        <v>-413</v>
+      </c>
+      <c r="Y12" s="173"/>
+      <c r="Z12" s="170">
         <f t="shared" si="2"/>
-        <v>-12535</v>
-      </c>
-      <c r="Z12" s="148">
+        <v>-12948</v>
+      </c>
+      <c r="AA12" s="148">
         <f t="shared" si="3"/>
-        <v>-0.12534999999999999</v>
-      </c>
-      <c r="AB12" s="133"/>
+        <v>-0.12948000000000001</v>
+      </c>
       <c r="AC12" s="133"/>
-    </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="AD12" s="133"/>
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A13" s="141" t="s">
         <v>212</v>
       </c>
@@ -7460,19 +7500,22 @@
       <c r="W13" s="146">
         <v>-40457</v>
       </c>
-      <c r="X13" s="173"/>
-      <c r="Y13" s="170">
+      <c r="X13" s="146">
+        <v>-15543</v>
+      </c>
+      <c r="Y13" s="173"/>
+      <c r="Z13" s="170">
         <f t="shared" si="2"/>
-        <v>106535</v>
-      </c>
-      <c r="Z13" s="148">
+        <v>90992</v>
+      </c>
+      <c r="AA13" s="148">
         <f t="shared" si="3"/>
-        <v>0.42614000000000002</v>
-      </c>
-      <c r="AB13" s="133"/>
+        <v>0.36396800000000007</v>
+      </c>
       <c r="AC13" s="133"/>
-    </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="AD13" s="133"/>
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A14" s="141" t="s">
         <v>51</v>
       </c>
@@ -7540,29 +7583,32 @@
       <c r="W14" s="146">
         <v>-37218</v>
       </c>
-      <c r="X14" s="173"/>
-      <c r="Y14" s="170">
+      <c r="X14" s="146">
+        <v>-17800</v>
+      </c>
+      <c r="Y14" s="173"/>
+      <c r="Z14" s="170">
         <f t="shared" si="2"/>
-        <v>139118</v>
-      </c>
-      <c r="Z14" s="148">
+        <v>121318</v>
+      </c>
+      <c r="AA14" s="148">
         <f t="shared" si="3"/>
-        <v>0.63235454545454539</v>
-      </c>
-      <c r="AB14" s="133"/>
-      <c r="AC14" s="192">
-        <f>AC7-AC9</f>
-        <v>4974.7047540000003</v>
-      </c>
-      <c r="AF14" s="132">
+        <v>0.55144545454545446</v>
+      </c>
+      <c r="AC14" s="133"/>
+      <c r="AD14" s="192">
+        <f>AD7-AD9</f>
+        <v>-17826.666701999999</v>
+      </c>
+      <c r="AG14" s="132">
         <v>-13200</v>
       </c>
-      <c r="AH14" s="132">
-        <f>AF14+AC14</f>
-        <v>-8225.2952459999997</v>
-      </c>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="AI14" s="132">
+        <f>AG14+AD14</f>
+        <v>-31026.666701999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A15" s="141" t="s">
         <v>43</v>
       </c>
@@ -7630,17 +7676,20 @@
       <c r="W15" s="146">
         <v>17900</v>
       </c>
-      <c r="X15" s="173"/>
-      <c r="Y15" s="170">
+      <c r="X15" s="146">
+        <v>17130</v>
+      </c>
+      <c r="Y15" s="173"/>
+      <c r="Z15" s="170">
         <f t="shared" si="2"/>
-        <v>-30633</v>
-      </c>
-      <c r="Z15" s="148">
+        <v>-13503</v>
+      </c>
+      <c r="AA15" s="148">
         <f t="shared" si="3"/>
-        <v>-0.30632999999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
+        <v>-0.13503000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A16" s="141" t="s">
         <v>24</v>
       </c>
@@ -7708,28 +7757,31 @@
       <c r="W16" s="146">
         <v>30270</v>
       </c>
-      <c r="X16" s="173"/>
-      <c r="Y16" s="170">
+      <c r="X16" s="146">
+        <v>157200</v>
+      </c>
+      <c r="Y16" s="173"/>
+      <c r="Z16" s="170">
         <f t="shared" si="2"/>
-        <v>428868</v>
-      </c>
-      <c r="Z16" s="148">
+        <v>586068</v>
+      </c>
+      <c r="AA16" s="148">
         <f t="shared" si="3"/>
-        <v>1.7154720000000001</v>
-      </c>
-      <c r="AH16" s="132">
+        <v>2.3442720000000001</v>
+      </c>
+      <c r="AI16" s="132">
         <v>4000000</v>
       </c>
-      <c r="AI16" s="132">
-        <f>AH16*7/100</f>
+      <c r="AJ16" s="132">
+        <f>AI16*7/100</f>
         <v>280000</v>
       </c>
-      <c r="AK16" s="132">
+      <c r="AL16" s="132">
         <f>15*12</f>
         <v>180</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="141" t="s">
         <v>23</v>
       </c>
@@ -7797,21 +7849,24 @@
       <c r="W17" s="146">
         <v>168000</v>
       </c>
-      <c r="X17" s="173"/>
-      <c r="Y17" s="170">
+      <c r="X17" s="146">
+        <v>-171000</v>
+      </c>
+      <c r="Y17" s="173"/>
+      <c r="Z17" s="170">
         <f t="shared" si="2"/>
-        <v>737424</v>
-      </c>
-      <c r="Z17" s="148">
+        <v>566424</v>
+      </c>
+      <c r="AA17" s="148">
         <f t="shared" si="3"/>
-        <v>1.8435600000000001</v>
-      </c>
-      <c r="AI17" s="132">
-        <f>AI16/12</f>
+        <v>1.4160600000000001</v>
+      </c>
+      <c r="AJ17" s="132">
+        <f>AJ16/12</f>
         <v>23333.333333333332</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" s="141" t="s">
         <v>165</v>
       </c>
@@ -7879,17 +7934,20 @@
       <c r="W18" s="146">
         <v>39300</v>
       </c>
-      <c r="X18" s="173"/>
-      <c r="Y18" s="170">
+      <c r="X18" s="146">
+        <v>32700</v>
+      </c>
+      <c r="Y18" s="173"/>
+      <c r="Z18" s="170">
         <f t="shared" si="2"/>
-        <v>719336</v>
-      </c>
-      <c r="Z18" s="148">
+        <v>752036</v>
+      </c>
+      <c r="AA18" s="148">
         <f t="shared" si="3"/>
-        <v>4.7955733333333326</v>
-      </c>
-    </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
+        <v>5.0135733333333325</v>
+      </c>
+    </row>
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" s="141" t="s">
         <v>110</v>
       </c>
@@ -7957,20 +8015,23 @@
       <c r="W19" s="146">
         <v>0</v>
       </c>
-      <c r="X19" s="173"/>
-      <c r="Y19" s="170">
+      <c r="X19" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="173"/>
+      <c r="Z19" s="170">
         <f t="shared" si="2"/>
         <v>-150688</v>
       </c>
-      <c r="Z19" s="148">
+      <c r="AA19" s="148">
         <f t="shared" si="3"/>
         <v>-1.3698909090909093</v>
       </c>
-      <c r="AD19" s="132">
+      <c r="AE19" s="132">
         <v>54000</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A20" s="141" t="s">
         <v>319</v>
       </c>
@@ -8038,20 +8099,23 @@
       <c r="W20" s="146">
         <v>0</v>
       </c>
-      <c r="X20" s="173"/>
-      <c r="Y20" s="170">
+      <c r="X20" s="146">
+        <v>140</v>
+      </c>
+      <c r="Y20" s="173"/>
+      <c r="Z20" s="170">
         <f t="shared" si="2"/>
-        <v>-110972</v>
-      </c>
-      <c r="Z20" s="148">
+        <v>-110832</v>
+      </c>
+      <c r="AA20" s="148">
         <f t="shared" si="3"/>
-        <v>-4.4388800000000002</v>
-      </c>
-      <c r="AD20" s="132">
+        <v>-4.4332799999999999</v>
+      </c>
+      <c r="AE20" s="132">
         <v>11100</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="141" t="s">
         <v>316</v>
       </c>
@@ -8119,20 +8183,21 @@
       <c r="W21" s="146">
         <v>0</v>
       </c>
-      <c r="X21" s="173"/>
-      <c r="Y21" s="170">
+      <c r="X21" s="146"/>
+      <c r="Y21" s="173"/>
+      <c r="Z21" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Z21" s="148">
+      <c r="AA21" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AD21" s="132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AE21" s="132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="141" t="s">
         <v>317</v>
       </c>
@@ -8200,21 +8265,24 @@
       <c r="W22" s="146">
         <v>0</v>
       </c>
-      <c r="X22" s="173"/>
-      <c r="Y22" s="170">
+      <c r="X22" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="173"/>
+      <c r="Z22" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Z22" s="148">
+      <c r="AA22" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AD22" s="132">
-        <f>SUM(AD19:AD21)</f>
+      <c r="AE22" s="132">
+        <f>SUM(AE19:AE21)</f>
         <v>65100</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="141" t="s">
         <v>32</v>
       </c>
@@ -8282,17 +8350,20 @@
       <c r="W23" s="146">
         <v>54387</v>
       </c>
-      <c r="X23" s="173"/>
-      <c r="Y23" s="170">
+      <c r="X23" s="146">
+        <v>-5748</v>
+      </c>
+      <c r="Y23" s="173"/>
+      <c r="Z23" s="170">
         <f t="shared" si="2"/>
-        <v>-21517</v>
-      </c>
-      <c r="Z23" s="148">
+        <v>-27265</v>
+      </c>
+      <c r="AA23" s="148">
         <f t="shared" si="3"/>
-        <v>-0.19560909090909087</v>
-      </c>
-    </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
+        <v>-0.24786363636363637</v>
+      </c>
+    </row>
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="141" t="s">
         <v>97</v>
       </c>
@@ -8360,17 +8431,20 @@
       <c r="W24" s="146">
         <v>77900</v>
       </c>
-      <c r="X24" s="173"/>
-      <c r="Y24" s="170">
+      <c r="X24" s="146">
+        <v>133200</v>
+      </c>
+      <c r="Y24" s="173"/>
+      <c r="Z24" s="170">
         <f t="shared" si="2"/>
-        <v>-699679</v>
-      </c>
-      <c r="Z24" s="148">
+        <v>-566479</v>
+      </c>
+      <c r="AA24" s="148">
         <f t="shared" si="3"/>
-        <v>-3.0420826086956523</v>
-      </c>
-    </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
+        <v>-2.4629521739130436</v>
+      </c>
+    </row>
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="141" t="s">
         <v>335</v>
       </c>
@@ -8424,17 +8498,20 @@
       <c r="W25" s="146">
         <v>71400</v>
       </c>
-      <c r="X25" s="173"/>
-      <c r="Y25" s="170">
+      <c r="X25" s="146">
+        <v>87920</v>
+      </c>
+      <c r="Y25" s="173"/>
+      <c r="Z25" s="170">
         <f t="shared" si="2"/>
-        <v>101071</v>
-      </c>
-      <c r="Z25" s="148">
+        <v>188991</v>
+      </c>
+      <c r="AA25" s="148">
         <f t="shared" si="3"/>
-        <v>5.0535500000000004</v>
-      </c>
-    </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
+        <v>9.4495500000000003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" s="141" t="s">
         <v>302</v>
       </c>
@@ -8500,17 +8577,20 @@
       <c r="W26" s="146">
         <v>-18145</v>
       </c>
-      <c r="X26" s="173"/>
-      <c r="Y26" s="170">
+      <c r="X26" s="146">
+        <v>14000</v>
+      </c>
+      <c r="Y26" s="173"/>
+      <c r="Z26" s="170">
         <f t="shared" si="2"/>
-        <v>-45804</v>
-      </c>
-      <c r="Z26" s="148">
+        <v>-31804</v>
+      </c>
+      <c r="AA26" s="148">
         <f t="shared" si="3"/>
-        <v>-0.91608000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
+        <v>-0.63607999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A27" s="141" t="s">
         <v>29</v>
       </c>
@@ -8578,17 +8658,20 @@
       <c r="W27" s="146">
         <v>397000</v>
       </c>
-      <c r="X27" s="173"/>
-      <c r="Y27" s="170">
+      <c r="X27" s="146">
+        <v>-482000</v>
+      </c>
+      <c r="Y27" s="173"/>
+      <c r="Z27" s="170">
         <f t="shared" si="2"/>
-        <v>2290800</v>
-      </c>
-      <c r="Z27" s="148">
+        <v>1808800</v>
+      </c>
+      <c r="AA27" s="148">
         <f t="shared" si="3"/>
-        <v>4.5815999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
+        <v>3.6175999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="141" t="s">
         <v>28</v>
       </c>
@@ -8656,17 +8739,20 @@
       <c r="W28" s="146">
         <v>-162700</v>
       </c>
-      <c r="X28" s="173"/>
-      <c r="Y28" s="170">
+      <c r="X28" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="173"/>
+      <c r="Z28" s="170">
         <f t="shared" si="2"/>
         <v>225891</v>
       </c>
-      <c r="Z28" s="148">
+      <c r="AA28" s="148">
         <f t="shared" si="3"/>
         <v>0.22589100000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="141" t="s">
         <v>332</v>
       </c>
@@ -8730,17 +8816,20 @@
       <c r="W29" s="146">
         <v>-28900</v>
       </c>
-      <c r="X29" s="173"/>
-      <c r="Y29" s="170">
+      <c r="X29" s="146">
+        <v>32266</v>
+      </c>
+      <c r="Y29" s="173"/>
+      <c r="Z29" s="170">
         <f t="shared" si="2"/>
-        <v>-4080</v>
-      </c>
-      <c r="Z29" s="148">
+        <v>28186</v>
+      </c>
+      <c r="AA29" s="148">
         <f t="shared" si="3"/>
-        <v>-8.1600000000000006E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
+        <v>0.56372</v>
+      </c>
+    </row>
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="141" t="s">
         <v>65</v>
       </c>
@@ -8808,17 +8897,20 @@
       <c r="W30" s="146">
         <v>0</v>
       </c>
-      <c r="X30" s="173"/>
-      <c r="Y30" s="170">
+      <c r="X30" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="173"/>
+      <c r="Z30" s="170">
         <f t="shared" si="2"/>
         <v>841174</v>
       </c>
-      <c r="Z30" s="148">
+      <c r="AA30" s="148">
         <f t="shared" si="3"/>
         <v>1.682348</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" s="140" t="s">
         <v>34</v>
       </c>
@@ -8886,17 +8978,20 @@
       <c r="W31" s="146">
         <v>0</v>
       </c>
-      <c r="X31" s="173"/>
-      <c r="Y31" s="170">
+      <c r="X31" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="173"/>
+      <c r="Z31" s="170">
         <f t="shared" si="2"/>
         <v>140133</v>
       </c>
-      <c r="Z31" s="148">
+      <c r="AA31" s="148">
         <f t="shared" si="3"/>
         <v>0.28026600000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A32" s="140" t="s">
         <v>131</v>
       </c>
@@ -8964,17 +9059,20 @@
       <c r="W32" s="146">
         <v>4974</v>
       </c>
-      <c r="X32" s="173"/>
-      <c r="Y32" s="170">
+      <c r="X32" s="146">
+        <v>-27000</v>
+      </c>
+      <c r="Y32" s="173"/>
+      <c r="Z32" s="170">
         <f t="shared" si="2"/>
-        <v>70166</v>
-      </c>
-      <c r="Z32" s="148">
+        <v>43166</v>
+      </c>
+      <c r="AA32" s="148">
         <f t="shared" si="3"/>
-        <v>1.4033199999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
+        <v>0.86331999999999998</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="43" t="s">
         <v>67</v>
       </c>
@@ -9042,18 +9140,21 @@
       <c r="W33" s="146">
         <v>38495</v>
       </c>
-      <c r="X33" s="173"/>
-      <c r="Y33" s="170">
+      <c r="X33" s="146">
+        <v>3700</v>
+      </c>
+      <c r="Y33" s="173"/>
+      <c r="Z33" s="170">
         <f t="shared" si="2"/>
-        <v>340337</v>
-      </c>
-      <c r="Z33" s="148">
+        <v>344037</v>
+      </c>
+      <c r="AA33" s="148">
         <f t="shared" si="3"/>
-        <v>8.5084250000000008</v>
-      </c>
-      <c r="AC33" s="133"/>
-    </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
+        <v>8.6009250000000002</v>
+      </c>
+      <c r="AD33" s="133"/>
+    </row>
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="141" t="s">
         <v>31</v>
       </c>
@@ -9121,21 +9222,24 @@
       <c r="W34" s="146">
         <v>16600</v>
       </c>
-      <c r="X34" s="173"/>
-      <c r="Y34" s="170">
+      <c r="X34" s="146">
+        <v>-60500</v>
+      </c>
+      <c r="Y34" s="173"/>
+      <c r="Z34" s="170">
         <f t="shared" si="2"/>
-        <v>371505</v>
-      </c>
-      <c r="Z34" s="148">
+        <v>311005</v>
+      </c>
+      <c r="AA34" s="148">
         <f t="shared" si="3"/>
-        <v>0.92876250000000005</v>
-      </c>
-      <c r="AB34" s="5"/>
-      <c r="AC34" s="133">
+        <v>0.77751250000000005</v>
+      </c>
+      <c r="AC34" s="5"/>
+      <c r="AD34" s="133">
         <v>46634</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="141" t="s">
         <v>104</v>
       </c>
@@ -9203,19 +9307,22 @@
       <c r="W35" s="146">
         <v>41600</v>
       </c>
-      <c r="X35" s="173"/>
-      <c r="Y35" s="170">
+      <c r="X35" s="146">
+        <v>60600</v>
+      </c>
+      <c r="Y35" s="173"/>
+      <c r="Z35" s="170">
         <f t="shared" si="2"/>
-        <v>-97365</v>
-      </c>
-      <c r="Z35" s="148">
+        <v>-36765</v>
+      </c>
+      <c r="AA35" s="148">
         <f t="shared" si="3"/>
-        <v>-0.97365000000000002</v>
-      </c>
-      <c r="AB35" s="5"/>
-      <c r="AC35" s="133"/>
-    </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
+        <v>-0.36764999999999998</v>
+      </c>
+      <c r="AC35" s="5"/>
+      <c r="AD35" s="133"/>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="141" t="s">
         <v>314</v>
       </c>
@@ -9281,24 +9388,27 @@
       <c r="W36" s="146">
         <v>0</v>
       </c>
-      <c r="X36" s="173"/>
-      <c r="Y36" s="170">
+      <c r="X36" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="173"/>
+      <c r="Z36" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Z36" s="148">
+      <c r="AA36" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AB36" s="133">
+      <c r="AC36" s="133">
         <v>233083</v>
       </c>
-      <c r="AC36" s="133">
-        <f>(AB37+AB36)/10000000*13780</f>
+      <c r="AD36" s="133">
+        <f>(AC37+AC36)/10000000*13780</f>
         <v>706.63839999999993</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="141" t="s">
         <v>229</v>
       </c>
@@ -9366,21 +9476,24 @@
       <c r="W37" s="146">
         <v>-6562</v>
       </c>
-      <c r="X37" s="173"/>
-      <c r="Y37" s="170">
+      <c r="X37" s="146">
+        <v>-17725</v>
+      </c>
+      <c r="Y37" s="173"/>
+      <c r="Z37" s="170">
         <f t="shared" si="2"/>
-        <v>-24327</v>
-      </c>
-      <c r="Z37" s="148">
+        <v>-42052</v>
+      </c>
+      <c r="AA37" s="148">
         <f t="shared" si="3"/>
-        <v>-0.48653999999999997</v>
-      </c>
-      <c r="AB37" s="133">
+        <v>-0.84104000000000001</v>
+      </c>
+      <c r="AC37" s="133">
         <v>279717</v>
       </c>
-      <c r="AC37" s="133"/>
-    </row>
-    <row r="38" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD37" s="133"/>
+    </row>
+    <row r="38" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="141" t="s">
         <v>45</v>
       </c>
@@ -9448,22 +9561,25 @@
       <c r="W38" s="146">
         <v>-219600</v>
       </c>
-      <c r="X38" s="173"/>
-      <c r="Y38" s="170">
+      <c r="X38" s="146">
+        <v>-306450</v>
+      </c>
+      <c r="Y38" s="173"/>
+      <c r="Z38" s="170">
         <f t="shared" si="2"/>
-        <v>728571</v>
-      </c>
-      <c r="Z38" s="148">
+        <v>422121</v>
+      </c>
+      <c r="AA38" s="148">
         <f t="shared" si="3"/>
-        <v>2.4285700000000001</v>
-      </c>
-      <c r="AB38" s="133"/>
-      <c r="AC38" s="133">
-        <f>+AC34-AC36</f>
+        <v>1.40707</v>
+      </c>
+      <c r="AC38" s="133"/>
+      <c r="AD38" s="133">
+        <f>+AD34-AD36</f>
         <v>45927.361599999997</v>
       </c>
     </row>
-    <row r="39" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="141" t="s">
         <v>292</v>
       </c>
@@ -9529,19 +9645,22 @@
       <c r="W39" s="146">
         <v>15022</v>
       </c>
-      <c r="X39" s="173"/>
-      <c r="Y39" s="170">
+      <c r="X39" s="146">
+        <v>-118577</v>
+      </c>
+      <c r="Y39" s="173"/>
+      <c r="Z39" s="170">
         <f t="shared" si="2"/>
-        <v>-72992</v>
-      </c>
-      <c r="Z39" s="148">
+        <v>-191569</v>
+      </c>
+      <c r="AA39" s="148">
         <f t="shared" si="3"/>
-        <v>-7.2991999999999999</v>
-      </c>
-      <c r="AB39" s="133"/>
+        <v>-19.1569</v>
+      </c>
       <c r="AC39" s="133"/>
-    </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AD39" s="133"/>
+    </row>
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="141" t="s">
         <v>132</v>
       </c>
@@ -9609,19 +9728,22 @@
       <c r="W40" s="146">
         <v>12700</v>
       </c>
-      <c r="X40" s="173"/>
-      <c r="Y40" s="170">
+      <c r="X40" s="146">
+        <v>-5383</v>
+      </c>
+      <c r="Y40" s="173"/>
+      <c r="Z40" s="170">
         <f t="shared" si="2"/>
-        <v>80741</v>
-      </c>
-      <c r="Z40" s="148">
+        <v>75358</v>
+      </c>
+      <c r="AA40" s="148">
         <f t="shared" si="3"/>
-        <v>1.6148199999999999</v>
-      </c>
-      <c r="AB40" s="133"/>
+        <v>1.5071600000000001</v>
+      </c>
       <c r="AC40" s="133"/>
-    </row>
-    <row r="41" spans="1:29" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD40" s="133"/>
+    </row>
+    <row r="41" spans="1:30" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="141" t="s">
         <v>48</v>
       </c>
@@ -9689,19 +9811,22 @@
       <c r="W41" s="146">
         <v>119000</v>
       </c>
-      <c r="X41" s="173"/>
-      <c r="Y41" s="170">
+      <c r="X41" s="146">
+        <v>216130</v>
+      </c>
+      <c r="Y41" s="173"/>
+      <c r="Z41" s="170">
         <f t="shared" si="2"/>
-        <v>-963743</v>
-      </c>
-      <c r="Z41" s="148">
+        <v>-747613</v>
+      </c>
+      <c r="AA41" s="148">
         <f t="shared" si="3"/>
-        <v>-9.6374300000000002</v>
-      </c>
-      <c r="AB41" s="133"/>
+        <v>-7.4761300000000004</v>
+      </c>
       <c r="AC41" s="133"/>
-    </row>
-    <row r="42" spans="1:29" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD41" s="133"/>
+    </row>
+    <row r="42" spans="1:30" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="141" t="s">
         <v>336</v>
       </c>
@@ -9755,19 +9880,22 @@
       <c r="W42" s="146">
         <v>136200</v>
       </c>
-      <c r="X42" s="173"/>
-      <c r="Y42" s="170">
+      <c r="X42" s="146">
+        <v>51600</v>
+      </c>
+      <c r="Y42" s="173"/>
+      <c r="Z42" s="170">
         <f t="shared" si="2"/>
-        <v>495990</v>
-      </c>
-      <c r="Z42" s="148">
+        <v>547590</v>
+      </c>
+      <c r="AA42" s="148">
         <f t="shared" si="3"/>
-        <v>9.9198000000000004</v>
-      </c>
-      <c r="AB42" s="133"/>
+        <v>10.9518</v>
+      </c>
       <c r="AC42" s="133"/>
-    </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AD42" s="133"/>
+    </row>
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="141" t="s">
         <v>301</v>
       </c>
@@ -9833,18 +9961,21 @@
       <c r="W43" s="146">
         <v>18400</v>
       </c>
-      <c r="X43" s="173"/>
-      <c r="Y43" s="170">
+      <c r="X43" s="146">
+        <v>2428</v>
+      </c>
+      <c r="Y43" s="173"/>
+      <c r="Z43" s="170">
         <f t="shared" si="2"/>
-        <v>-33213</v>
-      </c>
-      <c r="Z43" s="148">
+        <v>-30785</v>
+      </c>
+      <c r="AA43" s="148">
         <f t="shared" si="3"/>
-        <v>-0.66425999999999996</v>
-      </c>
-      <c r="AB43" s="133"/>
-    </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
+        <v>-0.61570000000000003</v>
+      </c>
+      <c r="AC43" s="133"/>
+    </row>
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="142" t="s">
         <v>168</v>
       </c>
@@ -9912,17 +10043,20 @@
       <c r="W44" s="146">
         <v>0</v>
       </c>
-      <c r="X44" s="173"/>
-      <c r="Y44" s="170">
+      <c r="X44" s="146">
+        <v>5500</v>
+      </c>
+      <c r="Y44" s="173"/>
+      <c r="Z44" s="170">
         <f t="shared" si="2"/>
-        <v>80210</v>
-      </c>
-      <c r="Z44" s="148">
+        <v>85710</v>
+      </c>
+      <c r="AA44" s="148">
         <f t="shared" si="3"/>
-        <v>0.20052500000000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
+        <v>0.21427499999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="142" t="s">
         <v>202</v>
       </c>
@@ -9990,17 +10124,20 @@
       <c r="W45" s="146">
         <v>-39900</v>
       </c>
-      <c r="X45" s="173"/>
-      <c r="Y45" s="170">
+      <c r="X45" s="146">
+        <v>196500</v>
+      </c>
+      <c r="Y45" s="173"/>
+      <c r="Z45" s="170">
         <f t="shared" si="2"/>
-        <v>8361</v>
-      </c>
-      <c r="Z45" s="148">
+        <v>204861</v>
+      </c>
+      <c r="AA45" s="148">
         <f t="shared" si="3"/>
-        <v>2.0902500000000001E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
+        <v>0.51215250000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="142" t="s">
         <v>33</v>
       </c>
@@ -10068,17 +10205,20 @@
       <c r="W46" s="146">
         <v>0</v>
       </c>
-      <c r="X46" s="173"/>
-      <c r="Y46" s="170">
+      <c r="X46" s="146">
+        <v>0</v>
+      </c>
+      <c r="Y46" s="173"/>
+      <c r="Z46" s="170">
         <f t="shared" si="2"/>
         <v>1105039</v>
       </c>
-      <c r="Z46" s="148">
+      <c r="AA46" s="148">
         <f t="shared" si="3"/>
         <v>3.6834633333333326</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="59" t="s">
         <v>306</v>
       </c>
@@ -10144,17 +10284,20 @@
       <c r="W47" s="150">
         <v>-181800</v>
       </c>
-      <c r="X47" s="173"/>
-      <c r="Y47" s="170">
+      <c r="X47" s="150">
+        <v>174900</v>
+      </c>
+      <c r="Y47" s="173"/>
+      <c r="Z47" s="170">
         <f t="shared" si="2"/>
-        <v>-3132740</v>
-      </c>
-      <c r="Z47" s="148">
+        <v>-2957840</v>
+      </c>
+      <c r="AA47" s="148">
         <f t="shared" si="3"/>
-        <v>-3.1327400000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
+        <v>-2.95784</v>
+      </c>
+    </row>
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59" t="s">
         <v>197</v>
       </c>
@@ -10222,17 +10365,20 @@
       <c r="W48" s="150">
         <v>45927</v>
       </c>
-      <c r="X48" s="173"/>
-      <c r="Y48" s="170">
+      <c r="X48" s="150">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="173"/>
+      <c r="Z48" s="170">
         <f t="shared" si="2"/>
         <v>61459</v>
       </c>
-      <c r="Z48" s="148">
+      <c r="AA48" s="148">
         <f t="shared" si="3"/>
         <v>1.2291799999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49" s="59" t="s">
         <v>213</v>
       </c>
@@ -10300,17 +10446,20 @@
       <c r="W49" s="150">
         <v>0</v>
       </c>
-      <c r="X49" s="173"/>
-      <c r="Y49" s="170">
+      <c r="X49" s="150">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="173"/>
+      <c r="Z49" s="170">
         <f t="shared" si="2"/>
         <v>369643</v>
       </c>
-      <c r="Z49" s="148">
+      <c r="AA49" s="148">
         <f t="shared" si="3"/>
         <v>0.56868153846153835</v>
       </c>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50" s="59" t="s">
         <v>214</v>
       </c>
@@ -10378,17 +10527,20 @@
       <c r="W50" s="150">
         <v>0</v>
       </c>
-      <c r="X50" s="173"/>
-      <c r="Y50" s="170">
+      <c r="X50" s="150">
+        <v>0</v>
+      </c>
+      <c r="Y50" s="173"/>
+      <c r="Z50" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Z50" s="148">
+      <c r="AA50" s="148">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A51" s="59" t="s">
         <v>49</v>
       </c>
@@ -10456,17 +10608,20 @@
       <c r="W51" s="150">
         <v>0</v>
       </c>
-      <c r="X51" s="173"/>
-      <c r="Y51" s="170">
+      <c r="X51" s="150">
+        <v>0</v>
+      </c>
+      <c r="Y51" s="173"/>
+      <c r="Z51" s="170">
         <f t="shared" si="2"/>
         <v>311687</v>
       </c>
-      <c r="Z51" s="148">
+      <c r="AA51" s="148">
         <f t="shared" si="3"/>
         <v>1.0389566666666668</v>
       </c>
     </row>
-    <row r="52" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52" s="59" t="s">
         <v>331</v>
       </c>
@@ -10534,17 +10689,20 @@
       <c r="W52" s="150">
         <v>13000</v>
       </c>
-      <c r="X52" s="173"/>
-      <c r="Y52" s="170">
+      <c r="X52" s="150">
+        <v>21100</v>
+      </c>
+      <c r="Y52" s="173"/>
+      <c r="Z52" s="170">
         <f t="shared" si="2"/>
-        <v>30634</v>
-      </c>
-      <c r="Z52" s="148">
+        <v>51734</v>
+      </c>
+      <c r="AA52" s="148">
         <f t="shared" si="3"/>
-        <v>0.30634</v>
-      </c>
-    </row>
-    <row r="53" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.51734000000000002</v>
+      </c>
+    </row>
+    <row r="53" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="59" t="s">
         <v>288</v>
       </c>
@@ -10612,17 +10770,20 @@
       <c r="W53" s="150">
         <v>94734</v>
       </c>
-      <c r="X53" s="173"/>
-      <c r="Y53" s="170">
+      <c r="X53" s="150">
+        <v>186200</v>
+      </c>
+      <c r="Y53" s="173"/>
+      <c r="Z53" s="170">
         <f t="shared" si="2"/>
-        <v>881323</v>
-      </c>
-      <c r="Z53" s="148">
+        <v>1067523</v>
+      </c>
+      <c r="AA53" s="148">
         <f t="shared" si="3"/>
-        <v>0.88132299999999997</v>
-      </c>
-    </row>
-    <row r="54" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1.067523</v>
+      </c>
+    </row>
+    <row r="54" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="24"/>
       <c r="B54" s="25"/>
       <c r="C54" s="26"/>
@@ -10631,7 +10792,7 @@
       <c r="F54" s="115"/>
       <c r="G54" s="16"/>
       <c r="H54" s="253">
-        <f t="shared" ref="H54:W54" si="4">SUM(H4:H53)</f>
+        <f t="shared" ref="H54:X54" si="4">SUM(H4:H53)</f>
         <v>38252</v>
       </c>
       <c r="I54" s="253">
@@ -10695,19 +10856,23 @@
         <v>584177</v>
       </c>
       <c r="X54" s="253">
-        <f>SUM(X4:X53)</f>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>214317</v>
       </c>
       <c r="Y54" s="253">
-        <f>SUM(H54:X54)</f>
-        <v>6781439</v>
-      </c>
-      <c r="Z54" s="254">
-        <f t="shared" ref="Z54" si="5">IFERROR(Y54/F54*100,0)/10000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <f>SUM(Y4:Y53)</f>
+        <v>0</v>
+      </c>
+      <c r="Z54" s="253">
+        <f>SUM(H54:Y54)</f>
+        <v>6995756</v>
+      </c>
+      <c r="AA54" s="254">
+        <f t="shared" ref="AA54" si="5">IFERROR(Z54/F54*100,0)/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="249"/>
       <c r="B55" s="249"/>
       <c r="C55" s="249"/>
@@ -10733,9 +10898,10 @@
       <c r="W55" s="249"/>
       <c r="X55" s="249"/>
       <c r="Y55" s="249"/>
-      <c r="Z55" s="251"/>
-    </row>
-    <row r="56" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="Z55" s="249"/>
+      <c r="AA55" s="251"/>
+    </row>
+    <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56" s="201" t="s">
         <v>241</v>
       </c>
@@ -10803,17 +10969,20 @@
       <c r="W56" s="161">
         <v>0</v>
       </c>
-      <c r="X56" s="245"/>
-      <c r="Y56" s="246">
-        <f>SUM(H56:X56)</f>
-        <v>28620</v>
-      </c>
-      <c r="Z56" s="247">
-        <f>IFERROR(Y56/F56*100,0)/10000000</f>
-        <v>9.5399999999999999E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X56" s="161">
+        <v>509300</v>
+      </c>
+      <c r="Y56" s="245"/>
+      <c r="Z56" s="246">
+        <f>SUM(H56:Y56)</f>
+        <v>537920</v>
+      </c>
+      <c r="AA56" s="247">
+        <f>IFERROR(Z56/F56*100,0)/10000000</f>
+        <v>1.7930666666666664</v>
+      </c>
+    </row>
+    <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57" s="201" t="s">
         <v>273</v>
       </c>
@@ -10879,17 +11048,20 @@
       <c r="W57" s="161">
         <v>24300</v>
       </c>
-      <c r="X57" s="173"/>
-      <c r="Y57" s="170">
-        <f>SUM(H57:X57)</f>
-        <v>-213294</v>
-      </c>
-      <c r="Z57" s="148">
-        <f>IFERROR(Y57/F57*100,0)/10000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X57" s="161">
+        <v>187300</v>
+      </c>
+      <c r="Y57" s="173"/>
+      <c r="Z57" s="170">
+        <f>SUM(H57:Y57)</f>
+        <v>-25994</v>
+      </c>
+      <c r="AA57" s="148">
+        <f>IFERROR(Z57/F57*100,0)/10000000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A58" s="201"/>
       <c r="B58" s="202" t="s">
         <v>338</v>
@@ -10931,11 +11103,17 @@
       <c r="W58" s="161">
         <v>0</v>
       </c>
-      <c r="X58" s="161"/>
-      <c r="Y58" s="257"/>
-      <c r="Z58" s="258"/>
-    </row>
-    <row r="59" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="X58" s="161">
+        <v>0</v>
+      </c>
+      <c r="Y58" s="161"/>
+      <c r="Z58" s="170">
+        <f t="shared" ref="Z58:Z59" si="6">SUM(H58:Y58)</f>
+        <v>0</v>
+      </c>
+      <c r="AA58" s="257"/>
+    </row>
+    <row r="59" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="201" t="s">
         <v>340</v>
       </c>
@@ -10979,11 +11157,17 @@
       <c r="W59" s="161">
         <v>1600</v>
       </c>
-      <c r="X59" s="161"/>
-      <c r="Y59" s="257"/>
-      <c r="Z59" s="258"/>
-    </row>
-    <row r="60" spans="1:30" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="X59" s="161">
+        <v>204500</v>
+      </c>
+      <c r="Y59" s="161"/>
+      <c r="Z59" s="170">
+        <f t="shared" si="6"/>
+        <v>41478</v>
+      </c>
+      <c r="AA59" s="257"/>
+    </row>
+    <row r="60" spans="1:31" s="248" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="199"/>
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
@@ -10992,51 +11176,51 @@
       <c r="F60" s="74"/>
       <c r="G60" s="17"/>
       <c r="H60" s="169">
-        <f t="shared" ref="H60:S60" si="6">SUM(H56:H57)</f>
+        <f t="shared" ref="H60:S60" si="7">SUM(H56:H57)</f>
         <v>5771</v>
       </c>
       <c r="I60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-81800</v>
       </c>
       <c r="J60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>309555</v>
       </c>
       <c r="K60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>15600</v>
       </c>
       <c r="L60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>149000</v>
       </c>
       <c r="M60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-9023</v>
       </c>
       <c r="N60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-50</v>
       </c>
       <c r="O60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-458665</v>
       </c>
       <c r="P60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-608</v>
       </c>
       <c r="Q60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-184264</v>
       </c>
       <c r="R60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>789</v>
       </c>
       <c r="S60" s="169">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>15771</v>
       </c>
       <c r="T60" s="169">
@@ -11056,73 +11240,77 @@
         <v>25900</v>
       </c>
       <c r="X60" s="169">
-        <f>SUM(X56:X57)</f>
-        <v>0</v>
-      </c>
-      <c r="Y60" s="256">
-        <f>SUM(H60:X60)</f>
-        <v>-288916</v>
-      </c>
-      <c r="Z60" s="172"/>
-    </row>
-    <row r="61" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AC61" s="133"/>
-    </row>
-    <row r="62" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AB62" s="133"/>
-    </row>
-    <row r="63" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AB63" s="5"/>
-      <c r="AC63" s="133"/>
-      <c r="AD63" s="236"/>
-    </row>
-    <row r="64" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AB64" s="133"/>
+        <f>SUM(X56:X59)</f>
+        <v>901100</v>
+      </c>
+      <c r="Y60" s="169">
+        <f>SUM(Y56:Y57)</f>
+        <v>0</v>
+      </c>
+      <c r="Z60" s="256">
+        <f>SUM(H60:Y60)</f>
+        <v>612184</v>
+      </c>
+      <c r="AA60" s="172"/>
+    </row>
+    <row r="61" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AD61" s="133"/>
+    </row>
+    <row r="62" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AC62" s="133"/>
+    </row>
+    <row r="63" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AC63" s="5"/>
+      <c r="AD63" s="133"/>
+      <c r="AE63" s="236"/>
+    </row>
+    <row r="64" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC64" s="133"/>
-      <c r="AD64" s="236"/>
-    </row>
-    <row r="65" spans="28:30" x14ac:dyDescent="0.25">
-      <c r="AB65" s="133"/>
+      <c r="AD64" s="133"/>
+      <c r="AE64" s="236"/>
+    </row>
+    <row r="65" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC65" s="133"/>
-      <c r="AD65" s="236"/>
-    </row>
-    <row r="66" spans="28:30" x14ac:dyDescent="0.25">
-      <c r="AB66" s="133"/>
+      <c r="AD65" s="133"/>
+      <c r="AE65" s="236"/>
+    </row>
+    <row r="66" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC66" s="133"/>
-      <c r="AD66" s="236"/>
-    </row>
-    <row r="67" spans="28:30" x14ac:dyDescent="0.25">
-      <c r="AB67" s="133"/>
+      <c r="AD66" s="133"/>
+      <c r="AE66" s="236"/>
+    </row>
+    <row r="67" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC67" s="133"/>
-      <c r="AD67" s="236"/>
-    </row>
-    <row r="68" spans="28:30" x14ac:dyDescent="0.25">
-      <c r="AB68" s="133"/>
-      <c r="AC68" s="236"/>
+      <c r="AD67" s="133"/>
+      <c r="AE67" s="236"/>
+    </row>
+    <row r="68" spans="29:31" x14ac:dyDescent="0.25">
+      <c r="AC68" s="133"/>
       <c r="AD68" s="236"/>
-    </row>
-    <row r="69" spans="28:30" x14ac:dyDescent="0.25">
-      <c r="AB69" s="236"/>
+      <c r="AE68" s="236"/>
+    </row>
+    <row r="69" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC69" s="236"/>
       <c r="AD69" s="236"/>
+      <c r="AE69" s="236"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2 A3:G3 Z54:Z55 Z60 H2:Z3 G38:X38 A4:X37 A56:Z59 A39:X54 A60:X60">
+  <conditionalFormatting sqref="G2 A3:G3 AA54:AA55 AA60 H2:AA3 G38:Y38 A4:Y37 A56:AA59 A39:Y54 A60:Y60">
     <cfRule type="expression" dxfId="537" priority="18">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y4:Z53">
+  <conditionalFormatting sqref="Z4:AA53">
     <cfRule type="expression" dxfId="536" priority="15">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y54">
+  <conditionalFormatting sqref="Z54">
     <cfRule type="expression" dxfId="535" priority="12">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y60">
+  <conditionalFormatting sqref="Z60">
     <cfRule type="expression" dxfId="534" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -11489,7 +11677,7 @@
       <c r="R6" s="158"/>
       <c r="S6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>123203</v>
+        <v>111320</v>
       </c>
       <c r="T6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11501,7 +11689,7 @@
       <c r="X6" s="131"/>
       <c r="Y6" s="153">
         <f t="shared" si="4"/>
-        <v>-429271</v>
+        <v>-441154</v>
       </c>
       <c r="Z6" s="167">
         <f t="shared" si="5"/>
@@ -11794,7 +11982,7 @@
       <c r="R10" s="158"/>
       <c r="S10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>380973</v>
+        <v>285473</v>
       </c>
       <c r="T10" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11805,7 +11993,7 @@
       <c r="W10" s="149"/>
       <c r="Y10" s="153">
         <f t="shared" ref="Y10:Y11" si="8">M10+P10+S10+V10</f>
-        <v>380973</v>
+        <v>285473</v>
       </c>
       <c r="Z10" s="167">
         <f t="shared" ref="Z10:Z11" si="9">(N10+Q10+T10+W10)</f>
@@ -11857,7 +12045,7 @@
       <c r="R11" s="158"/>
       <c r="S11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>252087</v>
+        <v>328587</v>
       </c>
       <c r="T11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11868,7 +12056,7 @@
       <c r="W11" s="149"/>
       <c r="Y11" s="153">
         <f t="shared" si="8"/>
-        <v>252087</v>
+        <v>328587</v>
       </c>
       <c r="Z11" s="167">
         <f t="shared" si="9"/>
@@ -11938,7 +12126,7 @@
       <c r="R12" s="158"/>
       <c r="S12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-8360</v>
+        <v>112840</v>
       </c>
       <c r="T12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -11949,7 +12137,7 @@
       <c r="W12" s="72"/>
       <c r="Y12" s="153">
         <f t="shared" si="4"/>
-        <v>-1184427</v>
+        <v>-1063227</v>
       </c>
       <c r="Z12" s="167">
         <f t="shared" si="5"/>
@@ -12019,7 +12207,7 @@
       <c r="R13" s="158"/>
       <c r="S13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>255986</v>
+        <v>266686</v>
       </c>
       <c r="T13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12030,7 +12218,7 @@
       <c r="W13" s="149"/>
       <c r="Y13" s="153">
         <f t="shared" si="4"/>
-        <v>-145889</v>
+        <v>-135189</v>
       </c>
       <c r="Z13" s="167">
         <f t="shared" si="5"/>
@@ -12100,7 +12288,7 @@
       <c r="R14" s="158"/>
       <c r="S14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>213427</v>
+        <v>276227</v>
       </c>
       <c r="T14" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12111,7 +12299,7 @@
       <c r="W14" s="149"/>
       <c r="Y14" s="153">
         <f t="shared" si="4"/>
-        <v>123498</v>
+        <v>186298</v>
       </c>
       <c r="Z14" s="167">
         <f t="shared" si="5"/>
@@ -12590,7 +12778,7 @@
       <c r="R20" s="158"/>
       <c r="S20" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>385774</v>
+        <v>271199</v>
       </c>
       <c r="T20" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12601,7 +12789,7 @@
       <c r="W20" s="72"/>
       <c r="Y20" s="153">
         <f t="shared" si="4"/>
-        <v>585826</v>
+        <v>471251</v>
       </c>
       <c r="Z20" s="167">
         <f t="shared" si="5"/>
@@ -12671,7 +12859,7 @@
       <c r="R21" s="158"/>
       <c r="S21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-12535</v>
+        <v>-12948</v>
       </c>
       <c r="T21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12682,7 +12870,7 @@
       <c r="W21" s="149"/>
       <c r="Y21" s="153">
         <f t="shared" si="4"/>
-        <v>-9960</v>
+        <v>-10373</v>
       </c>
       <c r="Z21" s="167">
         <f t="shared" si="5"/>
@@ -12842,7 +13030,7 @@
       <c r="R23" s="158"/>
       <c r="S23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>106535</v>
+        <v>90992</v>
       </c>
       <c r="T23" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12853,7 +13041,7 @@
       <c r="W23" s="72"/>
       <c r="Y23" s="153">
         <f t="shared" si="4"/>
-        <v>-144647</v>
+        <v>-160190</v>
       </c>
       <c r="Z23" s="167">
         <f t="shared" si="5"/>
@@ -12923,7 +13111,7 @@
       <c r="R24" s="158"/>
       <c r="S24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>139118</v>
+        <v>121318</v>
       </c>
       <c r="T24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -12934,7 +13122,7 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="153">
         <f t="shared" si="4"/>
-        <v>-64505</v>
+        <v>-82305</v>
       </c>
       <c r="Z24" s="167">
         <f t="shared" si="5"/>
@@ -13085,7 +13273,7 @@
       <c r="R26" s="158"/>
       <c r="S26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-30633</v>
+        <v>-13503</v>
       </c>
       <c r="T26" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13096,7 +13284,7 @@
       <c r="W26" s="72"/>
       <c r="Y26" s="153">
         <f t="shared" si="4"/>
-        <v>1715548</v>
+        <v>1732678</v>
       </c>
       <c r="Z26" s="167">
         <f t="shared" si="5"/>
@@ -13407,7 +13595,7 @@
       <c r="R30" s="158"/>
       <c r="S30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>428868</v>
+        <v>586068</v>
       </c>
       <c r="T30" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13418,7 +13606,7 @@
       <c r="W30" s="72"/>
       <c r="Y30" s="153">
         <f t="shared" si="4"/>
-        <v>807136</v>
+        <v>964336</v>
       </c>
       <c r="Z30" s="167">
         <f t="shared" si="5"/>
@@ -13488,7 +13676,7 @@
       <c r="R31" s="158"/>
       <c r="S31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>737424</v>
+        <v>566424</v>
       </c>
       <c r="T31" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13500,7 +13688,7 @@
       <c r="X31" s="1"/>
       <c r="Y31" s="153">
         <f t="shared" si="4"/>
-        <v>1616877</v>
+        <v>1445877</v>
       </c>
       <c r="Z31" s="167">
         <f t="shared" si="5"/>
@@ -13741,7 +13929,7 @@
       <c r="R34" s="158"/>
       <c r="S34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>719336</v>
+        <v>752036</v>
       </c>
       <c r="T34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13753,7 +13941,7 @@
       <c r="X34"/>
       <c r="Y34" s="153">
         <f t="shared" si="4"/>
-        <v>233331</v>
+        <v>266031</v>
       </c>
       <c r="Z34" s="167">
         <f t="shared" si="5"/>
@@ -13904,7 +14092,7 @@
       <c r="R36" s="158"/>
       <c r="S36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-21517</v>
+        <v>-27265</v>
       </c>
       <c r="T36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -13915,7 +14103,7 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="153">
         <f t="shared" si="4"/>
-        <v>-169144</v>
+        <v>-174892</v>
       </c>
       <c r="Z36" s="167">
         <f t="shared" si="5"/>
@@ -14073,7 +14261,7 @@
       <c r="R38" s="158"/>
       <c r="S38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-699679</v>
+        <v>-566479</v>
       </c>
       <c r="T38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14084,7 +14272,7 @@
       <c r="W38" s="72"/>
       <c r="Y38" s="153">
         <f t="shared" si="4"/>
-        <v>2202947</v>
+        <v>2336147</v>
       </c>
       <c r="Z38" s="167">
         <f t="shared" si="5"/>
@@ -14152,7 +14340,7 @@
       <c r="R39" s="158"/>
       <c r="S39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>101071</v>
+        <v>188991</v>
       </c>
       <c r="T39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14163,7 +14351,7 @@
       <c r="W39" s="149"/>
       <c r="Y39" s="153">
         <f t="shared" si="4"/>
-        <v>101071</v>
+        <v>188991</v>
       </c>
       <c r="Z39" s="167">
         <f t="shared" si="5"/>
@@ -14231,7 +14419,7 @@
       <c r="R40" s="158"/>
       <c r="S40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-45804</v>
+        <v>-31804</v>
       </c>
       <c r="T40" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14242,7 +14430,7 @@
       <c r="W40" s="149"/>
       <c r="Y40" s="153">
         <f t="shared" si="4"/>
-        <v>-89470</v>
+        <v>-75470</v>
       </c>
       <c r="Z40" s="167">
         <f t="shared" si="5"/>
@@ -14312,7 +14500,7 @@
       <c r="R41" s="158"/>
       <c r="S41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>2290800</v>
+        <v>1808800</v>
       </c>
       <c r="T41" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -14323,7 +14511,7 @@
       <c r="W41" s="72"/>
       <c r="Y41" s="153">
         <f t="shared" si="4"/>
-        <v>4831854</v>
+        <v>4349854</v>
       </c>
       <c r="Z41" s="167">
         <f t="shared" si="5"/>
@@ -14907,18 +15095,18 @@
       <c r="R48" s="158"/>
       <c r="S48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-4080</v>
+        <v>28186</v>
       </c>
       <c r="T48" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="U48" s="217"/>
-      <c r="V48" s="259"/>
+      <c r="V48" s="258"/>
       <c r="W48" s="149"/>
       <c r="Y48" s="153">
         <f t="shared" si="4"/>
-        <v>-4080</v>
+        <v>28186</v>
       </c>
       <c r="Z48" s="167">
         <f t="shared" si="5"/>
@@ -15152,7 +15340,7 @@
       <c r="R51" s="158"/>
       <c r="S51" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>70166</v>
+        <v>43166</v>
       </c>
       <c r="T51" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15163,7 +15351,7 @@
       <c r="W51" s="72"/>
       <c r="Y51" s="153">
         <f t="shared" si="4"/>
-        <v>-8884</v>
+        <v>-35884</v>
       </c>
       <c r="Z51" s="167">
         <f t="shared" si="5"/>
@@ -15321,7 +15509,7 @@
       <c r="R53" s="158"/>
       <c r="S53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>340337</v>
+        <v>344037</v>
       </c>
       <c r="T53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15332,7 +15520,7 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="153">
         <f t="shared" si="4"/>
-        <v>408602</v>
+        <v>412302</v>
       </c>
       <c r="Z53" s="167">
         <f t="shared" si="5"/>
@@ -15576,7 +15764,7 @@
       <c r="R56" s="158"/>
       <c r="S56" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>371505</v>
+        <v>311005</v>
       </c>
       <c r="T56" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15587,7 +15775,7 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="153">
         <f t="shared" si="4"/>
-        <v>566566</v>
+        <v>506066</v>
       </c>
       <c r="Z56" s="167">
         <f t="shared" si="5"/>
@@ -15657,7 +15845,7 @@
       <c r="R57" s="158"/>
       <c r="S57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-97365</v>
+        <v>-36765</v>
       </c>
       <c r="T57" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15668,7 +15856,7 @@
       <c r="W57" s="72"/>
       <c r="Y57" s="153">
         <f t="shared" si="4"/>
-        <v>562884</v>
+        <v>623484</v>
       </c>
       <c r="Z57" s="167">
         <f t="shared" si="5"/>
@@ -15819,7 +16007,7 @@
       <c r="R59" s="158"/>
       <c r="S59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-24327</v>
+        <v>-42052</v>
       </c>
       <c r="T59" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15831,7 +16019,7 @@
       <c r="X59" s="131"/>
       <c r="Y59" s="153">
         <f t="shared" si="4"/>
-        <v>-298352</v>
+        <v>-316077</v>
       </c>
       <c r="Z59" s="167">
         <f t="shared" si="5"/>
@@ -15902,7 +16090,7 @@
       <c r="R60" s="158"/>
       <c r="S60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>728571</v>
+        <v>422121</v>
       </c>
       <c r="T60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15913,7 +16101,7 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="153">
         <f t="shared" si="4"/>
-        <v>-3925764</v>
+        <v>-4232214</v>
       </c>
       <c r="Z60" s="167">
         <f t="shared" si="5"/>
@@ -16154,7 +16342,7 @@
       <c r="R63" s="158"/>
       <c r="S63" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-72992</v>
+        <v>-191569</v>
       </c>
       <c r="T63" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16165,7 +16353,7 @@
       <c r="W63" s="149"/>
       <c r="Y63" s="153">
         <f t="shared" si="4"/>
-        <v>-93113</v>
+        <v>-211690</v>
       </c>
       <c r="Z63" s="167">
         <f t="shared" si="5"/>
@@ -16235,7 +16423,7 @@
       <c r="R64" s="158"/>
       <c r="S64" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>80741</v>
+        <v>75358</v>
       </c>
       <c r="T64" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16247,7 +16435,7 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="153">
         <f t="shared" si="4"/>
-        <v>113432</v>
+        <v>108049</v>
       </c>
       <c r="Z64" s="167">
         <f t="shared" si="5"/>
@@ -16324,7 +16512,7 @@
       <c r="R65" s="158"/>
       <c r="S65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-963743</v>
+        <v>-747613</v>
       </c>
       <c r="T65" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16335,7 +16523,7 @@
       <c r="W65" s="72"/>
       <c r="Y65" s="153">
         <f t="shared" si="4"/>
-        <v>2715872</v>
+        <v>2932002</v>
       </c>
       <c r="Z65" s="167">
         <f t="shared" si="5"/>
@@ -16412,7 +16600,7 @@
       <c r="R66" s="158"/>
       <c r="S66" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>495990</v>
+        <v>547590</v>
       </c>
       <c r="T66" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16423,7 +16611,7 @@
       <c r="W66" s="149"/>
       <c r="Y66" s="153">
         <f t="shared" si="4"/>
-        <v>495990</v>
+        <v>547590</v>
       </c>
       <c r="Z66" s="167">
         <f t="shared" si="5"/>
@@ -16491,7 +16679,7 @@
       <c r="R67" s="158"/>
       <c r="S67" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-33213</v>
+        <v>-30785</v>
       </c>
       <c r="T67" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16502,7 +16690,7 @@
       <c r="W67" s="149"/>
       <c r="Y67" s="153">
         <f t="shared" si="4"/>
-        <v>-19922</v>
+        <v>-17494</v>
       </c>
       <c r="Z67" s="167">
         <f t="shared" si="5"/>
@@ -16660,7 +16848,7 @@
       <c r="R69" s="158"/>
       <c r="S69" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>80210</v>
+        <v>85710</v>
       </c>
       <c r="T69" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16671,7 +16859,7 @@
       <c r="W69" s="72"/>
       <c r="Y69" s="153">
         <f t="shared" si="4"/>
-        <v>1045083</v>
+        <v>1050583</v>
       </c>
       <c r="Z69" s="167">
         <f t="shared" si="5"/>
@@ -16823,7 +17011,7 @@
       <c r="R71" s="158"/>
       <c r="S71" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>8361</v>
+        <v>204861</v>
       </c>
       <c r="T71" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16835,7 +17023,7 @@
       <c r="X71" s="131"/>
       <c r="Y71" s="153">
         <f t="shared" ref="Y71:Y81" si="12">M71+P71+S71+V71</f>
-        <v>791142</v>
+        <v>987642</v>
       </c>
       <c r="Z71" s="167">
         <f t="shared" ref="Z71:Z81" si="13">(N71+Q71+T71+W71)</f>
@@ -16985,7 +17173,7 @@
       <c r="R73" s="158"/>
       <c r="S73" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-3132740</v>
+        <v>-2957840</v>
       </c>
       <c r="T73" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16996,7 +17184,7 @@
       <c r="W73" s="149"/>
       <c r="Y73" s="153">
         <f t="shared" si="12"/>
-        <v>-4095569</v>
+        <v>-3920669</v>
       </c>
       <c r="Z73" s="167">
         <f t="shared" si="13"/>
@@ -17544,7 +17732,7 @@
       <c r="R80" s="158"/>
       <c r="S80" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>30634</v>
+        <v>51734</v>
       </c>
       <c r="T80" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17555,7 +17743,7 @@
       <c r="W80" s="149"/>
       <c r="Y80" s="153">
         <f t="shared" si="12"/>
-        <v>30634</v>
+        <v>51734</v>
       </c>
       <c r="Z80" s="167">
         <f t="shared" si="13"/>
@@ -17623,7 +17811,7 @@
       <c r="R81" s="158"/>
       <c r="S81" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>881323</v>
+        <v>1067523</v>
       </c>
       <c r="T81" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17634,7 +17822,7 @@
       <c r="W81" s="149"/>
       <c r="Y81" s="153">
         <f t="shared" si="12"/>
-        <v>1372176</v>
+        <v>1558376</v>
       </c>
       <c r="Z81" s="167">
         <f t="shared" si="13"/>
@@ -17677,7 +17865,7 @@
       <c r="R82" s="122"/>
       <c r="S82" s="153">
         <f>SUM(S4:S81)</f>
-        <v>6892411</v>
+        <v>7106588</v>
       </c>
       <c r="T82" s="122"/>
       <c r="U82" s="122"/>
@@ -17685,7 +17873,7 @@
       <c r="W82" s="50"/>
       <c r="Y82" s="153">
         <f>SUM(Y4:Y81)</f>
-        <v>30161941</v>
+        <v>30376118</v>
       </c>
       <c r="Z82" s="160"/>
     </row>
@@ -19422,12 +19610,12 @@
         <v>0.5</v>
       </c>
       <c r="G4" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>123203</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>111320</v>
       </c>
       <c r="H4" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>2.4640599999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>2.2263999999999999</v>
       </c>
       <c r="I4" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19447,11 +19635,11 @@
       </c>
       <c r="M4" s="71">
         <f t="shared" ref="M4:N52" si="0">G4+I4+K4</f>
-        <v>123203</v>
+        <v>111320</v>
       </c>
       <c r="N4" s="165">
         <f t="shared" si="0"/>
-        <v>2.4640599999999999</v>
+        <v>2.2263999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -19474,12 +19662,12 @@
         <v>3.5</v>
       </c>
       <c r="G5" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>380973</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>285473</v>
       </c>
       <c r="H5" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.2699100000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.95157666666666674</v>
       </c>
       <c r="I5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19499,11 +19687,11 @@
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>380973</v>
+        <v>285473</v>
       </c>
       <c r="N5" s="165">
         <f t="shared" si="0"/>
-        <v>1.2699100000000001</v>
+        <v>0.95157666666666674</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -19526,12 +19714,12 @@
         <v>1</v>
       </c>
       <c r="G6" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>252087</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>328587</v>
       </c>
       <c r="H6" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>2.5208699999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>3.2858700000000001</v>
       </c>
       <c r="I6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19551,11 +19739,11 @@
       </c>
       <c r="M6" s="71">
         <f t="shared" si="0"/>
-        <v>252087</v>
+        <v>328587</v>
       </c>
       <c r="N6" s="165">
         <f t="shared" si="0"/>
-        <v>2.5208699999999999</v>
+        <v>3.2858700000000001</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -19578,12 +19766,12 @@
         <v>3</v>
       </c>
       <c r="G7" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-8360</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>112840</v>
       </c>
       <c r="H7" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-2.7866666666666661E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.37613333333333338</v>
       </c>
       <c r="I7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19603,11 +19791,11 @@
       </c>
       <c r="M7" s="71">
         <f t="shared" si="0"/>
-        <v>-8360</v>
+        <v>112840</v>
       </c>
       <c r="N7" s="165">
         <f t="shared" si="0"/>
-        <v>-2.7866666666666661E-2</v>
+        <v>0.37613333333333338</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -19630,12 +19818,12 @@
         <v>1.5</v>
       </c>
       <c r="G8" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>255986</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>266686</v>
       </c>
       <c r="H8" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.7065733333333335</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.7779066666666665</v>
       </c>
       <c r="I8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19655,11 +19843,11 @@
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>255986</v>
+        <v>266686</v>
       </c>
       <c r="N8" s="165">
         <f t="shared" si="0"/>
-        <v>1.7065733333333335</v>
+        <v>1.7779066666666665</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -19682,12 +19870,12 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>213427</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>276227</v>
       </c>
       <c r="H9" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>3.5571166666666674</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>4.6037833333333333</v>
       </c>
       <c r="I9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19707,11 +19895,11 @@
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>213427</v>
+        <v>276227</v>
       </c>
       <c r="N9" s="165">
         <f t="shared" si="0"/>
-        <v>3.5571166666666674</v>
+        <v>4.6037833333333333</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -19734,11 +19922,11 @@
         <v>15</v>
       </c>
       <c r="G10" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>-87379</v>
       </c>
       <c r="H10" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>-5.8252666666666661E-2</v>
       </c>
       <c r="I10" s="152">
@@ -19786,12 +19974,12 @@
         <v>6</v>
       </c>
       <c r="G11" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>385774</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>271199</v>
       </c>
       <c r="H11" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.64295666666666662</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.45199833333333339</v>
       </c>
       <c r="I11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19811,11 +19999,11 @@
       </c>
       <c r="M11" s="71">
         <f t="shared" si="0"/>
-        <v>385774</v>
+        <v>271199</v>
       </c>
       <c r="N11" s="165">
         <f t="shared" si="0"/>
-        <v>0.64295666666666662</v>
+        <v>0.45199833333333339</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -19838,12 +20026,12 @@
         <v>1</v>
       </c>
       <c r="G12" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-12535</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-12948</v>
       </c>
       <c r="H12" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.12534999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.12948000000000001</v>
       </c>
       <c r="I12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19863,11 +20051,11 @@
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>-12535</v>
+        <v>-12948</v>
       </c>
       <c r="N12" s="165">
         <f t="shared" si="0"/>
-        <v>-0.12534999999999999</v>
+        <v>-0.12948000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -19890,12 +20078,12 @@
         <v>1</v>
       </c>
       <c r="G13" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>106535</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>90992</v>
       </c>
       <c r="H13" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.42614000000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.36396800000000007</v>
       </c>
       <c r="I13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19915,11 +20103,11 @@
       </c>
       <c r="M13" s="71">
         <f t="shared" si="0"/>
-        <v>106535</v>
+        <v>90992</v>
       </c>
       <c r="N13" s="165">
         <f t="shared" si="0"/>
-        <v>0.42614000000000002</v>
+        <v>0.36396800000000007</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -19942,12 +20130,12 @@
         <v>1</v>
       </c>
       <c r="G14" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-30633</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-13503</v>
       </c>
       <c r="H14" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.30632999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.13503000000000001</v>
       </c>
       <c r="I14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -19967,11 +20155,11 @@
       </c>
       <c r="M14" s="71">
         <f t="shared" si="0"/>
-        <v>-30633</v>
+        <v>-13503</v>
       </c>
       <c r="N14" s="165">
         <f t="shared" si="0"/>
-        <v>-0.30632999999999999</v>
+        <v>-0.13503000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -19994,12 +20182,12 @@
         <v>0.2</v>
       </c>
       <c r="G15" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>139118</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>121318</v>
       </c>
       <c r="H15" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.63235454545454539</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.55144545454545446</v>
       </c>
       <c r="I15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20019,11 +20207,11 @@
       </c>
       <c r="M15" s="71">
         <f t="shared" si="0"/>
-        <v>139118</v>
+        <v>121318</v>
       </c>
       <c r="N15" s="165">
         <f t="shared" si="0"/>
-        <v>0.63235454545454539</v>
+        <v>0.55144545454545446</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -20046,12 +20234,12 @@
         <v>2.5</v>
       </c>
       <c r="G16" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>428868</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>586068</v>
       </c>
       <c r="H16" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.7154720000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>2.3442720000000001</v>
       </c>
       <c r="I16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20071,11 +20259,11 @@
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>428868</v>
+        <v>586068</v>
       </c>
       <c r="N16" s="165">
         <f t="shared" si="0"/>
-        <v>1.7154720000000001</v>
+        <v>2.3442720000000001</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -20098,12 +20286,12 @@
         <v>4</v>
       </c>
       <c r="G17" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>737424</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>566424</v>
       </c>
       <c r="H17" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.8435600000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.4160600000000001</v>
       </c>
       <c r="I17" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20123,11 +20311,11 @@
       </c>
       <c r="M17" s="71">
         <f t="shared" si="0"/>
-        <v>737424</v>
+        <v>566424</v>
       </c>
       <c r="N17" s="165">
         <f t="shared" si="0"/>
-        <v>1.8435600000000001</v>
+        <v>1.4160600000000001</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -20150,11 +20338,11 @@
         <v>0.25</v>
       </c>
       <c r="G18" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>-150688</v>
       </c>
       <c r="H18" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>-1.3698909090909093</v>
       </c>
       <c r="I18" s="152">
@@ -20202,12 +20390,12 @@
         <v>0.25</v>
       </c>
       <c r="G19" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-110972</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-110832</v>
       </c>
       <c r="H19" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-4.4388800000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-4.4332799999999999</v>
       </c>
       <c r="I19" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20227,11 +20415,11 @@
       </c>
       <c r="M19" s="71">
         <f t="shared" si="0"/>
-        <v>-110972</v>
+        <v>-110832</v>
       </c>
       <c r="N19" s="165">
         <f t="shared" si="0"/>
-        <v>-4.4388800000000002</v>
+        <v>-4.4332799999999999</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -20254,11 +20442,11 @@
         <v>2</v>
       </c>
       <c r="G20" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="152">
@@ -20306,12 +20494,12 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>719336</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>752036</v>
       </c>
       <c r="H21" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>4.7955733333333326</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>5.0135733333333325</v>
       </c>
       <c r="I21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20331,11 +20519,11 @@
       </c>
       <c r="M21" s="71">
         <f t="shared" si="0"/>
-        <v>719336</v>
+        <v>752036</v>
       </c>
       <c r="N21" s="165">
         <f t="shared" si="0"/>
-        <v>4.7955733333333326</v>
+        <v>5.0135733333333325</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -20358,12 +20546,12 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="G22" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-21517</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-27265</v>
       </c>
       <c r="H22" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.19560909090909087</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.24786363636363637</v>
       </c>
       <c r="I22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20383,11 +20571,11 @@
       </c>
       <c r="M22" s="71">
         <f t="shared" si="0"/>
-        <v>-21517</v>
+        <v>-27265</v>
       </c>
       <c r="N22" s="165">
         <f t="shared" si="0"/>
-        <v>-0.19560909090909087</v>
+        <v>-0.24786363636363637</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -20410,12 +20598,12 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G23" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-699679</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-566479</v>
       </c>
       <c r="H23" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-3.0420826086956523</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-2.4629521739130436</v>
       </c>
       <c r="I23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20435,11 +20623,11 @@
       </c>
       <c r="M23" s="71">
         <f t="shared" si="0"/>
-        <v>-699679</v>
+        <v>-566479</v>
       </c>
       <c r="N23" s="165">
         <f t="shared" si="0"/>
-        <v>-3.0420826086956523</v>
+        <v>-2.4629521739130436</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -20460,12 +20648,12 @@
         <v>0.2</v>
       </c>
       <c r="G24" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>101071</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>188991</v>
       </c>
       <c r="H24" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>5.0535500000000004</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>9.4495500000000003</v>
       </c>
       <c r="I24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20485,11 +20673,11 @@
       </c>
       <c r="M24" s="71">
         <f t="shared" ref="M24" si="1">G24+I24+K24</f>
-        <v>101071</v>
+        <v>188991</v>
       </c>
       <c r="N24" s="165">
         <f t="shared" ref="N24" si="2">H24+J24+L24</f>
-        <v>5.0535500000000004</v>
+        <v>9.4495500000000003</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -20510,12 +20698,12 @@
         <v>0.2</v>
       </c>
       <c r="G25" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-45804</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-31804</v>
       </c>
       <c r="H25" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.91608000000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.63607999999999998</v>
       </c>
       <c r="I25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20535,11 +20723,11 @@
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>-45804</v>
+        <v>-31804</v>
       </c>
       <c r="N25" s="165">
         <f t="shared" si="0"/>
-        <v>-0.91608000000000001</v>
+        <v>-0.63607999999999998</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -20562,12 +20750,12 @@
         <v>5</v>
       </c>
       <c r="G26" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>2290800</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1808800</v>
       </c>
       <c r="H26" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>4.5815999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>3.6175999999999999</v>
       </c>
       <c r="I26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20587,11 +20775,11 @@
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>2290800</v>
+        <v>1808800</v>
       </c>
       <c r="N26" s="165">
         <f t="shared" si="0"/>
-        <v>4.5815999999999999</v>
+        <v>3.6175999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -20614,11 +20802,11 @@
         <v>10</v>
       </c>
       <c r="G27" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>225891</v>
       </c>
       <c r="H27" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0.22589100000000001</v>
       </c>
       <c r="I27" s="152">
@@ -20665,12 +20853,12 @@
         <v>1</v>
       </c>
       <c r="G28" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-4080</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>28186</v>
       </c>
       <c r="H28" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-8.1600000000000006E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.56372</v>
       </c>
       <c r="I28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20690,11 +20878,11 @@
       </c>
       <c r="M28" s="71">
         <f t="shared" ref="M28" si="3">G28+I28+K28</f>
-        <v>-4080</v>
+        <v>28186</v>
       </c>
       <c r="N28" s="165">
         <f t="shared" ref="N28" si="4">H28+J28+L28</f>
-        <v>-8.1600000000000006E-2</v>
+        <v>0.56372</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -20717,11 +20905,11 @@
         <v>5</v>
       </c>
       <c r="G29" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>841174</v>
       </c>
       <c r="H29" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>1.682348</v>
       </c>
       <c r="I29" s="152">
@@ -20769,11 +20957,11 @@
         <v>5</v>
       </c>
       <c r="G30" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>140133</v>
       </c>
       <c r="H30" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0.28026600000000002</v>
       </c>
       <c r="I30" s="152">
@@ -20821,12 +21009,12 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>70166</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>43166</v>
       </c>
       <c r="H31" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.4033199999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.86331999999999998</v>
       </c>
       <c r="I31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20846,11 +21034,11 @@
       </c>
       <c r="M31" s="71">
         <f t="shared" si="0"/>
-        <v>70166</v>
+        <v>43166</v>
       </c>
       <c r="N31" s="165">
         <f t="shared" si="0"/>
-        <v>1.4033199999999999</v>
+        <v>0.86331999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -20873,12 +21061,12 @@
         <v>0.4</v>
       </c>
       <c r="G32" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>340337</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>344037</v>
       </c>
       <c r="H32" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>8.5084250000000008</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>8.6009250000000002</v>
       </c>
       <c r="I32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20898,11 +21086,11 @@
       </c>
       <c r="M32" s="71">
         <f t="shared" si="0"/>
-        <v>340337</v>
+        <v>344037</v>
       </c>
       <c r="N32" s="165">
         <f t="shared" si="0"/>
-        <v>8.5084250000000008</v>
+        <v>8.6009250000000002</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -20925,12 +21113,12 @@
         <v>4</v>
       </c>
       <c r="G33" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>371505</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>311005</v>
       </c>
       <c r="H33" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.92876250000000005</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.77751250000000005</v>
       </c>
       <c r="I33" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -20950,11 +21138,11 @@
       </c>
       <c r="M33" s="71">
         <f t="shared" si="0"/>
-        <v>371505</v>
+        <v>311005</v>
       </c>
       <c r="N33" s="165">
         <f t="shared" si="0"/>
-        <v>0.92876250000000005</v>
+        <v>0.77751250000000005</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -20977,12 +21165,12 @@
         <v>1</v>
       </c>
       <c r="G34" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-97365</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-36765</v>
       </c>
       <c r="H34" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.97365000000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.36764999999999998</v>
       </c>
       <c r="I34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21002,11 +21190,11 @@
       </c>
       <c r="M34" s="71">
         <f t="shared" si="0"/>
-        <v>-97365</v>
+        <v>-36765</v>
       </c>
       <c r="N34" s="165">
         <f t="shared" si="0"/>
-        <v>-0.97365000000000002</v>
+        <v>-0.36764999999999998</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -21027,11 +21215,11 @@
       </c>
       <c r="F35" s="155"/>
       <c r="G35" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H35" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I35" s="152">
@@ -21079,12 +21267,12 @@
         <v>0.5</v>
       </c>
       <c r="G36" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-24327</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-42052</v>
       </c>
       <c r="H36" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.48653999999999997</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.84104000000000001</v>
       </c>
       <c r="I36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21104,11 +21292,11 @@
       </c>
       <c r="M36" s="71">
         <f t="shared" si="0"/>
-        <v>-24327</v>
+        <v>-42052</v>
       </c>
       <c r="N36" s="165">
         <f t="shared" si="0"/>
-        <v>-0.48653999999999997</v>
+        <v>-0.84104000000000001</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -21131,12 +21319,12 @@
         <v>1</v>
       </c>
       <c r="G37" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>728571</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>422121</v>
       </c>
       <c r="H37" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>2.4285700000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.40707</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21156,11 +21344,11 @@
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>728571</v>
+        <v>422121</v>
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>2.4285700000000001</v>
+        <v>1.40707</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -21181,12 +21369,12 @@
         <v>0.1</v>
       </c>
       <c r="G38" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-72992</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-191569</v>
       </c>
       <c r="H38" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-7.2991999999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-19.1569</v>
       </c>
       <c r="I38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21206,11 +21394,11 @@
       </c>
       <c r="M38" s="71">
         <f t="shared" si="0"/>
-        <v>-72992</v>
+        <v>-191569</v>
       </c>
       <c r="N38" s="165">
         <f t="shared" si="0"/>
-        <v>-7.2991999999999999</v>
+        <v>-19.1569</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -21233,12 +21421,12 @@
         <v>1</v>
       </c>
       <c r="G39" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>80741</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>75358</v>
       </c>
       <c r="H39" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>1.6148199999999999</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.5071600000000001</v>
       </c>
       <c r="I39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21258,11 +21446,11 @@
       </c>
       <c r="M39" s="71">
         <f t="shared" si="0"/>
-        <v>80741</v>
+        <v>75358</v>
       </c>
       <c r="N39" s="165">
         <f t="shared" si="0"/>
-        <v>1.6148199999999999</v>
+        <v>1.5071600000000001</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -21285,12 +21473,12 @@
         <v>1</v>
       </c>
       <c r="G40" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-963743</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-747613</v>
       </c>
       <c r="H40" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-9.6374300000000002</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-7.4761300000000004</v>
       </c>
       <c r="I40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21310,11 +21498,11 @@
       </c>
       <c r="M40" s="71">
         <f t="shared" si="0"/>
-        <v>-963743</v>
+        <v>-747613</v>
       </c>
       <c r="N40" s="165">
         <f t="shared" si="0"/>
-        <v>-9.6374300000000002</v>
+        <v>-7.4761300000000004</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -21337,12 +21525,12 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>495990</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>547590</v>
       </c>
       <c r="H41" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>9.9198000000000004</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>10.9518</v>
       </c>
       <c r="I41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21362,11 +21550,11 @@
       </c>
       <c r="M41" s="71">
         <f t="shared" ref="M41" si="5">G41+I41+K41</f>
-        <v>495990</v>
+        <v>547590</v>
       </c>
       <c r="N41" s="165">
         <f t="shared" ref="N41" si="6">H41+J41+L41</f>
-        <v>9.9198000000000004</v>
+        <v>10.9518</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -21387,12 +21575,12 @@
         <v>0.1</v>
       </c>
       <c r="G42" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-33213</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-30785</v>
       </c>
       <c r="H42" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-0.66425999999999996</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-0.61570000000000003</v>
       </c>
       <c r="I42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21412,11 +21600,11 @@
       </c>
       <c r="M42" s="71">
         <f t="shared" si="0"/>
-        <v>-33213</v>
+        <v>-30785</v>
       </c>
       <c r="N42" s="165">
         <f t="shared" si="0"/>
-        <v>-0.66425999999999996</v>
+        <v>-0.61570000000000003</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -21439,11 +21627,11 @@
         <v>1</v>
       </c>
       <c r="G43" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>1105039</v>
       </c>
       <c r="H43" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>3.6834633333333326</v>
       </c>
       <c r="I43" s="152">
@@ -21485,11 +21673,11 @@
         <v>1</v>
       </c>
       <c r="G44" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H44" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I44" s="152">
@@ -21537,12 +21725,12 @@
         <v>4</v>
       </c>
       <c r="G45" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>80210</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>85710</v>
       </c>
       <c r="H45" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.20052500000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.21427499999999999</v>
       </c>
       <c r="I45" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21562,11 +21750,11 @@
       </c>
       <c r="M45" s="71">
         <f t="shared" si="0"/>
-        <v>80210</v>
+        <v>85710</v>
       </c>
       <c r="N45" s="165">
         <f t="shared" si="0"/>
-        <v>0.20052500000000001</v>
+        <v>0.21427499999999999</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -21589,12 +21777,12 @@
         <v>4</v>
       </c>
       <c r="G46" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>8361</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>204861</v>
       </c>
       <c r="H46" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>2.0902500000000001E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.51215250000000001</v>
       </c>
       <c r="I46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21614,11 +21802,11 @@
       </c>
       <c r="M46" s="71">
         <f t="shared" si="0"/>
-        <v>8361</v>
+        <v>204861</v>
       </c>
       <c r="N46" s="165">
         <f t="shared" si="0"/>
-        <v>2.0902500000000001E-2</v>
+        <v>0.51215250000000001</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -21639,12 +21827,12 @@
         <v>0.1</v>
       </c>
       <c r="G47" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-3132740</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-2957840</v>
       </c>
       <c r="H47" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-3.1327400000000001</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-2.95784</v>
       </c>
       <c r="I47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21664,11 +21852,11 @@
       </c>
       <c r="M47" s="71">
         <f t="shared" si="0"/>
-        <v>-3132740</v>
+        <v>-2957840</v>
       </c>
       <c r="N47" s="165">
         <f t="shared" si="0"/>
-        <v>-3.1327400000000001</v>
+        <v>-2.95784</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -21685,11 +21873,11 @@
       </c>
       <c r="F48" s="114"/>
       <c r="G48" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I48" s="152">
@@ -21737,11 +21925,11 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>61459</v>
       </c>
       <c r="H49" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>1.2291799999999999</v>
       </c>
       <c r="I49" s="152">
@@ -21789,11 +21977,11 @@
         <v>5</v>
       </c>
       <c r="G50" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>369643</v>
       </c>
       <c r="H50" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0.56868153846153835</v>
       </c>
       <c r="I50" s="152">
@@ -21841,11 +22029,11 @@
         <v>1</v>
       </c>
       <c r="G51" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I51" s="152">
@@ -21893,11 +22081,11 @@
         <v>2.5</v>
       </c>
       <c r="G52" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>311687</v>
       </c>
       <c r="H52" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>1.0389566666666668</v>
       </c>
       <c r="I52" s="152">
@@ -21945,12 +22133,12 @@
         <v>0.25</v>
       </c>
       <c r="G53" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>30634</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>51734</v>
       </c>
       <c r="H53" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.30634</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>0.51734000000000002</v>
       </c>
       <c r="I53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -21970,11 +22158,11 @@
       </c>
       <c r="M53" s="71">
         <f t="shared" ref="M53:N54" si="7">G53+I53+K53</f>
-        <v>30634</v>
+        <v>51734</v>
       </c>
       <c r="N53" s="165">
         <f t="shared" si="7"/>
-        <v>0.30634</v>
+        <v>0.51734000000000002</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -21997,12 +22185,12 @@
         <v>5</v>
       </c>
       <c r="G54" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>881323</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1067523</v>
       </c>
       <c r="H54" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>0.88132299999999997</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.067523</v>
       </c>
       <c r="I54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -22022,11 +22210,11 @@
       </c>
       <c r="M54" s="71">
         <f t="shared" si="7"/>
-        <v>881323</v>
+        <v>1067523</v>
       </c>
       <c r="N54" s="165">
         <f t="shared" si="7"/>
-        <v>0.88132299999999997</v>
+        <v>1.067523</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -22038,7 +22226,7 @@
       <c r="F55" s="233"/>
       <c r="G55" s="230">
         <f>SUM(G4:G54)</f>
-        <v>6781439</v>
+        <v>6995756</v>
       </c>
       <c r="H55" s="90"/>
       <c r="I55" s="230">
@@ -22053,7 +22241,7 @@
       <c r="L55" s="109"/>
       <c r="M55" s="230">
         <f>SUM(M4:M54)</f>
-        <v>6781439</v>
+        <v>6995756</v>
       </c>
       <c r="N55" s="234"/>
     </row>
@@ -22117,12 +22305,12 @@
       <c r="E59" s="208"/>
       <c r="F59" s="206"/>
       <c r="G59" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>28620</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>537920</v>
       </c>
       <c r="H59" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>9.5399999999999999E-2</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>1.7930666666666664</v>
       </c>
       <c r="I59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -22142,11 +22330,11 @@
       </c>
       <c r="M59" s="152">
         <f t="shared" ref="M59:N60" si="8">G59+I59+K59</f>
-        <v>28620</v>
+        <v>537920</v>
       </c>
       <c r="N59" s="166">
         <f t="shared" si="8"/>
-        <v>9.5399999999999999E-2</v>
+        <v>1.7930666666666664</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -22167,11 +22355,11 @@
       </c>
       <c r="F60" s="237"/>
       <c r="G60" s="152">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
-        <v>-213294</v>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
+        <v>-25994</v>
       </c>
       <c r="H60" s="154">
-        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADH$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DI$2,0),0),0)</f>
+        <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADI$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DJ$2,0),0),0)</f>
         <v>0</v>
       </c>
       <c r="I60" s="152">
@@ -22192,7 +22380,7 @@
       </c>
       <c r="M60" s="152">
         <f t="shared" si="8"/>
-        <v>-213294</v>
+        <v>-25994</v>
       </c>
       <c r="N60" s="166">
         <f t="shared" si="8"/>
@@ -22202,7 +22390,7 @@
     <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G61" s="93">
         <f>SUM(G59:G60)</f>
-        <v>-184674</v>
+        <v>511926</v>
       </c>
       <c r="H61" s="94"/>
       <c r="I61" s="93">
@@ -22217,7 +22405,7 @@
       <c r="L61" s="113"/>
       <c r="M61" s="93">
         <f>SUM(M59:M60)</f>
-        <v>-184674</v>
+        <v>511926</v>
       </c>
       <c r="N61" s="235"/>
     </row>

</xml_diff>

<commit_message>
Update Q1 FY2026-27 dashboard from Excel [Fri 10/30/2026]
</commit_message>
<xml_diff>
--- a/Quant Strategy(2026-27).xlsx
+++ b/Quant Strategy(2026-27).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21480" windowHeight="6690"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21480" windowHeight="6690" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="NOV-2026" sheetId="46" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3531" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3532" uniqueCount="346">
   <si>
     <t>Sudeep</t>
   </si>
@@ -2407,21 +2407,7 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="548">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="546">
     <dxf>
       <fill>
         <patternFill>
@@ -15185,7 +15171,7 @@
       <c r="R10" s="158"/>
       <c r="S10" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>385080</v>
+        <v>564375</v>
       </c>
       <c r="T10" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15196,7 +15182,7 @@
       <c r="W10" s="149"/>
       <c r="Y10" s="153">
         <f t="shared" ref="Y10:Y11" si="8">M10+P10+S10+V10</f>
-        <v>385080</v>
+        <v>564375</v>
       </c>
       <c r="Z10" s="167">
         <f t="shared" ref="Z10:Z11" si="9">(N10+Q10+T10+W10)</f>
@@ -15248,7 +15234,7 @@
       <c r="R11" s="158"/>
       <c r="S11" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>233472</v>
+        <v>282853</v>
       </c>
       <c r="T11" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15259,7 +15245,7 @@
       <c r="W11" s="149"/>
       <c r="Y11" s="153">
         <f t="shared" si="8"/>
-        <v>233472</v>
+        <v>282853</v>
       </c>
       <c r="Z11" s="167">
         <f t="shared" si="9"/>
@@ -15329,7 +15315,7 @@
       <c r="R12" s="158"/>
       <c r="S12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-92015</v>
+        <v>-140705</v>
       </c>
       <c r="T12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15340,7 +15326,7 @@
       <c r="W12" s="72"/>
       <c r="Y12" s="153">
         <f t="shared" si="4"/>
-        <v>-1268082</v>
+        <v>-1316772</v>
       </c>
       <c r="Z12" s="167">
         <f t="shared" si="5"/>
@@ -15410,7 +15396,7 @@
       <c r="R13" s="158"/>
       <c r="S13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>376935</v>
+        <v>416810</v>
       </c>
       <c r="T13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15421,7 +15407,7 @@
       <c r="W13" s="149"/>
       <c r="Y13" s="153">
         <f t="shared" si="4"/>
-        <v>-24940</v>
+        <v>14935</v>
       </c>
       <c r="Z13" s="167">
         <f t="shared" si="5"/>
@@ -15491,7 +15477,7 @@
       <c r="R14" s="158"/>
       <c r="S14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>154827</v>
+        <v>66341</v>
       </c>
       <c r="T14" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -15502,7 +15488,7 @@
       <c r="W14" s="149"/>
       <c r="Y14" s="153">
         <f t="shared" si="4"/>
-        <v>64898</v>
+        <v>-23588</v>
       </c>
       <c r="Z14" s="167">
         <f t="shared" si="5"/>
@@ -16062,7 +16048,7 @@
       <c r="R21" s="158"/>
       <c r="S21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-11570</v>
+        <v>-14872</v>
       </c>
       <c r="T21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16073,7 +16059,7 @@
       <c r="W21" s="149"/>
       <c r="Y21" s="153">
         <f t="shared" si="4"/>
-        <v>-8995</v>
+        <v>-12297</v>
       </c>
       <c r="Z21" s="167">
         <f t="shared" si="5"/>
@@ -16233,7 +16219,7 @@
       <c r="R23" s="158"/>
       <c r="S23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>65921</v>
+        <v>82977</v>
       </c>
       <c r="T23" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16244,7 +16230,7 @@
       <c r="W23" s="72"/>
       <c r="Y23" s="153">
         <f t="shared" si="4"/>
-        <v>-185261</v>
+        <v>-168205</v>
       </c>
       <c r="Z23" s="167">
         <f t="shared" si="5"/>
@@ -16314,7 +16300,7 @@
       <c r="R24" s="158"/>
       <c r="S24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>94772</v>
+        <v>120524</v>
       </c>
       <c r="T24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16325,7 +16311,7 @@
       <c r="W24" s="72"/>
       <c r="Y24" s="153">
         <f t="shared" si="4"/>
-        <v>-108851</v>
+        <v>-83099</v>
       </c>
       <c r="Z24" s="167">
         <f t="shared" si="5"/>
@@ -16476,7 +16462,7 @@
       <c r="R26" s="158"/>
       <c r="S26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-1980</v>
+        <v>-12790</v>
       </c>
       <c r="T26" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16487,7 +16473,7 @@
       <c r="W26" s="72"/>
       <c r="Y26" s="153">
         <f t="shared" si="4"/>
-        <v>1744201</v>
+        <v>1733391</v>
       </c>
       <c r="Z26" s="167">
         <f t="shared" si="5"/>
@@ -16798,7 +16784,7 @@
       <c r="R30" s="158"/>
       <c r="S30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>678723</v>
+        <v>730873</v>
       </c>
       <c r="T30" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16809,7 +16795,7 @@
       <c r="W30" s="72"/>
       <c r="Y30" s="153">
         <f t="shared" si="4"/>
-        <v>1056991</v>
+        <v>1109141</v>
       </c>
       <c r="Z30" s="167">
         <f t="shared" si="5"/>
@@ -16879,7 +16865,7 @@
       <c r="R31" s="158"/>
       <c r="S31" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>376524</v>
+        <v>493824</v>
       </c>
       <c r="T31" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -16891,7 +16877,7 @@
       <c r="X31" s="1"/>
       <c r="Y31" s="153">
         <f t="shared" si="4"/>
-        <v>1255977</v>
+        <v>1373277</v>
       </c>
       <c r="Z31" s="167">
         <f t="shared" si="5"/>
@@ -17132,7 +17118,7 @@
       <c r="R34" s="158"/>
       <c r="S34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>731166</v>
+        <v>688166</v>
       </c>
       <c r="T34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17144,7 +17130,7 @@
       <c r="X34"/>
       <c r="Y34" s="153">
         <f t="shared" si="4"/>
-        <v>245161</v>
+        <v>202161</v>
       </c>
       <c r="Z34" s="167">
         <f t="shared" si="5"/>
@@ -17295,7 +17281,7 @@
       <c r="R36" s="158"/>
       <c r="S36" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>23714</v>
+        <v>-24031</v>
       </c>
       <c r="T36" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17306,7 +17292,7 @@
       <c r="W36" s="72"/>
       <c r="Y36" s="153">
         <f t="shared" si="4"/>
-        <v>-123913</v>
+        <v>-171658</v>
       </c>
       <c r="Z36" s="167">
         <f t="shared" si="5"/>
@@ -17464,7 +17450,7 @@
       <c r="R38" s="158"/>
       <c r="S38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-294779</v>
+        <v>-356631</v>
       </c>
       <c r="T38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17475,7 +17461,7 @@
       <c r="W38" s="72"/>
       <c r="Y38" s="153">
         <f t="shared" si="4"/>
-        <v>2607847</v>
+        <v>2545995</v>
       </c>
       <c r="Z38" s="167">
         <f t="shared" si="5"/>
@@ -17543,7 +17529,7 @@
       <c r="R39" s="158"/>
       <c r="S39" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>159162</v>
+        <v>138037</v>
       </c>
       <c r="T39" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17554,7 +17540,7 @@
       <c r="W39" s="149"/>
       <c r="Y39" s="153">
         <f t="shared" si="4"/>
-        <v>159162</v>
+        <v>138037</v>
       </c>
       <c r="Z39" s="167">
         <f t="shared" si="5"/>
@@ -17622,7 +17608,7 @@
       <c r="R40" s="158"/>
       <c r="S40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-95559</v>
+        <v>-91206</v>
       </c>
       <c r="T40" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17633,7 +17619,7 @@
       <c r="W40" s="149"/>
       <c r="Y40" s="153">
         <f t="shared" si="4"/>
-        <v>-139225</v>
+        <v>-134872</v>
       </c>
       <c r="Z40" s="167">
         <f t="shared" si="5"/>
@@ -17703,7 +17689,7 @@
       <c r="R41" s="158"/>
       <c r="S41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>1961800</v>
+        <v>2229800</v>
       </c>
       <c r="T41" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -17714,7 +17700,7 @@
       <c r="W41" s="72"/>
       <c r="Y41" s="153">
         <f t="shared" si="4"/>
-        <v>4502854</v>
+        <v>4770854</v>
       </c>
       <c r="Z41" s="167">
         <f t="shared" si="5"/>
@@ -18298,7 +18284,7 @@
       <c r="R48" s="158"/>
       <c r="S48" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-37539</v>
+        <v>-91075</v>
       </c>
       <c r="T48" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -18309,7 +18295,7 @@
       <c r="W48" s="149"/>
       <c r="Y48" s="153">
         <f t="shared" si="4"/>
-        <v>-37539</v>
+        <v>-91075</v>
       </c>
       <c r="Z48" s="167">
         <f t="shared" si="5"/>
@@ -18460,7 +18446,7 @@
       <c r="R50" s="158"/>
       <c r="S50" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>177902</v>
+        <v>31502</v>
       </c>
       <c r="T50" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -18472,7 +18458,7 @@
       <c r="X50" s="1"/>
       <c r="Y50" s="153">
         <f t="shared" si="4"/>
-        <v>950773</v>
+        <v>804373</v>
       </c>
       <c r="Z50" s="167">
         <f t="shared" si="5"/>
@@ -18712,7 +18698,7 @@
       <c r="R53" s="158"/>
       <c r="S53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>347883</v>
+        <v>341988</v>
       </c>
       <c r="T53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -18723,7 +18709,7 @@
       <c r="W53" s="72"/>
       <c r="Y53" s="153">
         <f t="shared" si="4"/>
-        <v>416148</v>
+        <v>410253</v>
       </c>
       <c r="Z53" s="167">
         <f t="shared" si="5"/>
@@ -18967,7 +18953,7 @@
       <c r="R56" s="158"/>
       <c r="S56" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>300365</v>
+        <v>209201</v>
       </c>
       <c r="T56" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -18978,7 +18964,7 @@
       <c r="W56" s="72"/>
       <c r="Y56" s="153">
         <f t="shared" si="4"/>
-        <v>495426</v>
+        <v>404262</v>
       </c>
       <c r="Z56" s="167">
         <f t="shared" si="5"/>
@@ -19048,7 +19034,7 @@
       <c r="R57" s="158"/>
       <c r="S57" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>23642</v>
+        <v>-41268</v>
       </c>
       <c r="T57" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19059,7 +19045,7 @@
       <c r="W57" s="72"/>
       <c r="Y57" s="153">
         <f t="shared" si="4"/>
-        <v>683891</v>
+        <v>618981</v>
       </c>
       <c r="Z57" s="167">
         <f t="shared" si="5"/>
@@ -19293,7 +19279,7 @@
       <c r="R60" s="158"/>
       <c r="S60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>467721</v>
+        <v>225121</v>
       </c>
       <c r="T60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19304,7 +19290,7 @@
       <c r="W60" s="72"/>
       <c r="Y60" s="153">
         <f t="shared" si="4"/>
-        <v>-4186614</v>
+        <v>-4429214</v>
       </c>
       <c r="Z60" s="167">
         <f t="shared" si="5"/>
@@ -19545,7 +19531,7 @@
       <c r="R63" s="158"/>
       <c r="S63" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-225524</v>
+        <v>-217860</v>
       </c>
       <c r="T63" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19556,7 +19542,7 @@
       <c r="W63" s="149"/>
       <c r="Y63" s="153">
         <f t="shared" si="4"/>
-        <v>-245645</v>
+        <v>-237981</v>
       </c>
       <c r="Z63" s="167">
         <f t="shared" si="5"/>
@@ -19715,7 +19701,7 @@
       <c r="R65" s="158"/>
       <c r="S65" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-373613</v>
+        <v>-568413</v>
       </c>
       <c r="T65" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19726,7 +19712,7 @@
       <c r="W65" s="72"/>
       <c r="Y65" s="153">
         <f t="shared" si="4"/>
-        <v>3306002</v>
+        <v>3111202</v>
       </c>
       <c r="Z65" s="167">
         <f t="shared" si="5"/>
@@ -19803,7 +19789,7 @@
       <c r="R66" s="158"/>
       <c r="S66" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>591786</v>
+        <v>544786</v>
       </c>
       <c r="T66" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19814,7 +19800,7 @@
       <c r="W66" s="149"/>
       <c r="Y66" s="153">
         <f t="shared" si="4"/>
-        <v>591786</v>
+        <v>544786</v>
       </c>
       <c r="Z66" s="167">
         <f t="shared" si="5"/>
@@ -19882,7 +19868,7 @@
       <c r="R67" s="158"/>
       <c r="S67" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-55185</v>
+        <v>-46085</v>
       </c>
       <c r="T67" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19893,7 +19879,7 @@
       <c r="W67" s="149"/>
       <c r="Y67" s="153">
         <f t="shared" si="4"/>
-        <v>-41894</v>
+        <v>-32794</v>
       </c>
       <c r="Z67" s="167">
         <f t="shared" si="5"/>
@@ -19963,7 +19949,7 @@
       <c r="R68" s="158"/>
       <c r="S68" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>1112739</v>
+        <v>1111205</v>
       </c>
       <c r="T68" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -19974,7 +19960,7 @@
       <c r="W68" s="72"/>
       <c r="Y68" s="153">
         <f t="shared" si="4"/>
-        <v>1955840</v>
+        <v>1954306</v>
       </c>
       <c r="Z68" s="167">
         <f t="shared" si="5"/>
@@ -20214,7 +20200,7 @@
       <c r="R71" s="158"/>
       <c r="S71" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>203653</v>
+        <v>199806</v>
       </c>
       <c r="T71" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -20226,7 +20212,7 @@
       <c r="X71" s="131"/>
       <c r="Y71" s="153">
         <f t="shared" ref="Y71:Y81" si="12">M71+P71+S71+V71</f>
-        <v>986434</v>
+        <v>982587</v>
       </c>
       <c r="Z71" s="167">
         <f t="shared" ref="Z71:Z81" si="13">(N71+Q71+T71+W71)</f>
@@ -20376,7 +20362,7 @@
       <c r="R73" s="158"/>
       <c r="S73" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>-2661565</v>
+        <v>-2531865</v>
       </c>
       <c r="T73" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -20387,7 +20373,7 @@
       <c r="W73" s="149"/>
       <c r="Y73" s="153">
         <f t="shared" si="12"/>
-        <v>-3624394</v>
+        <v>-3494694</v>
       </c>
       <c r="Z73" s="167">
         <f t="shared" si="13"/>
@@ -20935,7 +20921,7 @@
       <c r="R80" s="158"/>
       <c r="S80" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>88156</v>
+        <v>94004</v>
       </c>
       <c r="T80" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -20946,7 +20932,7 @@
       <c r="W80" s="149"/>
       <c r="Y80" s="153">
         <f t="shared" si="12"/>
-        <v>88156</v>
+        <v>94004</v>
       </c>
       <c r="Z80" s="167">
         <f t="shared" si="13"/>
@@ -21014,7 +21000,7 @@
       <c r="R81" s="158"/>
       <c r="S81" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$2,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
-        <v>1297423</v>
+        <v>1294523</v>
       </c>
       <c r="T81" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$144,'FY-(26-27)Q3'!$A$4:$ABW$117,MATCH('FY-(26-27)Q1'!$S$2:$T$3,'FY-(26-27)Q3'!$A$2:$BX$2,0),0),0)</f>
@@ -21025,7 +21011,7 @@
       <c r="W81" s="149"/>
       <c r="Y81" s="153">
         <f t="shared" si="12"/>
-        <v>1788276</v>
+        <v>1785376</v>
       </c>
       <c r="Z81" s="167">
         <f t="shared" si="13"/>
@@ -21068,7 +21054,7 @@
       <c r="R82" s="122"/>
       <c r="S82" s="153">
         <f>SUM(S4:S81)</f>
-        <v>8298952</v>
+        <v>8024830</v>
       </c>
       <c r="T82" s="122"/>
       <c r="U82" s="122"/>
@@ -21076,7 +21062,7 @@
       <c r="W82" s="50"/>
       <c r="Y82" s="153">
         <f>SUM(Y4:Y81)</f>
-        <v>31568482</v>
+        <v>31294360</v>
       </c>
       <c r="Z82" s="160"/>
     </row>
@@ -22798,7 +22784,9 @@
       <c r="Z2" s="255">
         <v>46324</v>
       </c>
-      <c r="AA2" s="182"/>
+      <c r="AA2" s="182">
+        <v>46325</v>
+      </c>
       <c r="AB2" s="183" t="s">
         <v>325</v>
       </c>
@@ -22883,7 +22871,9 @@
       <c r="Z3" s="178" t="s">
         <v>236</v>
       </c>
-      <c r="AA3" s="179"/>
+      <c r="AA3" s="179" t="s">
+        <v>235</v>
+      </c>
       <c r="AB3" s="188"/>
       <c r="AC3" s="179"/>
       <c r="AJ3" s="132" t="s">
@@ -22970,7 +22960,9 @@
       <c r="Z4" s="157">
         <v>0</v>
       </c>
-      <c r="AA4" s="210"/>
+      <c r="AA4" s="210">
+        <v>0</v>
+      </c>
       <c r="AB4" s="170">
         <f t="shared" ref="AB4" si="0">SUM(H4:AA4)</f>
         <v>97836</v>
@@ -23063,14 +23055,16 @@
       <c r="Z5" s="146">
         <v>52300</v>
       </c>
-      <c r="AA5" s="173"/>
+      <c r="AA5" s="173">
+        <v>179295</v>
+      </c>
       <c r="AB5" s="170">
         <f t="shared" ref="AB5:AB53" si="2">SUM(H5:AA5)</f>
-        <v>385080</v>
+        <v>564375</v>
       </c>
       <c r="AC5" s="148">
         <f t="shared" ref="AC5:AC53" si="3">IFERROR(AB5/F5*100,0)/10000000</f>
-        <v>1.2836000000000001</v>
+        <v>1.8812500000000001</v>
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
@@ -23150,14 +23144,16 @@
       <c r="Z6" s="146">
         <v>-5500</v>
       </c>
-      <c r="AA6" s="173"/>
+      <c r="AA6" s="173">
+        <v>49381</v>
+      </c>
       <c r="AB6" s="170">
         <f t="shared" si="2"/>
-        <v>233472</v>
+        <v>282853</v>
       </c>
       <c r="AC6" s="148">
         <f t="shared" si="3"/>
-        <v>2.3347199999999999</v>
+        <v>2.8285300000000002</v>
       </c>
     </row>
     <row r="7" spans="1:40" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -23237,18 +23233,20 @@
       <c r="Z7" s="146">
         <v>53145</v>
       </c>
-      <c r="AA7" s="173"/>
+      <c r="AA7" s="173">
+        <v>-48690</v>
+      </c>
       <c r="AB7" s="170">
         <f t="shared" si="2"/>
-        <v>-92015</v>
+        <v>-140705</v>
       </c>
       <c r="AC7" s="148">
         <f t="shared" si="3"/>
-        <v>-0.30671666666666669</v>
+        <v>-0.46901666666666658</v>
       </c>
       <c r="AE7" s="5"/>
       <c r="AF7" s="133">
-        <v>1056</v>
+        <v>-140487</v>
       </c>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.25">
@@ -23328,17 +23326,19 @@
       <c r="Z8" s="146">
         <v>155900</v>
       </c>
-      <c r="AA8" s="173"/>
+      <c r="AA8" s="173">
+        <v>39875</v>
+      </c>
       <c r="AB8" s="170">
         <f t="shared" si="2"/>
-        <v>376935</v>
+        <v>416810</v>
       </c>
       <c r="AC8" s="148">
         <f t="shared" si="3"/>
-        <v>2.5129000000000001</v>
+        <v>2.7787333333333333</v>
       </c>
       <c r="AE8" s="133">
-        <v>94669</v>
+        <v>2216136</v>
       </c>
       <c r="AF8" s="133"/>
     </row>
@@ -23417,21 +23417,23 @@
       <c r="Z9" s="146">
         <v>-12900</v>
       </c>
-      <c r="AA9" s="173"/>
+      <c r="AA9" s="173">
+        <v>-88486</v>
+      </c>
       <c r="AB9" s="170">
         <f t="shared" si="2"/>
-        <v>154827</v>
+        <v>66341</v>
       </c>
       <c r="AC9" s="148">
         <f t="shared" si="3"/>
-        <v>2.5804499999999999</v>
+        <v>1.1056833333333334</v>
       </c>
       <c r="AE9" s="133">
-        <v>95725</v>
+        <v>2075648</v>
       </c>
       <c r="AF9" s="133">
         <f>(AE9+AE8)/10000000*13780</f>
-        <v>262.362932</v>
+        <v>5914.0783520000005</v>
       </c>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
@@ -23511,7 +23513,9 @@
       <c r="Z10" s="146">
         <v>0</v>
       </c>
-      <c r="AA10" s="173"/>
+      <c r="AA10" s="173">
+        <v>0</v>
+      </c>
       <c r="AB10" s="170">
         <f t="shared" si="2"/>
         <v>-87379</v>
@@ -23600,7 +23604,9 @@
       <c r="Z11" s="146">
         <v>0</v>
       </c>
-      <c r="AA11" s="173"/>
+      <c r="AA11" s="173">
+        <v>0</v>
+      </c>
       <c r="AB11" s="170">
         <f t="shared" si="2"/>
         <v>269024</v>
@@ -23689,14 +23695,16 @@
       <c r="Z12" s="146">
         <v>-1290</v>
       </c>
-      <c r="AA12" s="173"/>
+      <c r="AA12" s="173">
+        <v>-3302</v>
+      </c>
       <c r="AB12" s="170">
         <f t="shared" si="2"/>
-        <v>-11570</v>
+        <v>-14872</v>
       </c>
       <c r="AC12" s="148">
         <f t="shared" si="3"/>
-        <v>-0.1157</v>
+        <v>-0.14871999999999999</v>
       </c>
       <c r="AE12" s="133"/>
       <c r="AF12" s="133"/>
@@ -23778,14 +23786,16 @@
       <c r="Z13" s="146">
         <v>-2000</v>
       </c>
-      <c r="AA13" s="173"/>
+      <c r="AA13" s="173">
+        <v>17056</v>
+      </c>
       <c r="AB13" s="170">
         <f t="shared" si="2"/>
-        <v>65921</v>
+        <v>82977</v>
       </c>
       <c r="AC13" s="148">
         <f t="shared" si="3"/>
-        <v>0.26368399999999997</v>
+        <v>0.33190800000000004</v>
       </c>
       <c r="AE13" s="133"/>
       <c r="AF13" s="133"/>
@@ -23867,26 +23877,28 @@
       <c r="Z14" s="146">
         <v>0</v>
       </c>
-      <c r="AA14" s="173"/>
+      <c r="AA14" s="173">
+        <v>25752</v>
+      </c>
       <c r="AB14" s="170">
         <f t="shared" si="2"/>
-        <v>94772</v>
+        <v>120524</v>
       </c>
       <c r="AC14" s="148">
         <f t="shared" si="3"/>
-        <v>0.43078181818181815</v>
+        <v>0.54783636363636357</v>
       </c>
       <c r="AE14" s="133"/>
       <c r="AF14" s="192">
         <f>AF7-AF9</f>
-        <v>793.637068</v>
+        <v>-146401.07835200001</v>
       </c>
       <c r="AI14" s="132">
         <v>43814</v>
       </c>
       <c r="AK14" s="132">
         <f>AI14+AF14</f>
-        <v>44607.637067999996</v>
+        <v>-102587.07835200001</v>
       </c>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.25">
@@ -23966,14 +23978,16 @@
       <c r="Z15" s="146">
         <v>12400</v>
       </c>
-      <c r="AA15" s="173"/>
+      <c r="AA15" s="173">
+        <v>-10810</v>
+      </c>
       <c r="AB15" s="170">
         <f t="shared" si="2"/>
-        <v>-1980</v>
+        <v>-12790</v>
       </c>
       <c r="AC15" s="148">
         <f t="shared" si="3"/>
-        <v>-1.9800000000000002E-2</v>
+        <v>-0.12790000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.25">
@@ -24053,14 +24067,16 @@
       <c r="Z16" s="146">
         <v>103100</v>
       </c>
-      <c r="AA16" s="173"/>
+      <c r="AA16" s="173">
+        <v>52150</v>
+      </c>
       <c r="AB16" s="170">
         <f t="shared" si="2"/>
-        <v>678723</v>
+        <v>730873</v>
       </c>
       <c r="AC16" s="148">
         <f t="shared" si="3"/>
-        <v>2.7148919999999999</v>
+        <v>2.923492</v>
       </c>
       <c r="AK16" s="132">
         <v>4000000</v>
@@ -24151,14 +24167,16 @@
       <c r="Z17" s="146">
         <v>71600</v>
       </c>
-      <c r="AA17" s="173"/>
+      <c r="AA17" s="173">
+        <v>117300</v>
+      </c>
       <c r="AB17" s="170">
         <f t="shared" si="2"/>
-        <v>376524</v>
+        <v>493824</v>
       </c>
       <c r="AC17" s="148">
         <f t="shared" si="3"/>
-        <v>0.94130999999999998</v>
+        <v>1.2345600000000001</v>
       </c>
       <c r="AL17" s="132">
         <f>AL16/12</f>
@@ -24242,14 +24260,16 @@
       <c r="Z18" s="146">
         <v>75330</v>
       </c>
-      <c r="AA18" s="173"/>
+      <c r="AA18" s="173">
+        <v>-43000</v>
+      </c>
       <c r="AB18" s="170">
         <f t="shared" si="2"/>
-        <v>731166</v>
+        <v>688166</v>
       </c>
       <c r="AC18" s="148">
         <f t="shared" si="3"/>
-        <v>4.8744399999999999</v>
+        <v>4.5877733333333328</v>
       </c>
     </row>
     <row r="19" spans="1:38" x14ac:dyDescent="0.25">
@@ -24329,7 +24349,9 @@
       <c r="Z19" s="146">
         <v>0</v>
       </c>
-      <c r="AA19" s="173"/>
+      <c r="AA19" s="173">
+        <v>0</v>
+      </c>
       <c r="AB19" s="170">
         <f t="shared" si="2"/>
         <v>-150688</v>
@@ -24419,7 +24441,9 @@
       <c r="Z20" s="146">
         <v>0</v>
       </c>
-      <c r="AA20" s="173"/>
+      <c r="AA20" s="173">
+        <v>0</v>
+      </c>
       <c r="AB20" s="170">
         <f t="shared" si="2"/>
         <v>-110832</v>
@@ -24509,7 +24533,9 @@
       <c r="Z21" s="146">
         <v>0</v>
       </c>
-      <c r="AA21" s="173"/>
+      <c r="AA21" s="173">
+        <v>0</v>
+      </c>
       <c r="AB21" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -24599,7 +24625,9 @@
       <c r="Z22" s="146">
         <v>0</v>
       </c>
-      <c r="AA22" s="173"/>
+      <c r="AA22" s="173">
+        <v>0</v>
+      </c>
       <c r="AB22" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -24690,14 +24718,16 @@
       <c r="Z23" s="146">
         <v>10320</v>
       </c>
-      <c r="AA23" s="173"/>
+      <c r="AA23" s="173">
+        <v>-47745</v>
+      </c>
       <c r="AB23" s="170">
         <f t="shared" si="2"/>
-        <v>23714</v>
+        <v>-24031</v>
       </c>
       <c r="AC23" s="148">
         <f t="shared" si="3"/>
-        <v>0.21558181818181815</v>
+        <v>-0.21846363636363639</v>
       </c>
     </row>
     <row r="24" spans="1:38" x14ac:dyDescent="0.25">
@@ -24777,14 +24807,16 @@
       <c r="Z24" s="146">
         <v>253900</v>
       </c>
-      <c r="AA24" s="173"/>
+      <c r="AA24" s="173">
+        <v>-61852</v>
+      </c>
       <c r="AB24" s="170">
         <f t="shared" si="2"/>
-        <v>-294779</v>
+        <v>-356631</v>
       </c>
       <c r="AC24" s="148">
         <f t="shared" si="3"/>
-        <v>-1.2816478260869566</v>
+        <v>-1.5505695652173914</v>
       </c>
     </row>
     <row r="25" spans="1:38" x14ac:dyDescent="0.25">
@@ -24850,14 +24882,16 @@
       <c r="Z25" s="146">
         <v>-7955</v>
       </c>
-      <c r="AA25" s="173"/>
+      <c r="AA25" s="173">
+        <v>-21125</v>
+      </c>
       <c r="AB25" s="170">
         <f t="shared" si="2"/>
-        <v>159162</v>
+        <v>138037</v>
       </c>
       <c r="AC25" s="148">
         <f t="shared" si="3"/>
-        <v>7.9581</v>
+        <v>6.9018499999999996</v>
       </c>
     </row>
     <row r="26" spans="1:38" x14ac:dyDescent="0.25">
@@ -24935,14 +24969,16 @@
       <c r="Z26" s="146">
         <v>12900</v>
       </c>
-      <c r="AA26" s="173"/>
+      <c r="AA26" s="173">
+        <v>4353</v>
+      </c>
       <c r="AB26" s="170">
         <f t="shared" si="2"/>
-        <v>-95559</v>
+        <v>-91206</v>
       </c>
       <c r="AC26" s="148">
         <f t="shared" si="3"/>
-        <v>-1.9111800000000001</v>
+        <v>-1.82412</v>
       </c>
     </row>
     <row r="27" spans="1:38" x14ac:dyDescent="0.25">
@@ -25022,14 +25058,16 @@
       <c r="Z27" s="146">
         <v>478000</v>
       </c>
-      <c r="AA27" s="173"/>
+      <c r="AA27" s="173">
+        <v>268000</v>
+      </c>
       <c r="AB27" s="170">
         <f t="shared" si="2"/>
-        <v>1961800</v>
+        <v>2229800</v>
       </c>
       <c r="AC27" s="148">
         <f t="shared" si="3"/>
-        <v>3.9236</v>
+        <v>4.4596</v>
       </c>
     </row>
     <row r="28" spans="1:38" x14ac:dyDescent="0.25">
@@ -25109,7 +25147,9 @@
       <c r="Z28" s="146">
         <v>80700</v>
       </c>
-      <c r="AA28" s="173"/>
+      <c r="AA28" s="173">
+        <v>0</v>
+      </c>
       <c r="AB28" s="170">
         <f t="shared" si="2"/>
         <v>288559</v>
@@ -25192,14 +25232,16 @@
       <c r="Z29" s="146">
         <v>9050</v>
       </c>
-      <c r="AA29" s="173"/>
+      <c r="AA29" s="173">
+        <v>-53536</v>
+      </c>
       <c r="AB29" s="170">
         <f t="shared" si="2"/>
-        <v>-37539</v>
+        <v>-91075</v>
       </c>
       <c r="AC29" s="148">
         <f t="shared" si="3"/>
-        <v>-0.75078</v>
+        <v>-1.8214999999999999</v>
       </c>
     </row>
     <row r="30" spans="1:38" x14ac:dyDescent="0.25">
@@ -25279,7 +25321,9 @@
       <c r="Z30" s="146">
         <v>10953</v>
       </c>
-      <c r="AA30" s="173"/>
+      <c r="AA30" s="173">
+        <v>0</v>
+      </c>
       <c r="AB30" s="170">
         <f t="shared" si="2"/>
         <v>852127</v>
@@ -25366,14 +25410,16 @@
       <c r="Z31" s="146">
         <v>37769</v>
       </c>
-      <c r="AA31" s="173"/>
+      <c r="AA31" s="173">
+        <v>-146400</v>
+      </c>
       <c r="AB31" s="170">
         <f t="shared" si="2"/>
-        <v>177902</v>
+        <v>31502</v>
       </c>
       <c r="AC31" s="148">
         <f t="shared" si="3"/>
-        <v>0.35580400000000001</v>
+        <v>6.3004000000000004E-2</v>
       </c>
     </row>
     <row r="32" spans="1:38" x14ac:dyDescent="0.25">
@@ -25453,7 +25499,9 @@
       <c r="Z32" s="146">
         <v>800</v>
       </c>
-      <c r="AA32" s="173"/>
+      <c r="AA32" s="173">
+        <v>0</v>
+      </c>
       <c r="AB32" s="170">
         <f t="shared" si="2"/>
         <v>43966</v>
@@ -25540,14 +25588,16 @@
       <c r="Z33" s="146">
         <v>0</v>
       </c>
-      <c r="AA33" s="173"/>
+      <c r="AA33" s="173">
+        <v>-5895</v>
+      </c>
       <c r="AB33" s="170">
         <f t="shared" si="2"/>
-        <v>347883</v>
+        <v>341988</v>
       </c>
       <c r="AC33" s="148">
         <f t="shared" si="3"/>
-        <v>8.6970749999999999</v>
+        <v>8.5496999999999996</v>
       </c>
       <c r="AF33" s="133"/>
     </row>
@@ -25628,14 +25678,16 @@
       <c r="Z34" s="146">
         <v>91560</v>
       </c>
-      <c r="AA34" s="173"/>
+      <c r="AA34" s="173">
+        <v>-91164</v>
+      </c>
       <c r="AB34" s="170">
         <f t="shared" si="2"/>
-        <v>300365</v>
+        <v>209201</v>
       </c>
       <c r="AC34" s="148">
         <f t="shared" si="3"/>
-        <v>0.75091249999999998</v>
+        <v>0.52300250000000004</v>
       </c>
       <c r="AE34" s="5"/>
       <c r="AF34" s="133">
@@ -25719,14 +25771,16 @@
       <c r="Z35" s="146">
         <v>52587</v>
       </c>
-      <c r="AA35" s="173"/>
+      <c r="AA35" s="173">
+        <v>-64910</v>
+      </c>
       <c r="AB35" s="170">
         <f t="shared" si="2"/>
-        <v>23642</v>
+        <v>-41268</v>
       </c>
       <c r="AC35" s="148">
         <f t="shared" si="3"/>
-        <v>0.23641999999999999</v>
+        <v>-0.41267999999999999</v>
       </c>
       <c r="AE35" s="5"/>
       <c r="AF35" s="133"/>
@@ -25806,7 +25860,9 @@
       <c r="Z36" s="146">
         <v>0</v>
       </c>
-      <c r="AA36" s="173"/>
+      <c r="AA36" s="173">
+        <v>0</v>
+      </c>
       <c r="AB36" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -25900,7 +25956,9 @@
       <c r="Z37" s="146">
         <v>0</v>
       </c>
-      <c r="AA37" s="173"/>
+      <c r="AA37" s="173">
+        <v>0</v>
+      </c>
       <c r="AB37" s="170">
         <f t="shared" si="2"/>
         <v>-51900</v>
@@ -25991,14 +26049,16 @@
       <c r="Z38" s="146">
         <v>-10800</v>
       </c>
-      <c r="AA38" s="173"/>
+      <c r="AA38" s="173">
+        <v>-242600</v>
+      </c>
       <c r="AB38" s="170">
         <f t="shared" si="2"/>
-        <v>467721</v>
+        <v>225121</v>
       </c>
       <c r="AC38" s="148">
         <f t="shared" si="3"/>
-        <v>1.55907</v>
+        <v>0.75040333333333331</v>
       </c>
       <c r="AE38" s="133"/>
       <c r="AF38" s="133">
@@ -26081,14 +26141,16 @@
       <c r="Z39" s="146">
         <v>42700</v>
       </c>
-      <c r="AA39" s="173"/>
+      <c r="AA39" s="173">
+        <v>7664</v>
+      </c>
       <c r="AB39" s="170">
         <f t="shared" si="2"/>
-        <v>-225524</v>
+        <v>-217860</v>
       </c>
       <c r="AC39" s="148">
         <f t="shared" si="3"/>
-        <v>-22.552399999999999</v>
+        <v>-21.786000000000001</v>
       </c>
       <c r="AE39" s="133"/>
       <c r="AF39" s="133"/>
@@ -26170,7 +26232,9 @@
       <c r="Z40" s="146">
         <v>0</v>
       </c>
-      <c r="AA40" s="173"/>
+      <c r="AA40" s="173">
+        <v>0</v>
+      </c>
       <c r="AB40" s="170">
         <f t="shared" si="2"/>
         <v>63458</v>
@@ -26259,14 +26323,16 @@
       <c r="Z41" s="146">
         <v>175600</v>
       </c>
-      <c r="AA41" s="173"/>
+      <c r="AA41" s="173">
+        <v>-194800</v>
+      </c>
       <c r="AB41" s="170">
         <f t="shared" si="2"/>
-        <v>-373613</v>
+        <v>-568413</v>
       </c>
       <c r="AC41" s="148">
         <f t="shared" si="3"/>
-        <v>-3.7361300000000002</v>
+        <v>-5.6841299999999997</v>
       </c>
       <c r="AE41" s="133"/>
       <c r="AF41" s="133"/>
@@ -26334,14 +26400,16 @@
       <c r="Z42" s="146">
         <v>96000</v>
       </c>
-      <c r="AA42" s="173"/>
+      <c r="AA42" s="173">
+        <v>-47000</v>
+      </c>
       <c r="AB42" s="170">
         <f t="shared" si="2"/>
-        <v>591786</v>
+        <v>544786</v>
       </c>
       <c r="AC42" s="148">
         <f t="shared" si="3"/>
-        <v>11.83572</v>
+        <v>10.895720000000001</v>
       </c>
       <c r="AE42" s="133"/>
       <c r="AF42" s="133"/>
@@ -26421,14 +26489,16 @@
       <c r="Z43" s="146">
         <v>18300</v>
       </c>
-      <c r="AA43" s="173"/>
+      <c r="AA43" s="173">
+        <v>9100</v>
+      </c>
       <c r="AB43" s="170">
         <f t="shared" si="2"/>
-        <v>-55185</v>
+        <v>-46085</v>
       </c>
       <c r="AC43" s="148">
         <f t="shared" si="3"/>
-        <v>-1.1036999999999999</v>
+        <v>-0.92169999999999996</v>
       </c>
       <c r="AE43" s="133"/>
     </row>
@@ -26509,7 +26579,9 @@
       <c r="Z44" s="146">
         <v>23600</v>
       </c>
-      <c r="AA44" s="173"/>
+      <c r="AA44" s="173">
+        <v>0</v>
+      </c>
       <c r="AB44" s="170">
         <f t="shared" si="2"/>
         <v>139410</v>
@@ -26596,14 +26668,16 @@
       <c r="Z45" s="146">
         <v>-2050</v>
       </c>
-      <c r="AA45" s="173"/>
+      <c r="AA45" s="173">
+        <v>-3847</v>
+      </c>
       <c r="AB45" s="170">
         <f t="shared" si="2"/>
-        <v>203653</v>
+        <v>199806</v>
       </c>
       <c r="AC45" s="148">
         <f t="shared" si="3"/>
-        <v>0.50913249999999999</v>
+        <v>0.49951499999999999</v>
       </c>
     </row>
     <row r="46" spans="1:32" x14ac:dyDescent="0.25">
@@ -26683,14 +26757,16 @@
       <c r="Z46" s="146">
         <v>0</v>
       </c>
-      <c r="AA46" s="173"/>
+      <c r="AA46" s="173">
+        <v>-1534</v>
+      </c>
       <c r="AB46" s="170">
         <f t="shared" si="2"/>
-        <v>1112739</v>
+        <v>1111205</v>
       </c>
       <c r="AC46" s="148">
         <f t="shared" si="3"/>
-        <v>3.70913</v>
+        <v>3.704016666666667</v>
       </c>
     </row>
     <row r="47" spans="1:32" x14ac:dyDescent="0.25">
@@ -26768,14 +26844,16 @@
       <c r="Z47" s="150">
         <v>224175</v>
       </c>
-      <c r="AA47" s="173"/>
+      <c r="AA47" s="173">
+        <v>129700</v>
+      </c>
       <c r="AB47" s="170">
         <f t="shared" si="2"/>
-        <v>-2661565</v>
+        <v>-2531865</v>
       </c>
       <c r="AC47" s="148">
         <f t="shared" si="3"/>
-        <v>-2.661565</v>
+        <v>-2.5318649999999998</v>
       </c>
     </row>
     <row r="48" spans="1:32" x14ac:dyDescent="0.25">
@@ -26855,7 +26933,9 @@
       <c r="Z48" s="150">
         <v>0</v>
       </c>
-      <c r="AA48" s="173"/>
+      <c r="AA48" s="173">
+        <v>0</v>
+      </c>
       <c r="AB48" s="170">
         <f t="shared" si="2"/>
         <v>58584</v>
@@ -26942,7 +27022,9 @@
       <c r="Z49" s="150">
         <v>0</v>
       </c>
-      <c r="AA49" s="173"/>
+      <c r="AA49" s="173">
+        <v>0</v>
+      </c>
       <c r="AB49" s="170">
         <f t="shared" si="2"/>
         <v>369643</v>
@@ -27029,7 +27111,9 @@
       <c r="Z50" s="150">
         <v>0</v>
       </c>
-      <c r="AA50" s="173"/>
+      <c r="AA50" s="173">
+        <v>0</v>
+      </c>
       <c r="AB50" s="170">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -27116,7 +27200,9 @@
       <c r="Z51" s="150">
         <v>90588</v>
       </c>
-      <c r="AA51" s="173"/>
+      <c r="AA51" s="173">
+        <v>0</v>
+      </c>
       <c r="AB51" s="170">
         <f t="shared" si="2"/>
         <v>402275</v>
@@ -27203,14 +27289,16 @@
       <c r="Z52" s="150">
         <v>32675</v>
       </c>
-      <c r="AA52" s="173"/>
+      <c r="AA52" s="173">
+        <v>5848</v>
+      </c>
       <c r="AB52" s="170">
         <f t="shared" si="2"/>
-        <v>88156</v>
+        <v>94004</v>
       </c>
       <c r="AC52" s="148">
         <f t="shared" si="3"/>
-        <v>0.88156000000000001</v>
+        <v>0.94003999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -27290,14 +27378,16 @@
       <c r="Z53" s="150">
         <v>170000</v>
       </c>
-      <c r="AA53" s="173"/>
+      <c r="AA53" s="173">
+        <v>-2900</v>
+      </c>
       <c r="AB53" s="170">
         <f t="shared" si="2"/>
-        <v>1297423</v>
+        <v>1294523</v>
       </c>
       <c r="AC53" s="148">
         <f t="shared" si="3"/>
-        <v>1.297423</v>
+        <v>1.2945230000000001</v>
       </c>
     </row>
     <row r="54" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -27386,11 +27476,11 @@
       </c>
       <c r="AA54" s="253">
         <f>SUM(AA4:AA53)</f>
-        <v>0</v>
+        <v>-274122</v>
       </c>
       <c r="AB54" s="253">
         <f>SUM(H54:AA54)</f>
-        <v>8188120</v>
+        <v>7913998</v>
       </c>
       <c r="AC54" s="254">
         <f t="shared" ref="AC54" si="5">IFERROR(AB54/F54*100,0)/10000000</f>
@@ -27505,14 +27595,16 @@
       <c r="Z56" s="161">
         <v>-18346</v>
       </c>
-      <c r="AA56" s="245"/>
+      <c r="AA56" s="245">
+        <v>1255</v>
+      </c>
       <c r="AB56" s="246">
         <f>SUM(H56:AA56)</f>
-        <v>553584</v>
+        <v>554839</v>
       </c>
       <c r="AC56" s="247">
         <f>IFERROR(AB56/F56*100,0)/10000000</f>
-        <v>1.84528</v>
+        <v>1.8494633333333337</v>
       </c>
     </row>
     <row r="57" spans="1:33" x14ac:dyDescent="0.25">
@@ -27590,10 +27682,12 @@
       <c r="Z57" s="161">
         <v>0</v>
       </c>
-      <c r="AA57" s="173"/>
+      <c r="AA57" s="173">
+        <v>10100</v>
+      </c>
       <c r="AB57" s="170">
         <f>SUM(H57:AA57)</f>
-        <v>-25994</v>
+        <v>-15894</v>
       </c>
       <c r="AC57" s="148">
         <f>IFERROR(AB57/F57*100,0)/10000000</f>
@@ -27653,7 +27747,9 @@
       <c r="Z58" s="161">
         <v>0</v>
       </c>
-      <c r="AA58" s="161"/>
+      <c r="AA58" s="161">
+        <v>0</v>
+      </c>
       <c r="AB58" s="170">
         <f t="shared" ref="AB58:AB59" si="6">SUM(H58:AA58)</f>
         <v>0</v>
@@ -27715,7 +27811,9 @@
       <c r="Z59" s="161">
         <v>452800</v>
       </c>
-      <c r="AA59" s="161"/>
+      <c r="AA59" s="161">
+        <v>0</v>
+      </c>
       <c r="AB59" s="170">
         <f t="shared" si="6"/>
         <v>533178</v>
@@ -27807,12 +27905,12 @@
         <v>434454</v>
       </c>
       <c r="AA60" s="169">
-        <f>SUM(AA56:AA57)</f>
-        <v>0</v>
+        <f>SUM(AA56:AA59)</f>
+        <v>11355</v>
       </c>
       <c r="AB60" s="256">
         <f>SUM(H60:AA60)</f>
-        <v>1119548</v>
+        <v>1130903</v>
       </c>
       <c r="AC60" s="172"/>
     </row>
@@ -28040,11 +28138,11 @@
       </c>
       <c r="G5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>385080</v>
+        <v>564375</v>
       </c>
       <c r="H5" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1.2836000000000001</v>
+        <v>1.8812500000000001</v>
       </c>
       <c r="I5" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28064,11 +28162,11 @@
       </c>
       <c r="M5" s="71">
         <f t="shared" si="0"/>
-        <v>385080</v>
+        <v>564375</v>
       </c>
       <c r="N5" s="165">
         <f t="shared" si="0"/>
-        <v>1.2836000000000001</v>
+        <v>1.8812500000000001</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -28092,11 +28190,11 @@
       </c>
       <c r="G6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>233472</v>
+        <v>282853</v>
       </c>
       <c r="H6" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>2.3347199999999999</v>
+        <v>2.8285300000000002</v>
       </c>
       <c r="I6" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28116,11 +28214,11 @@
       </c>
       <c r="M6" s="71">
         <f t="shared" si="0"/>
-        <v>233472</v>
+        <v>282853</v>
       </c>
       <c r="N6" s="165">
         <f t="shared" si="0"/>
-        <v>2.3347199999999999</v>
+        <v>2.8285300000000002</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -28144,11 +28242,11 @@
       </c>
       <c r="G7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-92015</v>
+        <v>-140705</v>
       </c>
       <c r="H7" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-0.30671666666666669</v>
+        <v>-0.46901666666666658</v>
       </c>
       <c r="I7" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28168,11 +28266,11 @@
       </c>
       <c r="M7" s="71">
         <f t="shared" si="0"/>
-        <v>-92015</v>
+        <v>-140705</v>
       </c>
       <c r="N7" s="165">
         <f t="shared" si="0"/>
-        <v>-0.30671666666666669</v>
+        <v>-0.46901666666666658</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -28196,11 +28294,11 @@
       </c>
       <c r="G8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>376935</v>
+        <v>416810</v>
       </c>
       <c r="H8" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>2.5129000000000001</v>
+        <v>2.7787333333333333</v>
       </c>
       <c r="I8" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28220,11 +28318,11 @@
       </c>
       <c r="M8" s="71">
         <f t="shared" si="0"/>
-        <v>376935</v>
+        <v>416810</v>
       </c>
       <c r="N8" s="165">
         <f t="shared" si="0"/>
-        <v>2.5129000000000001</v>
+        <v>2.7787333333333333</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -28248,11 +28346,11 @@
       </c>
       <c r="G9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>154827</v>
+        <v>66341</v>
       </c>
       <c r="H9" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>2.5804499999999999</v>
+        <v>1.1056833333333334</v>
       </c>
       <c r="I9" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28272,11 +28370,11 @@
       </c>
       <c r="M9" s="71">
         <f t="shared" si="0"/>
-        <v>154827</v>
+        <v>66341</v>
       </c>
       <c r="N9" s="165">
         <f t="shared" si="0"/>
-        <v>2.5804499999999999</v>
+        <v>1.1056833333333334</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -28404,11 +28502,11 @@
       </c>
       <c r="G12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-11570</v>
+        <v>-14872</v>
       </c>
       <c r="H12" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-0.1157</v>
+        <v>-0.14871999999999999</v>
       </c>
       <c r="I12" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28428,11 +28526,11 @@
       </c>
       <c r="M12" s="71">
         <f t="shared" si="0"/>
-        <v>-11570</v>
+        <v>-14872</v>
       </c>
       <c r="N12" s="165">
         <f t="shared" si="0"/>
-        <v>-0.1157</v>
+        <v>-0.14871999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -28456,11 +28554,11 @@
       </c>
       <c r="G13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>65921</v>
+        <v>82977</v>
       </c>
       <c r="H13" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.26368399999999997</v>
+        <v>0.33190800000000004</v>
       </c>
       <c r="I13" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28480,11 +28578,11 @@
       </c>
       <c r="M13" s="71">
         <f t="shared" si="0"/>
-        <v>65921</v>
+        <v>82977</v>
       </c>
       <c r="N13" s="165">
         <f t="shared" si="0"/>
-        <v>0.26368399999999997</v>
+        <v>0.33190800000000004</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -28508,11 +28606,11 @@
       </c>
       <c r="G14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-1980</v>
+        <v>-12790</v>
       </c>
       <c r="H14" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-1.9800000000000002E-2</v>
+        <v>-0.12790000000000001</v>
       </c>
       <c r="I14" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28532,11 +28630,11 @@
       </c>
       <c r="M14" s="71">
         <f t="shared" si="0"/>
-        <v>-1980</v>
+        <v>-12790</v>
       </c>
       <c r="N14" s="165">
         <f t="shared" si="0"/>
-        <v>-1.9800000000000002E-2</v>
+        <v>-0.12790000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -28560,11 +28658,11 @@
       </c>
       <c r="G15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>94772</v>
+        <v>120524</v>
       </c>
       <c r="H15" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.43078181818181815</v>
+        <v>0.54783636363636357</v>
       </c>
       <c r="I15" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28584,11 +28682,11 @@
       </c>
       <c r="M15" s="71">
         <f t="shared" si="0"/>
-        <v>94772</v>
+        <v>120524</v>
       </c>
       <c r="N15" s="165">
         <f t="shared" si="0"/>
-        <v>0.43078181818181815</v>
+        <v>0.54783636363636357</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -28612,11 +28710,11 @@
       </c>
       <c r="G16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>678723</v>
+        <v>730873</v>
       </c>
       <c r="H16" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>2.7148919999999999</v>
+        <v>2.923492</v>
       </c>
       <c r="I16" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28636,11 +28734,11 @@
       </c>
       <c r="M16" s="71">
         <f t="shared" si="0"/>
-        <v>678723</v>
+        <v>730873</v>
       </c>
       <c r="N16" s="165">
         <f t="shared" si="0"/>
-        <v>2.7148919999999999</v>
+        <v>2.923492</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -28664,11 +28762,11 @@
       </c>
       <c r="G17" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>376524</v>
+        <v>493824</v>
       </c>
       <c r="H17" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.94130999999999998</v>
+        <v>1.2345600000000001</v>
       </c>
       <c r="I17" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28688,11 +28786,11 @@
       </c>
       <c r="M17" s="71">
         <f t="shared" si="0"/>
-        <v>376524</v>
+        <v>493824</v>
       </c>
       <c r="N17" s="165">
         <f t="shared" si="0"/>
-        <v>0.94130999999999998</v>
+        <v>1.2345600000000001</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -28872,11 +28970,11 @@
       </c>
       <c r="G21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>731166</v>
+        <v>688166</v>
       </c>
       <c r="H21" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>4.8744399999999999</v>
+        <v>4.5877733333333328</v>
       </c>
       <c r="I21" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28896,11 +28994,11 @@
       </c>
       <c r="M21" s="71">
         <f t="shared" si="0"/>
-        <v>731166</v>
+        <v>688166</v>
       </c>
       <c r="N21" s="165">
         <f t="shared" si="0"/>
-        <v>4.8744399999999999</v>
+        <v>4.5877733333333328</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -28924,11 +29022,11 @@
       </c>
       <c r="G22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>23714</v>
+        <v>-24031</v>
       </c>
       <c r="H22" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.21558181818181815</v>
+        <v>-0.21846363636363639</v>
       </c>
       <c r="I22" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -28948,11 +29046,11 @@
       </c>
       <c r="M22" s="71">
         <f t="shared" si="0"/>
-        <v>23714</v>
+        <v>-24031</v>
       </c>
       <c r="N22" s="165">
         <f t="shared" si="0"/>
-        <v>0.21558181818181815</v>
+        <v>-0.21846363636363639</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -28976,11 +29074,11 @@
       </c>
       <c r="G23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-294779</v>
+        <v>-356631</v>
       </c>
       <c r="H23" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-1.2816478260869566</v>
+        <v>-1.5505695652173914</v>
       </c>
       <c r="I23" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29000,11 +29098,11 @@
       </c>
       <c r="M23" s="71">
         <f t="shared" si="0"/>
-        <v>-294779</v>
+        <v>-356631</v>
       </c>
       <c r="N23" s="165">
         <f t="shared" si="0"/>
-        <v>-1.2816478260869566</v>
+        <v>-1.5505695652173914</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -29026,11 +29124,11 @@
       </c>
       <c r="G24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>159162</v>
+        <v>138037</v>
       </c>
       <c r="H24" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>7.9581</v>
+        <v>6.9018499999999996</v>
       </c>
       <c r="I24" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29050,11 +29148,11 @@
       </c>
       <c r="M24" s="71">
         <f t="shared" ref="M24" si="1">G24+I24+K24</f>
-        <v>159162</v>
+        <v>138037</v>
       </c>
       <c r="N24" s="165">
         <f t="shared" ref="N24" si="2">H24+J24+L24</f>
-        <v>7.9581</v>
+        <v>6.9018499999999996</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -29076,11 +29174,11 @@
       </c>
       <c r="G25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-95559</v>
+        <v>-91206</v>
       </c>
       <c r="H25" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-1.9111800000000001</v>
+        <v>-1.82412</v>
       </c>
       <c r="I25" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29100,11 +29198,11 @@
       </c>
       <c r="M25" s="71">
         <f t="shared" si="0"/>
-        <v>-95559</v>
+        <v>-91206</v>
       </c>
       <c r="N25" s="165">
         <f t="shared" si="0"/>
-        <v>-1.9111800000000001</v>
+        <v>-1.82412</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -29128,11 +29226,11 @@
       </c>
       <c r="G26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1961800</v>
+        <v>2229800</v>
       </c>
       <c r="H26" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>3.9236</v>
+        <v>4.4596</v>
       </c>
       <c r="I26" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29152,11 +29250,11 @@
       </c>
       <c r="M26" s="71">
         <f t="shared" si="0"/>
-        <v>1961800</v>
+        <v>2229800</v>
       </c>
       <c r="N26" s="165">
         <f t="shared" si="0"/>
-        <v>3.9236</v>
+        <v>4.4596</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -29231,11 +29329,11 @@
       </c>
       <c r="G28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-37539</v>
+        <v>-91075</v>
       </c>
       <c r="H28" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-0.75078</v>
+        <v>-1.8214999999999999</v>
       </c>
       <c r="I28" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29255,11 +29353,11 @@
       </c>
       <c r="M28" s="71">
         <f t="shared" ref="M28" si="3">G28+I28+K28</f>
-        <v>-37539</v>
+        <v>-91075</v>
       </c>
       <c r="N28" s="165">
         <f t="shared" ref="N28" si="4">H28+J28+L28</f>
-        <v>-0.75078</v>
+        <v>-1.8214999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -29335,11 +29433,11 @@
       </c>
       <c r="G30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>177902</v>
+        <v>31502</v>
       </c>
       <c r="H30" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.35580400000000001</v>
+        <v>6.3004000000000004E-2</v>
       </c>
       <c r="I30" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29359,11 +29457,11 @@
       </c>
       <c r="M30" s="71">
         <f t="shared" si="0"/>
-        <v>177902</v>
+        <v>31502</v>
       </c>
       <c r="N30" s="165">
         <f t="shared" si="0"/>
-        <v>0.35580400000000001</v>
+        <v>6.3004000000000004E-2</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -29439,11 +29537,11 @@
       </c>
       <c r="G32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>347883</v>
+        <v>341988</v>
       </c>
       <c r="H32" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>8.6970749999999999</v>
+        <v>8.5496999999999996</v>
       </c>
       <c r="I32" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29463,11 +29561,11 @@
       </c>
       <c r="M32" s="71">
         <f t="shared" si="0"/>
-        <v>347883</v>
+        <v>341988</v>
       </c>
       <c r="N32" s="165">
         <f t="shared" si="0"/>
-        <v>8.6970749999999999</v>
+        <v>8.5496999999999996</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -29491,11 +29589,11 @@
       </c>
       <c r="G33" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>300365</v>
+        <v>209201</v>
       </c>
       <c r="H33" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.75091249999999998</v>
+        <v>0.52300250000000004</v>
       </c>
       <c r="I33" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29515,11 +29613,11 @@
       </c>
       <c r="M33" s="71">
         <f t="shared" si="0"/>
-        <v>300365</v>
+        <v>209201</v>
       </c>
       <c r="N33" s="165">
         <f t="shared" si="0"/>
-        <v>0.75091249999999998</v>
+        <v>0.52300250000000004</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -29543,11 +29641,11 @@
       </c>
       <c r="G34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>23642</v>
+        <v>-41268</v>
       </c>
       <c r="H34" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.23641999999999999</v>
+        <v>-0.41267999999999999</v>
       </c>
       <c r="I34" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29567,11 +29665,11 @@
       </c>
       <c r="M34" s="71">
         <f t="shared" si="0"/>
-        <v>23642</v>
+        <v>-41268</v>
       </c>
       <c r="N34" s="165">
         <f t="shared" si="0"/>
-        <v>0.23641999999999999</v>
+        <v>-0.41267999999999999</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -29697,11 +29795,11 @@
       </c>
       <c r="G37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>467721</v>
+        <v>225121</v>
       </c>
       <c r="H37" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1.55907</v>
+        <v>0.75040333333333331</v>
       </c>
       <c r="I37" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29721,11 +29819,11 @@
       </c>
       <c r="M37" s="71">
         <f t="shared" si="0"/>
-        <v>467721</v>
+        <v>225121</v>
       </c>
       <c r="N37" s="165">
         <f t="shared" si="0"/>
-        <v>1.55907</v>
+        <v>0.75040333333333331</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -29747,11 +29845,11 @@
       </c>
       <c r="G38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-225524</v>
+        <v>-217860</v>
       </c>
       <c r="H38" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-22.552399999999999</v>
+        <v>-21.786000000000001</v>
       </c>
       <c r="I38" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29771,11 +29869,11 @@
       </c>
       <c r="M38" s="71">
         <f t="shared" si="0"/>
-        <v>-225524</v>
+        <v>-217860</v>
       </c>
       <c r="N38" s="165">
         <f t="shared" si="0"/>
-        <v>-22.552399999999999</v>
+        <v>-21.786000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -29851,11 +29949,11 @@
       </c>
       <c r="G40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-373613</v>
+        <v>-568413</v>
       </c>
       <c r="H40" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-3.7361300000000002</v>
+        <v>-5.6841299999999997</v>
       </c>
       <c r="I40" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29875,11 +29973,11 @@
       </c>
       <c r="M40" s="71">
         <f t="shared" si="0"/>
-        <v>-373613</v>
+        <v>-568413</v>
       </c>
       <c r="N40" s="165">
         <f t="shared" si="0"/>
-        <v>-3.7361300000000002</v>
+        <v>-5.6841299999999997</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -29903,11 +30001,11 @@
       </c>
       <c r="G41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>591786</v>
+        <v>544786</v>
       </c>
       <c r="H41" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>11.83572</v>
+        <v>10.895720000000001</v>
       </c>
       <c r="I41" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29927,11 +30025,11 @@
       </c>
       <c r="M41" s="71">
         <f t="shared" ref="M41" si="5">G41+I41+K41</f>
-        <v>591786</v>
+        <v>544786</v>
       </c>
       <c r="N41" s="165">
         <f t="shared" ref="N41" si="6">H41+J41+L41</f>
-        <v>11.83572</v>
+        <v>10.895720000000001</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -29953,11 +30051,11 @@
       </c>
       <c r="G42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-55185</v>
+        <v>-46085</v>
       </c>
       <c r="H42" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-1.1036999999999999</v>
+        <v>-0.92169999999999996</v>
       </c>
       <c r="I42" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -29977,11 +30075,11 @@
       </c>
       <c r="M42" s="71">
         <f t="shared" si="0"/>
-        <v>-55185</v>
+        <v>-46085</v>
       </c>
       <c r="N42" s="165">
         <f t="shared" si="0"/>
-        <v>-1.1036999999999999</v>
+        <v>-0.92169999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -30005,11 +30103,11 @@
       </c>
       <c r="G43" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1112739</v>
+        <v>1111205</v>
       </c>
       <c r="H43" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>3.70913</v>
+        <v>3.704016666666667</v>
       </c>
       <c r="I43" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30029,11 +30127,11 @@
       </c>
       <c r="M43" s="71">
         <f t="shared" si="0"/>
-        <v>1112739</v>
+        <v>1111205</v>
       </c>
       <c r="N43" s="165">
         <f t="shared" si="0"/>
-        <v>3.70913</v>
+        <v>3.704016666666667</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -30155,11 +30253,11 @@
       </c>
       <c r="G46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>203653</v>
+        <v>199806</v>
       </c>
       <c r="H46" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.50913249999999999</v>
+        <v>0.49951499999999999</v>
       </c>
       <c r="I46" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30179,11 +30277,11 @@
       </c>
       <c r="M46" s="71">
         <f t="shared" si="0"/>
-        <v>203653</v>
+        <v>199806</v>
       </c>
       <c r="N46" s="165">
         <f t="shared" si="0"/>
-        <v>0.50913249999999999</v>
+        <v>0.49951499999999999</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -30205,11 +30303,11 @@
       </c>
       <c r="G47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-2661565</v>
+        <v>-2531865</v>
       </c>
       <c r="H47" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-2.661565</v>
+        <v>-2.5318649999999998</v>
       </c>
       <c r="I47" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30229,11 +30327,11 @@
       </c>
       <c r="M47" s="71">
         <f t="shared" si="0"/>
-        <v>-2661565</v>
+        <v>-2531865</v>
       </c>
       <c r="N47" s="165">
         <f t="shared" si="0"/>
-        <v>-2.661565</v>
+        <v>-2.5318649999999998</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -30511,11 +30609,11 @@
       </c>
       <c r="G53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>88156</v>
+        <v>94004</v>
       </c>
       <c r="H53" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>0.88156000000000001</v>
+        <v>0.94003999999999999</v>
       </c>
       <c r="I53" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30535,11 +30633,11 @@
       </c>
       <c r="M53" s="71">
         <f t="shared" ref="M53:N54" si="7">G53+I53+K53</f>
-        <v>88156</v>
+        <v>94004</v>
       </c>
       <c r="N53" s="165">
         <f t="shared" si="7"/>
-        <v>0.88156000000000001</v>
+        <v>0.94003999999999999</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -30563,11 +30661,11 @@
       </c>
       <c r="G54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1297423</v>
+        <v>1294523</v>
       </c>
       <c r="H54" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1.297423</v>
+        <v>1.2945230000000001</v>
       </c>
       <c r="I54" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30587,11 +30685,11 @@
       </c>
       <c r="M54" s="71">
         <f t="shared" si="7"/>
-        <v>1297423</v>
+        <v>1294523</v>
       </c>
       <c r="N54" s="165">
         <f t="shared" si="7"/>
-        <v>1.297423</v>
+        <v>1.2945230000000001</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -30603,7 +30701,7 @@
       <c r="F55" s="233"/>
       <c r="G55" s="230">
         <f>SUM(G4:G54)</f>
-        <v>8188120</v>
+        <v>7913998</v>
       </c>
       <c r="H55" s="90"/>
       <c r="I55" s="230">
@@ -30618,7 +30716,7 @@
       <c r="L55" s="109"/>
       <c r="M55" s="230">
         <f>SUM(M4:M54)</f>
-        <v>8188120</v>
+        <v>7913998</v>
       </c>
       <c r="N55" s="234"/>
     </row>
@@ -30683,11 +30781,11 @@
       <c r="F59" s="206"/>
       <c r="G59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>553584</v>
+        <v>554839</v>
       </c>
       <c r="H59" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>1.84528</v>
+        <v>1.8494633333333337</v>
       </c>
       <c r="I59" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'[1]NOV-2026'!$A$4:$ADL$124,MATCH('FY-(26-27)Q3'!$I$2:$J$2,'[1]NOV-2026'!$A$2:$DM$2,0),0),0)</f>
@@ -30707,11 +30805,11 @@
       </c>
       <c r="M59" s="152">
         <f t="shared" ref="M59:N60" si="8">G59+I59+K59</f>
-        <v>553584</v>
+        <v>554839</v>
       </c>
       <c r="N59" s="166">
         <f t="shared" si="8"/>
-        <v>1.84528</v>
+        <v>1.8494633333333337</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -30733,7 +30831,7 @@
       <c r="F60" s="237"/>
       <c r="G60" s="152">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
-        <v>-25994</v>
+        <v>-15894</v>
       </c>
       <c r="H60" s="154">
         <f>IFERROR(VLOOKUP($A$3:$A$116,'OCT-2026'!$A$4:$ADK$120,MATCH('FY-(26-27)Q3'!$G$2:$H$2,'OCT-2026'!$A$2:$DL$2,0),0),0)</f>
@@ -30757,7 +30855,7 @@
       </c>
       <c r="M60" s="152">
         <f t="shared" si="8"/>
-        <v>-25994</v>
+        <v>-15894</v>
       </c>
       <c r="N60" s="166">
         <f t="shared" si="8"/>
@@ -30767,7 +30865,7 @@
     <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G61" s="93">
         <f>SUM(G59:G60)</f>
-        <v>527590</v>
+        <v>538945</v>
       </c>
       <c r="H61" s="94"/>
       <c r="I61" s="93">
@@ -30782,7 +30880,7 @@
       <c r="L61" s="113"/>
       <c r="M61" s="93">
         <f>SUM(M59:M60)</f>
-        <v>527590</v>
+        <v>538945</v>
       </c>
       <c r="N61" s="235"/>
     </row>

</xml_diff>